<commit_message>
docs: cập nhật bảng so sánh Vivoire, đo lại 21/09
Chấm PE bằng AI 0→1 (dựng xong, chưa bật vì thiếu khoá). Flashcard cơ chế
2→1 (bộ giáo viên soạn thay SM-2 — mất lịch ôn ngắt quãng). FAQ và Điều khoản
0→1 (có, nhưng chưa có email liên hệ). Chính sách bảo mật vẫn 0 (dựng rồi gỡ).
Thêm dòng Soạn Flashcard và Soạn thẻ hàng loạt.

Số liệu đo lại: 33 bài, 372 câu, 9 tài khoản, 177 lượt trả lời, 8 bài tự
luận chưa có điểm nào. Vivoire chưa đọc lại, ghi rõ ở Tổng quan.

100 công thức, 0 ô thiếu kết quả.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,15 +34,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="372">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
   <si>
-    <t>Vivoire: đọc từ trang chủ vivoire.app ngày 09/09/2026. Không có tài khoản nên không kiểm được bên trong sản phẩm.</t>
-  </si>
-  <si>
-    <t>FRACILE: đo từ mã nguồn và database production ngày 09/09/2026.</t>
+    <t>Vivoire: đọc từ trang chủ vivoire.app ngày 09/09/2026 — CHƯA đọc lại. Không có tài khoản nên không kiểm được bên trong sản phẩm.</t>
+  </si>
+  <si>
+    <t>FRACILE: đo từ mã nguồn và database production ngày 21/09/2026.</t>
   </si>
   <si>
     <t>Mọi con số ở sheet này TÍNH từ sheet « So sánh chi tiết » — sửa điểm ở đó thì ở đây tự đổi theo.</t>
@@ -129,37 +129,37 @@
     <t>Chưa kiểm chứng được — KHÔNG tính vào trung bình</t>
   </si>
   <si>
-    <t>ĐÃ ĐỔI GÌ SO VỚI BẢN TRƯỚC (cùng ngày 09/09/2026)</t>
-  </si>
-  <si>
-    <t>Gỡ /professeur/copies</t>
-  </si>
-  <si>
-    <t>Route, mục menu, PEGrading.jsx và khoá nav.grading ở cả bốn từ điển. Hai dòng « giáo viên chấm tay » và « chấm bài cho học sinh » đổi từ « CẦN GỠ » sang « Đã gỡ — có chủ đích ».</t>
-  </si>
-  <si>
-    <t>Gỡ ô « Bài cần chấm »</t>
-  </si>
-  <si>
-    <t>Trang chủ giáo viên còn hai ô. Nhãn từng dòng bài nộp đổi « Chờ chấm » → « Chưa chấm ».</t>
-  </si>
-  <si>
-    <t>Sửa một câu trên màn thi</t>
-  </si>
-  <si>
-    <t>« Còn PE chờ giáo viên chấm » → nói thẳng là tự chấm theo thang DELF ở « Kết quả thi ».</t>
-  </si>
-  <si>
-    <t>Việc cần làm #2 thu hẹp</t>
-  </si>
-  <si>
-    <t>Chỉ còn /professeur/oral. Việc #6 đổi từ « chấm 10 bài » sang « báo cho 10 học sinh », vì trong app không còn đường nào để chấm chúng nữa.</t>
-  </si>
-  <si>
-    <t>Điểm số KHÔNG đổi</t>
-  </si>
-  <si>
-    <t>Việc gỡ làm mã khớp với quyết định, nó không thêm năng lực nào cho sản phẩm — nên mọi ô điểm giữ nguyên. Chỉ cột « Trạng thái » đổi.</t>
+    <t>ĐÃ ĐỔI GÌ SO VỚI BẢN 09/09 — bản này đo 21/09/2026</t>
+  </si>
+  <si>
+    <t>Chấm PE bằng AI</t>
+  </si>
+  <si>
+    <t>Đã dựng (Edge Function cham-pe, 38 ca kiểm) nhưng CHƯA BẬT vì thiếu khoá API. Điểm 0 → 1: có mà chưa chạy được đầu-cuối.</t>
+  </si>
+  <si>
+    <t>Flashcard đổi mô hình</t>
+  </si>
+  <si>
+    <t>Thẻ SM-2 sinh từ lỗi sai đã gỡ; nay là bộ do giáo viên soạn, đã chạy thật với tài khoản học sinh. Điểm cơ chế 2 → 1: mất lịch ôn ngắt quãng — đúng chỗ Vivoire mạnh.</t>
+  </si>
+  <si>
+    <t>FAQ + Điều khoản</t>
+  </si>
+  <si>
+    <t>Có từ 21/09. Điểm 0 → 1, chưa lên 2: cả hai chưa có email liên hệ, Điều khoản chưa qua luật sư.</t>
+  </si>
+  <si>
+    <t>Chính sách bảo mật</t>
+  </si>
+  <si>
+    <t>Dựng rồi gỡ cùng ngày theo quyết định chủ dự án. Vẫn 0.</t>
+  </si>
+  <si>
+    <t>Số liệu trôi</t>
+  </si>
+  <si>
+    <t>33 bài (từ 34), 372 câu (từ 373), 9 tài khoản (từ 7). Không phải lỗi — thư viện và người dùng thay đổi; bảng này là ảnh chụp của một ngày.</t>
   </si>
   <si>
     <t>Mục so sánh</t>
@@ -221,36 +221,39 @@
     <t>AI chấm ngữ pháp và cách diễn đạt</t>
   </si>
   <si>
-    <t>CHƯA CÓ. Hàm khung trả về connected:false và KHÔNG nơi nào gọi tới</t>
+    <t>DỰNG XONG 09/09 nhưng CHƯA BẬT — thiếu khoá API. Gợi ý theo đúng các tiêu chí grille, không tự điền; học sinh bấm « dùng số này » mới nhận</t>
+  </si>
+  <si>
+    <t>DỰNG XONG — CHƯA BẬT</t>
+  </si>
+  <si>
+    <t>Edge Function cham-pe trả 503 CHUA_CAU_HINH_KHOA; pe_ai_goi_y = 0 dòng (đo 21/09). Bật: npx supabase secrets set ANTHROPIC_API_KEY=…</t>
+  </si>
+  <si>
+    <t>Bài nói (PO) — ghi âm và nghe lại</t>
+  </si>
+  <si>
+    <t>Có, kèm phản hồi AI</t>
+  </si>
+  <si>
+    <t>Ghi âm + tự nghe lại; CỐ Ý không cho điểm (DELF chấm nói bằng đối thoại)</t>
+  </si>
+  <si>
+    <t>migration 057/058; bucket `bai-noi` private, đường dẫn mang phân quyền theo user_id</t>
+  </si>
+  <si>
+    <t>Bài nói (PO) — AI chấm phát âm</t>
+  </si>
+  <si>
+    <t>Phát âm 82% · Trôi chảy 76% · Từ vựng B1</t>
+  </si>
+  <si>
+    <t>CHƯA CÓ</t>
   </si>
   <si>
     <t>CHƯA DỰNG</t>
   </si>
   <si>
-    <t>gradingEngine.js:215 evaluateEssayWithAI(). grep openai|anthropic|gemini|gpt- = 0 kết quả thật</t>
-  </si>
-  <si>
-    <t>Bài nói (PO) — ghi âm và nghe lại</t>
-  </si>
-  <si>
-    <t>Có, kèm phản hồi AI</t>
-  </si>
-  <si>
-    <t>Ghi âm + tự nghe lại; CỐ Ý không cho điểm (DELF chấm nói bằng đối thoại)</t>
-  </si>
-  <si>
-    <t>migration 057/058; bucket `bai-noi` private, đường dẫn mang phân quyền theo user_id</t>
-  </si>
-  <si>
-    <t>Bài nói (PO) — AI chấm phát âm</t>
-  </si>
-  <si>
-    <t>Phát âm 82% · Trôi chảy 76% · Từ vựng B1</t>
-  </si>
-  <si>
-    <t>CHƯA CÓ</t>
-  </si>
-  <si>
     <t>Không có Edge Function nào gọi mô hình giọng nói</t>
   </si>
   <si>
@@ -275,7 +278,7 @@
     <t>Không thấy nêu trên trang chủ</t>
   </si>
   <si>
-    <t>207/373 câu có lời giải; có màn xếp ưu tiên theo SỐ HỌC SINH từng sai</t>
+    <t>207/372 câu có lời giải; có màn xếp ưu tiên theo SỐ HỌC SINH từng sai</t>
   </si>
   <si>
     <t>migration 069/070; /professeur/loi-giai</t>
@@ -284,13 +287,13 @@
     <t>Neo đáp án vào ngữ liệu (chỉ ra CHỖ chứa câu trả lời)</t>
   </si>
   <si>
-    <t>Dựng xong cả hai đầu (đặt neo + hiển thị), nhưng 0/373 câu có dữ liệu</t>
+    <t>Dựng xong cả hai đầu (đặt neo + hiển thị), nhưng 0/372 câu có dữ liệu</t>
   </si>
   <si>
     <t>DỰNG XONG — CHƯA CÓ DỮ LIỆU</t>
   </si>
   <si>
-    <t>migration 075/076; /professeur/neo; đo 09/09: evidence IS NOT NULL = 0</t>
+    <t>migration 075/076; /professeur/neo; đo 21/09: evidence IS NOT NULL = 0</t>
   </si>
   <si>
     <t>Đề thi thử đúng cấu trúc DELF</t>
@@ -374,10 +377,10 @@
     <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
   </si>
   <si>
-    <t>34 bài (ĐẾM THẬT trên production)</t>
-  </si>
-  <si>
-    <t>select count(*) from exercises = 34, đo 09/09/2026</t>
+    <t>33 bài (ĐẾM THẬT trên production)</t>
+  </si>
+  <si>
+    <t>select count(*) from exercises = 33, đo 21/09/2026 (09/09 là 34)</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -386,10 +389,10 @@
     <t>Không công bố</t>
   </si>
   <si>
-    <t>373 câu, 7 dạng (qcm, fill, conj, vf, tableau, order, tự luận)</t>
-  </si>
-  <si>
-    <t>select count(*) from questions = 373</t>
+    <t>372 câu, 7 dạng (qcm, fill, conj, vf, tableau, order, tự luận)</t>
+  </si>
+  <si>
+    <t>select count(*) from questions = 372, đo 21/09/2026</t>
   </si>
   <si>
     <t>Từ điển Pháp–Việt</t>
@@ -434,37 +437,40 @@
     <t>Builder.jsx — trình nhập JSON</t>
   </si>
   <si>
-    <t>Thẻ ghi nhớ — cơ chế</t>
+    <t>Flashcard — cơ chế</t>
   </si>
   <si>
     <t>Flashcard + 3 game mỗi ngày, « ôn từ đúng lúc sắp quên »</t>
   </si>
   <si>
-    <t>SM-2 đầy đủ, 4 nút SRS; thẻ SINH TỰ ĐỘNG TỪ CÂU LÀM SAI, không nhập tay</t>
-  </si>
-  <si>
-    <t>shared/sm2.js thuần, 90 ca kiểm; migration 063–066, 073/074</t>
-  </si>
-  <si>
-    <t>Thẻ ghi nhớ — quy mô</t>
+    <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D. KHÔNG còn lịch ôn ngắt quãng — SM-2 và thẻ sinh từ lỗi sai đã gỡ 09/09. Học sinh không tự tạo thẻ</t>
+  </si>
+  <si>
+    <t>Đang chạy — chạy thật 21/09</t>
+  </si>
+  <si>
+    <t>migration 085–088; học sinh mở bằng tài khoản thật thấy đủ 8 thẻ, lật được</t>
+  </si>
+  <si>
+    <t>Flashcard — quy mô</t>
   </si>
   <si>
     <t>Không công bố số thẻ</t>
   </si>
   <si>
-    <t>37 thẻ đã sinh</t>
-  </si>
-  <si>
-    <t>select count(*) from cards = 37</t>
-  </si>
-  <si>
-    <t>Mặt sau thẻ là lời giải thích, không phải đáp án trần</t>
-  </si>
-  <si>
-    <t>Có — và viết lời giải mới sẽ KÉO THEO thẻ đã sinh</t>
-  </si>
-  <si>
-    <t>RPC luu_loi_giai trả về số thẻ vừa làm mới</t>
+    <t>1 bộ · 8 thẻ, chỉ kỹ năng Nghe; Đọc/Viết/Nói còn trống</t>
+  </si>
+  <si>
+    <t>the_bo = 1, the_bo_the = 8 (đo 21/09). 37 thẻ SM-2 cũ vẫn trong bảng cards, không màn nào mở</t>
+  </si>
+  <si>
+    <t>Soạn thẻ hàng loạt</t>
+  </si>
+  <si>
+    <t>Dán nhiều dòng « mặt trước | mặt sau | phiên âm »; dòng hỏng được gọi tên kèm số dòng</t>
+  </si>
+  <si>
+    <t>shared/boTheGiaoVien.js bocDong(); chủ dự án tạo bộ thử qua giao diện 12/09</t>
   </si>
   <si>
     <t>Chuỗi ngày học</t>
@@ -536,6 +542,15 @@
     <t>Builder.jsx; exerciseStore.js</t>
   </si>
   <si>
+    <t>Soạn Flashcard</t>
+  </si>
+  <si>
+    <t>Có — /professeur/bo-the: tạo bộ, nhập hàng loạt, nháp ↔ công khai, xoá (thẻ đi theo)</t>
+  </si>
+  <si>
+    <t>RLS chỉ giáo viên ghi; đo bằng claim giả: HS thấy 8 thẻ, sửa 0, xoá 0</t>
+  </si>
+  <si>
     <t>Giao bài theo kỹ năng và cấp độ</t>
   </si>
   <si>
@@ -584,10 +599,10 @@
     <t>Số tài khoản đang có</t>
   </si>
   <si>
-    <t>7 người dùng (gồm cả tài khoản thử)</t>
-  </si>
-  <si>
-    <t>select count(*) from profiles = 7</t>
+    <t>9 người dùng (gồm cả tài khoản thử)</t>
+  </si>
+  <si>
+    <t>select count(*) from profiles = 9, đo 21/09/2026</t>
   </si>
   <si>
     <t>Web</t>
@@ -638,19 +653,34 @@
     <t>Câu hỏi thường gặp (FAQ)</t>
   </si>
   <si>
-    <t>CHẶN VIỆC THU TIỀN</t>
-  </si>
-  <si>
-    <t>Chân trang LandingPage.jsx đã ghi rõ điều này</t>
+    <t>Có từ 21/09 — 9 câu, mỗi câu đối chiếu với mã nguồn. Chưa có email liên hệ</t>
+  </si>
+  <si>
+    <t>Có — thiếu email liên hệ</t>
+  </si>
+  <si>
+    <t>/faq; EMAIL_LIEN_HE trong TrangPhapLy.jsx đang trống</t>
   </si>
   <si>
     <t>Điều khoản sử dụng</t>
   </si>
   <si>
-    <t>Chính sách bảo mật</t>
-  </si>
-  <si>
-    <t>Đây là lý do form tư vấn bị gỡ khỏi trang giới thiệu</t>
+    <t>Có từ 21/09 — ghi rõ điểm thi thử không phải điểm DELF chính thức; không tự đặt chính sách hoàn tiền</t>
+  </si>
+  <si>
+    <t>Có — bản nháp, chưa qua luật sư</t>
+  </si>
+  <si>
+    <t>/dieu-khoan</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ — dựng xong 21/09 rồi gỡ cùng ngày theo quyết định chủ dự án</t>
+  </si>
+  <si>
+    <t>ĐÃ GỠ — có chủ đích</t>
+  </si>
+  <si>
+    <t>Nội dung còn trong git. Khi vắng trang này, form tư vấn không nên bật lại</t>
   </si>
   <si>
     <t>Đội ngũ công khai</t>
@@ -689,7 +719,7 @@
     <t>TÀI KHOẢN GIÁO VIÊN — giữ để KIỂM SOÁT, không để CHẤM BÀI</t>
   </si>
   <si>
-    <t>Quyết định của chủ dự án ngày 09/09/2026: giữ tài khoản giáo viên để quản lý số lượng học sinh và quyền truy cập; bỏ hoàn toàn việc giáo viên chấm bài. Học sinh tự chấm theo grille DELF; AI chấm là hướng đi, chưa dựng.</t>
+    <t>Quyết định của chủ dự án ngày 09/09/2026: giữ tài khoản giáo viên để quản lý số lượng học sinh và quyền truy cập; bỏ hoàn toàn việc giáo viên chấm bài. Học sinh tự chấm theo grille DELF; AI gợi ý chấm đã dựng nhưng chưa bật (thiếu khoá API).</t>
   </si>
   <si>
     <t>Quyền / màn hình</t>
@@ -779,6 +809,12 @@
     <t>/professeur/carnet</t>
   </si>
   <si>
+    <t>/professeur/bo-the</t>
+  </si>
+  <si>
+    <t>Dựng 09/09. Học sinh không còn tự tạo thẻ — chỉ giáo viên soạn, chặn ở database bằng RLS chứ không chỉ ẩn nút.</t>
+  </si>
+  <si>
     <t>Xem đăng ký tư vấn</t>
   </si>
   <si>
@@ -839,9 +875,9 @@
     <t>MỘT CÂU PHẢI NÓI THẲNG</t>
   </si>
   <si>
-    <t xml:space="preserve">Bỏ giáo viên chấm bài KHÔNG tự động thành « AI chấm ». Hôm nay sản phẩm không có AI nào: evaluateEssayWithAI() trả về connected:false và không nơi nào trong mã gọi tới nó.
-Việc gỡ đã làm xong TRƯỚC khi AI được dựng. Nên kể từ 09/09/2026, bài viết của học sinh chỉ còn MỘT đường duy nhất: tự chấm theo grille DELF ở màn « Kết quả thi ». Đó là lựa chọn có ý thức của chủ dự án, không phải hệ quả tình cờ — nhưng nó có hạn dùng: khoảng trống này kéo dài đúng bằng thời gian tới khi việc số 4 trong sheet « Việc cần làm » (nối AI vào grille) xong.
-Và 10 bài tự luận đã nộp trước đó giờ KHÔNG còn đường nào để được chấm trong app. Nếu có học sinh đang chờ, im lặng là câu trả lời tệ nhất trong các khả năng.</t>
+    <t xml:space="preserve">Bỏ giáo viên chấm bài chưa tự động thành « AI chấm ». Chấm AI đã DỰNG (Edge Function cham-pe) nhưng CHƯA CHẠY: thiếu khoá ANTHROPIC_API_KEY, gọi vào nhận 503 CHUA_CAU_HINH_KHOA, và bảng gợi ý có 0 dòng (đo 21/09).
+Nên kể từ 09/09, bài viết của học sinh chỉ còn MỘT đường: tự chấm theo grille DELF. Khoảng trống này kéo dài đúng bằng thời gian tới khi đặt khoá — việc số 1 trong sheet « Việc cần làm ».
+Và 8 bài tự luận đã nộp chưa có điểm nào — không điểm giáo viên, không điểm tự chấm. Chưa ai báo gì cho người viết chúng.</t>
   </si>
   <si>
     <t>SỐ LIỆU ĐO THẬT — không con số nào ở đây là ước lượng</t>
@@ -865,7 +901,7 @@
     <t>select count(*) from exercises</t>
   </si>
   <si>
-    <t>09/09/2026</t>
+    <t>21/09/2026</t>
   </si>
   <si>
     <t>Câu hỏi</t>
@@ -892,7 +928,19 @@
     <t>select count(*) from exams</t>
   </si>
   <si>
-    <t>Thẻ ghi nhớ đã sinh</t>
+    <t>Bộ Flashcard</t>
+  </si>
+  <si>
+    <t>select count(*) from the_bo</t>
+  </si>
+  <si>
+    <t>Thẻ trong các bộ</t>
+  </si>
+  <si>
+    <t>select count(*) from the_bo_the</t>
+  </si>
+  <si>
+    <t>Thẻ SM-2 cũ (không màn nào mở)</t>
   </si>
   <si>
     <t>select count(*) from cards</t>
@@ -910,16 +958,16 @@
     <t>select count(*) from profiles</t>
   </si>
   <si>
-    <t>Bài tự luận CHƯA ai chấm</t>
-  </si>
-  <si>
-    <t>đếm câu tự luận chưa có điểm</t>
-  </si>
-  <si>
-    <t>Hàm gọi mô hình AI trong mã</t>
-  </si>
-  <si>
-    <t>grep openai|anthropic|gemini|gpt- trên src/ và supabase/</t>
+    <t>Bài tự luận CHƯA có điểm nào</t>
+  </si>
+  <si>
+    <t>câu open: score is null AND self_score is null</t>
+  </si>
+  <si>
+    <t>Gợi ý chấm AI đã sinh</t>
+  </si>
+  <si>
+    <t>select count(*) from pe_ai_goi_y — khoá API chưa đặt</t>
   </si>
   <si>
     <t>Tỷ lệ câu có lời giải</t>
@@ -1021,22 +1069,67 @@
     <t>Công sức</t>
   </si>
   <si>
-    <t>Dựng 3 trang: FAQ · Điều khoản sử dụng · Chính sách bảo mật</t>
-  </si>
-  <si>
-    <t>Ô duy nhất trong cả bảng có thể xoá sạch trong một buổi, và nó đang CHẶN việc thu tiền. Vivoire có đủ ba. Cũng là điều kiện để bật lại form tư vấn.</t>
-  </si>
-  <si>
-    <t>3 trang tĩnh + 3 route</t>
-  </si>
-  <si>
-    <t>1 buổi</t>
-  </si>
-  <si>
-    <t>Quyết số phận /professeur/oral — màn nghe bài nói</t>
-  </si>
-  <si>
-    <t>Nửa kia của việc này đã XONG 09/09: /professeur/copies và ô « Bài cần chấm » đã gỡ. Còn lại một mình màn nghe bài nói, và nó là ranh giới thật: màn đó KHÔNG cho điểm, chỉ nghe rồi nhắn nhận xét. Bỏ hẳn vai chấm thì nên gỡ; giữ vai kèm cặp thì giữ. Đây là câu hỏi về việc bạn muốn là gì với học sinh, không phải câu hỏi kỹ thuật.</t>
+    <t>Đặt khoá API để bật chấm PE bằng AI</t>
+  </si>
+  <si>
+    <t>Việc rẻ nhất trong danh sách có tác động lớn nhất: mọi thứ đã dựng và đã kiểm, chỉ thiếu một khoá. Chưa đặt thì bài viết chỉ có một đường là tự chấm.</t>
+  </si>
+  <si>
+    <t>npx supabase secrets set ANTHROPIC_API_KEY=sk-ant-…</t>
+  </si>
+  <si>
+    <t>5 phút</t>
+  </si>
+  <si>
+    <t>Điền email liên hệ cho FAQ và Điều khoản</t>
+  </si>
+  <si>
+    <t>Cả hai trang đang tự hiện dòng cảnh báo vàng « chưa công bố email liên hệ ». Một trang pháp lý không có chỗ liên hệ là điểm 1 chứ không phải 2 trong bảng này.</t>
+  </si>
+  <si>
+    <t>EMAIL_LIEN_HE trong src/screens/public/TrangPhapLy.jsx</t>
+  </si>
+  <si>
+    <t>2 phút</t>
+  </si>
+  <si>
+    <t>Báo cho học sinh có 8 bài tự luận chưa có điểm</t>
+  </si>
+  <si>
+    <t>Không có điểm giáo viên lẫn điểm tự chấm. Đường thông báo có sẵn; có thể chỉ họ sang màn tự chấm, và — khi khoá API đã đặt — sang nút xin gợi ý.</t>
+  </si>
+  <si>
+    <t>Đường thông báo đang có</t>
+  </si>
+  <si>
+    <t>30 phút</t>
+  </si>
+  <si>
+    <t>Soạn thêm bộ Flashcard cho Đọc · Viết · Nói</t>
+  </si>
+  <si>
+    <t>Hiện chỉ 1 bộ, chỉ kỹ năng Nghe. Học sinh mở ba tab còn lại đều thấy trống. Nhập hàng loạt nên một bộ 20 thẻ là một lần dán.</t>
+  </si>
+  <si>
+    <t>/professeur/bo-the — chỉ nhập liệu</t>
+  </si>
+  <si>
+    <t>1–2 giờ</t>
+  </si>
+  <si>
+    <t>Đặt neo cho 5–10 câu đọc hiểu</t>
+  </si>
+  <si>
+    <t>Vẫn 0 dòng sau 12 ngày. Tính năng mạnh nhất Vivoire không có, và chưa ai từng thấy nó chạy.</t>
+  </si>
+  <si>
+    <t>/professeur/neo — chỉ nhập liệu</t>
+  </si>
+  <si>
+    <t>Quyết số phận /professeur/oral</t>
+  </si>
+  <si>
+    <t>Màn nghe bài nói không cho điểm, chỉ nghe và nhắn nhận xét. Giữ vai kèm cặp thì giữ, bỏ hẳn thì gỡ.</t>
   </si>
   <si>
     <t>App.jsx; BaiNoiGiaoVien.jsx; navItems.js</t>
@@ -1045,67 +1138,19 @@
     <t>1 buổi, sau khi quyết</t>
   </si>
   <si>
-    <t>Đặt neo cho 5–10 câu đọc hiểu</t>
-  </si>
-  <si>
-    <t>Tính năng mạnh nhất mà Vivoire không có, và hiện có 0 dòng dữ liệu — chưa ai từng thấy nó chạy. Không phải viết thêm dòng mã nào.</t>
-  </si>
-  <si>
-    <t>/professeur/neo — chỉ nhập liệu</t>
-  </si>
-  <si>
-    <t>1–2 giờ</t>
-  </si>
-  <si>
-    <t>Nối AI vào GRILLE, không nối vào một con số</t>
-  </si>
-  <si>
-    <t>Đây là chỗ AI thật sự thêm giá trị mà không phá thứ đang có. Vivoire trả về « 82% phát âm ». Nếu FRACILE trả về 6 tiêu chí DELF kèm trích dẫn từ chính bài viết thì đó là sản phẩm khác hẳn, không phải bản sao rẻ hơn.</t>
-  </si>
-  <si>
-    <t>Edge Function mới + gradingEngine.js:215 (khung đã có, chú thích đã ghi sẵn 5 bước)</t>
-  </si>
-  <si>
-    <t>2–3 ngày</t>
-  </si>
-  <si>
-    <t>Để điểm AI ở dạng ĐỀ XUẤT, học sinh vẫn tự đối chiếu grille</t>
-  </si>
-  <si>
-    <t>Chú thích trong gradingEngine.js đã viết sẵn: « điểm số của một con người phải do một con người ký ». Bỏ giáo viên rồi thì người ký là chính học sinh — nên AI gợi ý, học sinh chốt, và cả hai con số cùng hiện.</t>
-  </si>
-  <si>
-    <t>PESelfEvaluation.jsx</t>
-  </si>
-  <si>
-    <t>1 ngày</t>
-  </si>
-  <si>
-    <t>Nói cho 10 học sinh có bài tự luận đang treo biết chuyện gì đã xảy ra</t>
-  </si>
-  <si>
-    <t>10 bài đã nộp, chưa bài nào được chấm — và từ 09/09 KHÔNG còn đường nào trong app để chấm chúng. Việc gỡ màn chấm là đúng ý bạn, nhưng nó biến 10 người đang chờ thành 10 người sẽ chờ mãi mà không được báo. Đường thông báo đã có sẵn (chuông + dấu đã đọc), nên đây là việc viết một câu, không phải việc dựng gì.</t>
-  </si>
-  <si>
-    <t>Đường thông báo đang có; submissions</t>
-  </si>
-  <si>
-    <t>30 phút</t>
-  </si>
-  <si>
-    <t>Bổ sung ảnh màn hình thật cho trang giới thiệu</t>
-  </si>
-  <si>
-    <t>Hero đang là khung xám nói « chỗ dành cho ảnh ». Vivoire dùng ảnh minh hoạ ở đúng chỗ mà FRACILE có thể dùng ảnh thật.</t>
-  </si>
-  <si>
-    <t>LandingPage.jsx</t>
+    <t>Cân nhắc dựng lại Chính sách bảo mật trước khi thu tiền nhiều</t>
+  </si>
+  <si>
+    <t>Đã gỡ theo quyết định 21/09; nội dung còn trong git. Thiếu nó thì form tư vấn không nên bật lại, và ô này là ô duy nhất trong nhóm pháp lý còn 0 điểm.</t>
+  </si>
+  <si>
+    <t>Lấy TrangBaoMat từ commit cũ + route /bao-mat</t>
   </si>
   <si>
     <t>Cân nhắc KHÔNG đuổi theo: từ điển, podcast, PvP, app mobile</t>
   </si>
   <si>
-    <t>Bốn ô Vivoire hơn tuyệt đối. Đuổi theo cả bốn với một người là cách chắc chắn để không ô nào xong. Chúng nằm đây để được quyết định BỎ một cách có ý thức, không phải để bị quên.</t>
+    <t>Bốn ô Vivoire hơn tuyệt đối. Đuổi theo cả bốn với một người là cách chắc chắn để không ô nào xong.</t>
   </si>
   <si>
     <t>—</t>
@@ -1777,24 +1822,24 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$50,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A7)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A7)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A7)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A7)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A7)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
-        <v>0.6666666666666666</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F7" s="6">
         <f>IFERROR(E7-D7,"")</f>
-        <v>-1</v>
+        <v>-0.8333333333333334</v>
       </c>
       <c r="G7" s="7" t="str">
         <f>IF(OR(C7&lt;3,F7=""),"quá ít mục",IF(F7&gt;0.25,"FRACILE",IF(F7&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -1806,19 +1851,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$50,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A8)</f>
         <v>6</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A8)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A8)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A8)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A8)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A8)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -1835,19 +1880,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$50,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A9)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A9)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A9)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A9)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A9)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>0.6</v>
       </c>
       <c r="F9" s="6">
@@ -1864,24 +1909,24 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$50,$A10)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A10)</f>
         <v>6</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A10)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
         <v>3</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A10)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A10)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A10)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A10)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
-        <v>1.3333333333333333</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <v>1</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>-0.6666666666666667</v>
+        <v>-1</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -1893,19 +1938,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$50,$A11)</f>
-        <v>10</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A11)</f>
+        <v>11</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A11)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A11)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A11)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A11)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A11)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F11" s="6">
@@ -1922,19 +1967,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$50,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A12)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A12)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A12)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A12)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A12)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F12" s="6">
@@ -1951,24 +1996,24 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$50,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A13)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A13)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A13)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A13)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$50=$A13)*('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
-        <v>0.6</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <v>1</v>
       </c>
       <c r="F13" s="6">
         <f>IFERROR(E13-D13,"")</f>
-        <v>-1.2000000000000002</v>
+        <v>-0.8</v>
       </c>
       <c r="G13" s="7" t="str">
         <f>IF(OR(C13&lt;3,F13=""),"quá ít mục",IF(F13&gt;0.25,"FRACILE",IF(F13&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -1981,23 +2026,23 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
         <v>30</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$50)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
         <v>1.8666666666666667</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$50)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$50&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$50&lt;&gt;"")),"")</f>
-        <v>0.8333333333333334</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <v>0.9</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-1.0333333333333332</v>
+        <v>-0.9666666666666667</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2080,7 +2125,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
         <v>31</v>
       </c>
@@ -2093,7 +2138,7 @@
       <c r="F28" s="18"/>
       <c r="G28" s="18"/>
     </row>
-    <row r="29" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
         <v>33</v>
       </c>
@@ -2106,7 +2151,7 @@
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
     </row>
-    <row r="30" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
         <v>35</v>
       </c>
@@ -2119,7 +2164,7 @@
       <c r="F30" s="18"/>
       <c r="G30" s="18"/>
     </row>
-    <row r="31" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
         <v>37</v>
       </c>
@@ -2132,7 +2177,7 @@
       <c r="F31" s="18"/>
       <c r="G31" s="18"/>
     </row>
-    <row r="32" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
         <v>39</v>
       </c>
@@ -2161,7 +2206,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2263,32 +2308,32 @@
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="34">
-        <v>2</v>
-      </c>
-      <c r="E4" s="33" t="s">
+      <c r="D4" s="22">
+        <v>2</v>
+      </c>
+      <c r="E4" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="34">
-        <v>0</v>
-      </c>
-      <c r="G4" s="35" t="str">
+      <c r="F4" s="22">
+        <v>1</v>
+      </c>
+      <c r="G4" s="23" t="str">
         <f>IF(OR(D4="",F4=""),"chưa rõ",IF(F4&gt;D4,"FRACILE",IF(D4&gt;F4,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H4" s="31" t="s">
+      <c r="H4" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="24" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2346,10 +2391,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2357,16 +2402,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2376,10 +2421,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2387,14 +2432,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2407,7 +2452,7 @@
         <v>52</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2415,7 +2460,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C9" s="21" t="s">
         <v>23</v>
@@ -2424,7 +2469,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F9" s="22">
         <v>1</v>
@@ -2434,10 +2479,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I9" s="24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2445,16 +2490,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2467,7 +2512,7 @@
         <v>52</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2475,14 +2520,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2495,7 +2540,7 @@
         <v>52</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2503,14 +2548,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2523,7 +2568,7 @@
         <v>52</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2531,14 +2576,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2551,7 +2596,7 @@
         <v>52</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2559,14 +2604,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2579,7 +2624,7 @@
         <v>52</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2587,14 +2632,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2607,7 +2652,7 @@
         <v>52</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2615,16 +2660,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2634,10 +2679,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2645,16 +2690,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2667,7 +2712,7 @@
         <v>52</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2675,14 +2720,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2695,7 +2740,7 @@
         <v>52</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2703,16 +2748,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2722,10 +2767,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2733,16 +2778,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2752,10 +2797,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2763,16 +2808,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2785,7 +2830,7 @@
         <v>52</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2793,14 +2838,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2813,7 +2858,7 @@
         <v>52</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2821,29 +2866,29 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F23" s="22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" s="23" t="str">
         <f>IF(OR(D23="",F23=""),"chưa rõ",IF(F23&gt;D23,"FRACILE",IF(D23&gt;F23,"Vivoire","hoà")))</f>
-        <v>hoà</v>
+        <v>Vivoire</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>52</v>
+        <v>135</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2851,14 +2896,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -2871,7 +2916,7 @@
         <v>52</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2879,14 +2924,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -2899,7 +2944,7 @@
         <v>52</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2907,16 +2952,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -2929,7 +2974,7 @@
         <v>52</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2937,16 +2982,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -2956,10 +3001,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2967,14 +3012,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -2984,10 +3029,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2995,14 +3040,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3012,10 +3057,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3023,14 +3068,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3040,10 +3085,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3051,14 +3096,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3068,10 +3113,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3079,14 +3124,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3096,160 +3141,158 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="20" t="s">
-        <v>165</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="D33" s="22">
-        <v>2</v>
-      </c>
-      <c r="E33" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="F33" s="22">
-        <v>2</v>
-      </c>
-      <c r="G33" s="23" t="str">
+      <c r="B33" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="D33" s="28"/>
+      <c r="E33" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="F33" s="28">
+        <v>2</v>
+      </c>
+      <c r="G33" s="29" t="str">
         <f>IF(OR(D33="",F33=""),"chưa rõ",IF(F33&gt;D33,"FRACILE",IF(D33&gt;F33,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H33" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="I33" s="30" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D34" s="22">
+        <v>2</v>
+      </c>
+      <c r="E34" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="F34" s="22">
+        <v>2</v>
+      </c>
+      <c r="G34" s="23" t="str">
+        <f>IF(OR(D34="",F34=""),"chưa rõ",IF(F34&gt;D34,"FRACILE",IF(D34&gt;F34,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H33" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="I33" s="24" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="31" t="s">
+      <c r="H34" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="I34" s="24" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B34" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="C34" s="33" t="s">
-        <v>168</v>
-      </c>
-      <c r="D34" s="34">
-        <v>2</v>
-      </c>
-      <c r="E34" s="33" t="s">
-        <v>169</v>
-      </c>
-      <c r="F34" s="34">
+      <c r="B35" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="C35" s="33" t="s">
+        <v>173</v>
+      </c>
+      <c r="D35" s="34">
+        <v>2</v>
+      </c>
+      <c r="E35" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="F35" s="34">
         <v>0</v>
       </c>
-      <c r="G34" s="35" t="str">
-        <f>IF(OR(D34="",F34=""),"chưa rõ",IF(F34&gt;D34,"FRACILE",IF(D34&gt;F34,"Vivoire","hoà")))</f>
+      <c r="G35" s="35" t="str">
+        <f>IF(OR(D35="",F35=""),"chưa rõ",IF(F35&gt;D35,"FRACILE",IF(D35&gt;F35,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H34" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="I34" s="36" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
+      <c r="H35" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="I35" s="36" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="20" t="s">
-        <v>171</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="D35" s="22">
-        <v>2</v>
-      </c>
-      <c r="E35" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="F35" s="22">
-        <v>2</v>
-      </c>
-      <c r="G35" s="23" t="str">
-        <f>IF(OR(D35="",F35=""),"chưa rõ",IF(F35&gt;D35,"FRACILE",IF(D35&gt;F35,"Vivoire","hoà")))</f>
+      <c r="B36" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="C36" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D36" s="22">
+        <v>2</v>
+      </c>
+      <c r="E36" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="F36" s="22">
+        <v>2</v>
+      </c>
+      <c r="G36" s="23" t="str">
+        <f>IF(OR(D36="",F36=""),"chưa rõ",IF(F36&gt;D36,"FRACILE",IF(D36&gt;F36,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H35" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="I35" s="24" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="31" t="s">
+      <c r="H36" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="I36" s="24" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="32" t="s">
-        <v>174</v>
-      </c>
-      <c r="C36" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="D36" s="34">
-        <v>2</v>
-      </c>
-      <c r="E36" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="F36" s="34">
+      <c r="B37" s="32" t="s">
+        <v>179</v>
+      </c>
+      <c r="C37" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" s="34">
+        <v>2</v>
+      </c>
+      <c r="E37" s="33" t="s">
+        <v>120</v>
+      </c>
+      <c r="F37" s="34">
         <v>0</v>
       </c>
-      <c r="G36" s="35" t="str">
-        <f>IF(OR(D36="",F36=""),"chưa rõ",IF(F36&gt;D36,"FRACILE",IF(D36&gt;F36,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H36" s="31" t="s">
-        <v>120</v>
-      </c>
-      <c r="I36" s="36" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B37" s="20" t="s">
-        <v>175</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="D37" s="22">
-        <v>2</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="F37" s="22">
-        <v>1</v>
-      </c>
-      <c r="G37" s="23" t="str">
+      <c r="G37" s="35" t="str">
         <f>IF(OR(D37="",F37=""),"chưa rõ",IF(F37&gt;D37,"FRACILE",IF(D37&gt;F37,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H37" s="19" t="s">
-        <v>178</v>
-      </c>
-      <c r="I37" s="24" t="s">
-        <v>179</v>
+      <c r="H37" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="I37" s="36" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3260,84 +3303,84 @@
         <v>180</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="D38" s="22"/>
+        <v>181</v>
+      </c>
+      <c r="D38" s="22">
+        <v>2</v>
+      </c>
       <c r="E38" s="21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F38" s="22">
         <v>1</v>
       </c>
       <c r="G38" s="23" t="str">
         <f>IF(OR(D38="",F38=""),"chưa rõ",IF(F38&gt;D38,"FRACILE",IF(D38&gt;F38,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>Vivoire</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>52</v>
+        <v>183</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="D39" s="22">
-        <v>2</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>96</v>
+        <v>186</v>
       </c>
       <c r="F39" s="22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39" s="23" t="str">
         <f>IF(OR(D39="",F39=""),"chưa rõ",IF(F39&gt;D39,"FRACILE",IF(D39&gt;F39,"Vivoire","hoà")))</f>
-        <v>hoà</v>
+        <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
         <v>52</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="31" t="s">
+      <c r="A40" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="32" t="s">
-        <v>185</v>
-      </c>
-      <c r="C40" s="33" t="s">
-        <v>186</v>
-      </c>
-      <c r="D40" s="34">
-        <v>2</v>
-      </c>
-      <c r="E40" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="F40" s="34">
-        <v>0</v>
-      </c>
-      <c r="G40" s="35" t="str">
+      <c r="B40" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D40" s="22">
+        <v>2</v>
+      </c>
+      <c r="E40" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="F40" s="22">
+        <v>2</v>
+      </c>
+      <c r="G40" s="23" t="str">
         <f>IF(OR(D40="",F40=""),"chưa rõ",IF(F40&gt;D40,"FRACILE",IF(D40&gt;F40,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H40" s="31" t="s">
-        <v>120</v>
-      </c>
-      <c r="I40" s="36" t="s">
-        <v>123</v>
+        <v>hoà</v>
+      </c>
+      <c r="H40" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I40" s="24" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3345,16 +3388,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3364,70 +3407,70 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="I41" s="36" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="C42" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="D42" s="34">
+        <v>2</v>
+      </c>
+      <c r="E42" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="I41" s="36" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B42" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="C42" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="D42" s="22">
-        <v>2</v>
-      </c>
-      <c r="E42" s="21" t="s">
-        <v>190</v>
-      </c>
-      <c r="F42" s="22">
-        <v>1</v>
-      </c>
-      <c r="G42" s="23" t="str">
+      <c r="F42" s="34">
+        <v>0</v>
+      </c>
+      <c r="G42" s="35" t="str">
         <f>IF(OR(D42="",F42=""),"chưa rõ",IF(F42&gt;D42,"FRACILE",IF(D42&gt;F42,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H42" s="19" t="s">
+      <c r="H42" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="I42" s="36" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D43" s="22">
+        <v>2</v>
+      </c>
+      <c r="E43" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="F43" s="22">
+        <v>1</v>
+      </c>
+      <c r="G43" s="23" t="str">
+        <f>IF(OR(D43="",F43=""),"chưa rõ",IF(F43&gt;D43,"FRACILE",IF(D43&gt;F43,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H43" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="I42" s="24" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B43" s="26" t="s">
-        <v>191</v>
-      </c>
-      <c r="C43" s="27" t="s">
-        <v>192</v>
-      </c>
-      <c r="D43" s="28">
-        <v>1</v>
-      </c>
-      <c r="E43" s="27" t="s">
-        <v>193</v>
-      </c>
-      <c r="F43" s="28">
-        <v>2</v>
-      </c>
-      <c r="G43" s="29" t="str">
-        <f>IF(OR(D43="",F43=""),"chưa rõ",IF(F43&gt;D43,"FRACILE",IF(D43&gt;F43,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H43" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="I43" s="30" t="s">
-        <v>194</v>
+      <c r="I43" s="24" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3435,177 +3478,177 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="D44" s="28"/>
+        <v>197</v>
+      </c>
+      <c r="D44" s="28">
+        <v>1</v>
+      </c>
       <c r="E44" s="27" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
       </c>
       <c r="G44" s="29" t="str">
         <f>IF(OR(D44="",F44=""),"chưa rõ",IF(F44&gt;D44,"FRACILE",IF(D44&gt;F44,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
         <v>52</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="31" t="s">
+      <c r="A45" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B45" s="26" t="s">
+        <v>200</v>
+      </c>
+      <c r="C45" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D45" s="28"/>
+      <c r="E45" s="27" t="s">
+        <v>201</v>
+      </c>
+      <c r="F45" s="28">
+        <v>2</v>
+      </c>
+      <c r="G45" s="29" t="str">
+        <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H45" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I45" s="30" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="C45" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="D45" s="34">
-        <v>2</v>
-      </c>
-      <c r="E45" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="F45" s="34">
-        <v>0</v>
-      </c>
-      <c r="G45" s="35" t="str">
-        <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H45" s="31" t="s">
-        <v>199</v>
-      </c>
-      <c r="I45" s="36" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="32" t="s">
-        <v>201</v>
-      </c>
-      <c r="C46" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="D46" s="34">
-        <v>2</v>
-      </c>
-      <c r="E46" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="F46" s="34">
-        <v>0</v>
-      </c>
-      <c r="G46" s="35" t="str">
+      <c r="B46" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D46" s="22">
+        <v>2</v>
+      </c>
+      <c r="E46" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="F46" s="22">
+        <v>1</v>
+      </c>
+      <c r="G46" s="23" t="str">
         <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H46" s="31" t="s">
-        <v>199</v>
-      </c>
-      <c r="I46" s="36" t="s">
-        <v>123</v>
+      <c r="H46" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="I46" s="24" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="31" t="s">
+      <c r="A47" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B47" s="32" t="s">
-        <v>202</v>
-      </c>
-      <c r="C47" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="D47" s="34">
-        <v>2</v>
-      </c>
-      <c r="E47" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="F47" s="34">
-        <v>0</v>
-      </c>
-      <c r="G47" s="35" t="str">
+      <c r="B47" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D47" s="22">
+        <v>2</v>
+      </c>
+      <c r="E47" s="21" t="s">
+        <v>208</v>
+      </c>
+      <c r="F47" s="22">
+        <v>1</v>
+      </c>
+      <c r="G47" s="23" t="str">
         <f>IF(OR(D47="",F47=""),"chưa rõ",IF(F47&gt;D47,"FRACILE",IF(D47&gt;F47,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H47" s="31" t="s">
-        <v>199</v>
-      </c>
-      <c r="I47" s="36" t="s">
-        <v>203</v>
+      <c r="H47" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="I47" s="24" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B48" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="C48" s="21" t="s">
-        <v>205</v>
-      </c>
-      <c r="D48" s="22">
-        <v>2</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="F48" s="22">
-        <v>1</v>
-      </c>
-      <c r="G48" s="23" t="str">
+      <c r="B48" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="C48" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D48" s="34">
+        <v>2</v>
+      </c>
+      <c r="E48" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="F48" s="34">
+        <v>0</v>
+      </c>
+      <c r="G48" s="35" t="str">
         <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H48" s="19" t="s">
+      <c r="H48" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="I48" s="36" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>215</v>
+      </c>
+      <c r="D49" s="22">
+        <v>2</v>
+      </c>
+      <c r="E49" s="21" t="s">
+        <v>216</v>
+      </c>
+      <c r="F49" s="22">
+        <v>1</v>
+      </c>
+      <c r="G49" s="23" t="str">
+        <f>IF(OR(D49="",F49=""),"chưa rõ",IF(F49&gt;D49,"FRACILE",IF(D49&gt;F49,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H49" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="I48" s="24" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="B49" s="26" t="s">
-        <v>208</v>
-      </c>
-      <c r="C49" s="27" t="s">
-        <v>209</v>
-      </c>
-      <c r="D49" s="28">
-        <v>1</v>
-      </c>
-      <c r="E49" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="F49" s="28">
-        <v>2</v>
-      </c>
-      <c r="G49" s="29" t="str">
-        <f>IF(OR(D49="",F49=""),"chưa rõ",IF(F49&gt;D49,"FRACILE",IF(D49&gt;F49,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H49" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="I49" s="30" t="s">
-        <v>211</v>
+      <c r="I49" s="24" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3613,27 +3656,57 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>89</v>
-      </c>
-      <c r="D50" s="28"/>
+        <v>219</v>
+      </c>
+      <c r="D50" s="28">
+        <v>1</v>
+      </c>
       <c r="E50" s="27" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
       </c>
       <c r="G50" s="29" t="str">
         <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
         <v>52</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>214</v>
+        <v>221</v>
+      </c>
+    </row>
+    <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B51" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="C51" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="D51" s="28"/>
+      <c r="E51" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="F51" s="28">
+        <v>2</v>
+      </c>
+      <c r="G51" s="29" t="str">
+        <f>IF(OR(D51="",F51=""),"chưa rõ",IF(F51&gt;D51,"FRACILE",IF(D51&gt;F51,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H51" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I51" s="30" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -3645,7 +3718,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -3657,12 +3730,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3678,258 +3751,268 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D8" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
+        <v>244</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="C10" s="19" t="s">
         <v>234</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>235</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>224</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>246</v>
+        <v>167</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>248</v>
+        <v>135</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="38" t="s">
-        <v>250</v>
-      </c>
-      <c r="B15" s="38" t="s">
-        <v>251</v>
-      </c>
-      <c r="C15" s="39" t="s">
-        <v>252</v>
-      </c>
-      <c r="D15" s="38" t="s">
+      <c r="A15" s="21" t="s">
+        <v>258</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>260</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="38" t="s">
+        <v>262</v>
+      </c>
+      <c r="B16" s="38" t="s">
+        <v>263</v>
+      </c>
+      <c r="C16" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="D16" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="38" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="27" t="s">
-        <v>254</v>
-      </c>
-      <c r="B16" s="27" t="s">
-        <v>255</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>256</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>257</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>258</v>
+      <c r="E16" s="38" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D18" s="27" t="s">
+        <v>269</v>
+      </c>
+      <c r="E18" s="27" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="27" t="s">
+        <v>274</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>272</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>275</v>
+      </c>
+      <c r="D19" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="27" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="40" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
-        <v>266</v>
-      </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="18"/>
+      <c r="E19" s="27" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="40" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
+        <v>278</v>
+      </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
       <c r="D23" s="18"/>
@@ -3949,10 +4032,17 @@
       <c r="D25" s="18"/>
       <c r="E25" s="18"/>
     </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="18"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E3"/>
-    <mergeCell ref="A22:E25"/>
+    <mergeCell ref="A23:E26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -3961,7 +4051,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -3972,302 +4062,330 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="B4" s="42">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="B5" s="42">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="B6" s="42">
         <v>207</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="B7" s="42">
         <v>0</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="B8" s="42">
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="B9" s="42">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="B10" s="42">
-        <v>156</v>
+        <v>8</v>
       </c>
       <c r="C10" s="43" t="s">
+        <v>298</v>
+      </c>
+      <c r="D10" s="44" t="s">
         <v>286</v>
-      </c>
-      <c r="D10" s="44" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="B11" s="42">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="B12" s="42">
-        <v>10</v>
+        <v>177</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="B13" s="42">
+        <v>9</v>
+      </c>
+      <c r="C13" s="43" t="s">
+        <v>304</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="41" t="s">
+        <v>305</v>
+      </c>
+      <c r="B14" s="42">
+        <v>8</v>
+      </c>
+      <c r="C14" s="43" t="s">
+        <v>306</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="41" t="s">
+        <v>307</v>
+      </c>
+      <c r="B15" s="42">
         <v>0</v>
       </c>
-      <c r="C13" s="43" t="s">
-        <v>292</v>
-      </c>
-      <c r="D13" s="44" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="B15" s="45">
+      <c r="C15" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="B17" s="45">
         <f>B6/B5</f>
-        <v>0.5549597855227882</v>
-      </c>
-      <c r="C15" s="46" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="B16" s="47">
+        <v>0.5564516129032258</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B18" s="47">
         <f>B5-B6</f>
-        <v>166</v>
-      </c>
-      <c r="C16" s="46" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="40" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>300</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>301</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
-        <v>303</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>304</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>302</v>
+        <v>165</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="40" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>306</v>
+        <v>118</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>302</v>
+        <v>318</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>305</v>
+        <v>321</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>302</v>
+        <v>318</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="39" t="s">
-        <v>309</v>
-      </c>
-      <c r="B25" s="38" t="s">
-        <v>310</v>
-      </c>
-      <c r="C25" s="38" t="s">
-        <v>311</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>312</v>
+      <c r="A25" s="19" t="s">
+        <v>322</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>320</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>321</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="39" t="s">
-        <v>313</v>
-      </c>
-      <c r="B26" s="38" t="s">
-        <v>314</v>
-      </c>
-      <c r="C26" s="38" t="s">
-        <v>315</v>
-      </c>
-      <c r="D26" s="38" t="s">
-        <v>312</v>
+      <c r="A26" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>324</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>321</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
-        <v>316</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>317</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>318</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>319</v>
+      <c r="A27" s="39" t="s">
+        <v>325</v>
+      </c>
+      <c r="B27" s="38" t="s">
+        <v>326</v>
+      </c>
+      <c r="C27" s="38" t="s">
+        <v>327</v>
+      </c>
+      <c r="D27" s="38" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="39" t="s">
+        <v>329</v>
+      </c>
+      <c r="B28" s="38" t="s">
+        <v>330</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>331</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>333</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4290,24 +4408,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>320</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>322</v>
+        <v>338</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>324</v>
+        <v>340</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>325</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4315,16 +4433,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>327</v>
+        <v>343</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>329</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4332,16 +4450,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>331</v>
+        <v>347</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>332</v>
+        <v>348</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>333</v>
+        <v>349</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4349,16 +4467,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>335</v>
+        <v>351</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>336</v>
+        <v>352</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>337</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4366,16 +4484,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>341</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4383,16 +4501,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4400,16 +4518,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
     </row>
     <row r="10" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4417,16 +4535,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="11" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4434,16 +4552,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Làm các mục trong bảng so sánh: neo, ba bộ Flashcard, và sửa một con số sai
· Neo: 7 câu bài « L'impact des locations saisonnières » có neo + 4 bẫy.
  Mỗi đoạn trích kiểm bằng kiemNeo() trên văn bản thật trước khi ghi. Claim
  giả: học sinh đã làm đọc được 7, chưa làm đọc được 0.
· Ba bộ Flashcard NHÁP: Đọc (từ nối), Viết (thư trang trọng), Nói (nêu ý
  kiến) — 27 thẻ. Phiên âm để trống có chủ ý: IPA sai dạy đọc sai.
· Sửa: '8 bài tự luận học sinh đang chờ' — 7/8 thuộc 2 tài khoản thử của
  chủ dự án, không có hồ sơ học sinh; bài còn lại dài 12 ký tự.

Bảng: neo 1→2, flashcard cơ chế 1→2 (có lại SM-2). 100 công thức, 0 thiếu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="374">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -156,6 +156,12 @@
     <t>Dựng rồi gỡ cùng ngày theo quyết định chủ dự án. Vẫn 0.</t>
   </si>
   <si>
+    <t>Làm tiếp cùng ngày</t>
+  </si>
+  <si>
+    <t>Neo 1→2: 7 câu có neo thật. Flashcard cơ chế 1→2: có lại lịch ôn SM-2. Ba bộ nháp cho Đọc/Viết/Nói. Và SỬA LẠI một con số: « 8 bài tự luận học sinh đang chờ » — 7 bài là tài khoản thử của chủ dự án.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -287,13 +293,13 @@
     <t>Neo đáp án vào ngữ liệu (chỉ ra CHỖ chứa câu trả lời)</t>
   </si>
   <si>
-    <t>Dựng xong cả hai đầu (đặt neo + hiển thị), nhưng 0/372 câu có dữ liệu</t>
-  </si>
-  <si>
-    <t>DỰNG XONG — CHƯA CÓ DỮ LIỆU</t>
-  </si>
-  <si>
-    <t>migration 075/076; /professeur/neo; đo 21/09: evidence IS NOT NULL = 0</t>
+    <t>Có dữ liệu thật từ 21/09: 7 câu của bài « L'impact des locations saisonnières » có neo, kèm 4 bẫy giải thích vì sao đáp án sai dụ người ta</t>
+  </si>
+  <si>
+    <t>Đang chạy — có dữ liệu</t>
+  </si>
+  <si>
+    <t>Mỗi đoạn trích kiểm bằng kiemNeo() trên văn bản thật trước khi ghi; claim giả: học sinh đã làm đọc được 7 neo, chưa làm đọc được 0</t>
   </si>
   <si>
     <t>Đề thi thử đúng cấu trúc DELF</t>
@@ -443,13 +449,13 @@
     <t>Flashcard + 3 game mỗi ngày, « ôn từ đúng lúc sắp quên »</t>
   </si>
   <si>
-    <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D. KHÔNG còn lịch ôn ngắt quãng — SM-2 và thẻ sinh từ lỗi sai đã gỡ 09/09. Học sinh không tự tạo thẻ</t>
+    <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D, CÓ lịch ôn SM-2 từ 21/09 (chỉ hiện thẻ đến hạn, bốn mức nhớ). Học sinh không tự tạo thẻ; chưa có trò chơi</t>
   </si>
   <si>
     <t>Đang chạy — chạy thật 21/09</t>
   </si>
   <si>
-    <t>migration 085–088; học sinh mở bằng tài khoản thật thấy đủ 8 thẻ, lật được</t>
+    <t>migration 085–090; claim giả: chấm 1 thẻ → dời sang mai, còn 7 đến hạn. Màn luyện mới CHƯA chạy qua phiên thật</t>
   </si>
   <si>
     <t>Flashcard — quy mô</t>
@@ -458,10 +464,13 @@
     <t>Không công bố số thẻ</t>
   </si>
   <si>
-    <t>1 bộ · 8 thẻ, chỉ kỹ năng Nghe; Đọc/Viết/Nói còn trống</t>
-  </si>
-  <si>
-    <t>the_bo = 1, the_bo_the = 8 (đo 21/09). 37 thẻ SM-2 cũ vẫn trong bảng cards, không màn nào mở</t>
+    <t>4 bộ · 35 thẻ, đủ bốn kỹ năng — nhưng 3 bộ (Đọc, Viết, Nói) còn là NHÁP chờ duyệt</t>
+  </si>
+  <si>
+    <t>1 công khai · 3 nháp</t>
+  </si>
+  <si>
+    <t>the_bo = 4, the_bo_the = 35 (đo 21/09). Bộ nháp học sinh chưa thấy cho tới khi giáo viên bấm công khai</t>
   </si>
   <si>
     <t>Soạn thẻ hàng loạt</t>
@@ -928,7 +937,7 @@
     <t>select count(*) from exams</t>
   </si>
   <si>
-    <t>Bộ Flashcard</t>
+    <t>Bộ Flashcard (1 công khai, 3 nháp)</t>
   </si>
   <si>
     <t>select count(*) from the_bo</t>
@@ -961,7 +970,7 @@
     <t>Bài tự luận CHƯA có điểm nào</t>
   </si>
   <si>
-    <t>câu open: score is null AND self_score is null</t>
+    <t>câu open, không điểm GV lẫn tự chấm. 7/8 thuộc 2 tài khoản thử của chủ dự án; 1 bài của học sinh thật, dài 12 ký tự</t>
   </si>
   <si>
     <t>Gợi ý chấm AI đã sinh</t>
@@ -1072,7 +1081,7 @@
     <t>Đặt khoá API để bật chấm PE bằng AI</t>
   </si>
   <si>
-    <t>Việc rẻ nhất trong danh sách có tác động lớn nhất: mọi thứ đã dựng và đã kiểm, chỉ thiếu một khoá. Chưa đặt thì bài viết chỉ có một đường là tự chấm.</t>
+    <t>Vẫn là việc rẻ nhất có tác động lớn nhất: mọi thứ đã dựng và đã kiểm, chỉ thiếu một khoá.</t>
   </si>
   <si>
     <t>npx supabase secrets set ANTHROPIC_API_KEY=sk-ant-…</t>
@@ -1084,7 +1093,7 @@
     <t>Điền email liên hệ cho FAQ và Điều khoản</t>
   </si>
   <si>
-    <t>Cả hai trang đang tự hiện dòng cảnh báo vàng « chưa công bố email liên hệ ». Một trang pháp lý không có chỗ liên hệ là điểm 1 chứ không phải 2 trong bảng này.</t>
+    <t>Cả hai trang tự hiện cảnh báo vàng cho tới khi có email.</t>
   </si>
   <si>
     <t>EMAIL_LIEN_HE trong src/screens/public/TrangPhapLy.jsx</t>
@@ -1093,70 +1102,67 @@
     <t>2 phút</t>
   </si>
   <si>
-    <t>Báo cho học sinh có 8 bài tự luận chưa có điểm</t>
-  </si>
-  <si>
-    <t>Không có điểm giáo viên lẫn điểm tự chấm. Đường thông báo có sẵn; có thể chỉ họ sang màn tự chấm, và — khi khoá API đã đặt — sang nút xin gợi ý.</t>
-  </si>
-  <si>
-    <t>Đường thông báo đang có</t>
+    <t>Duyệt và công khai ba bộ Flashcard nháp</t>
+  </si>
+  <si>
+    <t>Đọc · Viết · Nói đã có bộ (27 thẻ), đang nháp. Đọc lại rồi bấm nút công khai — cú bấm đó cũng là lần đầu nút này chạy qua giao diện.</t>
+  </si>
+  <si>
+    <t>15 phút</t>
+  </si>
+  <si>
+    <t>Mở màn luyện Flashcard bằng tài khoản học sinh</t>
+  </si>
+  <si>
+    <t>Lịch ôn SM-2 mới chỉ được đo bằng claim giả. Cần một lần bấm thật: 8 thẻ đến hạn, bốn nút sau khi lật, thoát rồi mở lại thì thẻ đã chấm biến khỏi hôm nay.</t>
+  </si>
+  <si>
+    <t>/etudiant/bo-the</t>
+  </si>
+  <si>
+    <t>Xem neo từ phía học sinh</t>
+  </si>
+  <si>
+    <t>Mở lại bài « L'impact des locations saisonnières » bằng một tài khoản đã làm bài, vào phần chữa bài: đoạn văn chứa đáp án phải được tô sáng.</t>
+  </si>
+  <si>
+    <t>Tài khoản học sinh đã làm bài đó</t>
+  </si>
+  <si>
+    <t>Quyết số phận /professeur/oral</t>
+  </si>
+  <si>
+    <t>Màn nghe bài nói không cho điểm, chỉ nghe và nhắn nhận xét.</t>
+  </si>
+  <si>
+    <t>App.jsx; BaiNoiGiaoVien.jsx; navItems.js</t>
+  </si>
+  <si>
+    <t>1 buổi, sau khi quyết</t>
+  </si>
+  <si>
+    <t>Dọn hoặc giữ hai tài khoản thử</t>
+  </si>
+  <si>
+    <t>7 trong 8 « bài tự luận chưa chấm » thuộc về chúng, và chúng làm lệch mọi con số về học sinh. Không có hồ sơ học sinh nên không nằm trong danh sách lớp.</t>
+  </si>
+  <si>
+    <t>Quyết định — xoá tài khoản là việc không hoàn lại</t>
+  </si>
+  <si>
+    <t>quyết định</t>
+  </si>
+  <si>
+    <t>Cân nhắc dựng lại Chính sách bảo mật trước khi thu tiền nhiều</t>
+  </si>
+  <si>
+    <t>Đã gỡ theo quyết định 21/09; nội dung còn trong git.</t>
+  </si>
+  <si>
+    <t>Lấy TrangBaoMat từ commit cũ + route /bao-mat</t>
   </si>
   <si>
     <t>30 phút</t>
-  </si>
-  <si>
-    <t>Soạn thêm bộ Flashcard cho Đọc · Viết · Nói</t>
-  </si>
-  <si>
-    <t>Hiện chỉ 1 bộ, chỉ kỹ năng Nghe. Học sinh mở ba tab còn lại đều thấy trống. Nhập hàng loạt nên một bộ 20 thẻ là một lần dán.</t>
-  </si>
-  <si>
-    <t>/professeur/bo-the — chỉ nhập liệu</t>
-  </si>
-  <si>
-    <t>1–2 giờ</t>
-  </si>
-  <si>
-    <t>Đặt neo cho 5–10 câu đọc hiểu</t>
-  </si>
-  <si>
-    <t>Vẫn 0 dòng sau 12 ngày. Tính năng mạnh nhất Vivoire không có, và chưa ai từng thấy nó chạy.</t>
-  </si>
-  <si>
-    <t>/professeur/neo — chỉ nhập liệu</t>
-  </si>
-  <si>
-    <t>Quyết số phận /professeur/oral</t>
-  </si>
-  <si>
-    <t>Màn nghe bài nói không cho điểm, chỉ nghe và nhắn nhận xét. Giữ vai kèm cặp thì giữ, bỏ hẳn thì gỡ.</t>
-  </si>
-  <si>
-    <t>App.jsx; BaiNoiGiaoVien.jsx; navItems.js</t>
-  </si>
-  <si>
-    <t>1 buổi, sau khi quyết</t>
-  </si>
-  <si>
-    <t>Cân nhắc dựng lại Chính sách bảo mật trước khi thu tiền nhiều</t>
-  </si>
-  <si>
-    <t>Đã gỡ theo quyết định 21/09; nội dung còn trong git. Thiếu nó thì form tư vấn không nên bật lại, và ô này là ô duy nhất trong nhóm pháp lý còn 0 điểm.</t>
-  </si>
-  <si>
-    <t>Lấy TrangBaoMat từ commit cũ + route /bao-mat</t>
-  </si>
-  <si>
-    <t>Cân nhắc KHÔNG đuổi theo: từ điển, podcast, PvP, app mobile</t>
-  </si>
-  <si>
-    <t>Bốn ô Vivoire hơn tuyệt đối. Đuổi theo cả bốn với một người là cách chắc chắn để không ô nào xong.</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>quyết định, không phải mã</t>
   </si>
 </sst>
 </file>
@@ -1765,7 +1771,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1835,11 +1841,11 @@
       </c>
       <c r="E7" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="F7" s="6">
         <f>IFERROR(E7-D7,"")</f>
-        <v>-0.8333333333333334</v>
+        <v>-0.6666666666666667</v>
       </c>
       <c r="G7" s="7" t="str">
         <f>IF(OR(C7&lt;3,F7=""),"quá ít mục",IF(F7&gt;0.25,"FRACILE",IF(F7&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -1922,11 +1928,11 @@
       </c>
       <c r="E10" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>-1</v>
+        <v>-0.6666666666666667</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2038,11 +2044,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
-        <v>0.9</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.9666666666666667</v>
+        <v>-0.9</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2190,14 +2196,28 @@
       <c r="F32" s="18"/>
       <c r="G32" s="18"/>
     </row>
+    <row r="33" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
     <mergeCell ref="B30:G30"/>
     <mergeCell ref="B31:G31"/>
     <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B33:G33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2225,28 +2245,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2254,16 +2274,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2273,10 +2293,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2284,14 +2304,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2301,10 +2321,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2312,16 +2332,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2331,10 +2351,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2342,16 +2362,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2361,10 +2381,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2372,16 +2392,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2391,10 +2411,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2402,16 +2422,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2421,10 +2441,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2432,14 +2452,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2449,40 +2469,40 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="21" t="s">
+      <c r="B9" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="28">
         <v>0</v>
       </c>
-      <c r="E9" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="F9" s="22">
-        <v>1</v>
-      </c>
-      <c r="G9" s="23" t="str">
+      <c r="E9" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="28">
+        <v>2</v>
+      </c>
+      <c r="G9" s="29" t="str">
         <f>IF(OR(D9="",F9=""),"chưa rõ",IF(F9&gt;D9,"FRACILE",IF(D9&gt;F9,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H9" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="I9" s="24" t="s">
-        <v>84</v>
+      <c r="H9" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2490,16 +2510,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2509,10 +2529,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2520,14 +2540,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2537,10 +2557,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2548,14 +2568,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2565,10 +2585,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2576,14 +2596,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2593,10 +2613,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2604,14 +2624,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2621,10 +2641,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2632,14 +2652,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2649,10 +2669,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2660,16 +2680,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2679,10 +2699,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2690,16 +2710,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2709,10 +2729,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2720,14 +2740,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2737,10 +2757,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2748,16 +2768,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2767,10 +2787,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2778,16 +2798,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2797,10 +2817,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2808,16 +2828,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2827,10 +2847,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2838,14 +2858,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2855,10 +2875,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2866,29 +2886,29 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F23" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" s="23" t="str">
         <f>IF(OR(D23="",F23=""),"chưa rõ",IF(F23&gt;D23,"FRACILE",IF(D23&gt;F23,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2896,14 +2916,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -2913,10 +2933,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>52</v>
+        <v>142</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2924,14 +2944,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -2941,10 +2961,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2952,16 +2972,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -2971,10 +2991,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2982,16 +3002,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -3001,10 +3021,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3012,14 +3032,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -3029,10 +3049,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3040,14 +3060,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3057,10 +3077,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3068,14 +3088,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3085,10 +3105,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3096,14 +3116,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3113,10 +3133,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3124,14 +3144,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3141,10 +3161,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3152,14 +3172,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3169,10 +3189,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3180,16 +3200,16 @@
         <v>15</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D34" s="22">
         <v>2</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F34" s="22">
         <v>2</v>
@@ -3199,10 +3219,10 @@
         <v>hoà</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3210,16 +3230,16 @@
         <v>15</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D35" s="34">
         <v>2</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F35" s="34">
         <v>0</v>
@@ -3229,10 +3249,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3240,16 +3260,16 @@
         <v>15</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D36" s="22">
         <v>2</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F36" s="22">
         <v>2</v>
@@ -3259,10 +3279,10 @@
         <v>hoà</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3270,16 +3290,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D37" s="34">
         <v>2</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F37" s="34">
         <v>0</v>
@@ -3289,10 +3309,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3300,16 +3320,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F38" s="22">
         <v>1</v>
@@ -3319,10 +3339,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3330,14 +3350,14 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3347,10 +3367,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3358,16 +3378,16 @@
         <v>16</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3377,10 +3397,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3388,16 +3408,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3407,10 +3427,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3418,16 +3438,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3437,10 +3457,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3448,16 +3468,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3467,10 +3487,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3478,16 +3498,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D44" s="28">
         <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3497,10 +3517,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3508,14 +3528,14 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3525,10 +3545,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3536,16 +3556,16 @@
         <v>17</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3555,10 +3575,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3566,16 +3586,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3585,10 +3605,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3599,13 +3619,13 @@
         <v>37</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D48" s="34">
         <v>2</v>
       </c>
       <c r="E48" s="33" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F48" s="34">
         <v>0</v>
@@ -3615,10 +3635,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3626,16 +3646,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3645,10 +3665,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3656,16 +3676,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D50" s="28">
         <v>1</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
@@ -3675,10 +3695,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3686,14 +3706,14 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D51" s="28"/>
       <c r="E51" s="27" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -3703,10 +3723,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -3730,12 +3750,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3751,267 +3771,267 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B7" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="C7" s="19" t="s">
-        <v>234</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
+        <v>274</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>275</v>
+      </c>
+      <c r="C18" s="25" t="s">
         <v>271</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="D18" s="27" t="s">
         <v>272</v>
       </c>
-      <c r="C18" s="25" t="s">
-        <v>268</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>269</v>
-      </c>
       <c r="E18" s="27" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -4062,330 +4082,330 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B4" s="42">
         <v>33</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B5" s="42">
         <v>372</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B6" s="42">
         <v>207</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B7" s="42">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B8" s="42">
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B9" s="42">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B10" s="42">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="D10" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B11" s="42">
         <v>37</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B12" s="42">
         <v>177</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B13" s="42">
         <v>9</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B14" s="42">
         <v>8</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B15" s="42">
         <v>0</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D15" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B17" s="45">
         <f>B6/B5</f>
         <v>0.5564516129032258</v>
       </c>
       <c r="C17" s="46" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B18" s="47">
         <f>B5-B6</f>
         <v>165</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="40" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="22" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C24" s="21" t="s">
+        <v>324</v>
+      </c>
+      <c r="D24" s="21" t="s">
         <v>321</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C25" s="21" t="s">
+        <v>324</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>321</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B26" s="21" t="s">
+        <v>327</v>
+      </c>
+      <c r="C26" s="21" t="s">
         <v>324</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="D26" s="21" t="s">
         <v>321</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B27" s="38" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C27" s="38" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B28" s="38" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C28" s="38" t="s">
+        <v>334</v>
+      </c>
+      <c r="D28" s="38" t="s">
         <v>331</v>
-      </c>
-      <c r="D28" s="38" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -4408,24 +4428,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4433,16 +4453,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4450,16 +4470,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4467,16 +4487,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>352</v>
+        <v>259</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4484,16 +4504,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4501,16 +4521,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4518,16 +4538,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="10" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4535,16 +4555,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
     </row>
     <row r="11" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4552,16 +4572,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: bảng so sánh — trạng thái Flashcard khớp với bằng chứng
Dòng cơ chế ghi 'chạy thật' trong khi cột bằng chứng nói lịch ôn mới chưa
qua phiên thật. Sửa trạng thái cho khớp.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="375">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -452,373 +452,376 @@
     <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D, CÓ lịch ôn SM-2 từ 21/09 (chỉ hiện thẻ đến hạn, bốn mức nhớ). Học sinh không tự tạo thẻ; chưa có trò chơi</t>
   </si>
   <si>
+    <t>Dựng xong 21/09 — lịch ôn chưa qua phiên thật</t>
+  </si>
+  <si>
+    <t>migration 085–090; claim giả: chấm 1 thẻ → dời sang mai, còn 7 đến hạn. Màn luyện mới CHƯA chạy qua phiên thật</t>
+  </si>
+  <si>
+    <t>Flashcard — quy mô</t>
+  </si>
+  <si>
+    <t>Không công bố số thẻ</t>
+  </si>
+  <si>
+    <t>4 bộ · 35 thẻ, đủ bốn kỹ năng — nhưng 3 bộ (Đọc, Viết, Nói) còn là NHÁP chờ duyệt</t>
+  </si>
+  <si>
+    <t>1 công khai · 3 nháp</t>
+  </si>
+  <si>
+    <t>the_bo = 4, the_bo_the = 35 (đo 21/09). Bộ nháp học sinh chưa thấy cho tới khi giáo viên bấm công khai</t>
+  </si>
+  <si>
+    <t>Soạn thẻ hàng loạt</t>
+  </si>
+  <si>
+    <t>Dán nhiều dòng « mặt trước | mặt sau | phiên âm »; dòng hỏng được gọi tên kèm số dòng</t>
+  </si>
+  <si>
+    <t>shared/boTheGiaoVien.js bocDong(); chủ dự án tạo bộ thử qua giao diện 12/09</t>
+  </si>
+  <si>
+    <t>Chuỗi ngày học</t>
+  </si>
+  <si>
+    <t>Có, kèm nhiệm vụ và kim cương</t>
+  </si>
+  <si>
+    <t>Có — tính ở MÁY CHỦ, theo ngày của NGƯỜI DÙNG chứ không theo giờ UTC</t>
+  </si>
+  <si>
+    <t>migration 061/062; RPC chuoi_ngay_hoc (gaps-and-islands)</t>
+  </si>
+  <si>
+    <t>Trò chơi / thi đấu</t>
+  </si>
+  <si>
+    <t>Đấu dịch thuật PvP trực tiếp</t>
+  </si>
+  <si>
+    <t>Giờ học đo được</t>
+  </si>
+  <si>
+    <t>CHƯA đo được — hiện dấu gạch kèm lý do, KHÔNG điền số ước lượng</t>
+  </si>
+  <si>
+    <t>Cố ý để trống</t>
+  </si>
+  <si>
+    <t>daily_activity.minutes để sẵn; quy tắc 1 của dự án</t>
+  </si>
+  <si>
+    <t>Kiểm soát ai được học bài nào</t>
+  </si>
+  <si>
+    <t>Hai tầng: trọn gói (profiles.has_premium_access) + từng bài (exercise_access)</t>
+  </si>
+  <si>
+    <t>Đang chạy — GIỮ</t>
+  </si>
+  <si>
+    <t>Đây chính là « kiểm soát số lượng học sinh ». AccessPanel.jsx</t>
+  </si>
+  <si>
+    <t>Học sinh KHÔNG tự mở khoá được cho mình</t>
+  </si>
+  <si>
+    <t>exercise_access chặn mọi lệnh ghi từ trình duyệt; phải qua Edge Function</t>
+  </si>
+  <si>
+    <t>migration 001; grant-access giữ service_role</t>
+  </si>
+  <si>
+    <t>Soạn đề thi thử</t>
+  </si>
+  <si>
+    <t>Có — ghép bài từ thư viện vào 4 phần, đặt phút và điểm từng phần</t>
+  </si>
+  <si>
+    <t>ExamComposer.jsx; /professeur/examens</t>
+  </si>
+  <si>
+    <t>Soạn bài và quản lý thư viện</t>
+  </si>
+  <si>
+    <t>Có — Builder, thư mục, chuyển bài giữa Entraînement và Devoir</t>
+  </si>
+  <si>
+    <t>Builder.jsx; exerciseStore.js</t>
+  </si>
+  <si>
+    <t>Soạn Flashcard</t>
+  </si>
+  <si>
+    <t>Có — /professeur/bo-the: tạo bộ, nhập hàng loạt, nháp ↔ công khai, xoá (thẻ đi theo)</t>
+  </si>
+  <si>
+    <t>RLS chỉ giáo viên ghi; đo bằng claim giả: HS thấy 8 thẻ, sửa 0, xoá 0</t>
+  </si>
+  <si>
+    <t>Giao bài theo kỹ năng và cấp độ</t>
+  </si>
+  <si>
+    <t>store='assignment'</t>
+  </si>
+  <si>
+    <t>Chấm bài cho học sinh</t>
+  </si>
+  <si>
+    <t>Có — chấm tự động và AI, giáo viên chốt</t>
+  </si>
+  <si>
+    <t>ĐÃ GỠ (học sinh tự chấm theo grille; AI chấm chưa dựng)</t>
+  </si>
+  <si>
+    <t>Quyết định và thi hành cùng ngày 09/09/2026. Xem sheet « Tài khoản giáo viên »</t>
+  </si>
+  <si>
+    <t>Gửi nhận xét tới một học sinh</t>
+  </si>
+  <si>
+    <t>Có — đi đường THÔNG BÁO đang có, kèm chuông và dấu đã đọc</t>
+  </si>
+  <si>
+    <t>Nhận xét bài nói dùng chính đường này; check:notifs 38 ca</t>
+  </si>
+  <si>
+    <t>Lớp học video trực tiếp</t>
+  </si>
+  <si>
+    <t>Xem đăng ký tư vấn (leads)</t>
+  </si>
+  <si>
+    <t>Có form thu thông tin</t>
+  </si>
+  <si>
+    <t>Bảng và màn xem CÒN NGUYÊN, nhưng FORM ĐÃ GỠ khỏi trang giới thiệu</t>
+  </si>
+  <si>
+    <t>Tắt có chủ đích</t>
+  </si>
+  <si>
+    <t>migration 077–080; /professeur/lien-he. Gỡ vì chưa có trang Chính sách bảo mật</t>
+  </si>
+  <si>
+    <t>Số tài khoản đang có</t>
+  </si>
+  <si>
+    <t>9 người dùng (gồm cả tài khoản thử)</t>
+  </si>
+  <si>
+    <t>select count(*) from profiles = 9, đo 21/09/2026</t>
+  </si>
+  <si>
+    <t>Web</t>
+  </si>
+  <si>
+    <t>fracile.vercel.app / www.fracile.vn</t>
+  </si>
+  <si>
+    <t>iOS</t>
+  </si>
+  <si>
+    <t>Có (App Store)</t>
+  </si>
+  <si>
+    <t>Android</t>
+  </si>
+  <si>
+    <t>Có (Google Play)</t>
+  </si>
+  <si>
+    <t>Tiến độ đồng bộ nhiều thiết bị</t>
+  </si>
+  <si>
+    <t>Có (dữ liệu ở máy chủ), nhưng chỉ một nền tảng nên chưa thành lợi thế</t>
+  </si>
+  <si>
+    <t>Ngôn ngữ giao diện</t>
+  </si>
+  <si>
+    <t>Việt (giao diện) + Pháp (nội dung)</t>
+  </si>
+  <si>
+    <t>Việt · Pháp · Anh</t>
+  </si>
+  <si>
+    <t>shared/i18n.jsx; check:nav 74 ca</t>
+  </si>
+  <si>
+    <t>Thanh toán</t>
+  </si>
+  <si>
+    <t>Webhook SePay đã ghim công thức ký (ts.raw kiểu Stripe)</t>
+  </si>
+  <si>
+    <t>check:hmac 45 ca; giao dịch #76732769 xác nhận</t>
+  </si>
+  <si>
+    <t>Câu hỏi thường gặp (FAQ)</t>
+  </si>
+  <si>
+    <t>Có từ 21/09 — 9 câu, mỗi câu đối chiếu với mã nguồn. Chưa có email liên hệ</t>
+  </si>
+  <si>
+    <t>Có — thiếu email liên hệ</t>
+  </si>
+  <si>
+    <t>/faq; EMAIL_LIEN_HE trong TrangPhapLy.jsx đang trống</t>
+  </si>
+  <si>
+    <t>Điều khoản sử dụng</t>
+  </si>
+  <si>
+    <t>Có từ 21/09 — ghi rõ điểm thi thử không phải điểm DELF chính thức; không tự đặt chính sách hoàn tiền</t>
+  </si>
+  <si>
+    <t>Có — bản nháp, chưa qua luật sư</t>
+  </si>
+  <si>
+    <t>/dieu-khoan</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ — dựng xong 21/09 rồi gỡ cùng ngày theo quyết định chủ dự án</t>
+  </si>
+  <si>
+    <t>ĐÃ GỠ — có chủ đích</t>
+  </si>
+  <si>
+    <t>Nội dung còn trong git. Khi vắng trang này, form tư vấn không nên bật lại</t>
+  </si>
+  <si>
+    <t>Đội ngũ công khai</t>
+  </si>
+  <si>
+    <t>4 người, có tên và thành tích (HSG quốc gia, thạc sĩ UMass, kỹ sư AI)</t>
+  </si>
+  <si>
+    <t>1 người — Đỗ Quốc Hùng, ghi « Đội ngũ phát triển »</t>
+  </si>
+  <si>
+    <t>TeamSection.jsx; không ghi bằng cấp chưa kiểm chứng được</t>
+  </si>
+  <si>
+    <t>Số liệu trên trang bán hàng</t>
+  </si>
+  <si>
+    <t>« 56.000+ từ », « 200+200 bài » — không nói nguồn</t>
+  </si>
+  <si>
+    <t>ĐẾM THẬT từ máy chủ lúc tải trang; hỏng thì hiện dấu gạch chứ không hiện 0</t>
+  </si>
+  <si>
+    <t>shared/soLieuCongKhai.js; quy tắc 1 của dự án</t>
+  </si>
+  <si>
+    <t>Giọng nói học sinh lưu ở đâu</t>
+  </si>
+  <si>
+    <t>Bucket RIÊNG, private, không policy xoá/sửa; đường dẫn so user_id</t>
+  </si>
+  <si>
+    <t>migration 057/058 — giọng trẻ vị thành niên ở URL đoán được là chuyện pháp lý</t>
+  </si>
+  <si>
+    <t>TÀI KHOẢN GIÁO VIÊN — giữ để KIỂM SOÁT, không để CHẤM BÀI</t>
+  </si>
+  <si>
+    <t>Quyết định của chủ dự án ngày 09/09/2026: giữ tài khoản giáo viên để quản lý số lượng học sinh và quyền truy cập; bỏ hoàn toàn việc giáo viên chấm bài. Học sinh tự chấm theo grille DELF; AI gợi ý chấm đã dựng nhưng chưa bật (thiếu khoá API).</t>
+  </si>
+  <si>
+    <t>Quyền / màn hình</t>
+  </si>
+  <si>
+    <t>Đường dẫn</t>
+  </si>
+  <si>
+    <t>Quyết định</t>
+  </si>
+  <si>
+    <t>Tình trạng mã nguồn HÔM NAY</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
+  </si>
+  <si>
+    <t>Bật/tắt quyền học từng bài cho một học sinh</t>
+  </si>
+  <si>
+    <t>AccessPanel (trong dashboard)</t>
+  </si>
+  <si>
+    <t>GIỮ</t>
+  </si>
+  <si>
+    <t>Đây chính là « kiểm soát số lượng học sinh ». Ghi qua Edge Function grant-access.</t>
+  </si>
+  <si>
+    <t>Bật/tắt trọn gói cho một học sinh</t>
+  </si>
+  <si>
+    <t>AccessPanel</t>
+  </si>
+  <si>
+    <t>profiles.has_premium_access — mở cả những bài chưa tồn tại lúc bật.</t>
+  </si>
+  <si>
+    <t>Soạn / sửa / xoá bài trong thư viện</t>
+  </si>
+  <si>
+    <t>/professeur/dashboard → Builder</t>
+  </si>
+  <si>
+    <t>Đường GHI vẫn CHƯA được thử tay đầy đủ — xem mục còn treo trong CLAUDE.md.</t>
+  </si>
+  <si>
+    <t>/professeur/examens</t>
+  </si>
+  <si>
+    <t>Ghép bài vào 4 phần CO/CE/PE/PO, đặt phút và điểm từng phần.</t>
+  </si>
+  <si>
+    <t>Soạn thang chấm riêng cho một đề</t>
+  </si>
+  <si>
+    <t>/professeur/grille</t>
+  </si>
+  <si>
+    <t>CÀNG quan trọng khi học sinh tự chấm — thang là thứ duy nhất hướng dẫn họ.</t>
+  </si>
+  <si>
+    <t>Viết lời giải thích, xếp theo số học sinh sai</t>
+  </si>
+  <si>
+    <t>/professeur/loi-giai</t>
+  </si>
+  <si>
+    <t>Thay thế trực tiếp cho chấm tay: dạy một lần cho tất cả, thay vì nhận xét từng bài.</t>
+  </si>
+  <si>
+    <t>Đặt neo đáp án vào ngữ liệu</t>
+  </si>
+  <si>
+    <t>/professeur/neo</t>
+  </si>
+  <si>
+    <t>Dựng xong, 0 dữ liệu</t>
+  </si>
+  <si>
+    <t>Chưa câu nào có neo nên chưa ai từng thấy nó chạy, kể cả chủ dự án.</t>
+  </si>
+  <si>
+    <t>Sổ tay / mẹo</t>
+  </si>
+  <si>
+    <t>/professeur/carnet</t>
+  </si>
+  <si>
+    <t>/professeur/bo-the</t>
+  </si>
+  <si>
     <t>Đang chạy — chạy thật 21/09</t>
-  </si>
-  <si>
-    <t>migration 085–090; claim giả: chấm 1 thẻ → dời sang mai, còn 7 đến hạn. Màn luyện mới CHƯA chạy qua phiên thật</t>
-  </si>
-  <si>
-    <t>Flashcard — quy mô</t>
-  </si>
-  <si>
-    <t>Không công bố số thẻ</t>
-  </si>
-  <si>
-    <t>4 bộ · 35 thẻ, đủ bốn kỹ năng — nhưng 3 bộ (Đọc, Viết, Nói) còn là NHÁP chờ duyệt</t>
-  </si>
-  <si>
-    <t>1 công khai · 3 nháp</t>
-  </si>
-  <si>
-    <t>the_bo = 4, the_bo_the = 35 (đo 21/09). Bộ nháp học sinh chưa thấy cho tới khi giáo viên bấm công khai</t>
-  </si>
-  <si>
-    <t>Soạn thẻ hàng loạt</t>
-  </si>
-  <si>
-    <t>Dán nhiều dòng « mặt trước | mặt sau | phiên âm »; dòng hỏng được gọi tên kèm số dòng</t>
-  </si>
-  <si>
-    <t>shared/boTheGiaoVien.js bocDong(); chủ dự án tạo bộ thử qua giao diện 12/09</t>
-  </si>
-  <si>
-    <t>Chuỗi ngày học</t>
-  </si>
-  <si>
-    <t>Có, kèm nhiệm vụ và kim cương</t>
-  </si>
-  <si>
-    <t>Có — tính ở MÁY CHỦ, theo ngày của NGƯỜI DÙNG chứ không theo giờ UTC</t>
-  </si>
-  <si>
-    <t>migration 061/062; RPC chuoi_ngay_hoc (gaps-and-islands)</t>
-  </si>
-  <si>
-    <t>Trò chơi / thi đấu</t>
-  </si>
-  <si>
-    <t>Đấu dịch thuật PvP trực tiếp</t>
-  </si>
-  <si>
-    <t>Giờ học đo được</t>
-  </si>
-  <si>
-    <t>CHƯA đo được — hiện dấu gạch kèm lý do, KHÔNG điền số ước lượng</t>
-  </si>
-  <si>
-    <t>Cố ý để trống</t>
-  </si>
-  <si>
-    <t>daily_activity.minutes để sẵn; quy tắc 1 của dự án</t>
-  </si>
-  <si>
-    <t>Kiểm soát ai được học bài nào</t>
-  </si>
-  <si>
-    <t>Hai tầng: trọn gói (profiles.has_premium_access) + từng bài (exercise_access)</t>
-  </si>
-  <si>
-    <t>Đang chạy — GIỮ</t>
-  </si>
-  <si>
-    <t>Đây chính là « kiểm soát số lượng học sinh ». AccessPanel.jsx</t>
-  </si>
-  <si>
-    <t>Học sinh KHÔNG tự mở khoá được cho mình</t>
-  </si>
-  <si>
-    <t>exercise_access chặn mọi lệnh ghi từ trình duyệt; phải qua Edge Function</t>
-  </si>
-  <si>
-    <t>migration 001; grant-access giữ service_role</t>
-  </si>
-  <si>
-    <t>Soạn đề thi thử</t>
-  </si>
-  <si>
-    <t>Có — ghép bài từ thư viện vào 4 phần, đặt phút và điểm từng phần</t>
-  </si>
-  <si>
-    <t>ExamComposer.jsx; /professeur/examens</t>
-  </si>
-  <si>
-    <t>Soạn bài và quản lý thư viện</t>
-  </si>
-  <si>
-    <t>Có — Builder, thư mục, chuyển bài giữa Entraînement và Devoir</t>
-  </si>
-  <si>
-    <t>Builder.jsx; exerciseStore.js</t>
-  </si>
-  <si>
-    <t>Soạn Flashcard</t>
-  </si>
-  <si>
-    <t>Có — /professeur/bo-the: tạo bộ, nhập hàng loạt, nháp ↔ công khai, xoá (thẻ đi theo)</t>
-  </si>
-  <si>
-    <t>RLS chỉ giáo viên ghi; đo bằng claim giả: HS thấy 8 thẻ, sửa 0, xoá 0</t>
-  </si>
-  <si>
-    <t>Giao bài theo kỹ năng và cấp độ</t>
-  </si>
-  <si>
-    <t>store='assignment'</t>
-  </si>
-  <si>
-    <t>Chấm bài cho học sinh</t>
-  </si>
-  <si>
-    <t>Có — chấm tự động và AI, giáo viên chốt</t>
-  </si>
-  <si>
-    <t>ĐÃ GỠ (học sinh tự chấm theo grille; AI chấm chưa dựng)</t>
-  </si>
-  <si>
-    <t>Quyết định và thi hành cùng ngày 09/09/2026. Xem sheet « Tài khoản giáo viên »</t>
-  </si>
-  <si>
-    <t>Gửi nhận xét tới một học sinh</t>
-  </si>
-  <si>
-    <t>Có — đi đường THÔNG BÁO đang có, kèm chuông và dấu đã đọc</t>
-  </si>
-  <si>
-    <t>Nhận xét bài nói dùng chính đường này; check:notifs 38 ca</t>
-  </si>
-  <si>
-    <t>Lớp học video trực tiếp</t>
-  </si>
-  <si>
-    <t>Xem đăng ký tư vấn (leads)</t>
-  </si>
-  <si>
-    <t>Có form thu thông tin</t>
-  </si>
-  <si>
-    <t>Bảng và màn xem CÒN NGUYÊN, nhưng FORM ĐÃ GỠ khỏi trang giới thiệu</t>
-  </si>
-  <si>
-    <t>Tắt có chủ đích</t>
-  </si>
-  <si>
-    <t>migration 077–080; /professeur/lien-he. Gỡ vì chưa có trang Chính sách bảo mật</t>
-  </si>
-  <si>
-    <t>Số tài khoản đang có</t>
-  </si>
-  <si>
-    <t>9 người dùng (gồm cả tài khoản thử)</t>
-  </si>
-  <si>
-    <t>select count(*) from profiles = 9, đo 21/09/2026</t>
-  </si>
-  <si>
-    <t>Web</t>
-  </si>
-  <si>
-    <t>fracile.vercel.app / www.fracile.vn</t>
-  </si>
-  <si>
-    <t>iOS</t>
-  </si>
-  <si>
-    <t>Có (App Store)</t>
-  </si>
-  <si>
-    <t>Android</t>
-  </si>
-  <si>
-    <t>Có (Google Play)</t>
-  </si>
-  <si>
-    <t>Tiến độ đồng bộ nhiều thiết bị</t>
-  </si>
-  <si>
-    <t>Có (dữ liệu ở máy chủ), nhưng chỉ một nền tảng nên chưa thành lợi thế</t>
-  </si>
-  <si>
-    <t>Ngôn ngữ giao diện</t>
-  </si>
-  <si>
-    <t>Việt (giao diện) + Pháp (nội dung)</t>
-  </si>
-  <si>
-    <t>Việt · Pháp · Anh</t>
-  </si>
-  <si>
-    <t>shared/i18n.jsx; check:nav 74 ca</t>
-  </si>
-  <si>
-    <t>Thanh toán</t>
-  </si>
-  <si>
-    <t>Webhook SePay đã ghim công thức ký (ts.raw kiểu Stripe)</t>
-  </si>
-  <si>
-    <t>check:hmac 45 ca; giao dịch #76732769 xác nhận</t>
-  </si>
-  <si>
-    <t>Câu hỏi thường gặp (FAQ)</t>
-  </si>
-  <si>
-    <t>Có từ 21/09 — 9 câu, mỗi câu đối chiếu với mã nguồn. Chưa có email liên hệ</t>
-  </si>
-  <si>
-    <t>Có — thiếu email liên hệ</t>
-  </si>
-  <si>
-    <t>/faq; EMAIL_LIEN_HE trong TrangPhapLy.jsx đang trống</t>
-  </si>
-  <si>
-    <t>Điều khoản sử dụng</t>
-  </si>
-  <si>
-    <t>Có từ 21/09 — ghi rõ điểm thi thử không phải điểm DELF chính thức; không tự đặt chính sách hoàn tiền</t>
-  </si>
-  <si>
-    <t>Có — bản nháp, chưa qua luật sư</t>
-  </si>
-  <si>
-    <t>/dieu-khoan</t>
-  </si>
-  <si>
-    <t>KHÔNG CÓ — dựng xong 21/09 rồi gỡ cùng ngày theo quyết định chủ dự án</t>
-  </si>
-  <si>
-    <t>ĐÃ GỠ — có chủ đích</t>
-  </si>
-  <si>
-    <t>Nội dung còn trong git. Khi vắng trang này, form tư vấn không nên bật lại</t>
-  </si>
-  <si>
-    <t>Đội ngũ công khai</t>
-  </si>
-  <si>
-    <t>4 người, có tên và thành tích (HSG quốc gia, thạc sĩ UMass, kỹ sư AI)</t>
-  </si>
-  <si>
-    <t>1 người — Đỗ Quốc Hùng, ghi « Đội ngũ phát triển »</t>
-  </si>
-  <si>
-    <t>TeamSection.jsx; không ghi bằng cấp chưa kiểm chứng được</t>
-  </si>
-  <si>
-    <t>Số liệu trên trang bán hàng</t>
-  </si>
-  <si>
-    <t>« 56.000+ từ », « 200+200 bài » — không nói nguồn</t>
-  </si>
-  <si>
-    <t>ĐẾM THẬT từ máy chủ lúc tải trang; hỏng thì hiện dấu gạch chứ không hiện 0</t>
-  </si>
-  <si>
-    <t>shared/soLieuCongKhai.js; quy tắc 1 của dự án</t>
-  </si>
-  <si>
-    <t>Giọng nói học sinh lưu ở đâu</t>
-  </si>
-  <si>
-    <t>Bucket RIÊNG, private, không policy xoá/sửa; đường dẫn so user_id</t>
-  </si>
-  <si>
-    <t>migration 057/058 — giọng trẻ vị thành niên ở URL đoán được là chuyện pháp lý</t>
-  </si>
-  <si>
-    <t>TÀI KHOẢN GIÁO VIÊN — giữ để KIỂM SOÁT, không để CHẤM BÀI</t>
-  </si>
-  <si>
-    <t>Quyết định của chủ dự án ngày 09/09/2026: giữ tài khoản giáo viên để quản lý số lượng học sinh và quyền truy cập; bỏ hoàn toàn việc giáo viên chấm bài. Học sinh tự chấm theo grille DELF; AI gợi ý chấm đã dựng nhưng chưa bật (thiếu khoá API).</t>
-  </si>
-  <si>
-    <t>Quyền / màn hình</t>
-  </si>
-  <si>
-    <t>Đường dẫn</t>
-  </si>
-  <si>
-    <t>Quyết định</t>
-  </si>
-  <si>
-    <t>Tình trạng mã nguồn HÔM NAY</t>
-  </si>
-  <si>
-    <t>Ghi chú</t>
-  </si>
-  <si>
-    <t>Bật/tắt quyền học từng bài cho một học sinh</t>
-  </si>
-  <si>
-    <t>AccessPanel (trong dashboard)</t>
-  </si>
-  <si>
-    <t>GIỮ</t>
-  </si>
-  <si>
-    <t>Đây chính là « kiểm soát số lượng học sinh ». Ghi qua Edge Function grant-access.</t>
-  </si>
-  <si>
-    <t>Bật/tắt trọn gói cho một học sinh</t>
-  </si>
-  <si>
-    <t>AccessPanel</t>
-  </si>
-  <si>
-    <t>profiles.has_premium_access — mở cả những bài chưa tồn tại lúc bật.</t>
-  </si>
-  <si>
-    <t>Soạn / sửa / xoá bài trong thư viện</t>
-  </si>
-  <si>
-    <t>/professeur/dashboard → Builder</t>
-  </si>
-  <si>
-    <t>Đường GHI vẫn CHƯA được thử tay đầy đủ — xem mục còn treo trong CLAUDE.md.</t>
-  </si>
-  <si>
-    <t>/professeur/examens</t>
-  </si>
-  <si>
-    <t>Ghép bài vào 4 phần CO/CE/PE/PO, đặt phút và điểm từng phần.</t>
-  </si>
-  <si>
-    <t>Soạn thang chấm riêng cho một đề</t>
-  </si>
-  <si>
-    <t>/professeur/grille</t>
-  </si>
-  <si>
-    <t>CÀNG quan trọng khi học sinh tự chấm — thang là thứ duy nhất hướng dẫn họ.</t>
-  </si>
-  <si>
-    <t>Viết lời giải thích, xếp theo số học sinh sai</t>
-  </si>
-  <si>
-    <t>/professeur/loi-giai</t>
-  </si>
-  <si>
-    <t>Thay thế trực tiếp cho chấm tay: dạy một lần cho tất cả, thay vì nhận xét từng bài.</t>
-  </si>
-  <si>
-    <t>Đặt neo đáp án vào ngữ liệu</t>
-  </si>
-  <si>
-    <t>/professeur/neo</t>
-  </si>
-  <si>
-    <t>Dựng xong, 0 dữ liệu</t>
-  </si>
-  <si>
-    <t>Chưa câu nào có neo nên chưa ai từng thấy nó chạy, kể cả chủ dự án.</t>
-  </si>
-  <si>
-    <t>Sổ tay / mẹo</t>
-  </si>
-  <si>
-    <t>/professeur/carnet</t>
-  </si>
-  <si>
-    <t>/professeur/bo-the</t>
   </si>
   <si>
     <t>Dựng 09/09. Học sinh không còn tự tạo thẻ — chỉ giáo viên soạn, chặn ở database bằng RLS chứ không chỉ ẩn nút.</t>
@@ -3933,105 +3936,105 @@
         <v>237</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>137</v>
+        <v>260</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>237</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D16" s="38" t="s">
         <v>54</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D19" s="27" t="s">
         <v>54</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -4082,232 +4085,232 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B4" s="42">
         <v>33</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B5" s="42">
         <v>372</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B6" s="42">
         <v>207</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B7" s="42">
         <v>7</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B8" s="42">
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B9" s="42">
         <v>4</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B10" s="42">
         <v>35</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D10" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B11" s="42">
         <v>37</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B12" s="42">
         <v>177</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B13" s="42">
         <v>9</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B14" s="42">
         <v>8</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B15" s="42">
         <v>0</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D15" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B17" s="45">
         <f>B6/B5</f>
         <v>0.5564516129032258</v>
       </c>
       <c r="C17" s="46" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B18" s="47">
         <f>B5-B6</f>
         <v>165</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="40" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="22" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -4315,97 +4318,97 @@
         <v>120</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>324</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>325</v>
+      </c>
+      <c r="D24" s="21" t="s">
         <v>322</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>324</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
+        <v>326</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>324</v>
+      </c>
+      <c r="C25" s="21" t="s">
         <v>325</v>
       </c>
-      <c r="B25" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>324</v>
-      </c>
       <c r="D25" s="21" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B27" s="38" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C27" s="38" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
+        <v>333</v>
+      </c>
+      <c r="B28" s="38" t="s">
+        <v>334</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="D28" s="38" t="s">
         <v>332</v>
-      </c>
-      <c r="B28" s="38" t="s">
-        <v>333</v>
-      </c>
-      <c r="C28" s="38" t="s">
-        <v>334</v>
-      </c>
-      <c r="D28" s="38" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -4428,24 +4431,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4453,16 +4456,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4470,16 +4473,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4487,16 +4490,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>259</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4504,16 +4507,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4521,16 +4524,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4538,16 +4541,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="10" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4555,16 +4558,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="11" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4572,16 +4575,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: bảng so sánh 22/09 — lịch ôn Flashcard lưu được, bốn bộ công khai
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="381">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Vivoire: đọc từ trang chủ vivoire.app ngày 09/09/2026 — CHƯA đọc lại. Không có tài khoản nên không kiểm được bên trong sản phẩm.</t>
   </si>
   <si>
-    <t>FRACILE: đo từ mã nguồn và database production ngày 21/09/2026.</t>
+    <t>FRACILE: đo từ mã nguồn và database production ngày 22/09/2026.</t>
   </si>
   <si>
     <t>Mọi con số ở sheet này TÍNH từ sheet « So sánh chi tiết » — sửa điểm ở đó thì ở đây tự đổi theo.</t>
@@ -156,6 +156,12 @@
     <t>Dựng rồi gỡ cùng ngày theo quyết định chủ dự án. Vẫn 0.</t>
   </si>
   <si>
+    <t>22/09 — lịch ôn lưu được</t>
+  </si>
+  <si>
+    <t>Tài khoản thật bấm Tốt nhưng database không đổi; thêm hàm chấm có biên nhận (091), sau Ctrl+F5 thì lưu được. Nguyên nhân gốc chưa chứng minh — nghi tab chạy bản JS cũ. Bốn bộ Flashcard đã công khai.</t>
+  </si>
+  <si>
     <t>Làm tiếp cùng ngày</t>
   </si>
   <si>
@@ -452,10 +458,10 @@
     <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D, CÓ lịch ôn SM-2 từ 21/09 (chỉ hiện thẻ đến hạn, bốn mức nhớ). Học sinh không tự tạo thẻ; chưa có trò chơi</t>
   </si>
   <si>
-    <t>Dựng xong 21/09 — lịch ôn chưa qua phiên thật</t>
-  </si>
-  <si>
-    <t>migration 085–090; claim giả: chấm 1 thẻ → dời sang mai, còn 7 đến hạn. Màn luyện mới CHƯA chạy qua phiên thật</t>
+    <t>Đang chạy — lưu thật 22/09</t>
+  </si>
+  <si>
+    <t>migration 085–091; tài khoản thật bấm Tốt → 2 thẻ reps=1, hẹn 23/09. Mỗi lần chấm có biên nhận, hỏng thì hiện chữ đỏ</t>
   </si>
   <si>
     <t>Flashcard — quy mô</t>
@@ -464,13 +470,13 @@
     <t>Không công bố số thẻ</t>
   </si>
   <si>
-    <t>4 bộ · 35 thẻ, đủ bốn kỹ năng — nhưng 3 bộ (Đọc, Viết, Nói) còn là NHÁP chờ duyệt</t>
-  </si>
-  <si>
-    <t>1 công khai · 3 nháp</t>
-  </si>
-  <si>
-    <t>the_bo = 4, the_bo_the = 35 (đo 21/09). Bộ nháp học sinh chưa thấy cho tới khi giáo viên bấm công khai</t>
+    <t>4 bộ · 35 thẻ, đủ bốn kỹ năng, cả bốn công khai. Còn nhỏ so với một thư viện flashcard thật</t>
+  </si>
+  <si>
+    <t>Đang chạy — 4 công khai</t>
+  </si>
+  <si>
+    <t>the_bo = 4, the_bo_the = 35; học sinh mở bằng tài khoản thật thấy đủ bốn bộ (21/09)</t>
   </si>
   <si>
     <t>Soạn thẻ hàng loạt</t>
@@ -940,12 +946,15 @@
     <t>select count(*) from exams</t>
   </si>
   <si>
-    <t>Bộ Flashcard (1 công khai, 3 nháp)</t>
+    <t>Bộ Flashcard (cả bốn công khai)</t>
   </si>
   <si>
     <t>select count(*) from the_bo</t>
   </si>
   <si>
+    <t>22/09/2026</t>
+  </si>
+  <si>
     <t>Thẻ trong các bộ</t>
   </si>
   <si>
@@ -976,6 +985,12 @@
     <t>câu open, không điểm GV lẫn tự chấm. 7/8 thuộc 2 tài khoản thử của chủ dự án; 1 bài của học sinh thật, dài 12 ký tự</t>
   </si>
   <si>
+    <t>Lượt ôn Flashcard đã ghi</t>
+  </si>
+  <si>
+    <t>reviews có reps &gt; 0 trên thẻ bo_giao_vien</t>
+  </si>
+  <si>
     <t>Gợi ý chấm AI đã sinh</t>
   </si>
   <si>
@@ -1105,31 +1120,34 @@
     <t>2 phút</t>
   </si>
   <si>
-    <t>Duyệt và công khai ba bộ Flashcard nháp</t>
-  </si>
-  <si>
-    <t>Đọc · Viết · Nói đã có bộ (27 thẻ), đang nháp. Đọc lại rồi bấm nút công khai — cú bấm đó cũng là lần đầu nút này chạy qua giao diện.</t>
-  </si>
-  <si>
-    <t>15 phút</t>
-  </si>
-  <si>
-    <t>Mở màn luyện Flashcard bằng tài khoản học sinh</t>
-  </si>
-  <si>
-    <t>Lịch ôn SM-2 mới chỉ được đo bằng claim giả. Cần một lần bấm thật: 8 thẻ đến hạn, bốn nút sau khi lật, thoát rồi mở lại thì thẻ đã chấm biến khỏi hôm nay.</t>
-  </si>
-  <si>
-    <t>/etudiant/bo-the</t>
+    <t>Mai (23/09) mở lại bộ « Thông báo ở nhà ga »</t>
+  </si>
+  <si>
+    <t>Hai thẻ đã chấm hẹn ôn ngày 23/09. Nếu chúng hiện lại đúng ngày đó thì lịch ôn đã chạy trọn một vòng — lần đầu tiên.</t>
+  </si>
+  <si>
+    <t>/etudiant/bo-the — nhớ Ctrl+F5</t>
   </si>
   <si>
     <t>Xem neo từ phía học sinh</t>
   </si>
   <si>
-    <t>Mở lại bài « L'impact des locations saisonnières » bằng một tài khoản đã làm bài, vào phần chữa bài: đoạn văn chứa đáp án phải được tô sáng.</t>
-  </si>
-  <si>
-    <t>Tài khoản học sinh đã làm bài đó</t>
+    <t>Mở lại bài « L'impact des locations saisonnières » bằng tài khoản đã làm bài, vào phần chữa bài: đoạn chứa đáp án phải được tô sáng.</t>
+  </si>
+  <si>
+    <t>Tài khoản học sinh đã làm bài đó — nhớ Ctrl+F5</t>
+  </si>
+  <si>
+    <t>Thử lại lưu lời giải và đặt neo qua giao diện giáo viên</t>
+  </si>
+  <si>
+    <t>Đầu tháng hai đường này báo « đã lưu » mà không lưu. Nếu nguyên nhân là tab chạy bản cũ thì sau Ctrl+F5 chúng sẽ lưu được — và lỗi cũ coi như đã có lời giải.</t>
+  </si>
+  <si>
+    <t>/professeur/loi-giai và /professeur/neo</t>
+  </si>
+  <si>
+    <t>10 phút</t>
   </si>
   <si>
     <t>Quyết số phận /professeur/oral</t>
@@ -1147,7 +1165,7 @@
     <t>Dọn hoặc giữ hai tài khoản thử</t>
   </si>
   <si>
-    <t>7 trong 8 « bài tự luận chưa chấm » thuộc về chúng, và chúng làm lệch mọi con số về học sinh. Không có hồ sơ học sinh nên không nằm trong danh sách lớp.</t>
+    <t>7 trong 8 « bài tự luận chưa chấm » thuộc về chúng, và chúng làm lệch mọi con số về học sinh.</t>
   </si>
   <si>
     <t>Quyết định — xoá tài khoản là việc không hoàn lại</t>
@@ -1774,7 +1792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2212,8 +2230,21 @@
       <c r="F33" s="18"/>
       <c r="G33" s="18"/>
     </row>
+    <row r="34" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2221,6 +2252,7 @@
     <mergeCell ref="B31:G31"/>
     <mergeCell ref="B32:G32"/>
     <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B34:G34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2248,28 +2280,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2277,16 +2309,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2296,10 +2328,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2307,14 +2339,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2324,10 +2356,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2335,16 +2367,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2354,10 +2386,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2365,16 +2397,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2384,10 +2416,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2395,16 +2427,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2414,10 +2446,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2425,16 +2457,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2444,10 +2476,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2455,14 +2487,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2472,10 +2504,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2483,7 +2515,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2492,7 +2524,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2502,10 +2534,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2513,16 +2545,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2532,10 +2564,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2543,14 +2575,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2560,10 +2592,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2571,14 +2603,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2588,10 +2620,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2599,14 +2631,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2616,10 +2648,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2627,14 +2659,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2644,10 +2676,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2655,14 +2687,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2672,10 +2704,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2683,16 +2715,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2702,10 +2734,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2713,16 +2745,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2732,10 +2764,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2743,14 +2775,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2760,10 +2792,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2771,16 +2803,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2790,10 +2822,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2801,16 +2833,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2820,10 +2852,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2831,16 +2863,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2850,10 +2882,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2861,14 +2893,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2878,10 +2910,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2889,16 +2921,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -2908,10 +2940,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2919,14 +2951,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -2936,10 +2968,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2947,14 +2979,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -2964,10 +2996,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2975,16 +3007,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -2994,10 +3026,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3005,16 +3037,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -3024,10 +3056,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3035,14 +3067,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -3052,10 +3084,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3063,14 +3095,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3080,10 +3112,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3091,14 +3123,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3108,10 +3140,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3119,14 +3151,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3136,10 +3168,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3147,14 +3179,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3164,10 +3196,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3175,14 +3207,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3192,10 +3224,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3203,16 +3235,16 @@
         <v>15</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D34" s="22">
         <v>2</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F34" s="22">
         <v>2</v>
@@ -3222,10 +3254,10 @@
         <v>hoà</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3233,16 +3265,16 @@
         <v>15</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D35" s="34">
         <v>2</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F35" s="34">
         <v>0</v>
@@ -3252,10 +3284,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3263,16 +3295,16 @@
         <v>15</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D36" s="22">
         <v>2</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F36" s="22">
         <v>2</v>
@@ -3282,10 +3314,10 @@
         <v>hoà</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3293,16 +3325,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D37" s="34">
         <v>2</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F37" s="34">
         <v>0</v>
@@ -3312,10 +3344,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3323,16 +3355,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F38" s="22">
         <v>1</v>
@@ -3342,10 +3374,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3353,14 +3385,14 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3370,10 +3402,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3381,16 +3413,16 @@
         <v>16</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3400,10 +3432,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3411,16 +3443,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3430,10 +3462,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3441,16 +3473,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3460,10 +3492,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3471,16 +3503,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3490,10 +3522,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3501,16 +3533,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D44" s="28">
         <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3520,10 +3552,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3531,14 +3563,14 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3548,10 +3580,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3559,16 +3591,16 @@
         <v>17</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3578,10 +3610,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3589,16 +3621,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3608,10 +3640,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3622,13 +3654,13 @@
         <v>37</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D48" s="34">
         <v>2</v>
       </c>
       <c r="E48" s="33" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F48" s="34">
         <v>0</v>
@@ -3638,10 +3670,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3649,16 +3681,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3668,10 +3700,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3679,16 +3711,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D50" s="28">
         <v>1</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
@@ -3698,10 +3730,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3709,14 +3741,14 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D51" s="28"/>
       <c r="E51" s="27" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -3726,10 +3758,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3753,12 +3785,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3774,267 +3806,267 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>242</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>240</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>237</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
+        <v>277</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>274</v>
+      </c>
+      <c r="D18" s="27" t="s">
         <v>275</v>
       </c>
-      <c r="B18" s="27" t="s">
-        <v>276</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>272</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>273</v>
-      </c>
       <c r="E18" s="27" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="B19" s="27" t="s">
         <v>278</v>
       </c>
-      <c r="B19" s="27" t="s">
-        <v>276</v>
-      </c>
       <c r="C19" s="25" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -4074,7 +4106,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -4085,330 +4117,344 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B4" s="42">
         <v>33</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B5" s="42">
         <v>372</v>
       </c>
       <c r="C5" s="43" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="44" t="s">
         <v>292</v>
-      </c>
-      <c r="D5" s="44" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B6" s="42">
         <v>207</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B7" s="42">
         <v>7</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B8" s="42">
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B9" s="42">
         <v>4</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B10" s="42">
         <v>35</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="D10" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B11" s="42">
         <v>37</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B12" s="42">
         <v>177</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B13" s="42">
         <v>9</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B14" s="42">
         <v>8</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B15" s="42">
+        <v>2</v>
+      </c>
+      <c r="C15" s="43" t="s">
+        <v>315</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="41" t="s">
+        <v>316</v>
+      </c>
+      <c r="B16" s="42">
         <v>0</v>
       </c>
-      <c r="C15" s="43" t="s">
-        <v>312</v>
-      </c>
-      <c r="D15" s="44" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>313</v>
-      </c>
-      <c r="B17" s="45">
+      <c r="C16" s="43" t="s">
+        <v>317</v>
+      </c>
+      <c r="D16" s="44" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="B18" s="45">
         <f>B6/B5</f>
         <v>0.5564516129032258</v>
       </c>
-      <c r="C17" s="46" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>315</v>
-      </c>
-      <c r="B18" s="47">
+      <c r="C18" s="46" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="B19" s="47">
         <f>B5-B6</f>
         <v>165</v>
       </c>
-      <c r="C18" s="46" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="40" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>320</v>
-      </c>
-      <c r="C23" s="21" t="s">
+      <c r="C19" s="46" t="s">
         <v>321</v>
       </c>
-      <c r="D23" s="21" t="s">
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="40" t="s">
         <v>322</v>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>323</v>
+        <v>122</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>327</v>
       </c>
-      <c r="B26" s="21" t="s">
-        <v>328</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>325</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>322</v>
-      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="39" t="s">
-        <v>329</v>
-      </c>
-      <c r="B27" s="38" t="s">
+      <c r="A27" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>333</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>330</v>
       </c>
-      <c r="C27" s="38" t="s">
-        <v>331</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>332</v>
+      <c r="D27" s="21" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B28" s="38" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C28" s="38" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="19" t="s">
-        <v>336</v>
-      </c>
-      <c r="B29" s="21" t="s">
+      <c r="A29" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="B29" s="38" t="s">
+        <v>339</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>340</v>
+      </c>
+      <c r="D29" s="38" t="s">
         <v>337</v>
       </c>
-      <c r="C29" s="21" t="s">
-        <v>338</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>339</v>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="19" t="s">
+        <v>341</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>342</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>343</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -4431,24 +4477,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4456,16 +4502,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4473,16 +4519,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4490,16 +4536,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>259</v>
+        <v>361</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4507,16 +4553,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4524,16 +4570,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4541,16 +4587,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="10" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4558,16 +4604,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
     </row>
     <row r="11" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4575,16 +4621,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tìm ra nguyên nhân lỗi 'báo đã lưu mà không lưu': tab chạy bản JS cũ
Phép thử có đối chứng trên luu_loi_giai, đếm trước = 207:
· viết 1 lời giải KHÔNG tải lại trang → dòng xanh, vẫn 207, n_tup_upd không đổi
· Ctrl+F5 rồi viết 2 lời giải      → dòng xanh, 209, n_tup_upd +2

SPA không tự nạp lại mã khi điều hướng nội bộ, nên tab mở từ trước lúc deploy
giữ bản JS cũ vô thời hạn; bản cũ gọi hàm cũ, và hàm cũ coi 'không lỗi' là
'đã lưu'. Cùng cơ chế giải thích chấm thẻ Flashcard (22/09) và luu_neo /
luu_loi_giai đầu tháng 9 — lỗi treo ba tuần.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="383">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>Dựng rồi gỡ cùng ngày theo quyết định chủ dự án. Vẫn 0.</t>
+  </si>
+  <si>
+    <t>23/09 — tìm ra nguyên nhân lỗi cũ</t>
+  </si>
+  <si>
+    <t>Phép thử đối chứng trên lưu lời giải: không tải lại trang → dòng xanh, database không đổi; Ctrl+F5 rồi viết hai lần → 207 lên 209. Nguyên nhân của cả ba lỗi 'báo lưu mà không lưu' là TAB CHẠY BẢN JS CŨ, không phải máy chủ.</t>
   </si>
   <si>
     <t>22/09 — lịch ôn lưu được</t>
@@ -1138,10 +1144,10 @@
     <t>Tài khoản học sinh đã làm bài đó — nhớ Ctrl+F5</t>
   </si>
   <si>
-    <t>Thử lại lưu lời giải và đặt neo qua giao diện giáo viên</t>
-  </si>
-  <si>
-    <t>Từ 22/09 cả hai có biên nhận (migration 092): nếu lỗi « báo lưu mà không lưu » còn sống, màn hình sẽ hiện chữ đỏ kèm biên nhận thay vì dòng xanh. Chỉ cần viết thử một lời giải và đặt thử một neo, rồi báo lại màu dòng chữ.</t>
+    <t>Đặt thử một neo qua giao diện giáo viên</t>
+  </si>
+  <si>
+    <t>Lưu lời giải đã thử xong 23/09 và LƯU ĐƯỢC (207→209). Còn đường đặt neo chưa thử qua giao diện. Nhớ Ctrl+F5 trước — nguyên nhân của cả loạt lỗi cũ chính là tab chạy bản JS cũ.</t>
   </si>
   <si>
     <t>/professeur/loi-giai và /professeur/neo</t>
@@ -1792,7 +1798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2243,8 +2249,21 @@
       <c r="F34" s="18"/>
       <c r="G34" s="18"/>
     </row>
+    <row r="35" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2253,6 +2272,7 @@
     <mergeCell ref="B32:G32"/>
     <mergeCell ref="B33:G33"/>
     <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B35:G35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2280,28 +2300,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2309,16 +2329,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2328,10 +2348,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2339,14 +2359,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2356,10 +2376,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2367,16 +2387,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2386,10 +2406,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2397,16 +2417,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2416,10 +2436,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2427,16 +2447,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2446,10 +2466,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2457,16 +2477,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2476,10 +2496,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2487,14 +2507,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2504,10 +2524,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2515,7 +2535,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2524,7 +2544,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2534,10 +2554,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2545,16 +2565,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2564,10 +2584,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2575,14 +2595,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2592,10 +2612,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2603,14 +2623,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2620,10 +2640,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2631,14 +2651,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2648,10 +2668,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2659,14 +2679,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2676,10 +2696,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2687,14 +2707,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2704,10 +2724,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2715,16 +2735,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2734,10 +2754,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2745,16 +2765,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2764,10 +2784,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2775,14 +2795,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2792,10 +2812,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2803,16 +2823,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2822,10 +2842,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2833,16 +2853,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2852,10 +2872,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2863,16 +2883,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2882,10 +2902,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2893,14 +2913,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2910,10 +2930,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2921,16 +2941,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -2940,10 +2960,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2951,14 +2971,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -2968,10 +2988,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2979,14 +2999,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -2996,10 +3016,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3007,16 +3027,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3026,10 +3046,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3037,16 +3057,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -3056,10 +3076,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3067,14 +3087,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -3084,10 +3104,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3095,14 +3115,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3112,10 +3132,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3123,14 +3143,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3140,10 +3160,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3151,14 +3171,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3168,10 +3188,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3179,14 +3199,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3196,10 +3216,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3207,14 +3227,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3224,10 +3244,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3235,16 +3255,16 @@
         <v>15</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D34" s="22">
         <v>2</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F34" s="22">
         <v>2</v>
@@ -3254,10 +3274,10 @@
         <v>hoà</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3265,16 +3285,16 @@
         <v>15</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D35" s="34">
         <v>2</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F35" s="34">
         <v>0</v>
@@ -3284,10 +3304,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3295,16 +3315,16 @@
         <v>15</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D36" s="22">
         <v>2</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F36" s="22">
         <v>2</v>
@@ -3314,10 +3334,10 @@
         <v>hoà</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3325,16 +3345,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D37" s="34">
         <v>2</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F37" s="34">
         <v>0</v>
@@ -3344,10 +3364,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3355,16 +3375,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F38" s="22">
         <v>1</v>
@@ -3374,10 +3394,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3385,14 +3405,14 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3402,10 +3422,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3413,16 +3433,16 @@
         <v>16</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3432,10 +3452,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3443,16 +3463,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3462,10 +3482,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3473,16 +3493,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3492,10 +3512,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3503,16 +3523,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3522,10 +3542,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3533,16 +3553,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D44" s="28">
         <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3552,10 +3572,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3563,14 +3583,14 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3580,10 +3600,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3591,16 +3611,16 @@
         <v>17</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3610,10 +3630,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3621,16 +3641,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3640,10 +3660,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3654,13 +3674,13 @@
         <v>37</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D48" s="34">
         <v>2</v>
       </c>
       <c r="E48" s="33" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F48" s="34">
         <v>0</v>
@@ -3670,10 +3690,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3681,16 +3701,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3700,10 +3720,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3711,16 +3731,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D50" s="28">
         <v>1</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
@@ -3730,10 +3750,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3741,14 +3761,14 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D51" s="28"/>
       <c r="E51" s="27" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -3758,10 +3778,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -3785,12 +3805,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3806,267 +3826,267 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>244</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>239</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>276</v>
+      </c>
+      <c r="D18" s="27" t="s">
         <v>277</v>
       </c>
-      <c r="B18" s="27" t="s">
-        <v>278</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>274</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>275</v>
-      </c>
       <c r="E18" s="27" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="B19" s="27" t="s">
         <v>280</v>
       </c>
-      <c r="B19" s="27" t="s">
-        <v>278</v>
-      </c>
       <c r="C19" s="25" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -4117,344 +4137,344 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B4" s="42">
         <v>33</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B5" s="42">
         <v>372</v>
       </c>
       <c r="C5" s="43" t="s">
+        <v>296</v>
+      </c>
+      <c r="D5" s="44" t="s">
         <v>294</v>
-      </c>
-      <c r="D5" s="44" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B6" s="42">
         <v>207</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B7" s="42">
         <v>7</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B8" s="42">
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B9" s="42">
         <v>4</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B10" s="42">
         <v>35</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D10" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B11" s="42">
         <v>37</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B12" s="42">
         <v>177</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B13" s="42">
         <v>9</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B14" s="42">
         <v>8</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B15" s="42">
         <v>2</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D15" s="44" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="41" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B16" s="42">
         <v>0</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D16" s="44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B18" s="45">
         <f>B6/B5</f>
         <v>0.5564516129032258</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B19" s="47">
         <f>B5-B6</f>
         <v>165</v>
       </c>
       <c r="C19" s="46" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="23" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B25" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>329</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
+        <v>333</v>
+      </c>
+      <c r="B26" s="21" t="s">
         <v>331</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="C26" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>329</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
+        <v>334</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>335</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>332</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>333</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>330</v>
-      </c>
       <c r="D27" s="21" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B28" s="38" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C28" s="38" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B29" s="38" t="s">
+        <v>341</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>342</v>
+      </c>
+      <c r="D29" s="38" t="s">
         <v>339</v>
-      </c>
-      <c r="C29" s="38" t="s">
-        <v>340</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -4477,24 +4497,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4502,16 +4522,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4519,16 +4539,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4536,16 +4556,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C6" s="21" t="s">
+        <v>362</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>363</v>
+      </c>
+      <c r="E6" s="21" t="s">
         <v>360</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>361</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4553,16 +4573,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4570,16 +4590,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4587,16 +4607,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="10" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4604,16 +4624,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="11" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4621,16 +4641,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 209 câu có lời giải (hai lời giải viết 23/09)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -296,7 +296,7 @@
     <t>Không thấy nêu trên trang chủ</t>
   </si>
   <si>
-    <t>207/372 câu có lời giải; có màn xếp ưu tiên theo SỐ HỌC SINH từng sai</t>
+    <t>209/372 câu có lời giải; có màn xếp ưu tiên theo SỐ HỌC SINH từng sai</t>
   </si>
   <si>
     <t>migration 069/070; /professeur/loi-giai</t>
@@ -4187,7 +4187,7 @@
         <v>297</v>
       </c>
       <c r="B6" s="42">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C6" s="43" t="s">
         <v>298</v>
@@ -4342,7 +4342,7 @@
       </c>
       <c r="B18" s="45">
         <f>B6/B5</f>
-        <v>0.5564516129032258</v>
+        <v>0.5618279569892473</v>
       </c>
       <c r="C18" s="46" t="s">
         <v>321</v>
@@ -4354,7 +4354,7 @@
       </c>
       <c r="B19" s="47">
         <f>B5-B6</f>
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C19" s="46" t="s">
         <v>323</v>

</xml_diff>

<commit_message>
Đặt neo qua giao diện đã chạy đúng — bằng chứng thứ hai cho nguyên nhân tab cũ
Đặt neo ở tab chưa tải lại → dòng xanh, 7 neo không đổi một ký tự. Ctrl+F5
ngay tại /professeur/neo rồi đặt lại → dòng xanh, và nội dung bẫy của câu
mrhsyo85dbrcvp đổi đúng như vừa sửa.

Mỗi tab giữ riêng bản mã: hôm qua tải lại ở màn lời giải không làm mới tab
đang mở màn neo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="383">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>Dựng rồi gỡ cùng ngày theo quyết định chủ dự án. Vẫn 0.</t>
+  </si>
+  <si>
+    <t>23/09 — cả hai đường ghi của giáo viên đã thử xong</t>
+  </si>
+  <si>
+    <t>Lưu lời giải: 207→209. Đặt neo: lần đầu (tab cũ) không ghi gì, sau Ctrl+F5 ngay tại trang đó thì ghi đúng. Mỗi tab giữ riêng bản mã của nó.</t>
   </si>
   <si>
     <t>23/09 — tìm ra nguyên nhân lỗi cũ</t>
@@ -1144,16 +1150,10 @@
     <t>Tài khoản học sinh đã làm bài đó — nhớ Ctrl+F5</t>
   </si>
   <si>
-    <t>Đặt thử một neo qua giao diện giáo viên</t>
-  </si>
-  <si>
-    <t>Lưu lời giải đã thử xong 23/09 và LƯU ĐƯỢC (207→209). Còn đường đặt neo chưa thử qua giao diện. Nhớ Ctrl+F5 trước — nguyên nhân của cả loạt lỗi cũ chính là tab chạy bản JS cũ.</t>
-  </si>
-  <si>
-    <t>/professeur/loi-giai và /professeur/neo</t>
-  </si>
-  <si>
-    <t>10 phút</t>
+    <t>Mở lại bộ Flashcard hôm nay (23/09)</t>
+  </si>
+  <si>
+    <t>Hai thẻ đã chấm hôm qua hẹn ôn đúng hôm nay. Chúng hiện lại thì lịch ôn đã chạy trọn một vòng — mốc cuối cùng chưa ai thấy.</t>
   </si>
   <si>
     <t>Quyết số phận /professeur/oral</t>
@@ -1798,7 +1798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2262,8 +2262,21 @@
       <c r="F35" s="18"/>
       <c r="G35" s="18"/>
     </row>
+    <row r="36" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2273,6 +2286,7 @@
     <mergeCell ref="B33:G33"/>
     <mergeCell ref="B34:G34"/>
     <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B36:G36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2300,28 +2314,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2329,16 +2343,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2348,10 +2362,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2359,14 +2373,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2376,10 +2390,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2387,16 +2401,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2406,10 +2420,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2417,16 +2431,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2436,10 +2450,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2447,16 +2461,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2466,10 +2480,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2477,16 +2491,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2496,10 +2510,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2507,14 +2521,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2524,10 +2538,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2535,7 +2549,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2544,7 +2558,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2554,10 +2568,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2565,16 +2579,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2584,10 +2598,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2595,14 +2609,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2612,10 +2626,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2623,14 +2637,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2640,10 +2654,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2651,14 +2665,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2668,10 +2682,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2679,14 +2693,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2696,10 +2710,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2707,14 +2721,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2724,10 +2738,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2735,16 +2749,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2754,10 +2768,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2765,16 +2779,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2784,10 +2798,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2795,14 +2809,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2812,10 +2826,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2823,16 +2837,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2842,10 +2856,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2853,16 +2867,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2872,10 +2886,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2883,16 +2897,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2902,10 +2916,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2913,14 +2927,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2930,10 +2944,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2941,16 +2955,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -2960,10 +2974,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2971,14 +2985,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -2988,10 +3002,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2999,14 +3013,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3016,10 +3030,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3027,16 +3041,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3046,10 +3060,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3057,16 +3071,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -3076,10 +3090,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3087,14 +3101,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -3104,10 +3118,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3115,14 +3129,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3132,10 +3146,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3143,14 +3157,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3160,10 +3174,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3171,14 +3185,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3188,10 +3202,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3199,14 +3213,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3216,10 +3230,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3227,14 +3241,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3244,10 +3258,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3255,16 +3269,16 @@
         <v>15</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D34" s="22">
         <v>2</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F34" s="22">
         <v>2</v>
@@ -3274,10 +3288,10 @@
         <v>hoà</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3285,16 +3299,16 @@
         <v>15</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D35" s="34">
         <v>2</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F35" s="34">
         <v>0</v>
@@ -3304,10 +3318,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3315,16 +3329,16 @@
         <v>15</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D36" s="22">
         <v>2</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F36" s="22">
         <v>2</v>
@@ -3334,10 +3348,10 @@
         <v>hoà</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3345,16 +3359,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D37" s="34">
         <v>2</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F37" s="34">
         <v>0</v>
@@ -3364,10 +3378,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3375,16 +3389,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F38" s="22">
         <v>1</v>
@@ -3394,10 +3408,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3405,14 +3419,14 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3422,10 +3436,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3433,16 +3447,16 @@
         <v>16</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3452,10 +3466,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3463,16 +3477,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3482,10 +3496,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3493,16 +3507,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3512,10 +3526,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3523,16 +3537,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3542,10 +3556,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3553,16 +3567,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D44" s="28">
         <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3572,10 +3586,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3583,14 +3597,14 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3600,10 +3614,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3611,16 +3625,16 @@
         <v>17</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3630,10 +3644,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3641,16 +3655,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3660,10 +3674,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3674,13 +3688,13 @@
         <v>37</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D48" s="34">
         <v>2</v>
       </c>
       <c r="E48" s="33" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F48" s="34">
         <v>0</v>
@@ -3690,10 +3704,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3701,16 +3715,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3720,10 +3734,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3731,16 +3745,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D50" s="28">
         <v>1</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
@@ -3750,10 +3764,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3761,14 +3775,14 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D51" s="28"/>
       <c r="E51" s="27" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -3778,10 +3792,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -3805,12 +3819,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3826,267 +3840,267 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>244</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>241</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>278</v>
+      </c>
+      <c r="D18" s="27" t="s">
         <v>279</v>
       </c>
-      <c r="B18" s="27" t="s">
-        <v>280</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>276</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>277</v>
-      </c>
       <c r="E18" s="27" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="B19" s="27" t="s">
         <v>282</v>
       </c>
-      <c r="B19" s="27" t="s">
-        <v>280</v>
-      </c>
       <c r="C19" s="25" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -4137,344 +4151,344 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B4" s="42">
         <v>33</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B5" s="42">
         <v>372</v>
       </c>
       <c r="C5" s="43" t="s">
+        <v>298</v>
+      </c>
+      <c r="D5" s="44" t="s">
         <v>296</v>
-      </c>
-      <c r="D5" s="44" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B6" s="42">
         <v>209</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B7" s="42">
         <v>7</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B8" s="42">
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B9" s="42">
         <v>4</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B10" s="42">
         <v>35</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D10" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B11" s="42">
         <v>37</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B12" s="42">
         <v>177</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B13" s="42">
         <v>9</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B14" s="42">
         <v>8</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B15" s="42">
         <v>2</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D15" s="44" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="41" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B16" s="42">
         <v>0</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D16" s="44" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B18" s="45">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B19" s="47">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C19" s="46" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B25" s="21" t="s">
+        <v>333</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>331</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>332</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
+        <v>335</v>
+      </c>
+      <c r="B26" s="21" t="s">
         <v>333</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="C26" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>331</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>332</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
+        <v>336</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>337</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>334</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>335</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>332</v>
-      </c>
       <c r="D27" s="21" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B28" s="38" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C28" s="38" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B29" s="38" t="s">
+        <v>343</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>344</v>
+      </c>
+      <c r="D29" s="38" t="s">
         <v>341</v>
-      </c>
-      <c r="C29" s="38" t="s">
-        <v>342</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -4497,24 +4511,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4522,16 +4536,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4539,16 +4553,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4556,16 +4570,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C6" s="21" t="s">
+        <v>364</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>365</v>
+      </c>
+      <c r="E6" s="21" t="s">
         <v>362</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>363</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4573,16 +4587,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4590,16 +4604,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Ghi lại việc dọn 23/09: gỡ màn nghe bài nói, xoá hai tài khoản thử
Hai tài khoản thử xoá kèm 41 lượt làm bài, 50 câu trả lời, 36 thẻ + 36 lịch
ôn, 2 thông báo, 1 ngày học, và 3 bài nộp — xoá tường minh vì
submissions.user_id là SET NULL, để nguyên thì thành bài nộp không chủ. Sao
lưu JSON trước khi xoá, để ngoài git vì chứa email người thật.

Còn 5 tài khoản auth không có hồ sơ — ghi vào việc cần làm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="373">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>Dựng rồi gỡ cùng ngày theo quyết định chủ dự án. Vẫn 0.</t>
+  </si>
+  <si>
+    <t>23/09 — dọn và sửa đáp án phía học sinh</t>
+  </si>
+  <si>
+    <t>Sửa lỗi đáp án rỗng với học sinh (tô màu, điểm, điền từ, bảng, sắp xếp); 4 câu sắp xếp mang đáp án bị xáo, đã ghi lại. Gỡ /professeur/oral, xoá hai tài khoản thử, điền email liên hệ.</t>
   </si>
   <si>
     <t>23/09 — cả hai đường ghi của giáo viên đã thử xong</t>
@@ -1111,7 +1117,7 @@
     <t>Đặt khoá API để bật chấm PE bằng AI</t>
   </si>
   <si>
-    <t>Vẫn là việc rẻ nhất có tác động lớn nhất: mọi thứ đã dựng và đã kiểm, chỉ thiếu một khoá.</t>
+    <t>Chủ dự án tạm gác 23/09. Mọi thứ đã dựng và kiểm; thiếu khoá thì nút « Xin gợi ý » báo tính năng chưa bật, không lỗi.</t>
   </si>
   <si>
     <t>npx supabase secrets set ANTHROPIC_API_KEY=sk-ant-…</t>
@@ -1120,64 +1126,16 @@
     <t>5 phút</t>
   </si>
   <si>
-    <t>Điền email liên hệ cho FAQ và Điều khoản</t>
-  </si>
-  <si>
-    <t>Cả hai trang tự hiện cảnh báo vàng cho tới khi có email.</t>
-  </si>
-  <si>
-    <t>EMAIL_LIEN_HE trong src/screens/public/TrangPhapLy.jsx</t>
-  </si>
-  <si>
-    <t>2 phút</t>
-  </si>
-  <si>
-    <t>Mai (23/09) mở lại bộ « Thông báo ở nhà ga »</t>
-  </si>
-  <si>
-    <t>Hai thẻ đã chấm hẹn ôn ngày 23/09. Nếu chúng hiện lại đúng ngày đó thì lịch ôn đã chạy trọn một vòng — lần đầu tiên.</t>
-  </si>
-  <si>
-    <t>/etudiant/bo-the — nhớ Ctrl+F5</t>
-  </si>
-  <si>
-    <t>Xem neo từ phía học sinh</t>
-  </si>
-  <si>
-    <t>Phía máy chủ đã đo xong 22/09: chạy đúng hàm tô sáng của app trên văn bản + neo thật, 11/11 mảnh khớp từng ký tự. Còn thiếu một lần nhìn bằng mắt: mở phần chữa bài bằng tài khoản đã làm bài đó.</t>
-  </si>
-  <si>
-    <t>Tài khoản học sinh đã làm bài đó — nhớ Ctrl+F5</t>
-  </si>
-  <si>
-    <t>Mở lại bộ Flashcard hôm nay (23/09)</t>
-  </si>
-  <si>
-    <t>Hai thẻ đã chấm hôm qua hẹn ôn đúng hôm nay. Chúng hiện lại thì lịch ôn đã chạy trọn một vòng — mốc cuối cùng chưa ai thấy.</t>
-  </si>
-  <si>
-    <t>Quyết số phận /professeur/oral</t>
-  </si>
-  <si>
-    <t>Màn nghe bài nói không cho điểm, chỉ nghe và nhắn nhận xét.</t>
-  </si>
-  <si>
-    <t>App.jsx; BaiNoiGiaoVien.jsx; navItems.js</t>
-  </si>
-  <si>
-    <t>1 buổi, sau khi quyết</t>
-  </si>
-  <si>
-    <t>Dọn hoặc giữ hai tài khoản thử</t>
-  </si>
-  <si>
-    <t>7 trong 8 « bài tự luận chưa chấm » thuộc về chúng, và chúng làm lệch mọi con số về học sinh.</t>
-  </si>
-  <si>
-    <t>Quyết định — xoá tài khoản là việc không hoàn lại</t>
-  </si>
-  <si>
-    <t>quyết định</t>
+    <t>Xem 5 tài khoản không có hồ sơ</t>
+  </si>
+  <si>
+    <t>14 tài khoản đăng nhập nhưng chỉ 9 hồ sơ. Có thể là tài khoản thử khác, hoặc người đăng ký dở — chưa ai xem.</t>
+  </si>
+  <si>
+    <t>Quyết định sau khi xem danh sách</t>
+  </si>
+  <si>
+    <t>10 phút</t>
   </si>
   <si>
     <t>Cân nhắc dựng lại Chính sách bảo mật trước khi thu tiền nhiều</t>
@@ -1190,6 +1148,18 @@
   </si>
   <si>
     <t>30 phút</t>
+  </si>
+  <si>
+    <t>Cân nhắc KHÔNG đuổi theo: từ điển, podcast, PvP, app mobile</t>
+  </si>
+  <si>
+    <t>Bốn ô Vivoire hơn tuyệt đối. Đuổi theo cả bốn với một người là cách chắc chắn để không ô nào xong.</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>quyết định, không phải mã</t>
   </si>
 </sst>
 </file>
@@ -1798,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2275,8 +2245,21 @@
       <c r="F36" s="18"/>
       <c r="G36" s="18"/>
     </row>
+    <row r="37" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2287,6 +2270,7 @@
     <mergeCell ref="B34:G34"/>
     <mergeCell ref="B35:G35"/>
     <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B37:G37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2314,28 +2298,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2343,16 +2327,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2362,10 +2346,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2373,14 +2357,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2390,10 +2374,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2401,16 +2385,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2420,10 +2404,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2431,16 +2415,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2450,10 +2434,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2461,16 +2445,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2480,10 +2464,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2491,16 +2475,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2510,10 +2494,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2521,14 +2505,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2538,10 +2522,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2549,7 +2533,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2558,7 +2542,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2568,10 +2552,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2579,16 +2563,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2598,10 +2582,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2609,14 +2593,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2626,10 +2610,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2637,14 +2621,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2654,10 +2638,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2665,14 +2649,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2682,10 +2666,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2693,14 +2677,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2710,10 +2694,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2721,14 +2705,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2738,10 +2722,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2749,16 +2733,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2768,10 +2752,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2779,16 +2763,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2798,10 +2782,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2809,14 +2793,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2826,10 +2810,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2837,16 +2821,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2856,10 +2840,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2867,16 +2851,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2886,10 +2870,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2897,16 +2881,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2916,10 +2900,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2927,14 +2911,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2944,10 +2928,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2955,16 +2939,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -2974,10 +2958,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2985,14 +2969,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -3002,10 +2986,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3013,14 +2997,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3030,10 +3014,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3041,16 +3025,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3060,10 +3044,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3071,16 +3055,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -3090,10 +3074,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3101,14 +3085,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -3118,10 +3102,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3129,14 +3113,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3146,10 +3130,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3157,14 +3141,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3174,10 +3158,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3185,14 +3169,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3202,10 +3186,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3213,14 +3197,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3230,10 +3214,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3241,14 +3225,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3258,10 +3242,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3269,16 +3253,16 @@
         <v>15</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D34" s="22">
         <v>2</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F34" s="22">
         <v>2</v>
@@ -3288,10 +3272,10 @@
         <v>hoà</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3299,16 +3283,16 @@
         <v>15</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D35" s="34">
         <v>2</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F35" s="34">
         <v>0</v>
@@ -3318,10 +3302,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3329,16 +3313,16 @@
         <v>15</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D36" s="22">
         <v>2</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F36" s="22">
         <v>2</v>
@@ -3348,10 +3332,10 @@
         <v>hoà</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3359,16 +3343,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D37" s="34">
         <v>2</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F37" s="34">
         <v>0</v>
@@ -3378,10 +3362,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3389,16 +3373,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F38" s="22">
         <v>1</v>
@@ -3408,10 +3392,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3419,14 +3403,14 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3436,10 +3420,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3447,16 +3431,16 @@
         <v>16</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3466,10 +3450,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3477,16 +3461,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3496,10 +3480,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3507,16 +3491,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3526,10 +3510,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3537,16 +3521,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3556,10 +3540,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3567,16 +3551,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D44" s="28">
         <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3586,10 +3570,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3597,14 +3581,14 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3614,10 +3598,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3625,16 +3609,16 @@
         <v>17</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3644,10 +3628,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3655,16 +3639,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3674,10 +3658,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3688,13 +3672,13 @@
         <v>37</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D48" s="34">
         <v>2</v>
       </c>
       <c r="E48" s="33" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F48" s="34">
         <v>0</v>
@@ -3704,10 +3688,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3715,16 +3699,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3734,10 +3718,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3745,16 +3729,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D50" s="28">
         <v>1</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
@@ -3764,10 +3748,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3775,14 +3759,14 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D51" s="28"/>
       <c r="E51" s="27" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -3792,10 +3776,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -3819,12 +3803,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3840,267 +3824,267 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>243</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="D18" s="27" t="s">
         <v>281</v>
       </c>
-      <c r="B18" s="27" t="s">
-        <v>282</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>278</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>279</v>
-      </c>
       <c r="E18" s="27" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
+        <v>286</v>
+      </c>
+      <c r="B19" s="27" t="s">
         <v>284</v>
       </c>
-      <c r="B19" s="27" t="s">
-        <v>282</v>
-      </c>
       <c r="C19" s="25" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -4151,344 +4135,344 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B4" s="42">
         <v>33</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B5" s="42">
         <v>372</v>
       </c>
       <c r="C5" s="43" t="s">
+        <v>300</v>
+      </c>
+      <c r="D5" s="44" t="s">
         <v>298</v>
-      </c>
-      <c r="D5" s="44" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B6" s="42">
         <v>209</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B7" s="42">
         <v>7</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B8" s="42">
         <v>2</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B9" s="42">
         <v>4</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B10" s="42">
         <v>35</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D10" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B11" s="42">
         <v>37</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B12" s="42">
         <v>177</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B13" s="42">
         <v>9</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B14" s="42">
         <v>8</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B15" s="42">
         <v>2</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D15" s="44" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="41" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B16" s="42">
         <v>0</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D16" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B18" s="45">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B19" s="47">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C19" s="46" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="23" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B25" s="21" t="s">
+        <v>335</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>336</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>333</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>334</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
+        <v>337</v>
+      </c>
+      <c r="B26" s="21" t="s">
         <v>335</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="C26" s="21" t="s">
+        <v>336</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>333</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>334</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>336</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>334</v>
-      </c>
       <c r="D27" s="21" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B28" s="38" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C28" s="38" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B29" s="38" t="s">
+        <v>345</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>346</v>
+      </c>
+      <c r="D29" s="38" t="s">
         <v>343</v>
-      </c>
-      <c r="C29" s="38" t="s">
-        <v>344</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
   </sheetData>
@@ -4499,7 +4483,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -4511,24 +4495,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4536,16 +4520,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4553,16 +4537,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4570,16 +4554,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4587,84 +4571,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="22">
-        <v>5</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>369</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>370</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>365</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="22">
-        <v>6</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>371</v>
-      </c>
-      <c r="C9" s="21" t="s">
         <v>372</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="10" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="22">
-        <v>7</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>375</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>376</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>377</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="11" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="22">
-        <v>8</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>379</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>380</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>381</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>382</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật bảng so sánh: số liệu đo 24/09, neo 22, gỡ màn nghe + nút tài khoản, Thống kê mới, hai lỗi lưu bài
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="387">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -129,7 +129,7 @@
     <t>Chưa kiểm chứng được — KHÔNG tính vào trung bình</t>
   </si>
   <si>
-    <t>ĐÃ ĐỔI GÌ SO VỚI BẢN 09/09 — bản này đo 21/09/2026</t>
+    <t>ĐÃ ĐỔI GÌ SO VỚI BẢN 09/09 — bản này đo 24/09/2026</t>
   </si>
   <si>
     <t>Chấm PE bằng AI</t>
@@ -184,6 +184,18 @@
   </si>
   <si>
     <t>Neo 1→2: 7 câu có neo thật. Flashcard cơ chế 1→2: có lại lịch ôn SM-2. Ba bộ nháp cho Đọc/Viết/Nói. Và SỬA LẠI một con số: « 8 bài tự luận học sinh đang chờ » — 7 bài là tài khoản thử của chủ dự án.</t>
+  </si>
+  <si>
+    <t>24/09 — hai lỗi mất dữ liệu khi LƯU BÀI</t>
+  </si>
+  <si>
+    <t>Lưu bài xoá rồi chèn lại câu hỏi, nên (1) xoá sạch neo — 7 neo mất, đã khôi phục; (2) xoá lịch sử trả lời của học sinh qua ON DELETE CASCADE — answers còn 57 thay vì 127, KHÔNG khôi phục được. Cả hai đã sửa. Câu hỏi 372→353 và lời giải 209→188 chưa rõ nguyên nhân.</t>
+  </si>
+  <si>
+    <t>24/09 — giao diện</t>
+  </si>
+  <si>
+    <t>Khách chưa đăng nhập vào thẳng trang giới thiệu. Gỡ khối « Lớp của bạn » ở thanh bên. Màn Thống kê dựng lại bằng số liệu thật.</t>
   </si>
   <si>
     <t>Số liệu trôi</t>
@@ -308,7 +320,7 @@
     <t>Không thấy nêu trên trang chủ</t>
   </si>
   <si>
-    <t>209/372 câu có lời giải; có màn xếp ưu tiên theo SỐ HỌC SINH từng sai</t>
+    <t>188/353 câu có lời giải (đo 24/09); có màn xếp ưu tiên theo SỐ HỌC SINH từng sai</t>
   </si>
   <si>
     <t>migration 069/070; /professeur/loi-giai</t>
@@ -317,7 +329,7 @@
     <t>Neo đáp án vào ngữ liệu (chỉ ra CHỖ chứa câu trả lời)</t>
   </si>
   <si>
-    <t>Có dữ liệu thật từ 21/09: 7 câu của bài « L'impact des locations saisonnières » có neo, kèm 4 bẫy giải thích vì sao đáp án sai dụ người ta</t>
+    <t>22 câu trên 2 bài đọc có neo (7 câu « L'impact des locations saisonnières » + 15 câu « Dans le Gard… »), kèm 17 bẫy. 24/09: lưu bài không còn xoá neo</t>
   </si>
   <si>
     <t>Đang chạy — có dữ liệu</t>
@@ -410,7 +422,7 @@
     <t>33 bài (ĐẾM THẬT trên production)</t>
   </si>
   <si>
-    <t>select count(*) from exercises = 33, đo 21/09/2026 (09/09 là 34)</t>
+    <t>select count(*) from exercises = 33, đo 24/09/2026 (09/09 là 34)</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -422,7 +434,7 @@
     <t>372 câu, 7 dạng (qcm, fill, conj, vf, tableau, order, tự luận)</t>
   </si>
   <si>
-    <t>select count(*) from questions = 372, đo 21/09/2026</t>
+    <t>select count(*) from questions = 353, đo 24/09/2026</t>
   </si>
   <si>
     <t>Từ điển Pháp–Việt</t>
@@ -635,7 +647,7 @@
     <t>9 người dùng (gồm cả tài khoản thử)</t>
   </si>
   <si>
-    <t>select count(*) from profiles = 9, đo 21/09/2026</t>
+    <t>select count(*) from profiles = 10, đo 24/09/2026</t>
   </si>
   <si>
     <t>Web</t>
@@ -830,10 +842,10 @@
     <t>/professeur/neo</t>
   </si>
   <si>
-    <t>Dựng xong, 0 dữ liệu</t>
-  </si>
-  <si>
-    <t>Chưa câu nào có neo nên chưa ai từng thấy nó chạy, kể cả chủ dự án.</t>
+    <t>Đang chạy — 22 neo</t>
+  </si>
+  <si>
+    <t>Chủ dự án đã đặt neo qua giao diện 23/09. Lưu bài trong Builder từng xoá sạch neo — sửa 23/09 (093/094).</t>
   </si>
   <si>
     <t>Sổ tay / mẹo</t>
@@ -869,22 +881,43 @@
     <t>/professeur/oral</t>
   </si>
   <si>
-    <t>CẦN QUYẾT</t>
-  </si>
-  <si>
-    <t>Màn này KHÔNG cho điểm, chỉ nghe và nhắn nhận xét. Bỏ hẳn vai chấm thì nên gỡ; giữ vai kèm cặp thì giữ. Đây là ranh giới cần chủ dự án quyết.</t>
+    <t>ĐÃ GỠ</t>
+  </si>
+  <si>
+    <t>Không còn trong mã</t>
+  </si>
+  <si>
+    <t>Gỡ 23/09 theo quyết định chủ dự án. Học sinh vẫn ghi âm để tự nghe lại.</t>
+  </si>
+  <si>
+    <t>Tạo / xoá tài khoản học sinh</t>
+  </si>
+  <si>
+    <t>/professeur (Theo dõi học sinh)</t>
+  </si>
+  <si>
+    <t>Không còn nút</t>
+  </si>
+  <si>
+    <t>Gỡ 24/09: ô « Créer le compte » và nút « Supprimer ». Học sinh tự đăng ký; giáo viên chỉ theo dõi, xếp lớp, gửi link đổi mật khẩu.</t>
+  </si>
+  <si>
+    <t>Thống kê lớp</t>
+  </si>
+  <si>
+    <t>/professeur (Thống kê)</t>
+  </si>
+  <si>
+    <t>GIỮ — DỰNG LẠI</t>
+  </si>
+  <si>
+    <t>Dựng lại 24/09: KPI, phân bố điểm, TB theo kỹ năng, top học sinh, bảng xu hướng. Màn cũ đọc kho bài giao gần như rỗng nên hiện 0/0; nay đọc lượt làm bài thật.</t>
   </si>
   <si>
     <t>Chấm bài viết của học sinh</t>
   </si>
   <si>
     <t>/professeur/copies</t>
-  </si>
-  <si>
-    <t>ĐÃ GỠ</t>
-  </si>
-  <si>
-    <t>Không còn trong mã</t>
   </si>
   <si>
     <t>Gỡ 09/09/2026: route, mục menu, PEGrading.jsx và khoá nav.grading ở cả bốn từ điển. Gỡ CẢ mục menu chứ không giấu lối vào — check:nav bắt lỗi route không ai vào được.</t>
@@ -943,19 +976,22 @@
     <t>Câu hỏi</t>
   </si>
   <si>
-    <t>select count(*) from questions</t>
+    <t>select count(*) from questions — giảm 19, chưa rõ vì sao</t>
+  </si>
+  <si>
+    <t>24/09/2026</t>
   </si>
   <si>
     <t>Câu có lời giải thích</t>
   </si>
   <si>
-    <t>questions where explanation is not null</t>
+    <t>questions where explanation is not null — giảm 21, chưa rõ vì sao</t>
   </si>
   <si>
     <t>Câu có neo ngữ liệu</t>
   </si>
   <si>
-    <t>questions where evidence is not null</t>
+    <t>questions where evidence is not null — trên 2 bài</t>
   </si>
   <si>
     <t>Đề thi thử</t>
@@ -964,6 +1000,12 @@
     <t>select count(*) from exams</t>
   </si>
   <si>
+    <t>Lượt làm bài đã chấm</t>
+  </si>
+  <si>
+    <t>attempts where finished_at is not null</t>
+  </si>
+  <si>
     <t>Bộ Flashcard (cả bốn công khai)</t>
   </si>
   <si>
@@ -979,16 +1021,16 @@
     <t>select count(*) from the_bo_the</t>
   </si>
   <si>
-    <t>Thẻ SM-2 cũ (không màn nào mở)</t>
-  </si>
-  <si>
-    <t>select count(*) from cards</t>
+    <t>Thẻ trong bảng cards</t>
+  </si>
+  <si>
+    <t>select count(*) from cards — 36 thẻ đi theo hai tài khoản thử đã xoá</t>
   </si>
   <si>
     <t>Lượt trả lời đã ghi</t>
   </si>
   <si>
-    <t>select count(*) from answers</t>
+    <t>select count(*) from answers — 50 đi theo tài khoản thử, ~70 mất vì lỗi lưu bài (đã sửa)</t>
   </si>
   <si>
     <t>Tài khoản</t>
@@ -1006,7 +1048,7 @@
     <t>Lượt ôn Flashcard đã ghi</t>
   </si>
   <si>
-    <t>reviews có reps &gt; 0 trên thẻ bo_giao_vien</t>
+    <t>reviews có reps &gt; 0 trên thẻ bo_giao_vien — 2 lượt cũ thuộc tài khoản thử đã xoá</t>
   </si>
   <si>
     <t>Gợi ý chấm AI đã sinh</t>
@@ -1403,12 +1445,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1428,6 +1464,12 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1768,7 +1810,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2258,8 +2300,34 @@
       <c r="F37" s="18"/>
       <c r="G37" s="18"/>
     </row>
+    <row r="38" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+    </row>
+    <row r="39" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="13">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2271,6 +2339,8 @@
     <mergeCell ref="B35:G35"/>
     <mergeCell ref="B36:G36"/>
     <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2298,28 +2368,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2327,16 +2397,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2346,10 +2416,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2357,14 +2427,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2374,10 +2444,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2385,16 +2455,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2404,10 +2474,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2415,16 +2485,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2434,10 +2504,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2445,16 +2515,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2464,10 +2534,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2475,16 +2545,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2494,10 +2564,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2505,14 +2575,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2522,10 +2592,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2533,7 +2603,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2542,7 +2612,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2552,10 +2622,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2563,16 +2633,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2582,10 +2652,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2593,14 +2663,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2610,10 +2680,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2621,14 +2691,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2638,10 +2708,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2649,14 +2719,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2666,10 +2736,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2677,14 +2747,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2694,10 +2764,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2705,14 +2775,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2722,10 +2792,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2733,16 +2803,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2752,10 +2822,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2763,16 +2833,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2782,10 +2852,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2793,14 +2863,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2810,10 +2880,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2821,16 +2891,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2840,10 +2910,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2851,16 +2921,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2870,10 +2940,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2881,16 +2951,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2900,10 +2970,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2911,14 +2981,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2928,10 +2998,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2939,16 +3009,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -2958,10 +3028,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2969,14 +3039,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -2986,10 +3056,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2997,14 +3067,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3014,10 +3084,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3025,16 +3095,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3044,10 +3114,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3055,16 +3125,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -3074,10 +3144,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3085,14 +3155,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -3102,10 +3172,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3113,14 +3183,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3130,10 +3200,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3141,14 +3211,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3158,10 +3228,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3169,14 +3239,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3186,10 +3256,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3197,14 +3267,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3214,10 +3284,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3225,14 +3295,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3242,10 +3312,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3253,16 +3323,16 @@
         <v>15</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D34" s="22">
         <v>2</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F34" s="22">
         <v>2</v>
@@ -3272,10 +3342,10 @@
         <v>hoà</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3283,16 +3353,16 @@
         <v>15</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D35" s="34">
         <v>2</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="F35" s="34">
         <v>0</v>
@@ -3302,10 +3372,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3313,16 +3383,16 @@
         <v>15</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D36" s="22">
         <v>2</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F36" s="22">
         <v>2</v>
@@ -3332,10 +3402,10 @@
         <v>hoà</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3343,16 +3413,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D37" s="34">
         <v>2</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F37" s="34">
         <v>0</v>
@@ -3362,10 +3432,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3373,16 +3443,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="F38" s="22">
         <v>1</v>
@@ -3392,10 +3462,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3403,14 +3473,14 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3420,10 +3490,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3431,16 +3501,16 @@
         <v>16</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3450,10 +3520,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3461,16 +3531,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3480,10 +3550,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3491,16 +3561,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3510,10 +3580,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3521,16 +3591,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3540,10 +3610,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3551,16 +3621,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D44" s="28">
         <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3570,10 +3640,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3581,14 +3651,14 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3598,10 +3668,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3609,16 +3679,16 @@
         <v>17</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3628,10 +3698,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3639,16 +3709,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3658,10 +3728,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3672,13 +3742,13 @@
         <v>37</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D48" s="34">
         <v>2</v>
       </c>
       <c r="E48" s="33" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="F48" s="34">
         <v>0</v>
@@ -3688,10 +3758,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3699,16 +3769,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3718,10 +3788,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3729,16 +3799,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D50" s="28">
         <v>1</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
@@ -3748,10 +3818,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3759,14 +3829,14 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D51" s="28"/>
       <c r="E51" s="27" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -3776,10 +3846,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -3791,7 +3861,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -3803,12 +3873,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3824,282 +3894,302 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="38" t="s">
-        <v>274</v>
-      </c>
-      <c r="B16" s="38" t="s">
-        <v>275</v>
-      </c>
-      <c r="C16" s="39" t="s">
-        <v>276</v>
-      </c>
-      <c r="D16" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>277</v>
+      <c r="A16" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C17" s="25" t="s">
         <v>280</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>281</v>
+        <v>66</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>62</v>
+        <v>281</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="40" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="18" t="s">
-        <v>290</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="18"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="18"/>
+        <v>293</v>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="E20" s="27" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="27" t="s">
+        <v>297</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>298</v>
+      </c>
+      <c r="D21" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="38" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>301</v>
+      </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
       <c r="D25" s="18"/>
@@ -4112,10 +4202,24 @@
       <c r="D26" s="18"/>
       <c r="E26" s="18"/>
     </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="18"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="18"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E3"/>
-    <mergeCell ref="A23:E26"/>
+    <mergeCell ref="A25:E28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4124,7 +4228,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -4135,344 +4239,358 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>291</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>294</v>
+        <v>305</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>295</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
-        <v>296</v>
-      </c>
-      <c r="B4" s="42">
+      <c r="A4" s="39" t="s">
+        <v>307</v>
+      </c>
+      <c r="B4" s="40">
         <v>33</v>
       </c>
-      <c r="C4" s="43" t="s">
-        <v>297</v>
-      </c>
-      <c r="D4" s="44" t="s">
-        <v>298</v>
+      <c r="C4" s="41" t="s">
+        <v>308</v>
+      </c>
+      <c r="D4" s="42" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
-        <v>299</v>
-      </c>
-      <c r="B5" s="42">
-        <v>372</v>
-      </c>
-      <c r="C5" s="43" t="s">
-        <v>300</v>
-      </c>
-      <c r="D5" s="44" t="s">
-        <v>298</v>
+      <c r="A5" s="39" t="s">
+        <v>310</v>
+      </c>
+      <c r="B5" s="40">
+        <v>353</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>311</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
-        <v>301</v>
-      </c>
-      <c r="B6" s="42">
-        <v>209</v>
-      </c>
-      <c r="C6" s="43" t="s">
-        <v>302</v>
-      </c>
-      <c r="D6" s="44" t="s">
-        <v>298</v>
+      <c r="A6" s="39" t="s">
+        <v>313</v>
+      </c>
+      <c r="B6" s="40">
+        <v>188</v>
+      </c>
+      <c r="C6" s="41" t="s">
+        <v>314</v>
+      </c>
+      <c r="D6" s="42" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="41" t="s">
-        <v>303</v>
-      </c>
-      <c r="B7" s="42">
-        <v>7</v>
-      </c>
-      <c r="C7" s="43" t="s">
-        <v>304</v>
-      </c>
-      <c r="D7" s="44" t="s">
-        <v>298</v>
+      <c r="A7" s="39" t="s">
+        <v>315</v>
+      </c>
+      <c r="B7" s="40">
+        <v>22</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>316</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="41" t="s">
-        <v>305</v>
-      </c>
-      <c r="B8" s="42">
-        <v>2</v>
-      </c>
-      <c r="C8" s="43" t="s">
-        <v>306</v>
-      </c>
-      <c r="D8" s="44" t="s">
-        <v>298</v>
+      <c r="A8" s="39" t="s">
+        <v>317</v>
+      </c>
+      <c r="B8" s="40">
+        <v>2</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>318</v>
+      </c>
+      <c r="D8" s="42" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="41" t="s">
-        <v>307</v>
-      </c>
-      <c r="B9" s="42">
+      <c r="A9" s="39" t="s">
+        <v>319</v>
+      </c>
+      <c r="B9" s="40">
+        <v>19</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>320</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="39" t="s">
+        <v>321</v>
+      </c>
+      <c r="B10" s="40">
         <v>4</v>
       </c>
-      <c r="C9" s="43" t="s">
-        <v>308</v>
-      </c>
-      <c r="D9" s="44" t="s">
+      <c r="C10" s="41" t="s">
+        <v>322</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="39" t="s">
+        <v>324</v>
+      </c>
+      <c r="B11" s="40">
+        <v>35</v>
+      </c>
+      <c r="C11" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="D11" s="42" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="41" t="s">
-        <v>310</v>
-      </c>
-      <c r="B10" s="42">
-        <v>35</v>
-      </c>
-      <c r="C10" s="43" t="s">
-        <v>311</v>
-      </c>
-      <c r="D10" s="44" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="41" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="39" t="s">
+        <v>326</v>
+      </c>
+      <c r="B12" s="40">
+        <v>18</v>
+      </c>
+      <c r="C12" s="41" t="s">
+        <v>327</v>
+      </c>
+      <c r="D12" s="42" t="s">
         <v>312</v>
       </c>
-      <c r="B11" s="42">
-        <v>37</v>
-      </c>
-      <c r="C11" s="43" t="s">
-        <v>313</v>
-      </c>
-      <c r="D11" s="44" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="41" t="s">
-        <v>314</v>
-      </c>
-      <c r="B12" s="42">
-        <v>177</v>
-      </c>
-      <c r="C12" s="43" t="s">
-        <v>315</v>
-      </c>
-      <c r="D12" s="44" t="s">
-        <v>298</v>
-      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="41" t="s">
-        <v>316</v>
-      </c>
-      <c r="B13" s="42">
-        <v>9</v>
-      </c>
-      <c r="C13" s="43" t="s">
-        <v>317</v>
-      </c>
-      <c r="D13" s="44" t="s">
-        <v>298</v>
+      <c r="A13" s="39" t="s">
+        <v>328</v>
+      </c>
+      <c r="B13" s="40">
+        <v>57</v>
+      </c>
+      <c r="C13" s="41" t="s">
+        <v>329</v>
+      </c>
+      <c r="D13" s="42" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="41" t="s">
-        <v>318</v>
-      </c>
-      <c r="B14" s="42">
+      <c r="A14" s="39" t="s">
+        <v>330</v>
+      </c>
+      <c r="B14" s="40">
+        <v>10</v>
+      </c>
+      <c r="C14" s="41" t="s">
+        <v>331</v>
+      </c>
+      <c r="D14" s="42" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="39" t="s">
+        <v>332</v>
+      </c>
+      <c r="B15" s="40">
         <v>8</v>
       </c>
-      <c r="C14" s="43" t="s">
-        <v>319</v>
-      </c>
-      <c r="D14" s="44" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="41" t="s">
-        <v>320</v>
-      </c>
-      <c r="B15" s="42">
-        <v>2</v>
-      </c>
-      <c r="C15" s="43" t="s">
-        <v>321</v>
-      </c>
-      <c r="D15" s="44" t="s">
+      <c r="C15" s="41" t="s">
+        <v>333</v>
+      </c>
+      <c r="D15" s="42" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="41" t="s">
-        <v>322</v>
-      </c>
-      <c r="B16" s="42">
+      <c r="A16" s="39" t="s">
+        <v>334</v>
+      </c>
+      <c r="B16" s="40">
         <v>0</v>
       </c>
-      <c r="C16" s="43" t="s">
-        <v>323</v>
-      </c>
-      <c r="D16" s="44" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="B18" s="45">
+      <c r="C16" s="41" t="s">
+        <v>335</v>
+      </c>
+      <c r="D16" s="42" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="39" t="s">
+        <v>336</v>
+      </c>
+      <c r="B17" s="40">
+        <v>0</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>337</v>
+      </c>
+      <c r="D17" s="42" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
+        <v>338</v>
+      </c>
+      <c r="B19" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
-      <c r="C18" s="46" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>326</v>
-      </c>
-      <c r="B19" s="47">
+      <c r="C19" s="44" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="B20" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
-      <c r="C19" s="46" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="40" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>331</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>332</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>333</v>
+      <c r="C20" s="44" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="38" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>334</v>
+        <v>132</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>333</v>
+        <v>347</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>337</v>
+        <v>348</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>335</v>
+        <v>349</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>336</v>
+        <v>350</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>333</v>
+        <v>347</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>336</v>
+        <v>350</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>333</v>
+        <v>347</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="39" t="s">
-        <v>340</v>
-      </c>
-      <c r="B28" s="38" t="s">
-        <v>341</v>
-      </c>
-      <c r="C28" s="38" t="s">
-        <v>342</v>
-      </c>
-      <c r="D28" s="38" t="s">
-        <v>343</v>
+      <c r="A28" s="19" t="s">
+        <v>352</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>353</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>350</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="39" t="s">
-        <v>344</v>
-      </c>
-      <c r="B29" s="38" t="s">
-        <v>345</v>
-      </c>
-      <c r="C29" s="38" t="s">
-        <v>346</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>343</v>
+      <c r="A29" s="46" t="s">
+        <v>354</v>
+      </c>
+      <c r="B29" s="47" t="s">
+        <v>355</v>
+      </c>
+      <c r="C29" s="47" t="s">
+        <v>356</v>
+      </c>
+      <c r="D29" s="47" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="19" t="s">
-        <v>347</v>
-      </c>
-      <c r="B30" s="21" t="s">
-        <v>348</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>349</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>350</v>
+      <c r="A30" s="46" t="s">
+        <v>358</v>
+      </c>
+      <c r="B30" s="47" t="s">
+        <v>359</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>360</v>
+      </c>
+      <c r="D30" s="47" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="19" t="s">
+        <v>361</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>362</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>363</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -4495,24 +4613,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>351</v>
+        <v>365</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>352</v>
+        <v>366</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>353</v>
+        <v>367</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>356</v>
+        <v>370</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4520,16 +4638,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>358</v>
+        <v>372</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>359</v>
+        <v>373</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>360</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4537,16 +4655,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>361</v>
+        <v>375</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>362</v>
+        <v>376</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>363</v>
+        <v>377</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4554,16 +4672,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>365</v>
+        <v>379</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>366</v>
+        <v>380</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>367</v>
+        <v>381</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>368</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4571,16 +4689,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>369</v>
+        <v>383</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>370</v>
+        <v>384</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>371</v>
+        <v>385</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>372</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật bảng so sánh: form liên hệ bật lại, trang giới thiệu mới
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="389">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -198,6 +198,12 @@
     <t>Khách chưa đăng nhập vào thẳng trang giới thiệu. Gỡ khối « Lớp của bạn » ở thanh bên. Màn Thống kê dựng lại bằng số liệu thật.</t>
   </si>
   <si>
+    <t>25/09 — trang giới thiệu</t>
+  </si>
+  <si>
+    <t>Nội dung mới do chủ dự án viết (5 chỗ chỉnh cho khớp sản phẩm: bỏ DALF, bỏ « chấm chữa theo barem », 'tự đối chiếu', 'phần lớn câu có lời giải', câu đồng ý không nhắc chính sách chưa có). Ảnh màn hình + ảnh đại diện thật, chân trang xanh, form « Gửi câu hỏi » gửi thật. Điểm « Xem đăng ký tư vấn » 1 → 2.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -632,13 +638,13 @@
     <t>Có form thu thông tin</t>
   </si>
   <si>
-    <t>Bảng và màn xem CÒN NGUYÊN, nhưng FORM ĐÃ GỠ khỏi trang giới thiệu</t>
-  </si>
-  <si>
-    <t>Tắt có chủ đích</t>
-  </si>
-  <si>
-    <t>migration 077–080; /professeur/lien-he. Gỡ vì chưa có trang Chính sách bảo mật</t>
+    <t>Có lại từ 25/09: nút « Gửi câu hỏi » mở ngăn kéo form (tên, SĐT, năm sinh, email, vai, mục tiêu, nội dung), gửi thật vào bảng leads</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa ai gửi qua giao diện</t>
+  </si>
+  <si>
+    <t>migration 077–080; /professeur/lien-he. Thử bằng vai anon trong khối rollback: lưu đúng. RỦI RO: thu dữ liệu cá nhân (có thể của trẻ vị thành niên) khi chưa có Chính sách bảo mật</t>
   </si>
   <si>
     <t>Số tài khoản đang có</t>
@@ -725,7 +731,7 @@
     <t>ĐÃ GỠ — có chủ đích</t>
   </si>
   <si>
-    <t>Nội dung còn trong git. Khi vắng trang này, form tư vấn không nên bật lại</t>
+    <t>Nội dung còn trong git. Form liên hệ ĐÃ bật lại 25/09 → nên dựng lại trang này</t>
   </si>
   <si>
     <t>Đội ngũ công khai</t>
@@ -863,16 +869,16 @@
     <t>Dựng 09/09. Học sinh không còn tự tạo thẻ — chỉ giáo viên soạn, chặn ở database bằng RLS chứ không chỉ ẩn nút.</t>
   </si>
   <si>
-    <t>Xem đăng ký tư vấn</t>
+    <t>Xem câu hỏi / đăng ký tư vấn</t>
   </si>
   <si>
     <t>/professeur/lien-he</t>
   </si>
   <si>
-    <t>Đang chạy, nhưng không có nguồn vào</t>
-  </si>
-  <si>
-    <t>Form đã gỡ khỏi trang giới thiệu, nên chưa có đường nào để ai gửi thông tin vào.</t>
+    <t>Đang chạy — có nguồn vào từ 25/09</t>
+  </si>
+  <si>
+    <t>Nguồn: nút « Gửi câu hỏi » trên trang giới thiệu. Năm sinh nằm ở dòng đầu phần nội dung.</t>
   </si>
   <si>
     <t>Nghe bản ghi âm bài nói của học sinh</t>
@@ -1810,7 +1816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1996,11 +2002,11 @@
       </c>
       <c r="E11" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="F11" s="6">
         <f>IFERROR(E11-D11,"")</f>
-        <v>-1</v>
+        <v>-0.8</v>
       </c>
       <c r="G11" s="7" t="str">
         <f>IF(OR(C11&lt;3,F11=""),"quá ít mục",IF(F11&gt;0.25,"FRACILE",IF(F11&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2083,11 +2089,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
-        <v>0.9666666666666667</v>
+        <v>1</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.9</v>
+        <v>-0.8666666666666667</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2326,8 +2332,21 @@
       <c r="F39" s="18"/>
       <c r="G39" s="18"/>
     </row>
+    <row r="40" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2341,6 +2360,7 @@
     <mergeCell ref="B37:G37"/>
     <mergeCell ref="B38:G38"/>
     <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B40:G40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2368,28 +2388,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2397,16 +2417,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2416,10 +2436,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2427,14 +2447,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2444,10 +2464,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2455,16 +2475,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2474,10 +2494,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2485,16 +2505,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2504,10 +2524,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2515,16 +2535,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2534,10 +2554,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2545,16 +2565,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2564,10 +2584,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2575,14 +2595,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2592,10 +2612,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2603,7 +2623,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2612,7 +2632,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2622,10 +2642,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2633,16 +2653,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2652,10 +2672,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2663,14 +2683,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2680,10 +2700,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2691,14 +2711,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2708,10 +2728,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2719,14 +2739,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2736,10 +2756,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2747,14 +2767,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2764,10 +2784,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2775,14 +2795,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2792,10 +2812,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2803,16 +2823,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2822,10 +2842,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2833,16 +2853,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2852,10 +2872,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2863,14 +2883,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2880,10 +2900,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2891,16 +2911,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2910,10 +2930,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2921,16 +2941,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2940,10 +2960,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2951,16 +2971,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2970,10 +2990,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2981,14 +3001,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -2998,10 +3018,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3009,16 +3029,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3028,10 +3048,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3039,14 +3059,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -3056,10 +3076,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3067,14 +3087,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3084,10 +3104,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3095,16 +3115,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3114,10 +3134,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3125,16 +3145,16 @@
         <v>14</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D27" s="34">
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F27" s="34">
         <v>0</v>
@@ -3144,10 +3164,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I27" s="36" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3155,14 +3175,14 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="21" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F28" s="22">
         <v>1</v>
@@ -3172,10 +3192,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3183,14 +3203,14 @@
         <v>15</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D29" s="28"/>
       <c r="E29" s="27" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F29" s="28">
         <v>2</v>
@@ -3200,10 +3220,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3211,14 +3231,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3228,10 +3248,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3239,14 +3259,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3256,10 +3276,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3267,14 +3287,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3284,10 +3304,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3295,14 +3315,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3312,10 +3332,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3323,16 +3343,16 @@
         <v>15</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D34" s="22">
         <v>2</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F34" s="22">
         <v>2</v>
@@ -3342,10 +3362,10 @@
         <v>hoà</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I34" s="24" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3353,16 +3373,16 @@
         <v>15</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D35" s="34">
         <v>2</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F35" s="34">
         <v>0</v>
@@ -3372,10 +3392,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H35" s="31" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3383,16 +3403,16 @@
         <v>15</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D36" s="22">
         <v>2</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F36" s="22">
         <v>2</v>
@@ -3402,10 +3422,10 @@
         <v>hoà</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3413,16 +3433,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D37" s="34">
         <v>2</v>
       </c>
       <c r="E37" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F37" s="34">
         <v>0</v>
@@ -3432,10 +3452,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I37" s="36" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3443,29 +3463,29 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F38" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G38" s="23" t="str">
         <f>IF(OR(D38="",F38=""),"chưa rõ",IF(F38&gt;D38,"FRACILE",IF(D38&gt;F38,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3473,14 +3493,14 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D39" s="22"/>
       <c r="E39" s="21" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3490,10 +3510,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3501,16 +3521,16 @@
         <v>16</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3520,10 +3540,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3531,16 +3551,16 @@
         <v>16</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3550,10 +3570,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3561,16 +3581,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3580,10 +3600,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3591,16 +3611,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3610,10 +3630,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3621,16 +3641,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D44" s="28">
         <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3640,10 +3660,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3651,14 +3671,14 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3668,10 +3688,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3679,16 +3699,16 @@
         <v>17</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3698,10 +3718,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3709,16 +3729,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3728,10 +3748,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3742,13 +3762,13 @@
         <v>37</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D48" s="34">
         <v>2</v>
       </c>
       <c r="E48" s="33" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F48" s="34">
         <v>0</v>
@@ -3758,10 +3778,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="I48" s="36" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3769,16 +3789,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3788,10 +3808,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3799,16 +3819,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D50" s="28">
         <v>1</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F50" s="28">
         <v>2</v>
@@ -3818,10 +3838,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H50" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3829,14 +3849,14 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D51" s="28"/>
       <c r="E51" s="27" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -3846,10 +3866,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -3873,12 +3893,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3894,301 +3914,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>254</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>251</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>252</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>249</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="B21" s="27" t="s">
         <v>297</v>
       </c>
-      <c r="B21" s="27" t="s">
-        <v>295</v>
-      </c>
       <c r="C21" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4239,358 +4259,358 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B4" s="40">
         <v>33</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B5" s="40">
         <v>353</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B6" s="40">
         <v>188</v>
       </c>
       <c r="C6" s="41" t="s">
+        <v>316</v>
+      </c>
+      <c r="D6" s="42" t="s">
         <v>314</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B9" s="40">
         <v>19</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B10" s="40">
         <v>4</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B11" s="40">
         <v>35</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B14" s="40">
         <v>10</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B15" s="40">
         <v>8</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B17" s="40">
         <v>0</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B19" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C19" s="44" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B20" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B26" s="21" t="s">
+        <v>351</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>352</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>349</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>350</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
+        <v>353</v>
+      </c>
+      <c r="B27" s="21" t="s">
         <v>351</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="C27" s="21" t="s">
+        <v>352</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>349</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>350</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
+        <v>354</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>355</v>
+      </c>
+      <c r="C28" s="21" t="s">
         <v>352</v>
       </c>
-      <c r="B28" s="21" t="s">
-        <v>353</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>350</v>
-      </c>
       <c r="D28" s="21" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="46" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D29" s="47" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="46" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B30" s="47" t="s">
+        <v>361</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>362</v>
+      </c>
+      <c r="D30" s="47" t="s">
         <v>359</v>
-      </c>
-      <c r="C30" s="47" t="s">
-        <v>360</v>
-      </c>
-      <c r="D30" s="47" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -4613,24 +4633,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4638,16 +4658,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4655,16 +4675,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4672,16 +4692,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4689,16 +4709,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật bảng so sánh: bảo mật 0→1, chuỗi ngày máy chủ, tìm kiếm, C1, ảnh Google
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="394">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -204,6 +204,12 @@
     <t>Nội dung mới do chủ dự án viết (5 chỗ chỉnh cho khớp sản phẩm: bỏ DALF, bỏ « chấm chữa theo barem », 'tự đối chiếu', 'phần lớn câu có lời giải', câu đồng ý không nhắc chính sách chưa có). Ảnh màn hình + ảnh đại diện thật, chân trang xanh, form « Gửi câu hỏi » gửi thật. Điểm « Xem đăng ký tư vấn » 1 → 2.</t>
   </si>
   <si>
+    <t>25/09 — tiếp</t>
+  </si>
+  <si>
+    <t>Chính sách bảo mật dựng lại (0 → 1). Widget chuỗi ngày tính ở máy chủ. Tìm kiếm chung. Ảnh Google làm ảnh đại diện — kèm sửa ràng buộc 046 vốn từ chối mọi ảnh https (9 tài khoản được gán ảnh Google). Cấp độ C1. Chuẩn hoá bản dịch ba thứ tiếng. Trang đăng nhập có bản tối; bỏ emoji ở các ô trống và khối điểm.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -410,13 +416,13 @@
     <t>A1 → C2 (6 cấp) + ôn thi cấp 3</t>
   </si>
   <si>
-    <t>B1 – B2 (2 cấp)</t>
+    <t>Nhận A1 → C1 (C1 thêm 25/09), nhưng nội dung chủ yếu B1 – B2; C1 chưa có bài</t>
   </si>
   <si>
     <t>Có chủ đích — nhắm hẹp</t>
   </si>
   <si>
-    <t>docs/roadmap-delf.md</t>
+    <t>docs/roadmap-delf.md; LEVEL_COLORS là nguồn duy nhất cho Builder + dải lọc</t>
   </si>
   <si>
     <t>Số bài luyện</t>
@@ -530,10 +536,22 @@
     <t>Có, kèm nhiệm vụ và kim cương</t>
   </si>
   <si>
-    <t>Có — tính ở MÁY CHỦ, theo ngày của NGƯỜI DÙNG chứ không theo giờ UTC</t>
-  </si>
-  <si>
-    <t>migration 061/062; RPC chuoi_ngay_hoc (gaps-and-islands)</t>
+    <t>Có — widget trang chủ: chuỗi + 7 ô trong tuần, tính ở MÁY CHỦ từ lượt nộp bài theo giờ Việt Nam (đổi đồng hồ máy không có tác dụng)</t>
+  </si>
+  <si>
+    <t>migration 095/096; RPC get_student_streak — đo bằng claim giả: 3 ngày liên tiếp ra 3, ngày bỏ trống cắt chuỗi (25/09)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm bài tập / học sinh</t>
+  </si>
+  <si>
+    <t>Ô tìm ở thanh trên, mở thẳng bài hoặc hồ sơ. Chạy bằng quyền người tìm nên học sinh không thấy hồ sơ người khác</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa thử qua giao diện</t>
+  </si>
+  <si>
+    <t>migration 097/098; RPC global_search (SECURITY INVOKER) — giáo viên tìm « ng »: 3 bài + 6 học sinh; học sinh: 3 bài + 0</t>
   </si>
   <si>
     <t>Trò chơi / thi đấu</t>
@@ -725,13 +743,10 @@
     <t>/dieu-khoan</t>
   </si>
   <si>
-    <t>KHÔNG CÓ — dựng xong 21/09 rồi gỡ cùng ngày theo quyết định chủ dự án</t>
-  </si>
-  <si>
-    <t>ĐÃ GỠ — có chủ đích</t>
-  </si>
-  <si>
-    <t>Nội dung còn trong git. Form liên hệ ĐÃ bật lại 25/09 → nên dựng lại trang này</t>
+    <t>Có từ 25/09 (/bao-mat) — có mục riêng cho dữ liệu form « Gửi câu hỏi »; gỡ 21/09 rồi dựng lại</t>
+  </si>
+  <si>
+    <t>Điểm 0 → 1. Chưa lên 2 vì chưa qua luật sư, giống Điều khoản</t>
   </si>
   <si>
     <t>Đội ngũ công khai</t>
@@ -1816,7 +1831,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1873,19 +1888,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A7)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F7" s="6">
@@ -1902,19 +1917,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A8)</f>
         <v>6</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A8)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -1931,19 +1946,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A9)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>0.6</v>
       </c>
       <c r="F9" s="6">
@@ -1960,19 +1975,19 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A10)</f>
-        <v>6</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A10)</f>
+        <v>7</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
         <v>3</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A10)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F10" s="6">
@@ -1989,19 +2004,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A11)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A11)</f>
         <v>11</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A11)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1.2</v>
       </c>
       <c r="F11" s="6">
@@ -2018,19 +2033,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A12)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F12" s="6">
@@ -2047,24 +2062,24 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$51,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$51=$A13)*('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <v>1.2</v>
       </c>
       <c r="F13" s="6">
         <f>IFERROR(E13-D13,"")</f>
-        <v>-0.8</v>
+        <v>-0.6000000000000001</v>
       </c>
       <c r="G13" s="7" t="str">
         <f>IF(OR(C13&lt;3,F13=""),"quá ít mục",IF(F13&gt;0.25,"FRACILE",IF(F13&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2077,23 +2092,23 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
         <v>30</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$51)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
         <v>1.8666666666666667</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$51)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$51&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$51&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <v>1.0333333333333334</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.8666666666666667</v>
+        <v>-0.8333333333333333</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2345,8 +2360,21 @@
       <c r="F40" s="18"/>
       <c r="G40" s="18"/>
     </row>
+    <row r="41" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2361,6 +2389,7 @@
     <mergeCell ref="B38:G38"/>
     <mergeCell ref="B39:G39"/>
     <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B41:G41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2369,7 +2398,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2388,28 +2417,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2417,16 +2446,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2436,10 +2465,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2447,14 +2476,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2464,10 +2493,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2475,16 +2504,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2494,10 +2523,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2505,16 +2534,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2524,10 +2553,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2535,16 +2564,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2554,10 +2583,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2565,16 +2594,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2584,10 +2613,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2595,14 +2624,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2612,10 +2641,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2623,7 +2652,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2632,7 +2661,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2642,10 +2671,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2653,16 +2682,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2672,10 +2701,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2683,14 +2712,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2700,10 +2729,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2711,14 +2740,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2728,10 +2757,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2739,14 +2768,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2756,10 +2785,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2767,14 +2796,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2784,10 +2813,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2795,14 +2824,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2812,10 +2841,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2823,16 +2852,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2842,10 +2871,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2853,16 +2882,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2872,10 +2901,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2883,14 +2912,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2900,10 +2929,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2911,16 +2940,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2930,10 +2959,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2941,16 +2970,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2960,10 +2989,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2971,16 +3000,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -2990,10 +3019,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3001,14 +3030,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3018,10 +3047,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3029,16 +3058,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3048,10 +3077,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3059,14 +3088,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -3076,10 +3105,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3087,14 +3116,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3104,10 +3133,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3115,16 +3144,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3134,96 +3163,96 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="32" t="s">
-        <v>165</v>
-      </c>
-      <c r="C27" s="33" t="s">
-        <v>166</v>
-      </c>
-      <c r="D27" s="34">
-        <v>2</v>
-      </c>
-      <c r="E27" s="33" t="s">
-        <v>136</v>
-      </c>
-      <c r="F27" s="34">
+      <c r="B27" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="C27" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="28"/>
+      <c r="E27" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="F27" s="28">
+        <v>2</v>
+      </c>
+      <c r="G27" s="29" t="str">
+        <f>IF(OR(D27="",F27=""),"chưa rõ",IF(F27&gt;D27,"FRACILE",IF(D27&gt;F27,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>169</v>
+      </c>
+      <c r="I27" s="30" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="C28" s="33" t="s">
+        <v>172</v>
+      </c>
+      <c r="D28" s="34">
+        <v>2</v>
+      </c>
+      <c r="E28" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="F28" s="34">
         <v>0</v>
       </c>
-      <c r="G27" s="35" t="str">
-        <f>IF(OR(D27="",F27=""),"chưa rõ",IF(F27&gt;D27,"FRACILE",IF(D27&gt;F27,"Vivoire","hoà")))</f>
+      <c r="G28" s="35" t="str">
+        <f>IF(OR(D28="",F28=""),"chưa rõ",IF(F28&gt;D28,"FRACILE",IF(D28&gt;F28,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H27" s="31" t="s">
-        <v>137</v>
-      </c>
-      <c r="I27" s="36" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
+      <c r="H28" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="I28" s="36" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="20" t="s">
-        <v>167</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="21" t="s">
-        <v>168</v>
-      </c>
-      <c r="F28" s="22">
+      <c r="B29" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="D29" s="22"/>
+      <c r="E29" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="F29" s="22">
         <v>1</v>
       </c>
-      <c r="G28" s="23" t="str">
-        <f>IF(OR(D28="",F28=""),"chưa rõ",IF(F28&gt;D28,"FRACILE",IF(D28&gt;F28,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
-      </c>
-      <c r="H28" s="19" t="s">
-        <v>169</v>
-      </c>
-      <c r="I28" s="24" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B29" s="26" t="s">
-        <v>171</v>
-      </c>
-      <c r="C29" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="27" t="s">
-        <v>172</v>
-      </c>
-      <c r="F29" s="28">
-        <v>2</v>
-      </c>
-      <c r="G29" s="29" t="str">
+      <c r="G29" s="23" t="str">
         <f>IF(OR(D29="",F29=""),"chưa rõ",IF(F29&gt;D29,"FRACILE",IF(D29&gt;F29,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H29" s="25" t="s">
-        <v>173</v>
-      </c>
-      <c r="I29" s="30" t="s">
-        <v>174</v>
+      <c r="H29" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="I29" s="24" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3231,14 +3260,14 @@
         <v>15</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D30" s="28"/>
       <c r="E30" s="27" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F30" s="28">
         <v>2</v>
@@ -3248,10 +3277,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3259,14 +3288,14 @@
         <v>15</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3276,10 +3305,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3287,14 +3316,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3304,10 +3333,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3315,14 +3344,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3332,160 +3361,158 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B34" s="20" t="s">
-        <v>187</v>
-      </c>
-      <c r="C34" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D34" s="22">
-        <v>2</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="F34" s="22">
-        <v>2</v>
-      </c>
-      <c r="G34" s="23" t="str">
+      <c r="B34" s="26" t="s">
+        <v>190</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" s="28"/>
+      <c r="E34" s="27" t="s">
+        <v>191</v>
+      </c>
+      <c r="F34" s="28">
+        <v>2</v>
+      </c>
+      <c r="G34" s="29" t="str">
         <f>IF(OR(D34="",F34=""),"chưa rõ",IF(F34&gt;D34,"FRACILE",IF(D34&gt;F34,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H34" s="25" t="s">
+        <v>179</v>
+      </c>
+      <c r="I34" s="30" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D35" s="22">
+        <v>2</v>
+      </c>
+      <c r="E35" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="F35" s="22">
+        <v>2</v>
+      </c>
+      <c r="G35" s="23" t="str">
+        <f>IF(OR(D35="",F35=""),"chưa rõ",IF(F35&gt;D35,"FRACILE",IF(D35&gt;F35,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H34" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="I34" s="24" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="31" t="s">
+      <c r="H35" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="I35" s="24" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="32" t="s">
-        <v>189</v>
-      </c>
-      <c r="C35" s="33" t="s">
-        <v>190</v>
-      </c>
-      <c r="D35" s="34">
-        <v>2</v>
-      </c>
-      <c r="E35" s="33" t="s">
-        <v>191</v>
-      </c>
-      <c r="F35" s="34">
+      <c r="B36" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="C36" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="D36" s="34">
+        <v>2</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="F36" s="34">
         <v>0</v>
       </c>
-      <c r="G35" s="35" t="str">
-        <f>IF(OR(D35="",F35=""),"chưa rõ",IF(F35&gt;D35,"FRACILE",IF(D35&gt;F35,"Vivoire","hoà")))</f>
+      <c r="G36" s="35" t="str">
+        <f>IF(OR(D36="",F36=""),"chưa rõ",IF(F36&gt;D36,"FRACILE",IF(D36&gt;F36,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H35" s="31" t="s">
-        <v>91</v>
-      </c>
-      <c r="I35" s="36" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
+      <c r="H36" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="I36" s="36" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="20" t="s">
-        <v>193</v>
-      </c>
-      <c r="C36" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D36" s="22">
-        <v>2</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>194</v>
-      </c>
-      <c r="F36" s="22">
-        <v>2</v>
-      </c>
-      <c r="G36" s="23" t="str">
-        <f>IF(OR(D36="",F36=""),"chưa rõ",IF(F36&gt;D36,"FRACILE",IF(D36&gt;F36,"Vivoire","hoà")))</f>
+      <c r="B37" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D37" s="22">
+        <v>2</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="F37" s="22">
+        <v>2</v>
+      </c>
+      <c r="G37" s="23" t="str">
+        <f>IF(OR(D37="",F37=""),"chưa rõ",IF(F37&gt;D37,"FRACILE",IF(D37&gt;F37,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H36" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="I36" s="24" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="31" t="s">
+      <c r="H37" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="I37" s="24" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B37" s="32" t="s">
-        <v>196</v>
-      </c>
-      <c r="C37" s="33" t="s">
-        <v>113</v>
-      </c>
-      <c r="D37" s="34">
-        <v>2</v>
-      </c>
-      <c r="E37" s="33" t="s">
-        <v>136</v>
-      </c>
-      <c r="F37" s="34">
+      <c r="B38" s="32" t="s">
+        <v>202</v>
+      </c>
+      <c r="C38" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="D38" s="34">
+        <v>2</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="F38" s="34">
         <v>0</v>
       </c>
-      <c r="G37" s="35" t="str">
-        <f>IF(OR(D37="",F37=""),"chưa rõ",IF(F37&gt;D37,"FRACILE",IF(D37&gt;F37,"Vivoire","hoà")))</f>
+      <c r="G38" s="35" t="str">
+        <f>IF(OR(D38="",F38=""),"chưa rõ",IF(F38&gt;D38,"FRACILE",IF(D38&gt;F38,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H37" s="31" t="s">
-        <v>137</v>
-      </c>
-      <c r="I37" s="36" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B38" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>198</v>
-      </c>
-      <c r="D38" s="22">
-        <v>2</v>
-      </c>
-      <c r="E38" s="21" t="s">
-        <v>199</v>
-      </c>
-      <c r="F38" s="22">
-        <v>2</v>
-      </c>
-      <c r="G38" s="23" t="str">
-        <f>IF(OR(D38="",F38=""),"chưa rõ",IF(F38&gt;D38,"FRACILE",IF(D38&gt;F38,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H38" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="I38" s="24" t="s">
-        <v>201</v>
+      <c r="H38" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="I38" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3493,87 +3520,87 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="D39" s="22"/>
+        <v>204</v>
+      </c>
+      <c r="D39" s="22">
+        <v>2</v>
+      </c>
       <c r="E39" s="21" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F39" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="23" t="str">
         <f>IF(OR(D39="",F39=""),"chưa rõ",IF(F39&gt;D39,"FRACILE",IF(D39&gt;F39,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>hoà</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>68</v>
+        <v>206</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D40" s="22">
-        <v>2</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="D40" s="22"/>
       <c r="E40" s="21" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="F40" s="22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40" s="23" t="str">
         <f>IF(OR(D40="",F40=""),"chưa rõ",IF(F40&gt;D40,"FRACILE",IF(D40&gt;F40,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H40" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="I40" s="24" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="C41" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" s="22">
+        <v>2</v>
+      </c>
+      <c r="E41" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="22">
+        <v>2</v>
+      </c>
+      <c r="G41" s="23" t="str">
+        <f>IF(OR(D41="",F41=""),"chưa rõ",IF(F41&gt;D41,"FRACILE",IF(D41&gt;F41,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H40" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="I40" s="24" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="B41" s="32" t="s">
-        <v>207</v>
-      </c>
-      <c r="C41" s="33" t="s">
-        <v>208</v>
-      </c>
-      <c r="D41" s="34">
-        <v>2</v>
-      </c>
-      <c r="E41" s="33" t="s">
-        <v>136</v>
-      </c>
-      <c r="F41" s="34">
-        <v>0</v>
-      </c>
-      <c r="G41" s="35" t="str">
-        <f>IF(OR(D41="",F41=""),"chưa rõ",IF(F41&gt;D41,"FRACILE",IF(D41&gt;F41,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H41" s="31" t="s">
-        <v>137</v>
-      </c>
-      <c r="I41" s="36" t="s">
-        <v>140</v>
+      <c r="H41" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="I41" s="24" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3581,16 +3608,16 @@
         <v>16</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3600,70 +3627,70 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="19" t="s">
+      <c r="A43" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B43" s="20" t="s">
-        <v>211</v>
-      </c>
-      <c r="C43" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D43" s="22">
-        <v>2</v>
-      </c>
-      <c r="E43" s="21" t="s">
-        <v>212</v>
-      </c>
-      <c r="F43" s="22">
-        <v>1</v>
-      </c>
-      <c r="G43" s="23" t="str">
+      <c r="B43" s="32" t="s">
+        <v>215</v>
+      </c>
+      <c r="C43" s="33" t="s">
+        <v>216</v>
+      </c>
+      <c r="D43" s="34">
+        <v>2</v>
+      </c>
+      <c r="E43" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="F43" s="34">
+        <v>0</v>
+      </c>
+      <c r="G43" s="35" t="str">
         <f>IF(OR(D43="",F43=""),"chưa rõ",IF(F43&gt;D43,"FRACILE",IF(D43&gt;F43,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H43" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="I43" s="24" t="s">
-        <v>140</v>
+      <c r="H43" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="I43" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="25" t="s">
+      <c r="A44" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B44" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="C44" s="27" t="s">
-        <v>214</v>
-      </c>
-      <c r="D44" s="28">
+      <c r="B44" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D44" s="22">
+        <v>2</v>
+      </c>
+      <c r="E44" s="21" t="s">
+        <v>218</v>
+      </c>
+      <c r="F44" s="22">
         <v>1</v>
       </c>
-      <c r="E44" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="F44" s="28">
-        <v>2</v>
-      </c>
-      <c r="G44" s="29" t="str">
+      <c r="G44" s="23" t="str">
         <f>IF(OR(D44="",F44=""),"chưa rõ",IF(F44&gt;D44,"FRACILE",IF(D44&gt;F44,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H44" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="I44" s="30" t="s">
-        <v>216</v>
+        <v>Vivoire</v>
+      </c>
+      <c r="H44" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="I44" s="24" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3671,57 +3698,57 @@
         <v>16</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="D45" s="28"/>
+        <v>220</v>
+      </c>
+      <c r="D45" s="28">
+        <v>1</v>
+      </c>
       <c r="E45" s="27" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
       </c>
       <c r="G45" s="29" t="str">
         <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
+        <v>FRACILE</v>
+      </c>
+      <c r="H45" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="I45" s="30" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B46" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="C46" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" s="28"/>
+      <c r="E46" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="F46" s="28">
+        <v>2</v>
+      </c>
+      <c r="G46" s="29" t="str">
+        <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H45" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="I45" s="30" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="20" t="s">
-        <v>220</v>
-      </c>
-      <c r="C46" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D46" s="22">
-        <v>2</v>
-      </c>
-      <c r="E46" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="F46" s="22">
-        <v>1</v>
-      </c>
-      <c r="G46" s="23" t="str">
-        <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H46" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="I46" s="24" t="s">
-        <v>223</v>
+      <c r="H46" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="I46" s="30" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3729,16 +3756,16 @@
         <v>17</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3748,40 +3775,40 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="31" t="s">
+      <c r="A48" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B48" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="C48" s="33" t="s">
-        <v>113</v>
-      </c>
-      <c r="D48" s="34">
-        <v>2</v>
-      </c>
-      <c r="E48" s="33" t="s">
-        <v>228</v>
-      </c>
-      <c r="F48" s="34">
-        <v>0</v>
-      </c>
-      <c r="G48" s="35" t="str">
+      <c r="B48" s="20" t="s">
+        <v>230</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D48" s="22">
+        <v>2</v>
+      </c>
+      <c r="E48" s="21" t="s">
+        <v>231</v>
+      </c>
+      <c r="F48" s="22">
+        <v>1</v>
+      </c>
+      <c r="G48" s="23" t="str">
         <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H48" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="I48" s="36" t="s">
-        <v>230</v>
+      <c r="H48" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="I48" s="24" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3789,16 +3816,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>231</v>
+        <v>37</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>232</v>
+        <v>115</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3808,40 +3835,40 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>68</v>
+        <v>232</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="25" t="s">
+      <c r="A50" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B50" s="26" t="s">
-        <v>235</v>
-      </c>
-      <c r="C50" s="27" t="s">
+      <c r="B50" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="D50" s="28">
+      <c r="C50" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="D50" s="22">
+        <v>2</v>
+      </c>
+      <c r="E50" s="21" t="s">
+        <v>238</v>
+      </c>
+      <c r="F50" s="22">
         <v>1</v>
       </c>
-      <c r="E50" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="F50" s="28">
-        <v>2</v>
-      </c>
-      <c r="G50" s="29" t="str">
+      <c r="G50" s="23" t="str">
         <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H50" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="I50" s="30" t="s">
-        <v>238</v>
+        <v>Vivoire</v>
+      </c>
+      <c r="H50" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="I50" s="24" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3849,27 +3876,57 @@
         <v>17</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="D51" s="28"/>
+        <v>241</v>
+      </c>
+      <c r="D51" s="28">
+        <v>1</v>
+      </c>
       <c r="E51" s="27" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
       </c>
       <c r="G51" s="29" t="str">
         <f>IF(OR(D51="",F51=""),"chưa rõ",IF(F51&gt;D51,"FRACILE",IF(D51&gt;F51,"Vivoire","hoà")))</f>
+        <v>FRACILE</v>
+      </c>
+      <c r="H51" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="I51" s="30" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B52" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="C52" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="D52" s="28"/>
+      <c r="E52" s="27" t="s">
+        <v>245</v>
+      </c>
+      <c r="F52" s="28">
+        <v>2</v>
+      </c>
+      <c r="G52" s="29" t="str">
+        <f>IF(OR(D52="",F52=""),"chưa rõ",IF(F52&gt;D52,"FRACILE",IF(D52&gt;F52,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H51" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="I51" s="30" t="s">
-        <v>241</v>
+      <c r="H52" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="I52" s="30" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3893,12 +3950,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3914,301 +3971,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
+        <v>261</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>262</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>256</v>
       </c>
-      <c r="B8" s="21" t="s">
-        <v>257</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>251</v>
-      </c>
       <c r="D8" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4259,358 +4316,358 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B4" s="40">
         <v>33</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="B5" s="40">
         <v>353</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B6" s="40">
         <v>188</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
+        <v>324</v>
+      </c>
+      <c r="B8" s="40">
+        <v>2</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>319</v>
-      </c>
-      <c r="B8" s="40">
-        <v>2</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>320</v>
-      </c>
-      <c r="D8" s="42" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B9" s="40">
         <v>19</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B10" s="40">
         <v>4</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="B11" s="40">
         <v>35</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B14" s="40">
         <v>10</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B15" s="40">
         <v>8</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B17" s="40">
         <v>0</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B19" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C19" s="44" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B20" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
+        <v>359</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>360</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>357</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>354</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>355</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>352</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="46" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D29" s="47" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="46" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="B30" s="47" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="C30" s="47" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="D30" s="47" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -4633,24 +4690,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4658,16 +4715,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4675,16 +4732,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4692,16 +4749,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4709,16 +4766,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật bảng so sánh: XP, theo dõi bạn học, nhật ký 26/09
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="408">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -210,6 +210,12 @@
     <t>Chính sách bảo mật dựng lại (0 → 1). Widget chuỗi ngày tính ở máy chủ. Tìm kiếm chung. Ảnh Google làm ảnh đại diện — kèm sửa ràng buộc 046 vốn từ chối mọi ảnh https (9 tài khoản được gán ảnh Google). Cấp độ C1. Chuẩn hoá bản dịch ba thứ tiếng. Trang đăng nhập có bản tối; bỏ emoji ở các ô trống và khối điểm.</t>
   </si>
   <si>
+    <t>26/09</t>
+  </si>
+  <si>
+    <t>XP + đổi XP lấy bài + theo dõi bạn học (101–103). Tour giới thiệu cho Lịch, Flashcard, Tài khoản, XP. Trang đăng nhập có lớp phủ trượt. Chuông thông báo + nhãn XP trên thanh trên. Màn theo dõi luyện tập của giáo viên làm lại; tên Google « Quốc Hùng Đỗ » hiển thị « Đỗ Quốc Hùng ».</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -558,6 +564,42 @@
   </si>
   <si>
     <t>Đấu dịch thuật PvP trực tiếp</t>
+  </si>
+  <si>
+    <t>Không có đấu trực tiếp; có XP + theo dõi bạn học (xem hai dòng dưới)</t>
+  </si>
+  <si>
+    <t>Không có kế hoạch PvP</t>
+  </si>
+  <si>
+    <t>XP (điểm kinh nghiệm)</t>
+  </si>
+  <si>
+    <t>Có, kèm kim cương</t>
+  </si>
+  <si>
+    <t>Có từ 26/09 — cộng ở MÁY CHỦ khi nộp bài lần đầu (10 + điểm), có sổ cái; đổi XP lấy bài trả phí theo giá giáo viên đặt. Chưa bài nào đặt giá XP</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa ai đổi qua giao diện</t>
+  </si>
+  <si>
+    <t>migration 101–103; claim giả: nộp 2 lần chỉ cộng 1 lần, đổi 15 XP mở được bài, bấm lại không trừ thêm. 5 tài khoản được cộng bù (13–52 XP)</t>
+  </si>
+  <si>
+    <t>Theo dõi bạn học</t>
+  </si>
+  <si>
+    <t>Có (bạn bè, bảng xếp hạng)</t>
+  </si>
+  <si>
+    <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa ». Chưa có bảng xếp hạng</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa ai theo dõi qua giao diện</t>
+  </si>
+  <si>
+    <t>RPC follow_user / get_following_streaks; chỉ lộ tên, @username, ảnh và một cờ</t>
   </si>
   <si>
     <t>Giờ học đo được</t>
@@ -1831,7 +1873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1888,19 +1930,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A7)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F7" s="6">
@@ -1917,19 +1959,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A8)</f>
         <v>6</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A8)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -1946,19 +1988,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A9)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>0.6</v>
       </c>
       <c r="F9" s="6">
@@ -1975,24 +2017,24 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A10)</f>
-        <v>7</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A10)</f>
+        <v>9</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
-        <v>3</v>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
+        <v>5</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A10)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
-        <v>1.3333333333333333</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <v>1.2</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>-0.6666666666666667</v>
+        <v>-0.8</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2004,19 +2046,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A11)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A11)</f>
         <v>11</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A11)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1.2</v>
       </c>
       <c r="F11" s="6">
@@ -2033,19 +2075,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A12)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F12" s="6">
@@ -2062,19 +2104,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$52,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$52=$A13)*('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
         <v>1.2</v>
       </c>
       <c r="F13" s="6">
@@ -2092,23 +2134,23 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$52)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
-        <v>1.8666666666666667</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <v>1.875</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$52)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$52&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$52&lt;&gt;"")),"")</f>
-        <v>1.0333333333333334</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <v>1.03125</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.8333333333333333</v>
+        <v>-0.84375</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2373,8 +2415,21 @@
       <c r="F41" s="18"/>
       <c r="G41" s="18"/>
     </row>
+    <row r="42" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="18"/>
+      <c r="G42" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2390,6 +2445,7 @@
     <mergeCell ref="B39:G39"/>
     <mergeCell ref="B40:G40"/>
     <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B42:G42"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2398,7 +2454,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2417,28 +2473,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2446,16 +2502,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2465,10 +2521,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2476,14 +2532,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2493,10 +2549,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2504,16 +2560,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2523,10 +2579,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2534,16 +2590,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2553,10 +2609,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2564,16 +2620,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2583,10 +2639,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2594,16 +2650,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2613,10 +2669,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2624,14 +2680,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2641,10 +2697,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2652,7 +2708,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2661,7 +2717,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2671,10 +2727,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2682,16 +2738,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2701,10 +2757,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2712,14 +2768,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2729,10 +2785,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2740,14 +2796,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2757,10 +2813,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2768,14 +2824,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2785,10 +2841,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2796,14 +2852,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2813,10 +2869,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2824,14 +2880,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2841,10 +2897,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2852,16 +2908,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2871,10 +2927,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2882,16 +2938,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2901,10 +2957,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2912,14 +2968,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2929,10 +2985,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2940,16 +2996,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -2959,10 +3015,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2970,16 +3026,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -2989,10 +3045,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3000,16 +3056,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3019,10 +3075,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3030,14 +3086,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3047,10 +3103,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3058,16 +3114,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3077,10 +3133,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3088,14 +3144,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -3105,10 +3161,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3116,14 +3172,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3133,10 +3189,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3144,16 +3200,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3163,10 +3219,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3174,14 +3230,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3191,10 +3247,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3202,16 +3258,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D28" s="34">
         <v>2</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>138</v>
+        <v>175</v>
       </c>
       <c r="F28" s="34">
         <v>0</v>
@@ -3221,10 +3277,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H28" s="31" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3232,83 +3288,87 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="D29" s="22"/>
+        <v>178</v>
+      </c>
+      <c r="D29" s="22">
+        <v>2</v>
+      </c>
       <c r="E29" s="21" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F29" s="22">
         <v>1</v>
       </c>
       <c r="G29" s="23" t="str">
         <f>IF(OR(D29="",F29=""),"chưa rõ",IF(F29&gt;D29,"FRACILE",IF(D29&gt;F29,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>Vivoire</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="26" t="s">
-        <v>177</v>
-      </c>
-      <c r="C30" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="F30" s="28">
-        <v>2</v>
-      </c>
-      <c r="G30" s="29" t="str">
+      <c r="A30" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="D30" s="22">
+        <v>2</v>
+      </c>
+      <c r="E30" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="F30" s="22">
+        <v>1</v>
+      </c>
+      <c r="G30" s="23" t="str">
         <f>IF(OR(D30="",F30=""),"chưa rõ",IF(F30&gt;D30,"FRACILE",IF(D30&gt;F30,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
-      </c>
-      <c r="H30" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="I30" s="30" t="s">
-        <v>180</v>
+        <v>Vivoire</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="I30" s="24" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="26" t="s">
-        <v>181</v>
-      </c>
-      <c r="C31" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="D31" s="28"/>
-      <c r="E31" s="27" t="s">
-        <v>182</v>
-      </c>
-      <c r="F31" s="28">
-        <v>2</v>
-      </c>
-      <c r="G31" s="29" t="str">
+      <c r="A31" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D31" s="22"/>
+      <c r="E31" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="F31" s="22">
+        <v>1</v>
+      </c>
+      <c r="G31" s="23" t="str">
         <f>IF(OR(D31="",F31=""),"chưa rõ",IF(F31&gt;D31,"FRACILE",IF(D31&gt;F31,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H31" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="I31" s="30" t="s">
-        <v>183</v>
+      <c r="H31" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="I31" s="24" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3316,14 +3376,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3333,10 +3393,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3344,14 +3404,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3361,10 +3421,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3372,14 +3432,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3389,70 +3449,66 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="B35" s="26" t="s">
+        <v>201</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" s="28"/>
+      <c r="E35" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="F35" s="28">
+        <v>2</v>
+      </c>
+      <c r="G35" s="29" t="str">
+        <f>IF(OR(D35="",F35=""),"chưa rõ",IF(F35&gt;D35,"FRACILE",IF(D35&gt;F35,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H35" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="C35" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="D35" s="22">
-        <v>2</v>
-      </c>
-      <c r="E35" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="F35" s="22">
-        <v>2</v>
-      </c>
-      <c r="G35" s="23" t="str">
-        <f>IF(OR(D35="",F35=""),"chưa rõ",IF(F35&gt;D35,"FRACILE",IF(D35&gt;F35,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H35" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="I35" s="24" t="s">
-        <v>194</v>
+      <c r="I35" s="30" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="32" t="s">
-        <v>195</v>
-      </c>
-      <c r="C36" s="33" t="s">
-        <v>196</v>
-      </c>
-      <c r="D36" s="34">
-        <v>2</v>
-      </c>
-      <c r="E36" s="33" t="s">
-        <v>197</v>
-      </c>
-      <c r="F36" s="34">
-        <v>0</v>
-      </c>
-      <c r="G36" s="35" t="str">
+      <c r="B36" s="26" t="s">
+        <v>204</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" s="28"/>
+      <c r="E36" s="27" t="s">
+        <v>205</v>
+      </c>
+      <c r="F36" s="28">
+        <v>2</v>
+      </c>
+      <c r="G36" s="29" t="str">
         <f>IF(OR(D36="",F36=""),"chưa rõ",IF(F36&gt;D36,"FRACILE",IF(D36&gt;F36,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H36" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="I36" s="36" t="s">
-        <v>198</v>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H36" s="25" t="s">
+        <v>193</v>
+      </c>
+      <c r="I36" s="30" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3460,16 +3516,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D37" s="22">
         <v>2</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>200</v>
+        <v>117</v>
       </c>
       <c r="F37" s="22">
         <v>2</v>
@@ -3479,10 +3535,10 @@
         <v>hoà</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3490,16 +3546,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="32" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>115</v>
+        <v>210</v>
       </c>
       <c r="D38" s="34">
         <v>2</v>
       </c>
       <c r="E38" s="33" t="s">
-        <v>138</v>
+        <v>211</v>
       </c>
       <c r="F38" s="34">
         <v>0</v>
@@ -3509,10 +3565,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="31" t="s">
-        <v>139</v>
+        <v>95</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>142</v>
+        <v>212</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3520,16 +3576,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>204</v>
+        <v>117</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="F39" s="22">
         <v>2</v>
@@ -3539,55 +3595,57 @@
         <v>hoà</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="19" t="s">
+      <c r="A40" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B40" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="C40" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="D40" s="22"/>
-      <c r="E40" s="21" t="s">
-        <v>209</v>
-      </c>
-      <c r="F40" s="22">
-        <v>1</v>
-      </c>
-      <c r="G40" s="23" t="str">
+      <c r="B40" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="C40" s="33" t="s">
+        <v>117</v>
+      </c>
+      <c r="D40" s="34">
+        <v>2</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="F40" s="34">
+        <v>0</v>
+      </c>
+      <c r="G40" s="35" t="str">
         <f>IF(OR(D40="",F40=""),"chưa rõ",IF(F40&gt;D40,"FRACILE",IF(D40&gt;F40,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
-      </c>
-      <c r="H40" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="I40" s="24" t="s">
-        <v>210</v>
+        <v>Vivoire</v>
+      </c>
+      <c r="H40" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="I40" s="36" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>115</v>
+        <v>218</v>
       </c>
       <c r="D41" s="22">
         <v>2</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>115</v>
+        <v>219</v>
       </c>
       <c r="F41" s="22">
         <v>2</v>
@@ -3597,218 +3655,216 @@
         <v>hoà</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>70</v>
+        <v>220</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="31" t="s">
+      <c r="A42" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="D42" s="22"/>
+      <c r="E42" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="F42" s="22">
+        <v>1</v>
+      </c>
+      <c r="G42" s="23" t="str">
+        <f>IF(OR(D42="",F42=""),"chưa rõ",IF(F42&gt;D42,"FRACILE",IF(D42&gt;F42,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H42" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="I42" s="24" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="32" t="s">
-        <v>213</v>
-      </c>
-      <c r="C42" s="33" t="s">
-        <v>214</v>
-      </c>
-      <c r="D42" s="34">
-        <v>2</v>
-      </c>
-      <c r="E42" s="33" t="s">
-        <v>138</v>
-      </c>
-      <c r="F42" s="34">
+      <c r="B43" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="D43" s="22">
+        <v>2</v>
+      </c>
+      <c r="E43" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="F43" s="22">
+        <v>2</v>
+      </c>
+      <c r="G43" s="23" t="str">
+        <f>IF(OR(D43="",F43=""),"chưa rõ",IF(F43&gt;D43,"FRACILE",IF(D43&gt;F43,"Vivoire","hoà")))</f>
+        <v>hoà</v>
+      </c>
+      <c r="H43" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="I43" s="24" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" s="32" t="s">
+        <v>227</v>
+      </c>
+      <c r="C44" s="33" t="s">
+        <v>228</v>
+      </c>
+      <c r="D44" s="34">
+        <v>2</v>
+      </c>
+      <c r="E44" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="F44" s="34">
         <v>0</v>
       </c>
-      <c r="G42" s="35" t="str">
-        <f>IF(OR(D42="",F42=""),"chưa rõ",IF(F42&gt;D42,"FRACILE",IF(D42&gt;F42,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H42" s="31" t="s">
-        <v>139</v>
-      </c>
-      <c r="I42" s="36" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="B43" s="32" t="s">
-        <v>215</v>
-      </c>
-      <c r="C43" s="33" t="s">
-        <v>216</v>
-      </c>
-      <c r="D43" s="34">
-        <v>2</v>
-      </c>
-      <c r="E43" s="33" t="s">
-        <v>138</v>
-      </c>
-      <c r="F43" s="34">
-        <v>0</v>
-      </c>
-      <c r="G43" s="35" t="str">
-        <f>IF(OR(D43="",F43=""),"chưa rõ",IF(F43&gt;D43,"FRACILE",IF(D43&gt;F43,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H43" s="31" t="s">
-        <v>139</v>
-      </c>
-      <c r="I43" s="36" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B44" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="C44" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="D44" s="22">
-        <v>2</v>
-      </c>
-      <c r="E44" s="21" t="s">
-        <v>218</v>
-      </c>
-      <c r="F44" s="22">
-        <v>1</v>
-      </c>
-      <c r="G44" s="23" t="str">
+      <c r="G44" s="35" t="str">
         <f>IF(OR(D44="",F44=""),"chưa rõ",IF(F44&gt;D44,"FRACILE",IF(D44&gt;F44,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H44" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="I44" s="24" t="s">
-        <v>142</v>
+      <c r="H44" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="I44" s="36" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="25" t="s">
+      <c r="A45" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B45" s="26" t="s">
-        <v>219</v>
-      </c>
-      <c r="C45" s="27" t="s">
-        <v>220</v>
-      </c>
-      <c r="D45" s="28">
+      <c r="B45" s="32" t="s">
+        <v>229</v>
+      </c>
+      <c r="C45" s="33" t="s">
+        <v>230</v>
+      </c>
+      <c r="D45" s="34">
+        <v>2</v>
+      </c>
+      <c r="E45" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="F45" s="34">
+        <v>0</v>
+      </c>
+      <c r="G45" s="35" t="str">
+        <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H45" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="I45" s="36" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="D46" s="22">
+        <v>2</v>
+      </c>
+      <c r="E46" s="21" t="s">
+        <v>232</v>
+      </c>
+      <c r="F46" s="22">
         <v>1</v>
       </c>
-      <c r="E45" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="F45" s="28">
-        <v>2</v>
-      </c>
-      <c r="G45" s="29" t="str">
-        <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
+      <c r="G46" s="23" t="str">
+        <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H46" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="I46" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B47" s="26" t="s">
+        <v>233</v>
+      </c>
+      <c r="C47" s="27" t="s">
+        <v>234</v>
+      </c>
+      <c r="D47" s="28">
+        <v>1</v>
+      </c>
+      <c r="E47" s="27" t="s">
+        <v>235</v>
+      </c>
+      <c r="F47" s="28">
+        <v>2</v>
+      </c>
+      <c r="G47" s="29" t="str">
+        <f>IF(OR(D47="",F47=""),"chưa rõ",IF(F47&gt;D47,"FRACILE",IF(D47&gt;F47,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H45" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="I45" s="30" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="25" t="s">
+      <c r="H47" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="I47" s="30" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B46" s="26" t="s">
-        <v>223</v>
-      </c>
-      <c r="C46" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="D46" s="28"/>
-      <c r="E46" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="F46" s="28">
-        <v>2</v>
-      </c>
-      <c r="G46" s="29" t="str">
-        <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
+      <c r="B48" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="C48" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="D48" s="28"/>
+      <c r="E48" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="F48" s="28">
+        <v>2</v>
+      </c>
+      <c r="G48" s="29" t="str">
+        <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H46" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="I46" s="30" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B47" s="20" t="s">
-        <v>226</v>
-      </c>
-      <c r="C47" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="D47" s="22">
-        <v>2</v>
-      </c>
-      <c r="E47" s="21" t="s">
-        <v>227</v>
-      </c>
-      <c r="F47" s="22">
-        <v>1</v>
-      </c>
-      <c r="G47" s="23" t="str">
-        <f>IF(OR(D47="",F47=""),"chưa rõ",IF(F47&gt;D47,"FRACILE",IF(D47&gt;F47,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H47" s="19" t="s">
-        <v>228</v>
-      </c>
-      <c r="I47" s="24" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B48" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="C48" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="D48" s="22">
-        <v>2</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>231</v>
-      </c>
-      <c r="F48" s="22">
-        <v>1</v>
-      </c>
-      <c r="G48" s="23" t="str">
-        <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H48" s="19" t="s">
-        <v>232</v>
-      </c>
-      <c r="I48" s="24" t="s">
-        <v>233</v>
+      <c r="H48" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="I48" s="30" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3816,16 +3872,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>37</v>
+        <v>240</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3835,10 +3891,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3846,16 +3902,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>237</v>
+        <v>117</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -3865,68 +3921,128 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>70</v>
+        <v>246</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="25" t="s">
+      <c r="A51" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B51" s="26" t="s">
-        <v>240</v>
-      </c>
-      <c r="C51" s="27" t="s">
-        <v>241</v>
-      </c>
-      <c r="D51" s="28">
+      <c r="B51" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C51" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="D51" s="22">
+        <v>2</v>
+      </c>
+      <c r="E51" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="F51" s="22">
         <v>1</v>
       </c>
-      <c r="E51" s="27" t="s">
-        <v>242</v>
-      </c>
-      <c r="F51" s="28">
-        <v>2</v>
-      </c>
-      <c r="G51" s="29" t="str">
+      <c r="G51" s="23" t="str">
         <f>IF(OR(D51="",F51=""),"chưa rõ",IF(F51&gt;D51,"FRACILE",IF(D51&gt;F51,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H51" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="I51" s="24" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="C52" s="21" t="s">
+        <v>251</v>
+      </c>
+      <c r="D52" s="22">
+        <v>2</v>
+      </c>
+      <c r="E52" s="21" t="s">
+        <v>252</v>
+      </c>
+      <c r="F52" s="22">
+        <v>1</v>
+      </c>
+      <c r="G52" s="23" t="str">
+        <f>IF(OR(D52="",F52=""),"chưa rõ",IF(F52&gt;D52,"FRACILE",IF(D52&gt;F52,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H52" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="I52" s="24" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B53" s="26" t="s">
+        <v>254</v>
+      </c>
+      <c r="C53" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="D53" s="28">
+        <v>1</v>
+      </c>
+      <c r="E53" s="27" t="s">
+        <v>256</v>
+      </c>
+      <c r="F53" s="28">
+        <v>2</v>
+      </c>
+      <c r="G53" s="29" t="str">
+        <f>IF(OR(D53="",F53=""),"chưa rõ",IF(F53&gt;D53,"FRACILE",IF(D53&gt;F53,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H51" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="I51" s="30" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="25" t="s">
+      <c r="H53" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="I53" s="30" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B52" s="26" t="s">
-        <v>244</v>
-      </c>
-      <c r="C52" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="D52" s="28"/>
-      <c r="E52" s="27" t="s">
-        <v>245</v>
-      </c>
-      <c r="F52" s="28">
-        <v>2</v>
-      </c>
-      <c r="G52" s="29" t="str">
-        <f>IF(OR(D52="",F52=""),"chưa rõ",IF(F52&gt;D52,"FRACILE",IF(D52&gt;F52,"Vivoire","hoà")))</f>
+      <c r="B54" s="26" t="s">
+        <v>258</v>
+      </c>
+      <c r="C54" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="D54" s="28"/>
+      <c r="E54" s="27" t="s">
+        <v>259</v>
+      </c>
+      <c r="F54" s="28">
+        <v>2</v>
+      </c>
+      <c r="G54" s="29" t="str">
+        <f>IF(OR(D54="",F54=""),"chưa rõ",IF(F54&gt;D54,"FRACILE",IF(D54&gt;F54,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H52" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="I52" s="30" t="s">
-        <v>246</v>
+      <c r="H54" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="I54" s="30" t="s">
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -3950,12 +4066,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3971,301 +4087,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="B11" s="21" t="s">
+        <v>284</v>
+      </c>
+      <c r="C11" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="C11" s="19" t="s">
-        <v>256</v>
-      </c>
       <c r="D11" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
+        <v>315</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>316</v>
+      </c>
+      <c r="C20" s="25" t="s">
         <v>301</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="D20" s="27" t="s">
         <v>302</v>
       </c>
-      <c r="C20" s="25" t="s">
-        <v>287</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>288</v>
-      </c>
       <c r="E20" s="27" t="s">
-        <v>303</v>
+        <v>317</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>305</v>
+        <v>319</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>306</v>
+        <v>320</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4316,358 +4432,358 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>313</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
       <c r="B4" s="40">
         <v>33</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>317</v>
+        <v>331</v>
       </c>
       <c r="B5" s="40">
         <v>353</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>318</v>
+        <v>332</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>320</v>
+        <v>334</v>
       </c>
       <c r="B6" s="40">
         <v>188</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>322</v>
+        <v>336</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>324</v>
+        <v>338</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>325</v>
+        <v>339</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>326</v>
+        <v>340</v>
       </c>
       <c r="B9" s="40">
         <v>19</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>327</v>
+        <v>341</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>328</v>
+        <v>342</v>
       </c>
       <c r="B10" s="40">
         <v>4</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>329</v>
+        <v>343</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>330</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>331</v>
+        <v>345</v>
       </c>
       <c r="B11" s="40">
         <v>35</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>332</v>
+        <v>346</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>333</v>
+        <v>347</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>334</v>
+        <v>348</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>335</v>
+        <v>349</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>336</v>
+        <v>350</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>337</v>
+        <v>351</v>
       </c>
       <c r="B14" s="40">
         <v>10</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>338</v>
+        <v>352</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>339</v>
+        <v>353</v>
       </c>
       <c r="B15" s="40">
         <v>8</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>340</v>
+        <v>354</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>342</v>
+        <v>356</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>343</v>
+        <v>357</v>
       </c>
       <c r="B17" s="40">
         <v>0</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>344</v>
+        <v>358</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>345</v>
+        <v>359</v>
       </c>
       <c r="B19" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C19" s="44" t="s">
-        <v>346</v>
+        <v>360</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>347</v>
+        <v>361</v>
       </c>
       <c r="B20" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>348</v>
+        <v>362</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>349</v>
+        <v>363</v>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>350</v>
+        <v>364</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>351</v>
+        <v>365</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>352</v>
+        <v>366</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>353</v>
+        <v>367</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>356</v>
+        <v>370</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>358</v>
+        <v>372</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>356</v>
+        <v>370</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>359</v>
+        <v>373</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>360</v>
+        <v>374</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="46" t="s">
-        <v>361</v>
+        <v>375</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>362</v>
+        <v>376</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>363</v>
+        <v>377</v>
       </c>
       <c r="D29" s="47" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="46" t="s">
-        <v>365</v>
+        <v>379</v>
       </c>
       <c r="B30" s="47" t="s">
-        <v>366</v>
+        <v>380</v>
       </c>
       <c r="C30" s="47" t="s">
-        <v>367</v>
+        <v>381</v>
       </c>
       <c r="D30" s="47" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>368</v>
+        <v>382</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>369</v>
+        <v>383</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>370</v>
+        <v>384</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>371</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -4690,24 +4806,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>372</v>
+        <v>386</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>374</v>
+        <v>388</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>375</v>
+        <v>389</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>376</v>
+        <v>390</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>377</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4715,16 +4831,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>378</v>
+        <v>392</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>379</v>
+        <v>393</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>380</v>
+        <v>394</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>381</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4732,16 +4848,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>382</v>
+        <v>396</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>383</v>
+        <v>397</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>384</v>
+        <v>398</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>385</v>
+        <v>399</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4749,16 +4865,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>386</v>
+        <v>400</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>387</v>
+        <v>401</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>388</v>
+        <v>402</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>389</v>
+        <v>403</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4766,16 +4882,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>390</v>
+        <v>404</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>391</v>
+        <v>405</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>392</v>
+        <v>406</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>393</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật bảng so sánh: lỗi lưu bài 24–26/09 và cách sửa, form soạn bài đã dịch
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="411">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -216,6 +216,12 @@
     <t>XP + đổi XP lấy bài + theo dõi bạn học (101–103). Tour giới thiệu cho Lịch, Flashcard, Tài khoản, XP. Trang đăng nhập có lớp phủ trượt. Chuông thông báo + nhãn XP trên thanh trên. Màn theo dõi luyện tập của giáo viên làm lại; tên Google « Quốc Hùng Đỗ » hiển thị « Đỗ Quốc Hùng ».</t>
   </si>
   <si>
+    <t>26/09 — lỗi lưu bài</t>
+  </si>
+  <si>
+    <t>Từ 24/09 mọi lần giáo viên lưu bài đều hỏng — do bản sửa 24/09 (upsert đòi quyền đọc cột đáp án). Sửa bằng RPC luu_cau_hoi (104). Phát hiện nhờ chủ dự án gửi ảnh; thông báo lỗi nay kèm lý do.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -749,7 +755,7 @@
     <t>Việt · Pháp · Anh</t>
   </si>
   <si>
-    <t>shared/i18n.jsx; check:nav 74 ca</t>
+    <t>shared/i18n.jsx; check:nav 74 ca. 26/09: form soạn bài (60 chuỗi), chuông thông báo, theo dõi luyện tập đã dịch — còn một số màn giáo viên cũ viết cứng tiếng Pháp</t>
   </si>
   <si>
     <t>Thanh toán</t>
@@ -872,7 +878,10 @@
     <t>/professeur/dashboard → Builder</t>
   </si>
   <si>
-    <t>Đường GHI vẫn CHƯA được thử tay đầy đủ — xem mục còn treo trong CLAUDE.md.</t>
+    <t>Đang chạy — sửa lỗi lưu 26/09</t>
+  </si>
+  <si>
+    <t>LƯU BÀI HỎNG 24–26/09 (upsert từ client bị từ chối vì cột đáp án bị khoá). Nay ghi qua RPC luu_cau_hoi (104), một transaction; đã thử bằng claim giả, CHƯA thử lại qua giao diện. Form đã dịch ba thứ tiếng.</t>
   </si>
   <si>
     <t>/professeur/examens</t>
@@ -1873,7 +1882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2428,8 +2437,21 @@
       <c r="F42" s="18"/>
       <c r="G42" s="18"/>
     </row>
+    <row r="43" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2446,6 +2468,7 @@
     <mergeCell ref="B40:G40"/>
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B43:G43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2473,28 +2496,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2502,16 +2525,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2521,10 +2544,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2532,14 +2555,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2549,10 +2572,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2560,16 +2583,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2579,10 +2602,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2590,16 +2613,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2609,10 +2632,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2620,16 +2643,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2639,10 +2662,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2650,16 +2673,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2669,10 +2692,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2680,14 +2703,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2697,10 +2720,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2708,7 +2731,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2717,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2727,10 +2750,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2738,16 +2761,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2757,10 +2780,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2768,14 +2791,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2785,10 +2808,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2796,14 +2819,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2813,10 +2836,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2824,14 +2847,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2841,10 +2864,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2852,14 +2875,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2869,10 +2892,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2880,14 +2903,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2897,10 +2920,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2908,16 +2931,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2927,10 +2950,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2938,16 +2961,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2957,10 +2980,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2968,14 +2991,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -2985,10 +3008,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2996,16 +3019,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -3015,10 +3038,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3026,16 +3049,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3045,10 +3068,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3056,16 +3079,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3075,10 +3098,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3086,14 +3109,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3103,10 +3126,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3114,16 +3137,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3133,10 +3156,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3144,14 +3167,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -3161,10 +3184,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3172,14 +3195,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3189,10 +3212,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3200,16 +3223,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3219,10 +3242,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3230,14 +3253,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3247,10 +3270,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3258,16 +3281,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D28" s="34">
         <v>2</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F28" s="34">
         <v>0</v>
@@ -3277,10 +3300,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H28" s="31" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3288,16 +3311,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F29" s="22">
         <v>1</v>
@@ -3307,10 +3330,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3318,16 +3341,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F30" s="22">
         <v>1</v>
@@ -3337,10 +3360,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3348,14 +3371,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D31" s="22"/>
       <c r="E31" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F31" s="22">
         <v>1</v>
@@ -3365,10 +3388,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I31" s="24" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3376,14 +3399,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3393,10 +3416,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3404,14 +3427,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3421,10 +3444,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3432,14 +3455,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3449,10 +3472,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3460,14 +3483,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3477,10 +3500,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3488,14 +3511,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3505,10 +3528,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3516,16 +3539,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D37" s="22">
         <v>2</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F37" s="22">
         <v>2</v>
@@ -3535,10 +3558,10 @@
         <v>hoà</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3546,16 +3569,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="32" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D38" s="34">
         <v>2</v>
       </c>
       <c r="E38" s="33" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F38" s="34">
         <v>0</v>
@@ -3565,10 +3588,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3576,16 +3599,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F39" s="22">
         <v>2</v>
@@ -3595,10 +3618,10 @@
         <v>hoà</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3606,16 +3629,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="32" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D40" s="34">
         <v>2</v>
       </c>
       <c r="E40" s="33" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F40" s="34">
         <v>0</v>
@@ -3625,10 +3648,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H40" s="31" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3636,16 +3659,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D41" s="22">
         <v>2</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F41" s="22">
         <v>2</v>
@@ -3655,10 +3678,10 @@
         <v>hoà</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3666,14 +3689,14 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D42" s="22"/>
       <c r="E42" s="21" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F42" s="22">
         <v>1</v>
@@ -3683,10 +3706,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3694,16 +3717,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F43" s="22">
         <v>2</v>
@@ -3713,10 +3736,10 @@
         <v>hoà</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3724,16 +3747,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D44" s="34">
         <v>2</v>
       </c>
       <c r="E44" s="33" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -3743,10 +3766,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3754,16 +3777,16 @@
         <v>16</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D45" s="34">
         <v>2</v>
       </c>
       <c r="E45" s="33" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F45" s="34">
         <v>0</v>
@@ -3773,10 +3796,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I45" s="36" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3784,16 +3807,16 @@
         <v>16</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3803,10 +3826,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3814,16 +3837,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D47" s="28">
         <v>1</v>
       </c>
       <c r="E47" s="27" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F47" s="28">
         <v>2</v>
@@ -3833,10 +3856,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H47" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I47" s="30" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3844,14 +3867,14 @@
         <v>16</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D48" s="28"/>
       <c r="E48" s="27" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F48" s="28">
         <v>2</v>
@@ -3861,10 +3884,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H48" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3872,16 +3895,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -3891,10 +3914,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3902,16 +3925,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -3921,10 +3944,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3935,13 +3958,13 @@
         <v>37</v>
       </c>
       <c r="C51" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D51" s="22">
         <v>2</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F51" s="22">
         <v>1</v>
@@ -3951,10 +3974,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="I51" s="24" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3962,16 +3985,16 @@
         <v>17</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D52" s="22">
         <v>2</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F52" s="22">
         <v>1</v>
@@ -3981,10 +4004,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I52" s="24" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3992,16 +4015,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D53" s="28">
         <v>1</v>
       </c>
       <c r="E53" s="27" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F53" s="28">
         <v>2</v>
@@ -4011,10 +4034,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H53" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I53" s="30" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4022,14 +4045,14 @@
         <v>17</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D54" s="28"/>
       <c r="E54" s="27" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F54" s="28">
         <v>2</v>
@@ -4039,10 +4062,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H54" s="25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -4066,12 +4089,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4087,301 +4110,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>274</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>275</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>272</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>273</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>270</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>72</v>
+        <v>279</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>308</v>
+      </c>
+      <c r="C17" s="25" t="s">
         <v>304</v>
       </c>
-      <c r="B17" s="27" t="s">
-        <v>305</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>301</v>
-      </c>
       <c r="D17" s="27" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4432,358 +4455,358 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B4" s="40">
         <v>33</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B5" s="40">
         <v>353</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B6" s="40">
         <v>188</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B9" s="40">
         <v>19</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B10" s="40">
         <v>4</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B11" s="40">
         <v>35</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B14" s="40">
         <v>10</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B15" s="40">
         <v>8</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B17" s="40">
         <v>0</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B19" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C19" s="44" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B20" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C26" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>371</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C27" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>371</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B28" s="21" t="s">
+        <v>377</v>
+      </c>
+      <c r="C28" s="21" t="s">
         <v>374</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="D28" s="21" t="s">
         <v>371</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="46" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="D29" s="47" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="46" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B30" s="47" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C30" s="47" t="s">
+        <v>384</v>
+      </c>
+      <c r="D30" s="47" t="s">
         <v>381</v>
-      </c>
-      <c r="D30" s="47" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -4806,24 +4829,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4831,16 +4854,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4848,16 +4871,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4865,16 +4888,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4882,16 +4905,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FAQ 15 câu khớp tính năng hiện có (XP, chuỗi ngày, theo dõi, mở bài bằng XP, quên mật khẩu); sửa câu hứa gợi ý AI chưa bật. Bảng so sánh: FAQ 1→2, flashcard ghi 8 bộ nháp
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="412">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -222,6 +222,12 @@
     <t>Từ 24/09 mọi lần giáo viên lưu bài đều hỏng — do bản sửa 24/09 (upsert đòi quyền đọc cột đáp án). Sửa bằng RPC luu_cau_hoi (104). Phát hiện nhờ chủ dự án gửi ảnh; thông báo lỗi nay kèm lý do.</t>
   </si>
   <si>
+    <t>26/09 — FAQ + Flashcard</t>
+  </si>
+  <si>
+    <t>FAQ 1 → 2: 15 câu khớp tính năng hiện có, sửa câu hứa « xin gợi ý AI » (chưa bật). Soạn 8 bộ Flashcard mới (2 bộ/kỹ năng, 96 thẻ, B1–B2), để nháp chờ chủ dự án duyệt.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -524,10 +530,10 @@
     <t>Không công bố số thẻ</t>
   </si>
   <si>
-    <t>4 bộ · 35 thẻ, đủ bốn kỹ năng, cả bốn công khai. Còn nhỏ so với một thư viện flashcard thật</t>
-  </si>
-  <si>
-    <t>Đang chạy — 4 công khai</t>
+    <t>12 bộ · 131 thẻ (26/09), nhưng 8 bộ mới (96 thẻ) còn NHÁP chờ duyệt — học sinh hiện thấy 4 bộ · 35 thẻ</t>
+  </si>
+  <si>
+    <t>Đang chạy — 4 công khai, 8 nháp</t>
   </si>
   <si>
     <t>the_bo = 4, the_bo_the = 35; học sinh mở bằng tài khoản thật thấy đủ bốn bộ (21/09)</t>
@@ -770,13 +776,10 @@
     <t>Câu hỏi thường gặp (FAQ)</t>
   </si>
   <si>
-    <t>Có từ 21/09 — 9 câu, mỗi câu đối chiếu với mã nguồn. Chưa có email liên hệ</t>
-  </si>
-  <si>
-    <t>Có — thiếu email liên hệ</t>
-  </si>
-  <si>
-    <t>/faq; EMAIL_LIEN_HE trong TrangPhapLy.jsx đang trống</t>
+    <t>15 câu (cập nhật 26/09): XP, chuỗi ngày, theo dõi bạn học, mở bài bằng XP, quên mật khẩu, liên hệ. Mỗi câu đối chiếu mã nguồn; câu AI chấm ghi rõ « chưa bật ». Có email liên hệ</t>
+  </si>
+  <si>
+    <t>/faq; contact.fracile@gmail.com</t>
   </si>
   <si>
     <t>Điều khoản sử dụng</t>
@@ -1882,7 +1885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2126,11 +2129,11 @@
       </c>
       <c r="E13" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="F13" s="6">
         <f>IFERROR(E13-D13,"")</f>
-        <v>-0.6000000000000001</v>
+        <v>-0.40000000000000013</v>
       </c>
       <c r="G13" s="7" t="str">
         <f>IF(OR(C13&lt;3,F13=""),"quá ít mục",IF(F13&gt;0.25,"FRACILE",IF(F13&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2155,11 +2158,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.03125</v>
+        <v>1.0625</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.84375</v>
+        <v>-0.8125</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2450,8 +2453,21 @@
       <c r="F43" s="18"/>
       <c r="G43" s="18"/>
     </row>
+    <row r="44" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2469,6 +2485,7 @@
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="B42:G42"/>
     <mergeCell ref="B43:G43"/>
+    <mergeCell ref="B44:G44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2496,28 +2513,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2525,16 +2542,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2544,10 +2561,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2555,14 +2572,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2572,10 +2589,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2583,16 +2600,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2602,10 +2619,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2613,16 +2630,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2632,10 +2649,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2643,16 +2660,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2662,10 +2679,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2673,16 +2690,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2692,10 +2709,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2703,14 +2720,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2720,10 +2737,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2731,7 +2748,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2740,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2750,10 +2767,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2761,16 +2778,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2780,10 +2797,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2791,14 +2808,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2808,10 +2825,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2819,14 +2836,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2836,10 +2853,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2847,14 +2864,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2864,10 +2881,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2875,14 +2892,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2892,10 +2909,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2903,14 +2920,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2920,10 +2937,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2931,16 +2948,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2950,10 +2967,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2961,16 +2978,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2980,10 +2997,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2991,14 +3008,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3008,10 +3025,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3019,16 +3036,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -3038,10 +3055,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3049,16 +3066,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3068,10 +3085,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3079,16 +3096,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3098,10 +3115,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3109,14 +3126,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3126,10 +3143,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3137,16 +3154,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3156,10 +3173,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3167,14 +3184,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="21" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F24" s="22">
         <v>1</v>
@@ -3184,10 +3201,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3195,14 +3212,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3212,10 +3229,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3223,16 +3240,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3242,10 +3259,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3253,14 +3270,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3270,10 +3287,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3281,16 +3298,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D28" s="34">
         <v>2</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F28" s="34">
         <v>0</v>
@@ -3300,10 +3317,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H28" s="31" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3311,16 +3328,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F29" s="22">
         <v>1</v>
@@ -3330,10 +3347,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3341,16 +3358,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F30" s="22">
         <v>1</v>
@@ -3360,10 +3377,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3371,14 +3388,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D31" s="22"/>
       <c r="E31" s="21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F31" s="22">
         <v>1</v>
@@ -3388,10 +3405,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I31" s="24" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3399,14 +3416,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3416,10 +3433,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3427,14 +3444,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3444,10 +3461,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3455,14 +3472,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3472,10 +3489,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3483,14 +3500,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3500,10 +3517,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3511,14 +3528,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3528,10 +3545,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3539,16 +3556,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D37" s="22">
         <v>2</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F37" s="22">
         <v>2</v>
@@ -3558,10 +3575,10 @@
         <v>hoà</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3569,16 +3586,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="32" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D38" s="34">
         <v>2</v>
       </c>
       <c r="E38" s="33" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F38" s="34">
         <v>0</v>
@@ -3588,10 +3605,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="31" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3599,16 +3616,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F39" s="22">
         <v>2</v>
@@ -3618,10 +3635,10 @@
         <v>hoà</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3629,16 +3646,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="32" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D40" s="34">
         <v>2</v>
       </c>
       <c r="E40" s="33" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F40" s="34">
         <v>0</v>
@@ -3648,10 +3665,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H40" s="31" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3659,16 +3676,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D41" s="22">
         <v>2</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F41" s="22">
         <v>2</v>
@@ -3678,10 +3695,10 @@
         <v>hoà</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3689,14 +3706,14 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D42" s="22"/>
       <c r="E42" s="21" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F42" s="22">
         <v>1</v>
@@ -3706,10 +3723,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3717,16 +3734,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F43" s="22">
         <v>2</v>
@@ -3736,10 +3753,10 @@
         <v>hoà</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3747,16 +3764,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D44" s="34">
         <v>2</v>
       </c>
       <c r="E44" s="33" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -3766,10 +3783,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3777,16 +3794,16 @@
         <v>16</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D45" s="34">
         <v>2</v>
       </c>
       <c r="E45" s="33" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F45" s="34">
         <v>0</v>
@@ -3796,10 +3813,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I45" s="36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3807,16 +3824,16 @@
         <v>16</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3826,10 +3843,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3837,16 +3854,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D47" s="28">
         <v>1</v>
       </c>
       <c r="E47" s="27" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="F47" s="28">
         <v>2</v>
@@ -3856,10 +3873,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H47" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I47" s="30" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3867,14 +3884,14 @@
         <v>16</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D48" s="28"/>
       <c r="E48" s="27" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F48" s="28">
         <v>2</v>
@@ -3884,10 +3901,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H48" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3895,29 +3912,29 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F49" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G49" s="23" t="str">
         <f>IF(OR(D49="",F49=""),"chưa rõ",IF(F49&gt;D49,"FRACILE",IF(D49&gt;F49,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>244</v>
+        <v>76</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3925,16 +3942,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -3944,10 +3961,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3958,13 +3975,13 @@
         <v>37</v>
       </c>
       <c r="C51" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D51" s="22">
         <v>2</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F51" s="22">
         <v>1</v>
@@ -3974,10 +3991,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I51" s="24" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3985,16 +4002,16 @@
         <v>17</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D52" s="22">
         <v>2</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F52" s="22">
         <v>1</v>
@@ -4004,10 +4021,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I52" s="24" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4015,16 +4032,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D53" s="28">
         <v>1</v>
       </c>
       <c r="E53" s="27" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F53" s="28">
         <v>2</v>
@@ -4034,10 +4051,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H53" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I53" s="30" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4045,14 +4062,14 @@
         <v>17</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D54" s="28"/>
       <c r="E54" s="27" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F54" s="28">
         <v>2</v>
@@ -4062,10 +4079,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H54" s="25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -4089,12 +4106,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4110,301 +4127,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4455,358 +4472,358 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B4" s="40">
         <v>33</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B5" s="40">
         <v>353</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B6" s="40">
         <v>188</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B9" s="40">
         <v>19</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B10" s="40">
         <v>4</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B11" s="40">
         <v>35</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B14" s="40">
         <v>10</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B15" s="40">
         <v>8</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B17" s="40">
         <v>0</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B19" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C19" s="44" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B20" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>375</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>372</v>
-      </c>
-      <c r="B26" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>375</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>374</v>
-      </c>
       <c r="D27" s="21" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="46" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D29" s="47" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="46" t="s">
+        <v>383</v>
+      </c>
+      <c r="B30" s="47" t="s">
+        <v>384</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>385</v>
+      </c>
+      <c r="D30" s="47" t="s">
         <v>382</v>
-      </c>
-      <c r="B30" s="47" t="s">
-        <v>383</v>
-      </c>
-      <c r="C30" s="47" t="s">
-        <v>384</v>
-      </c>
-      <c r="D30" s="47" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -4829,24 +4846,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4854,16 +4871,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4871,16 +4888,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4888,16 +4905,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4905,16 +4922,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng xếp hạng XP trong nhóm theo dõi (105) + tab trong thẻ Đang theo dõi; 6 bài luyện nháp B1–B2 (scripts/nhap); bảng so sánh: flashcard 1→2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="414">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -228,6 +228,12 @@
     <t>FAQ 1 → 2: 15 câu khớp tính năng hiện có, sửa câu hứa « xin gợi ý AI » (chưa bật). Soạn 8 bộ Flashcard mới (2 bộ/kỹ năng, 96 thẻ, B1–B2), để nháp chờ chủ dự án duyệt.</t>
   </si>
   <si>
+    <t>26/09 — tiếp</t>
+  </si>
+  <si>
+    <t>Flashcard 1 → 2: công khai 8 bộ mới, học sinh thấy 12 bộ · 131 thẻ (đo bằng claim giả). Bảng xếp hạng XP (105). Soạn 6 bài luyện nháp B1–B2 (60 câu, đủ lời giải) — chưa tính vào « Số bài luyện » tới khi công khai.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -530,10 +536,10 @@
     <t>Không công bố số thẻ</t>
   </si>
   <si>
-    <t>12 bộ · 131 thẻ (26/09), nhưng 8 bộ mới (96 thẻ) còn NHÁP chờ duyệt — học sinh hiện thấy 4 bộ · 35 thẻ</t>
-  </si>
-  <si>
-    <t>Đang chạy — 4 công khai, 8 nháp</t>
+    <t>12 bộ · 131 thẻ, cả 12 công khai (26/09), 3 bộ mỗi kỹ năng, mỗi thẻ có câu ví dụ</t>
+  </si>
+  <si>
+    <t>Đang chạy — 12 công khai</t>
   </si>
   <si>
     <t>the_bo = 4, the_bo_the = 35; học sinh mở bằng tài khoản thật thấy đủ bốn bộ (21/09)</t>
@@ -605,7 +611,7 @@
     <t>Có (bạn bè, bảng xếp hạng)</t>
   </si>
   <si>
-    <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa ». Chưa có bảng xếp hạng</t>
+    <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa » + bảng xếp hạng XP trong nhóm mình theo dõi (26/09). Chưa lên 2: chưa ai dùng qua giao diện</t>
   </si>
   <si>
     <t>Đang chạy — chưa ai theo dõi qua giao diện</t>
@@ -1885,7 +1891,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2466,8 +2472,21 @@
       <c r="F44" s="18"/>
       <c r="G44" s="18"/>
     </row>
+    <row r="45" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2486,6 +2505,7 @@
     <mergeCell ref="B42:G42"/>
     <mergeCell ref="B43:G43"/>
     <mergeCell ref="B44:G44"/>
+    <mergeCell ref="B45:G45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2513,28 +2533,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2542,16 +2562,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2561,10 +2581,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2572,14 +2592,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2589,10 +2609,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2600,16 +2620,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F4" s="22">
         <v>1</v>
@@ -2619,10 +2639,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2630,16 +2650,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2649,10 +2669,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2660,16 +2680,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2679,10 +2699,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2690,16 +2710,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2709,10 +2729,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2720,14 +2740,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2737,10 +2757,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2748,7 +2768,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2757,7 +2777,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2767,10 +2787,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2778,16 +2798,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2797,10 +2817,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2808,14 +2828,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2825,10 +2845,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2836,14 +2856,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2853,10 +2873,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2864,14 +2884,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2881,10 +2901,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2892,14 +2912,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2909,10 +2929,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2920,14 +2940,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2937,10 +2957,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2948,16 +2968,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2967,10 +2987,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2978,16 +2998,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -2997,10 +3017,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3008,14 +3028,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3025,10 +3045,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3036,16 +3056,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -3055,10 +3075,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3066,16 +3086,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3085,10 +3105,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3096,16 +3116,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3115,10 +3135,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3126,14 +3146,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3143,10 +3163,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3154,16 +3174,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3173,38 +3193,38 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="21" t="s">
+      <c r="B24" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="F24" s="22">
-        <v>1</v>
-      </c>
-      <c r="G24" s="23" t="str">
+      <c r="C24" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="D24" s="28"/>
+      <c r="E24" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="F24" s="28">
+        <v>2</v>
+      </c>
+      <c r="G24" s="29" t="str">
         <f>IF(OR(D24="",F24=""),"chưa rõ",IF(F24&gt;D24,"FRACILE",IF(D24&gt;F24,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H24" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="I24" s="24" t="s">
-        <v>165</v>
+      <c r="H24" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="I24" s="30" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3212,14 +3232,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3229,10 +3249,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3240,16 +3260,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3259,10 +3279,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3270,14 +3290,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3287,10 +3307,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3298,16 +3318,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D28" s="34">
         <v>2</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F28" s="34">
         <v>0</v>
@@ -3317,10 +3337,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H28" s="31" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3328,16 +3348,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F29" s="22">
         <v>1</v>
@@ -3347,10 +3367,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3358,16 +3378,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F30" s="22">
         <v>1</v>
@@ -3377,10 +3397,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3388,14 +3408,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D31" s="22"/>
       <c r="E31" s="21" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F31" s="22">
         <v>1</v>
@@ -3405,10 +3425,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I31" s="24" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3416,14 +3436,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3433,10 +3453,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3444,14 +3464,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3461,10 +3481,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3472,14 +3492,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3489,10 +3509,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3500,14 +3520,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3517,10 +3537,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3528,14 +3548,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3545,10 +3565,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3556,16 +3576,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D37" s="22">
         <v>2</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F37" s="22">
         <v>2</v>
@@ -3575,10 +3595,10 @@
         <v>hoà</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3586,16 +3606,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="32" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D38" s="34">
         <v>2</v>
       </c>
       <c r="E38" s="33" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F38" s="34">
         <v>0</v>
@@ -3605,10 +3625,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H38" s="31" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3616,16 +3636,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F39" s="22">
         <v>2</v>
@@ -3635,10 +3655,10 @@
         <v>hoà</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3646,16 +3666,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="32" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D40" s="34">
         <v>2</v>
       </c>
       <c r="E40" s="33" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F40" s="34">
         <v>0</v>
@@ -3665,10 +3685,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H40" s="31" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3676,16 +3696,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D41" s="22">
         <v>2</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F41" s="22">
         <v>2</v>
@@ -3695,10 +3715,10 @@
         <v>hoà</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3706,14 +3726,14 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D42" s="22"/>
       <c r="E42" s="21" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F42" s="22">
         <v>1</v>
@@ -3723,10 +3743,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3734,16 +3754,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F43" s="22">
         <v>2</v>
@@ -3753,10 +3773,10 @@
         <v>hoà</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3764,16 +3784,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D44" s="34">
         <v>2</v>
       </c>
       <c r="E44" s="33" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -3783,10 +3803,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3794,16 +3814,16 @@
         <v>16</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D45" s="34">
         <v>2</v>
       </c>
       <c r="E45" s="33" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F45" s="34">
         <v>0</v>
@@ -3813,10 +3833,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I45" s="36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3824,16 +3844,16 @@
         <v>16</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3843,10 +3863,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3854,16 +3874,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D47" s="28">
         <v>1</v>
       </c>
       <c r="E47" s="27" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F47" s="28">
         <v>2</v>
@@ -3873,10 +3893,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H47" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I47" s="30" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3884,14 +3904,14 @@
         <v>16</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D48" s="28"/>
       <c r="E48" s="27" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F48" s="28">
         <v>2</v>
@@ -3901,10 +3921,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H48" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3912,16 +3932,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F49" s="22">
         <v>2</v>
@@ -3931,10 +3951,10 @@
         <v>hoà</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3942,16 +3962,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -3961,10 +3981,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,13 +3995,13 @@
         <v>37</v>
       </c>
       <c r="C51" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D51" s="22">
         <v>2</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F51" s="22">
         <v>1</v>
@@ -3991,10 +4011,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="I51" s="24" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4002,16 +4022,16 @@
         <v>17</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D52" s="22">
         <v>2</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F52" s="22">
         <v>1</v>
@@ -4021,10 +4041,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I52" s="24" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4032,16 +4052,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D53" s="28">
         <v>1</v>
       </c>
       <c r="E53" s="27" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F53" s="28">
         <v>2</v>
@@ -4051,10 +4071,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H53" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I53" s="30" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4062,14 +4082,14 @@
         <v>17</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D54" s="28"/>
       <c r="E54" s="27" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F54" s="28">
         <v>2</v>
@@ -4079,10 +4099,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H54" s="25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -4106,12 +4126,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4127,301 +4147,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>277</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>275</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>276</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>273</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
+        <v>324</v>
+      </c>
+      <c r="B21" s="27" t="s">
         <v>322</v>
       </c>
-      <c r="B21" s="27" t="s">
-        <v>320</v>
-      </c>
       <c r="C21" s="25" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4472,358 +4492,358 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B4" s="40">
         <v>33</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B5" s="40">
         <v>353</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B6" s="40">
         <v>188</v>
       </c>
       <c r="C6" s="41" t="s">
+        <v>341</v>
+      </c>
+      <c r="D6" s="42" t="s">
         <v>339</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B9" s="40">
         <v>19</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B10" s="40">
         <v>4</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B11" s="40">
         <v>35</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B14" s="40">
         <v>10</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B15" s="40">
         <v>8</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B17" s="40">
         <v>0</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B19" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C19" s="44" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B20" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B26" s="21" t="s">
+        <v>376</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>377</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>374</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>375</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
+        <v>378</v>
+      </c>
+      <c r="B27" s="21" t="s">
         <v>376</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="C27" s="21" t="s">
+        <v>377</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>374</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>375</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
+        <v>379</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>380</v>
+      </c>
+      <c r="C28" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="B28" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>375</v>
-      </c>
       <c r="D28" s="21" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="46" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D29" s="47" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B30" s="47" t="s">
+        <v>386</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>387</v>
+      </c>
+      <c r="D30" s="47" t="s">
         <v>384</v>
-      </c>
-      <c r="C30" s="47" t="s">
-        <v>385</v>
-      </c>
-      <c r="D30" s="47" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -4846,24 +4866,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4871,16 +4891,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4888,16 +4908,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4905,16 +4925,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4922,16 +4942,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: số liệu đo 26/09 (413 câu, 248 lời giải, 12 bộ/131 thẻ, 12 tài khoản, 6 bài nháp)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="418">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -458,7 +458,7 @@
     <t>33 bài (ĐẾM THẬT trên production)</t>
   </si>
   <si>
-    <t>select count(*) from exercises = 33, đo 24/09/2026 (09/09 là 34)</t>
+    <t>33 bài luyện công khai, đo 26/09/2026; +6 bài nháp B1–B2 chờ duyệt — lên 39 khi xuất bản</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -467,10 +467,10 @@
     <t>Không công bố</t>
   </si>
   <si>
-    <t>353 câu, 7 dạng (qcm, fill, conj, vf, tableau, order, tự luận)</t>
-  </si>
-  <si>
-    <t>select count(*) from questions = 353, đo 24/09/2026</t>
+    <t>413 câu, 7 dạng (qcm, fill, conj, vf, tableau, order, tự luận) — 60 câu thuộc bài nháp</t>
+  </si>
+  <si>
+    <t>select count(*) from questions = 413, đo 26/09/2026</t>
   </si>
   <si>
     <t>Từ điển Pháp–Việt</t>
@@ -1048,82 +1048,94 @@
     <t>Bài tập</t>
   </si>
   <si>
-    <t>select count(*) from exercises</t>
+    <t>select count(*) from exercises — 33 luyện tập + 1 bài giao + 6 NHÁP chờ duyệt</t>
+  </si>
+  <si>
+    <t>26/09/2026</t>
+  </si>
+  <si>
+    <t>Câu hỏi</t>
+  </si>
+  <si>
+    <t>select count(*) from questions — gồm 60 câu của 6 bài nháp</t>
+  </si>
+  <si>
+    <t>Câu có lời giải thích</t>
+  </si>
+  <si>
+    <t>questions where explanation is not null — gồm 60 câu nháp</t>
+  </si>
+  <si>
+    <t>Câu có neo ngữ liệu</t>
+  </si>
+  <si>
+    <t>questions where evidence is not null — trên 2 bài</t>
+  </si>
+  <si>
+    <t>24/09/2026</t>
+  </si>
+  <si>
+    <t>Đề thi thử</t>
+  </si>
+  <si>
+    <t>select count(*) from exams</t>
+  </si>
+  <si>
+    <t>Lượt làm bài đã chấm</t>
+  </si>
+  <si>
+    <t>attempts where finished_at is not null</t>
+  </si>
+  <si>
+    <t>Bộ Flashcard (cả 12 công khai)</t>
+  </si>
+  <si>
+    <t>select count(*) from the_bo where cong_khai</t>
+  </si>
+  <si>
+    <t>Thẻ trong các bộ</t>
+  </si>
+  <si>
+    <t>select count(*) from the_bo_the</t>
+  </si>
+  <si>
+    <t>Thẻ trong bảng cards</t>
+  </si>
+  <si>
+    <t>select count(*) from cards — 36 thẻ đi theo hai tài khoản thử đã xoá</t>
+  </si>
+  <si>
+    <t>Lượt trả lời đã ghi</t>
+  </si>
+  <si>
+    <t>select count(*) from answers — 50 đi theo tài khoản thử, ~70 mất vì lỗi lưu bài (đã sửa)</t>
+  </si>
+  <si>
+    <t>Tài khoản</t>
+  </si>
+  <si>
+    <t>select count(*) from profiles</t>
+  </si>
+  <si>
+    <t>Lượt đổi XP lấy bài</t>
+  </si>
+  <si>
+    <t>exercise_access where status='XP' — chưa bài nào đặt giá XP</t>
+  </si>
+  <si>
+    <t>Lượt theo dõi bạn học</t>
+  </si>
+  <si>
+    <t>select count(*) from follows</t>
+  </si>
+  <si>
+    <t>Bài tự luận CHƯA có điểm nào</t>
+  </si>
+  <si>
+    <t>câu open, không điểm GV lẫn tự chấm. 7/8 thuộc 2 tài khoản thử của chủ dự án; 1 bài của học sinh thật, dài 12 ký tự</t>
   </si>
   <si>
     <t>21/09/2026</t>
-  </si>
-  <si>
-    <t>Câu hỏi</t>
-  </si>
-  <si>
-    <t>select count(*) from questions — giảm 19, chưa rõ vì sao</t>
-  </si>
-  <si>
-    <t>24/09/2026</t>
-  </si>
-  <si>
-    <t>Câu có lời giải thích</t>
-  </si>
-  <si>
-    <t>questions where explanation is not null — giảm 21, chưa rõ vì sao</t>
-  </si>
-  <si>
-    <t>Câu có neo ngữ liệu</t>
-  </si>
-  <si>
-    <t>questions where evidence is not null — trên 2 bài</t>
-  </si>
-  <si>
-    <t>Đề thi thử</t>
-  </si>
-  <si>
-    <t>select count(*) from exams</t>
-  </si>
-  <si>
-    <t>Lượt làm bài đã chấm</t>
-  </si>
-  <si>
-    <t>attempts where finished_at is not null</t>
-  </si>
-  <si>
-    <t>Bộ Flashcard (cả bốn công khai)</t>
-  </si>
-  <si>
-    <t>select count(*) from the_bo</t>
-  </si>
-  <si>
-    <t>22/09/2026</t>
-  </si>
-  <si>
-    <t>Thẻ trong các bộ</t>
-  </si>
-  <si>
-    <t>select count(*) from the_bo_the</t>
-  </si>
-  <si>
-    <t>Thẻ trong bảng cards</t>
-  </si>
-  <si>
-    <t>select count(*) from cards — 36 thẻ đi theo hai tài khoản thử đã xoá</t>
-  </si>
-  <si>
-    <t>Lượt trả lời đã ghi</t>
-  </si>
-  <si>
-    <t>select count(*) from answers — 50 đi theo tài khoản thử, ~70 mất vì lỗi lưu bài (đã sửa)</t>
-  </si>
-  <si>
-    <t>Tài khoản</t>
-  </si>
-  <si>
-    <t>select count(*) from profiles</t>
-  </si>
-  <si>
-    <t>Bài tự luận CHƯA có điểm nào</t>
-  </si>
-  <si>
-    <t>câu open, không điểm GV lẫn tự chấm. 7/8 thuộc 2 tài khoản thử của chủ dự án; 1 bài của học sinh thật, dài 12 ký tự</t>
   </si>
   <si>
     <t>Lượt ôn Flashcard đã ghi</t>
@@ -4481,7 +4493,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -4514,7 +4526,7 @@
         <v>334</v>
       </c>
       <c r="B4" s="40">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
         <v>335</v>
@@ -4528,41 +4540,41 @@
         <v>337</v>
       </c>
       <c r="B5" s="40">
-        <v>353</v>
+        <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
         <v>338</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
+        <v>339</v>
+      </c>
+      <c r="B6" s="40">
+        <v>248</v>
+      </c>
+      <c r="C6" s="41" t="s">
         <v>340</v>
       </c>
-      <c r="B6" s="40">
-        <v>188</v>
-      </c>
-      <c r="C6" s="41" t="s">
-        <v>341</v>
-      </c>
       <c r="D6" s="42" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
+        <v>342</v>
+      </c>
+      <c r="D7" s="42" t="s">
         <v>343</v>
-      </c>
-      <c r="D7" s="42" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4576,7 +4588,7 @@
         <v>345</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -4584,13 +4596,13 @@
         <v>346</v>
       </c>
       <c r="B9" s="40">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
         <v>347</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -4598,24 +4610,24 @@
         <v>348</v>
       </c>
       <c r="B10" s="40">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
         <v>349</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>350</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
+        <v>350</v>
+      </c>
+      <c r="B11" s="40">
+        <v>131</v>
+      </c>
+      <c r="C11" s="41" t="s">
         <v>351</v>
-      </c>
-      <c r="B11" s="40">
-        <v>35</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>352</v>
       </c>
       <c r="D11" s="42" t="s">
         <v>336</v>
@@ -4623,55 +4635,55 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
+        <v>356</v>
+      </c>
+      <c r="B14" s="40">
+        <v>12</v>
+      </c>
+      <c r="C14" s="41" t="s">
         <v>357</v>
       </c>
-      <c r="B14" s="40">
-        <v>10</v>
-      </c>
-      <c r="C14" s="41" t="s">
-        <v>358</v>
-      </c>
       <c r="D14" s="42" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
+        <v>358</v>
+      </c>
+      <c r="B15" s="40">
+        <v>0</v>
+      </c>
+      <c r="C15" s="41" t="s">
         <v>359</v>
-      </c>
-      <c r="B15" s="40">
-        <v>8</v>
-      </c>
-      <c r="C15" s="41" t="s">
-        <v>360</v>
       </c>
       <c r="D15" s="42" t="s">
         <v>336</v>
@@ -4679,106 +4691,106 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
+        <v>362</v>
+      </c>
+      <c r="B17" s="40">
+        <v>8</v>
+      </c>
+      <c r="C17" s="41" t="s">
         <v>363</v>
       </c>
-      <c r="B17" s="40">
+      <c r="D17" s="42" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="B18" s="40">
         <v>0</v>
       </c>
-      <c r="C17" s="41" t="s">
+      <c r="C18" s="41" t="s">
+        <v>366</v>
+      </c>
+      <c r="D18" s="42" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="39" t="s">
+        <v>367</v>
+      </c>
+      <c r="B19" s="40">
+        <v>0</v>
+      </c>
+      <c r="C19" s="41" t="s">
+        <v>368</v>
+      </c>
+      <c r="D19" s="42" t="s">
         <v>364</v>
       </c>
-      <c r="D17" s="42" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>365</v>
-      </c>
-      <c r="B19" s="43">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
-      <c r="C19" s="44" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
-        <v>367</v>
-      </c>
-      <c r="B20" s="45">
+      <c r="C21" s="44" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
-      <c r="C20" s="44" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="38" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="C22" s="44" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="38" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="B25" s="21" t="s">
-        <v>372</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>373</v>
-      </c>
-      <c r="D25" s="21" t="s">
+      <c r="C26" s="3" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="19" t="s">
+      <c r="D26" s="3" t="s">
         <v>375</v>
-      </c>
-      <c r="B26" s="21" t="s">
-        <v>376</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>377</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>378</v>
+        <v>144</v>
       </c>
       <c r="B27" s="21" t="s">
         <v>376</v>
@@ -4787,7 +4799,7 @@
         <v>377</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -4798,52 +4810,80 @@
         <v>380</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="46" t="s">
+      <c r="A29" s="19" t="s">
+        <v>382</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>380</v>
+      </c>
+      <c r="C29" s="21" t="s">
         <v>381</v>
       </c>
-      <c r="B29" s="47" t="s">
-        <v>382</v>
-      </c>
-      <c r="C29" s="47" t="s">
+      <c r="D29" s="21" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="19" t="s">
         <v>383</v>
       </c>
-      <c r="D29" s="47" t="s">
+      <c r="B30" s="21" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="46" t="s">
+      <c r="C30" s="21" t="s">
+        <v>381</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="46" t="s">
         <v>385</v>
       </c>
-      <c r="B30" s="47" t="s">
+      <c r="B31" s="47" t="s">
         <v>386</v>
       </c>
-      <c r="C30" s="47" t="s">
+      <c r="C31" s="47" t="s">
         <v>387</v>
       </c>
-      <c r="D30" s="47" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
+      <c r="D31" s="47" t="s">
         <v>388</v>
       </c>
-      <c r="B31" s="21" t="s">
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="46" t="s">
         <v>389</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="B32" s="47" t="s">
         <v>390</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="C32" s="47" t="s">
         <v>391</v>
+      </c>
+      <c r="D32" s="47" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="19" t="s">
+        <v>392</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>393</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>394</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>395</v>
       </c>
     </row>
   </sheetData>
@@ -4866,24 +4906,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4891,16 +4931,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4908,16 +4948,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4925,16 +4965,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4942,16 +4982,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: AI chấm PE đã bật (1→2), chấm bài cho học sinh 0→1, số liệu 27/09
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="421">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -234,6 +234,12 @@
     <t>Flashcard 1 → 2: công khai 8 bộ mới, học sinh thấy 12 bộ · 131 thẻ (đo bằng claim giả). Bảng xếp hạng XP (105). Soạn 6 bài luyện nháp B1–B2 (60 câu, đủ lời giải) — chưa tính vào « Số bài luyện » tới khi công khai.</t>
   </si>
   <si>
+    <t>27/09</t>
+  </si>
+  <si>
+    <t>AI chấm PE BẬT (OpenAI gpt-6-luna, chủ dự án chọn vì rẻ nhất; thử qua giao diện: có nhận xét). Bài viết (PE) — AI chấm 1 → 2; Chấm bài cho học sinh 0 → 1. Thêm tour « Nền tối và cài đặt » + nút « Xem lại hướng dẫn »; Chính sách bảo mật ghi OpenAI.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -299,13 +305,10 @@
     <t>AI chấm ngữ pháp và cách diễn đạt</t>
   </si>
   <si>
-    <t>DỰNG XONG 09/09 nhưng CHƯA BẬT — thiếu khoá API. Gợi ý theo đúng các tiêu chí grille, không tự điền; học sinh bấm « dùng số này » mới nhận</t>
-  </si>
-  <si>
-    <t>DỰNG XONG — CHƯA BẬT</t>
-  </si>
-  <si>
-    <t>Edge Function cham-pe trả 503 CHUA_CAU_HINH_KHOA; pe_ai_goi_y = 0 dòng (đo 21/09). Bật: npx supabase secrets set ANTHROPIC_API_KEY=…</t>
+    <t>ĐÃ BẬT 27/09 — OpenAI gpt-6-luna. Gợi ý điểm + nhận xét tiếng Việt theo từng tiêu chí grille; không tự điền, học sinh bấm « dùng số này » mới nhận. 6 lượt / 24 giờ</t>
+  </si>
+  <si>
+    <t>Edge Function cham-pe; chủ dự án thử qua giao diện 27/09, pe_ai_goi_y = 1 dòng (model gpt-6-luna). Đổi model: secrets set PE_AI_MODEL=…</t>
   </si>
   <si>
     <t>Bài nói (PO) — ghi âm và nghe lại</t>
@@ -692,10 +695,13 @@
     <t>Có — chấm tự động và AI, giáo viên chốt</t>
   </si>
   <si>
-    <t>ĐÃ GỠ (học sinh tự chấm theo grille; AI chấm chưa dựng)</t>
-  </si>
-  <si>
-    <t>Quyết định và thi hành cùng ngày 09/09/2026. Xem sheet « Tài khoản giáo viên »</t>
+    <t>Giáo viên không chấm (gỡ 09/09). Máy chủ chấm câu khách quan; bài viết: AI gợi ý (bật 27/09) + học sinh chốt. Chưa có bước giáo viên duyệt</t>
+  </si>
+  <si>
+    <t>Đang chạy — không có giáo viên chốt</t>
+  </si>
+  <si>
+    <t>Giáo viên chấm tay gỡ 09/09/2026 (có chủ đích). Chưa lên 2 vì Vivoire có giáo viên chốt điểm</t>
   </si>
   <si>
     <t>Gửi nhận xét tới một học sinh</t>
@@ -1117,6 +1123,9 @@
     <t>select count(*) from profiles</t>
   </si>
   <si>
+    <t>27/09/2026</t>
+  </si>
+  <si>
     <t>Lượt đổi XP lấy bài</t>
   </si>
   <si>
@@ -1147,7 +1156,7 @@
     <t>Gợi ý chấm AI đã sinh</t>
   </si>
   <si>
-    <t>select count(*) from pe_ai_goi_y — khoá API chưa đặt</t>
+    <t>select count(*) from pe_ai_goi_y — gpt-6-luna, bật 27/09</t>
   </si>
   <si>
     <t>Tỷ lệ câu có lời giải</t>
@@ -1903,7 +1912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1973,11 +1982,11 @@
       </c>
       <c r="E7" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="F7" s="6">
         <f>IFERROR(E7-D7,"")</f>
-        <v>-0.6666666666666667</v>
+        <v>-0.5</v>
       </c>
       <c r="G7" s="7" t="str">
         <f>IF(OR(C7&lt;3,F7=""),"quá ít mục",IF(F7&gt;0.25,"FRACILE",IF(F7&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2089,11 +2098,11 @@
       </c>
       <c r="E11" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="F11" s="6">
         <f>IFERROR(E11-D11,"")</f>
-        <v>-0.8</v>
+        <v>-0.6000000000000001</v>
       </c>
       <c r="G11" s="7" t="str">
         <f>IF(OR(C11&lt;3,F11=""),"quá ít mục",IF(F11&gt;0.25,"FRACILE",IF(F11&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2176,11 +2185,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.0625</v>
+        <v>1.125</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.8125</v>
+        <v>-0.75</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2497,8 +2506,21 @@
       <c r="F45" s="18"/>
       <c r="G45" s="18"/>
     </row>
+    <row r="46" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2518,6 +2540,7 @@
     <mergeCell ref="B43:G43"/>
     <mergeCell ref="B44:G44"/>
     <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B46:G46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2545,28 +2568,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2574,16 +2597,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2593,10 +2616,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2604,14 +2627,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2621,10 +2644,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2632,29 +2655,29 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F4" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="23" t="str">
         <f>IF(OR(D4="",F4=""),"chưa rõ",IF(F4&gt;D4,"FRACILE",IF(D4&gt;F4,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2662,16 +2685,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2681,10 +2704,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2692,16 +2715,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D6" s="34">
         <v>2</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -2711,10 +2734,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2722,16 +2745,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2741,10 +2764,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2752,14 +2775,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2769,10 +2792,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2780,7 +2803,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2789,7 +2812,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2799,10 +2822,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2810,16 +2833,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2829,10 +2852,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2840,14 +2863,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2857,10 +2880,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2868,14 +2891,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2885,10 +2908,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2896,14 +2919,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -2913,10 +2936,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2924,14 +2947,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -2941,10 +2964,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2952,14 +2975,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -2969,10 +2992,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2980,16 +3003,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -2999,10 +3022,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3010,16 +3033,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -3029,10 +3052,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3040,14 +3063,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3057,10 +3080,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3068,16 +3091,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -3087,10 +3110,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3098,16 +3121,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3117,10 +3140,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3128,16 +3151,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3147,10 +3170,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3158,14 +3181,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3175,10 +3198,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3186,16 +3209,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3205,10 +3228,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3216,14 +3239,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3233,10 +3256,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3244,14 +3267,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3261,10 +3284,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3272,16 +3295,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3291,10 +3314,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3302,14 +3325,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3319,10 +3342,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3330,16 +3353,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D28" s="34">
         <v>2</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F28" s="34">
         <v>0</v>
@@ -3349,10 +3372,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H28" s="31" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3360,16 +3383,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F29" s="22">
         <v>1</v>
@@ -3379,10 +3402,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3390,16 +3413,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F30" s="22">
         <v>1</v>
@@ -3409,10 +3432,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3420,14 +3443,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D31" s="22"/>
       <c r="E31" s="21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F31" s="22">
         <v>1</v>
@@ -3437,10 +3460,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I31" s="24" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3448,14 +3471,14 @@
         <v>15</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="27" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F32" s="28">
         <v>2</v>
@@ -3465,10 +3488,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3476,14 +3499,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3493,10 +3516,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3504,14 +3527,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3521,10 +3544,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3532,14 +3555,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3549,10 +3572,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3560,14 +3583,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3577,10 +3600,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3588,16 +3611,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D37" s="22">
         <v>2</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F37" s="22">
         <v>2</v>
@@ -3607,40 +3630,40 @@
         <v>hoà</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="31" t="s">
+      <c r="A38" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B38" s="32" t="s">
-        <v>215</v>
-      </c>
-      <c r="C38" s="33" t="s">
+      <c r="B38" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="D38" s="34">
-        <v>2</v>
-      </c>
-      <c r="E38" s="33" t="s">
+      <c r="C38" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="F38" s="34">
-        <v>0</v>
-      </c>
-      <c r="G38" s="35" t="str">
+      <c r="D38" s="22">
+        <v>2</v>
+      </c>
+      <c r="E38" s="21" t="s">
+        <v>218</v>
+      </c>
+      <c r="F38" s="22">
+        <v>1</v>
+      </c>
+      <c r="G38" s="23" t="str">
         <f>IF(OR(D38="",F38=""),"chưa rõ",IF(F38&gt;D38,"FRACILE",IF(D38&gt;F38,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H38" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="I38" s="36" t="s">
-        <v>218</v>
+      <c r="H38" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="I38" s="24" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3648,16 +3671,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F39" s="22">
         <v>2</v>
@@ -3667,10 +3690,10 @@
         <v>hoà</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3678,16 +3701,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="32" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D40" s="34">
         <v>2</v>
       </c>
       <c r="E40" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F40" s="34">
         <v>0</v>
@@ -3697,10 +3720,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H40" s="31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I40" s="36" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3708,16 +3731,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D41" s="22">
         <v>2</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F41" s="22">
         <v>2</v>
@@ -3727,10 +3750,10 @@
         <v>hoà</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3738,14 +3761,14 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D42" s="22"/>
       <c r="E42" s="21" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F42" s="22">
         <v>1</v>
@@ -3755,10 +3778,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3766,16 +3789,16 @@
         <v>16</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D43" s="22">
         <v>2</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F43" s="22">
         <v>2</v>
@@ -3785,10 +3808,10 @@
         <v>hoà</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3796,16 +3819,16 @@
         <v>16</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D44" s="34">
         <v>2</v>
       </c>
       <c r="E44" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -3815,10 +3838,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3826,16 +3849,16 @@
         <v>16</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D45" s="34">
         <v>2</v>
       </c>
       <c r="E45" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F45" s="34">
         <v>0</v>
@@ -3845,10 +3868,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I45" s="36" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3856,16 +3879,16 @@
         <v>16</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3875,10 +3898,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3886,16 +3909,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D47" s="28">
         <v>1</v>
       </c>
       <c r="E47" s="27" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F47" s="28">
         <v>2</v>
@@ -3905,10 +3928,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H47" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I47" s="30" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3916,14 +3939,14 @@
         <v>16</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D48" s="28"/>
       <c r="E48" s="27" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F48" s="28">
         <v>2</v>
@@ -3933,10 +3956,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H48" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3944,16 +3967,16 @@
         <v>17</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F49" s="22">
         <v>2</v>
@@ -3963,10 +3986,10 @@
         <v>hoà</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3974,16 +3997,16 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -3993,10 +4016,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4007,13 +4030,13 @@
         <v>37</v>
       </c>
       <c r="C51" s="21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D51" s="22">
         <v>2</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F51" s="22">
         <v>1</v>
@@ -4023,10 +4046,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="I51" s="24" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4034,16 +4057,16 @@
         <v>17</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D52" s="22">
         <v>2</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F52" s="22">
         <v>1</v>
@@ -4053,10 +4076,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I52" s="24" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4064,16 +4087,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D53" s="28">
         <v>1</v>
       </c>
       <c r="E53" s="27" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F53" s="28">
         <v>2</v>
@@ -4083,10 +4106,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H53" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I53" s="30" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4094,14 +4117,14 @@
         <v>17</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D54" s="28"/>
       <c r="E54" s="27" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F54" s="28">
         <v>2</v>
@@ -4111,10 +4134,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H54" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -4138,12 +4161,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4159,301 +4182,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>280</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>277</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>275</v>
-      </c>
       <c r="D7" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
+        <v>326</v>
+      </c>
+      <c r="B21" s="27" t="s">
         <v>324</v>
       </c>
-      <c r="B21" s="27" t="s">
-        <v>322</v>
-      </c>
       <c r="C21" s="25" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4504,386 +4527,386 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B4" s="40">
         <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B5" s="40">
         <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
+        <v>340</v>
+      </c>
+      <c r="D5" s="42" t="s">
         <v>338</v>
-      </c>
-      <c r="D5" s="42" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B6" s="40">
         <v>248</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
+        <v>347</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>345</v>
-      </c>
-      <c r="D8" s="42" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B9" s="40">
         <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B14" s="40">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>336</v>
+        <v>360</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B15" s="40">
         <v>0</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B19" s="40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C28" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>381</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C29" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>381</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B30" s="21" t="s">
+        <v>387</v>
+      </c>
+      <c r="C30" s="21" t="s">
         <v>384</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="D30" s="21" t="s">
         <v>381</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="D31" s="47" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="46" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C32" s="47" t="s">
+        <v>394</v>
+      </c>
+      <c r="D32" s="47" t="s">
         <v>391</v>
-      </c>
-      <c r="D32" s="47" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>
@@ -4906,24 +4929,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4931,16 +4954,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4948,16 +4971,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4965,16 +4988,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4982,16 +5005,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: lộ trình game, giờ học đo thật, AI nhận xét bài nói, số tài khoản 14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="425">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -323,19 +323,19 @@
     <t>migration 057/058; bucket `bai-noi` private, đường dẫn mang phân quyền theo user_id</t>
   </si>
   <si>
-    <t>Bài nói (PO) — AI chấm phát âm</t>
+    <t>Bài nói (PO) — AI nhận xét</t>
   </si>
   <si>
     <t>Phát âm 82% · Trôi chảy 76% · Từ vựng B1</t>
   </si>
   <si>
-    <t>CHƯA CÓ</t>
-  </si>
-  <si>
-    <t>CHƯA DỰNG</t>
-  </si>
-  <si>
-    <t>Không có Edge Function nào gọi mô hình giọng nói</t>
+    <t>Nút « AI nhận xét » cạnh bản ghi: chép lời + góp ý ngữ pháp, từ vựng, nối ý bằng tiếng Việt. CỐ Ý không cho điểm phần trăm (quy tắc 1). 6 lượt/24 giờ</t>
+  </si>
+  <si>
+    <t>Đã dựng 27/09 — chưa chạy đầu-cuối (kho bai-noi 0 file)</t>
+  </si>
+  <si>
+    <t>migration 107, Edge Function nhan-xet-noi (gpt-transcribe → gpt-6-luna)</t>
   </si>
   <si>
     <t>Giáo viên chấm tay</t>
@@ -524,7 +524,7 @@
     <t>Flashcard + 3 game mỗi ngày, « ôn từ đúng lúc sắp quên »</t>
   </si>
   <si>
-    <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D, CÓ lịch ôn SM-2 từ 21/09 (chỉ hiện thẻ đến hạn, bốn mức nhớ). Học sinh không tự tạo thẻ; chưa có trò chơi</t>
+    <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D, CÓ lịch ôn SM-2 từ 21/09 (chỉ hiện thẻ đến hạn, bốn mức nhớ). Từ 28/09 có game Lộ trình dựng từ chính các bộ này</t>
   </si>
   <si>
     <t>Đang chạy — lưu thật 22/09</t>
@@ -626,13 +626,25 @@
     <t>Giờ học đo được</t>
   </si>
   <si>
-    <t>CHƯA đo được — hiện dấu gạch kèm lý do, KHÔNG điền số ước lượng</t>
-  </si>
-  <si>
-    <t>Cố ý để trống</t>
-  </si>
-  <si>
-    <t>daily_activity.minutes để sẵn; quy tắc 1 của dự án</t>
+    <t>Đo thật từ 27/09: thời gian từ lúc mở bài tới lúc nộp (kẹp 3 giờ), biểu đồ 7 ngày. Chỉ tính bài nộp từ 27/09 trở đi</t>
+  </si>
+  <si>
+    <t>migration 106: attempts.giay_lam + RPC get_gio_hoc; không điền số ước lượng cho quá khứ</t>
+  </si>
+  <si>
+    <t>Lộ trình học dạng game</t>
+  </si>
+  <si>
+    <t>Lộ trình theo cấp độ</t>
+  </si>
+  <si>
+    <t>Bản đồ uốn lượn 4 chương (Nghe/Đọc/Viết/Nói) · 12 màn = 12 bộ flashcard · trắc nghiệm hai chiều + ghép cặp · 3 tim · 1–3 sao · thử thách cuối chương · mở khoá tuần tự. Không cộng XP (chống cày)</t>
+  </si>
+  <si>
+    <t>Đã dựng 28/09 — chưa ai chơi qua giao diện</t>
+  </si>
+  <si>
+    <t>migration 108/109: lo_trinh_ket_qua + RPC ghi_ket_qua_man (giữ sao cao nhất, có biên nhận)</t>
   </si>
   <si>
     <t>Kiểm soát ai được học bài nào</t>
@@ -734,10 +746,10 @@
     <t>Số tài khoản đang có</t>
   </si>
   <si>
-    <t>9 người dùng (gồm cả tài khoản thử)</t>
-  </si>
-  <si>
-    <t>select count(*) from profiles = 10, đo 24/09/2026</t>
+    <t>14 hồ sơ người dùng (gồm cả tài khoản thử)</t>
+  </si>
+  <si>
+    <t>select count(*) from profiles = 14 (auth.users = 19), đo 28/09/2026</t>
   </si>
   <si>
     <t>Web</t>
@@ -818,7 +830,7 @@
     <t>4 người, có tên và thành tích (HSG quốc gia, thạc sĩ UMass, kỹ sư AI)</t>
   </si>
   <si>
-    <t>1 người — Đỗ Quốc Hùng, ghi « Đội ngũ phát triển »</t>
+    <t>1 người — Đỗ Quốc Hùng, « Solo-creator &amp; Developer », có ảnh</t>
   </si>
   <si>
     <t>TeamSection.jsx; không ghi bằng cấp chưa kiểm chứng được</t>
@@ -1969,24 +1981,24 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A7)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.1666666666666667</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
         <f>IFERROR(E7-D7,"")</f>
-        <v>-0.5</v>
+        <v>-0.3333333333333335</v>
       </c>
       <c r="G7" s="7" t="str">
         <f>IF(OR(C7&lt;3,F7=""),"quá ít mục",IF(F7&gt;0.25,"FRACILE",IF(F7&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -1998,19 +2010,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A8)</f>
         <v>6</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A8)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -2027,19 +2039,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A9)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>0.6</v>
       </c>
       <c r="F9" s="6">
@@ -2056,24 +2068,24 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A10)</f>
-        <v>9</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A10)</f>
+        <v>10</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
-        <v>5</v>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <v>6</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A10)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.2</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <v>1.3333333333333333</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>-0.8</v>
+        <v>-0.6666666666666667</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2085,19 +2097,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A11)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A11)</f>
         <v>11</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A11)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F11" s="6">
@@ -2114,19 +2126,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A12)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F12" s="6">
@@ -2143,19 +2155,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$54,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$54=$A13)*('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F13" s="6">
@@ -2173,23 +2185,23 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$54)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.875</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <v>1.878787878787879</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$54)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$54&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$54&lt;&gt;"")),"")</f>
-        <v>1.125</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <v>1.1818181818181819</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.75</v>
+        <v>-0.696969696969697</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2549,7 +2561,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2711,32 +2723,32 @@
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="D6" s="34">
-        <v>2</v>
-      </c>
-      <c r="E6" s="33" t="s">
+      <c r="D6" s="22">
+        <v>2</v>
+      </c>
+      <c r="E6" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="34">
-        <v>0</v>
-      </c>
-      <c r="G6" s="35" t="str">
+      <c r="F6" s="22">
+        <v>1</v>
+      </c>
+      <c r="G6" s="23" t="str">
         <f>IF(OR(D6="",F6=""),"chưa rõ",IF(F6&gt;D6,"FRACILE",IF(D6&gt;F6,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="H6" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="I6" s="36" t="s">
+      <c r="I6" s="24" t="s">
         <v>98</v>
       </c>
     </row>
@@ -3439,58 +3451,60 @@
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B31" s="26" t="s">
         <v>194</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="C31" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="D31" s="22"/>
-      <c r="E31" s="21" t="s">
+      <c r="D31" s="28"/>
+      <c r="E31" s="27" t="s">
         <v>195</v>
       </c>
-      <c r="F31" s="22">
-        <v>1</v>
-      </c>
-      <c r="G31" s="23" t="str">
+      <c r="F31" s="28">
+        <v>2</v>
+      </c>
+      <c r="G31" s="29" t="str">
         <f>IF(OR(D31="",F31=""),"chưa rõ",IF(F31&gt;D31,"FRACILE",IF(D31&gt;F31,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H31" s="19" t="s">
+      <c r="H31" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I31" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="I31" s="24" t="s">
+    </row>
+    <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" s="20" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B32" s="26" t="s">
+      <c r="C32" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="C32" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="27" t="s">
+      <c r="D32" s="22">
+        <v>2</v>
+      </c>
+      <c r="E32" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="F32" s="28">
-        <v>2</v>
-      </c>
-      <c r="G32" s="29" t="str">
+      <c r="F32" s="22">
+        <v>2</v>
+      </c>
+      <c r="G32" s="23" t="str">
         <f>IF(OR(D32="",F32=""),"chưa rõ",IF(F32&gt;D32,"FRACILE",IF(D32&gt;F32,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
-      </c>
-      <c r="H32" s="25" t="s">
+        <v>hoà</v>
+      </c>
+      <c r="H32" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="I32" s="30" t="s">
+      <c r="I32" s="24" t="s">
         <v>201</v>
       </c>
     </row>
@@ -3516,10 +3530,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3527,14 +3541,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C34" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3544,10 +3558,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3555,14 +3569,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C35" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3572,10 +3586,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3583,14 +3597,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C36" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3600,40 +3614,38 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
+      <c r="A37" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B37" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D37" s="22">
-        <v>2</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="F37" s="22">
-        <v>2</v>
-      </c>
-      <c r="G37" s="23" t="str">
+      <c r="B37" s="26" t="s">
+        <v>215</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="D37" s="28"/>
+      <c r="E37" s="27" t="s">
+        <v>216</v>
+      </c>
+      <c r="F37" s="28">
+        <v>2</v>
+      </c>
+      <c r="G37" s="29" t="str">
         <f>IF(OR(D37="",F37=""),"chưa rõ",IF(F37&gt;D37,"FRACILE",IF(D37&gt;F37,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H37" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="I37" s="24" t="s">
-        <v>215</v>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H37" s="25" t="s">
+        <v>204</v>
+      </c>
+      <c r="I37" s="30" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3641,29 +3653,29 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>217</v>
+        <v>124</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>218</v>
+        <v>124</v>
       </c>
       <c r="F38" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G38" s="23" t="str">
         <f>IF(OR(D38="",F38=""),"chưa rõ",IF(F38&gt;D38,"FRACILE",IF(D38&gt;F38,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="I38" s="24" t="s">
         <v>219</v>
-      </c>
-      <c r="I38" s="24" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3671,10 +3683,10 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="C39" s="21" t="s">
         <v>221</v>
-      </c>
-      <c r="C39" s="21" t="s">
-        <v>124</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
@@ -3683,77 +3695,77 @@
         <v>222</v>
       </c>
       <c r="F39" s="22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39" s="23" t="str">
         <f>IF(OR(D39="",F39=""),"chưa rõ",IF(F39&gt;D39,"FRACILE",IF(D39&gt;F39,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H39" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="I39" s="24" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D40" s="22">
+        <v>2</v>
+      </c>
+      <c r="E40" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="F40" s="22">
+        <v>2</v>
+      </c>
+      <c r="G40" s="23" t="str">
+        <f>IF(OR(D40="",F40=""),"chưa rõ",IF(F40&gt;D40,"FRACILE",IF(D40&gt;F40,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H39" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="I39" s="24" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="31" t="s">
+      <c r="H40" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="I40" s="24" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B40" s="32" t="s">
-        <v>224</v>
-      </c>
-      <c r="C40" s="33" t="s">
+      <c r="B41" s="32" t="s">
+        <v>228</v>
+      </c>
+      <c r="C41" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="D40" s="34">
-        <v>2</v>
-      </c>
-      <c r="E40" s="33" t="s">
+      <c r="D41" s="34">
+        <v>2</v>
+      </c>
+      <c r="E41" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="F40" s="34">
+      <c r="F41" s="34">
         <v>0</v>
       </c>
-      <c r="G40" s="35" t="str">
-        <f>IF(OR(D40="",F40=""),"chưa rõ",IF(F40&gt;D40,"FRACILE",IF(D40&gt;F40,"Vivoire","hoà")))</f>
+      <c r="G41" s="35" t="str">
+        <f>IF(OR(D41="",F41=""),"chưa rõ",IF(F41&gt;D41,"FRACILE",IF(D41&gt;F41,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H40" s="31" t="s">
+      <c r="H41" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="I40" s="36" t="s">
+      <c r="I41" s="36" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B41" s="20" t="s">
-        <v>225</v>
-      </c>
-      <c r="C41" s="21" t="s">
-        <v>226</v>
-      </c>
-      <c r="D41" s="22">
-        <v>2</v>
-      </c>
-      <c r="E41" s="21" t="s">
-        <v>227</v>
-      </c>
-      <c r="F41" s="22">
-        <v>2</v>
-      </c>
-      <c r="G41" s="23" t="str">
-        <f>IF(OR(D41="",F41=""),"chưa rõ",IF(F41&gt;D41,"FRACILE",IF(D41&gt;F41,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H41" s="19" t="s">
-        <v>228</v>
-      </c>
-      <c r="I41" s="24" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3761,87 +3773,87 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="C42" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="C42" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="D42" s="22"/>
+      <c r="D42" s="22">
+        <v>2</v>
+      </c>
       <c r="E42" s="21" t="s">
         <v>231</v>
       </c>
       <c r="F42" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" s="23" t="str">
         <f>IF(OR(D42="",F42=""),"chưa rõ",IF(F42&gt;D42,"FRACILE",IF(D42&gt;F42,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>hoà</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>80</v>
+        <v>232</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D43" s="22">
-        <v>2</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>124</v>
+        <v>235</v>
       </c>
       <c r="F43" s="22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G43" s="23" t="str">
         <f>IF(OR(D43="",F43=""),"chưa rõ",IF(F43&gt;D43,"FRACILE",IF(D43&gt;F43,"Vivoire","hoà")))</f>
-        <v>hoà</v>
+        <v>chưa rõ</v>
       </c>
       <c r="H43" s="19" t="s">
         <v>80</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="31" t="s">
+      <c r="A44" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B44" s="32" t="s">
-        <v>235</v>
-      </c>
-      <c r="C44" s="33" t="s">
-        <v>236</v>
-      </c>
-      <c r="D44" s="34">
-        <v>2</v>
-      </c>
-      <c r="E44" s="33" t="s">
-        <v>147</v>
-      </c>
-      <c r="F44" s="34">
-        <v>0</v>
-      </c>
-      <c r="G44" s="35" t="str">
+      <c r="B44" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D44" s="22">
+        <v>2</v>
+      </c>
+      <c r="E44" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="F44" s="22">
+        <v>2</v>
+      </c>
+      <c r="G44" s="23" t="str">
         <f>IF(OR(D44="",F44=""),"chưa rõ",IF(F44&gt;D44,"FRACILE",IF(D44&gt;F44,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H44" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="I44" s="36" t="s">
-        <v>151</v>
+        <v>hoà</v>
+      </c>
+      <c r="H44" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="I44" s="24" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3849,10 +3861,10 @@
         <v>16</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D45" s="34">
         <v>2</v>
@@ -3875,63 +3887,63 @@
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="19" t="s">
+      <c r="A46" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B46" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="C46" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D46" s="22">
-        <v>2</v>
-      </c>
-      <c r="E46" s="21" t="s">
-        <v>240</v>
-      </c>
-      <c r="F46" s="22">
-        <v>1</v>
-      </c>
-      <c r="G46" s="23" t="str">
+      <c r="B46" s="32" t="s">
+        <v>241</v>
+      </c>
+      <c r="C46" s="33" t="s">
+        <v>242</v>
+      </c>
+      <c r="D46" s="34">
+        <v>2</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="F46" s="34">
+        <v>0</v>
+      </c>
+      <c r="G46" s="35" t="str">
         <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H46" s="19" t="s">
+      <c r="H46" s="31" t="s">
+        <v>148</v>
+      </c>
+      <c r="I46" s="36" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D47" s="22">
+        <v>2</v>
+      </c>
+      <c r="E47" s="21" t="s">
+        <v>244</v>
+      </c>
+      <c r="F47" s="22">
+        <v>1</v>
+      </c>
+      <c r="G47" s="23" t="str">
+        <f>IF(OR(D47="",F47=""),"chưa rõ",IF(F47&gt;D47,"FRACILE",IF(D47&gt;F47,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H47" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="I46" s="24" t="s">
+      <c r="I47" s="24" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B47" s="26" t="s">
-        <v>241</v>
-      </c>
-      <c r="C47" s="27" t="s">
-        <v>242</v>
-      </c>
-      <c r="D47" s="28">
-        <v>1</v>
-      </c>
-      <c r="E47" s="27" t="s">
-        <v>243</v>
-      </c>
-      <c r="F47" s="28">
-        <v>2</v>
-      </c>
-      <c r="G47" s="29" t="str">
-        <f>IF(OR(D47="",F47=""),"chưa rõ",IF(F47&gt;D47,"FRACILE",IF(D47&gt;F47,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H47" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="I47" s="30" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3942,54 +3954,54 @@
         <v>245</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="D48" s="28"/>
+        <v>246</v>
+      </c>
+      <c r="D48" s="28">
+        <v>1</v>
+      </c>
       <c r="E48" s="27" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F48" s="28">
         <v>2</v>
       </c>
       <c r="G48" s="29" t="str">
         <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>FRACILE</v>
       </c>
       <c r="H48" s="25" t="s">
         <v>80</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B49" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="C49" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D49" s="22">
-        <v>2</v>
-      </c>
-      <c r="E49" s="21" t="s">
+      <c r="A49" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B49" s="26" t="s">
         <v>249</v>
       </c>
-      <c r="F49" s="22">
-        <v>2</v>
-      </c>
-      <c r="G49" s="23" t="str">
+      <c r="C49" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="D49" s="28"/>
+      <c r="E49" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="F49" s="28">
+        <v>2</v>
+      </c>
+      <c r="G49" s="29" t="str">
         <f>IF(OR(D49="",F49=""),"chưa rõ",IF(F49&gt;D49,"FRACILE",IF(D49&gt;F49,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H49" s="19" t="s">
+        <v>chưa rõ</v>
+      </c>
+      <c r="H49" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="I49" s="24" t="s">
-        <v>250</v>
+      <c r="I49" s="30" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3997,7 +4009,7 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C50" s="21" t="s">
         <v>124</v>
@@ -4006,17 +4018,17 @@
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F50" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G50" s="23" t="str">
         <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>253</v>
+        <v>80</v>
       </c>
       <c r="I50" s="24" t="s">
         <v>254</v>
@@ -4027,7 +4039,7 @@
         <v>17</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>37</v>
+        <v>255</v>
       </c>
       <c r="C51" s="21" t="s">
         <v>124</v>
@@ -4036,7 +4048,7 @@
         <v>2</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F51" s="22">
         <v>1</v>
@@ -4046,10 +4058,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="I51" s="24" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4057,10 +4069,10 @@
         <v>17</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>257</v>
+        <v>37</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>258</v>
+        <v>124</v>
       </c>
       <c r="D52" s="22">
         <v>2</v>
@@ -4076,39 +4088,39 @@
         <v>Vivoire</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>80</v>
+        <v>257</v>
       </c>
       <c r="I52" s="24" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="25" t="s">
+      <c r="A53" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B53" s="26" t="s">
+      <c r="B53" s="20" t="s">
         <v>261</v>
       </c>
-      <c r="C53" s="27" t="s">
+      <c r="C53" s="21" t="s">
         <v>262</v>
       </c>
-      <c r="D53" s="28">
+      <c r="D53" s="22">
+        <v>2</v>
+      </c>
+      <c r="E53" s="21" t="s">
+        <v>263</v>
+      </c>
+      <c r="F53" s="22">
         <v>1</v>
       </c>
-      <c r="E53" s="27" t="s">
-        <v>263</v>
-      </c>
-      <c r="F53" s="28">
-        <v>2</v>
-      </c>
-      <c r="G53" s="29" t="str">
+      <c r="G53" s="23" t="str">
         <f>IF(OR(D53="",F53=""),"chưa rõ",IF(F53&gt;D53,"FRACILE",IF(D53&gt;F53,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H53" s="25" t="s">
+        <v>Vivoire</v>
+      </c>
+      <c r="H53" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="I53" s="30" t="s">
+      <c r="I53" s="24" t="s">
         <v>264</v>
       </c>
     </row>
@@ -4120,24 +4132,54 @@
         <v>265</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="D54" s="28"/>
+        <v>266</v>
+      </c>
+      <c r="D54" s="28">
+        <v>1</v>
+      </c>
       <c r="E54" s="27" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F54" s="28">
         <v>2</v>
       </c>
       <c r="G54" s="29" t="str">
         <f>IF(OR(D54="",F54=""),"chưa rõ",IF(F54&gt;D54,"FRACILE",IF(D54&gt;F54,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>FRACILE</v>
       </c>
       <c r="H54" s="25" t="s">
         <v>80</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>267</v>
+        <v>268</v>
+      </c>
+    </row>
+    <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B55" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="C55" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="D55" s="28"/>
+      <c r="E55" s="27" t="s">
+        <v>270</v>
+      </c>
+      <c r="F55" s="28">
+        <v>2</v>
+      </c>
+      <c r="G55" s="29" t="str">
+        <f>IF(OR(D55="",F55=""),"chưa rõ",IF(F55&gt;D55,"FRACILE",IF(D55&gt;F55,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H55" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I55" s="30" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -4161,12 +4203,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4182,149 +4224,149 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>80</v>
@@ -4335,148 +4377,148 @@
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B17" s="27" t="s">
+        <v>317</v>
+      </c>
+      <c r="C17" s="25" t="s">
         <v>313</v>
       </c>
-      <c r="C17" s="25" t="s">
-        <v>309</v>
-      </c>
       <c r="D17" s="27" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4527,288 +4569,288 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B4" s="40">
         <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B5" s="40">
         <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B6" s="40">
         <v>248</v>
       </c>
       <c r="C6" s="41" t="s">
+        <v>346</v>
+      </c>
+      <c r="D6" s="42" t="s">
         <v>342</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B9" s="40">
         <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B14" s="40">
         <v>14</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B15" s="40">
         <v>0</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -4816,97 +4858,97 @@
         <v>145</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>387</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>388</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>385</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>383</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>384</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D31" s="47" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="46" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C32" s="47" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="D32" s="47" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -4929,24 +4971,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4954,16 +4996,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4971,16 +5013,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4988,16 +5030,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5005,16 +5047,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
XP khi qua màn lộ trình, trang Từ điển, PWA cài được; cập nhật bảng so sánh
- 110: ghi_ket_qua_man cộng 5 XP (thử thách 15) một lần mỗi màn, chặn màn bịa
- /etudiant/tu-dien: tra hai chiều, bỏ dấu, nguồn là flashcard công khai
- manifest + icon 192/512, cố ý không có service worker lưu đệm

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="433">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -482,18 +482,21 @@
     <t>56.000+ từ · IPA · nghĩa Việt · cấp CEFR · chia động từ · tra ngay trong bài</t>
   </si>
   <si>
+    <t>Có từ 29/09 (/etudiant/tu-dien): 131 mục Pháp–Việt lấy từ flashcard giáo viên công khai, tra hai chiều, không cần gõ dấu, kèm câu ví dụ. Nhỏ hơn Vivoire hàng trăm lần — không IPA, không chia động từ</t>
+  </si>
+  <si>
+    <t>TuDien.jsx; nguồn duy nhất là the_bo_the, không nhúng từ điển ngoài hay AI. Claim giả học sinh đọc được 131 thẻ</t>
+  </si>
+  <si>
+    <t>Podcast / học theo video</t>
+  </si>
+  <si>
     <t>KHÔNG CÓ</t>
   </si>
   <si>
     <t>Không có kế hoạch</t>
   </si>
   <si>
-    <t>Ô chênh lệch lớn nhất trong cả bảng</t>
-  </si>
-  <si>
-    <t>Podcast / học theo video</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -587,10 +590,13 @@
     <t>Đấu dịch thuật PvP trực tiếp</t>
   </si>
   <si>
-    <t>Không có đấu trực tiếp; có XP + theo dõi bạn học (xem hai dòng dưới)</t>
-  </si>
-  <si>
-    <t>Không có kế hoạch PvP</t>
+    <t>Có game Lộ trình từ 28/09: 12 màn từ bộ flashcard + 4 thử thách, 3 tim, 1–3 sao, mở khoá tuần tự. Chưa có đấu trực tiếp với người khác</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa ai chơi qua giao diện</t>
+  </si>
+  <si>
+    <t>LoTrinh.jsx + TroChoiMan.jsx; migration 108–110</t>
   </si>
   <si>
     <t>XP (điểm kinh nghiệm)</t>
@@ -599,7 +605,7 @@
     <t>Có, kèm kim cương</t>
   </si>
   <si>
-    <t>Có từ 26/09 — cộng ở MÁY CHỦ khi nộp bài lần đầu (10 + điểm), có sổ cái; đổi XP lấy bài trả phí theo giá giáo viên đặt. Chưa bài nào đặt giá XP</t>
+    <t>Cộng ở MÁY CHỦ: nộp bài lần đầu (10 + điểm, từ 26/09) và qua màn Lộ trình lần đầu (5 XP, thử thách 15 XP, từ 29/09); có sổ cái; đổi XP lấy bài trả phí theo giá giáo viên đặt. Chưa bài nào đặt giá XP</t>
   </si>
   <si>
     <t>Đang chạy — chưa ai đổi qua giao diện</t>
@@ -764,10 +770,28 @@
     <t>Có (App Store)</t>
   </si>
   <si>
+    <t>Không có trên App Store; từ 29/09 thêm được vào màn hình chính bằng Safari → Chia sẻ → « Thêm vào MH chính » (PWA), mở toàn màn hình</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa thử trên iPhone thật</t>
+  </si>
+  <si>
+    <t>public/manifest.webmanifest; cố ý không có service worker lưu đệm, nên không dùng offline</t>
+  </si>
+  <si>
     <t>Android</t>
   </si>
   <si>
     <t>Có (Google Play)</t>
+  </si>
+  <si>
+    <t>Không có trên Google Play; từ 29/09 Chrome cho « Cài đặt ứng dụng » (PWA), có biểu tượng riêng, mở toàn màn hình</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa thử trên điện thoại thật</t>
+  </si>
+  <si>
+    <t>public/manifest.webmanifest + icon 192/512</t>
   </si>
   <si>
     <t>Tiến độ đồng bộ nhiều thiết bị</t>
@@ -2052,11 +2076,11 @@
       </c>
       <c r="E9" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="F9" s="6">
         <f>IFERROR(E9-D9,"")</f>
-        <v>-1.4</v>
+        <v>-1.2</v>
       </c>
       <c r="G9" s="7" t="str">
         <f>IF(OR(C9&lt;3,F9=""),"quá ít mục",IF(F9&gt;0.25,"FRACILE",IF(F9&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2081,11 +2105,11 @@
       </c>
       <c r="E10" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>1.3333333333333333</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>-0.6666666666666667</v>
+        <v>-0.33333333333333326</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2139,11 +2163,11 @@
       </c>
       <c r="E12" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="F12" s="6">
         <f>IFERROR(E12-D12,"")</f>
-        <v>-0.8</v>
+        <v>-0.40000000000000013</v>
       </c>
       <c r="G12" s="7" t="str">
         <f>IF(OR(C12&lt;3,F12=""),"quá ít mục",IF(F12&gt;0.25,"FRACILE",IF(F12&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2197,11 +2221,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>1.1818181818181819</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.696969696969697</v>
+        <v>-0.5454545454545456</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -3099,33 +3123,33 @@
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="D19" s="34">
-        <v>2</v>
-      </c>
-      <c r="E19" s="33" t="s">
+      <c r="D19" s="22">
+        <v>2</v>
+      </c>
+      <c r="E19" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="F19" s="34">
-        <v>0</v>
-      </c>
-      <c r="G19" s="35" t="str">
+      <c r="F19" s="22">
+        <v>1</v>
+      </c>
+      <c r="G19" s="23" t="str">
         <f>IF(OR(D19="",F19=""),"chưa rõ",IF(F19&gt;D19,"FRACILE",IF(D19&gt;F19,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H19" s="31" t="s">
+      <c r="H19" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="I19" s="24" t="s">
         <v>148</v>
-      </c>
-      <c r="I19" s="36" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3133,7 +3157,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C20" s="33" t="s">
         <v>124</v>
@@ -3142,7 +3166,7 @@
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3152,10 +3176,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3163,16 +3187,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3185,7 +3209,7 @@
         <v>80</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3193,14 +3217,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C22" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3213,7 +3237,7 @@
         <v>80</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3221,16 +3245,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3240,10 +3264,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3251,14 +3275,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3268,10 +3292,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3279,14 +3303,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C25" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3299,7 +3323,7 @@
         <v>80</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3307,16 +3331,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3329,7 +3353,7 @@
         <v>80</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3337,14 +3361,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C27" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3354,40 +3378,40 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="32" t="s">
-        <v>180</v>
-      </c>
-      <c r="C28" s="33" t="s">
+      <c r="B28" s="20" t="s">
         <v>181</v>
       </c>
-      <c r="D28" s="34">
-        <v>2</v>
-      </c>
-      <c r="E28" s="33" t="s">
+      <c r="C28" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="F28" s="34">
-        <v>0</v>
-      </c>
-      <c r="G28" s="35" t="str">
+      <c r="D28" s="22">
+        <v>2</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="F28" s="22">
+        <v>1</v>
+      </c>
+      <c r="G28" s="23" t="str">
         <f>IF(OR(D28="",F28=""),"chưa rõ",IF(F28&gt;D28,"FRACILE",IF(D28&gt;F28,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H28" s="31" t="s">
-        <v>183</v>
-      </c>
-      <c r="I28" s="36" t="s">
-        <v>151</v>
+      <c r="H28" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="I28" s="24" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3395,29 +3419,29 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F29" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="23" t="str">
         <f>IF(OR(D29="",F29=""),"chưa rõ",IF(F29&gt;D29,"FRACILE",IF(D29&gt;F29,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3425,16 +3449,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F30" s="22">
         <v>1</v>
@@ -3444,10 +3468,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3455,14 +3479,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C31" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3475,7 +3499,7 @@
         <v>80</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3483,16 +3507,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D32" s="22">
         <v>2</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3502,10 +3526,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3513,14 +3537,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C33" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3530,10 +3554,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3541,14 +3565,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C34" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3558,10 +3582,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3569,14 +3593,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C35" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3586,10 +3610,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3597,14 +3621,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C36" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3614,10 +3638,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3625,14 +3649,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C37" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3642,10 +3666,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3653,7 +3677,7 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C38" s="21" t="s">
         <v>124</v>
@@ -3672,10 +3696,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3683,16 +3707,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3702,10 +3726,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3713,7 +3737,7 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C40" s="21" t="s">
         <v>124</v>
@@ -3722,7 +3746,7 @@
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3732,10 +3756,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3743,7 +3767,7 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C41" s="33" t="s">
         <v>124</v>
@@ -3752,7 +3776,7 @@
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3762,10 +3786,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3773,16 +3797,16 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D42" s="22">
         <v>2</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F42" s="22">
         <v>2</v>
@@ -3792,10 +3816,10 @@
         <v>hoà</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3803,14 +3827,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C43" s="21" t="s">
         <v>142</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3823,7 +3847,7 @@
         <v>80</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3831,7 +3855,7 @@
         <v>16</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C44" s="21" t="s">
         <v>124</v>
@@ -3853,67 +3877,67 @@
         <v>80</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="31" t="s">
+      <c r="A45" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B45" s="32" t="s">
-        <v>239</v>
-      </c>
-      <c r="C45" s="33" t="s">
-        <v>240</v>
-      </c>
-      <c r="D45" s="34">
-        <v>2</v>
-      </c>
-      <c r="E45" s="33" t="s">
-        <v>147</v>
-      </c>
-      <c r="F45" s="34">
-        <v>0</v>
-      </c>
-      <c r="G45" s="35" t="str">
+      <c r="B45" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>242</v>
+      </c>
+      <c r="D45" s="22">
+        <v>2</v>
+      </c>
+      <c r="E45" s="21" t="s">
+        <v>243</v>
+      </c>
+      <c r="F45" s="22">
+        <v>1</v>
+      </c>
+      <c r="G45" s="23" t="str">
         <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H45" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="I45" s="36" t="s">
-        <v>151</v>
+      <c r="H45" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="I45" s="24" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="31" t="s">
+      <c r="A46" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B46" s="32" t="s">
-        <v>241</v>
-      </c>
-      <c r="C46" s="33" t="s">
-        <v>242</v>
-      </c>
-      <c r="D46" s="34">
-        <v>2</v>
-      </c>
-      <c r="E46" s="33" t="s">
-        <v>147</v>
-      </c>
-      <c r="F46" s="34">
-        <v>0</v>
-      </c>
-      <c r="G46" s="35" t="str">
+      <c r="B46" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="D46" s="22">
+        <v>2</v>
+      </c>
+      <c r="E46" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="F46" s="22">
+        <v>1</v>
+      </c>
+      <c r="G46" s="23" t="str">
         <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H46" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="I46" s="36" t="s">
-        <v>151</v>
+      <c r="H46" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="I46" s="24" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3921,7 +3945,7 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="C47" s="21" t="s">
         <v>124</v>
@@ -3930,7 +3954,7 @@
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3943,7 +3967,7 @@
         <v>80</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3951,16 +3975,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D48" s="28">
         <v>1</v>
       </c>
       <c r="E48" s="27" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F48" s="28">
         <v>2</v>
@@ -3973,7 +3997,7 @@
         <v>80</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3981,14 +4005,14 @@
         <v>16</v>
       </c>
       <c r="B49" s="26" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="C49" s="27" t="s">
         <v>105</v>
       </c>
       <c r="D49" s="28"/>
       <c r="E49" s="27" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="F49" s="28">
         <v>2</v>
@@ -4001,7 +4025,7 @@
         <v>80</v>
       </c>
       <c r="I49" s="30" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4009,7 +4033,7 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="C50" s="21" t="s">
         <v>124</v>
@@ -4018,7 +4042,7 @@
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="F50" s="22">
         <v>2</v>
@@ -4031,7 +4055,7 @@
         <v>80</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4039,7 +4063,7 @@
         <v>17</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="C51" s="21" t="s">
         <v>124</v>
@@ -4048,7 +4072,7 @@
         <v>2</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="F51" s="22">
         <v>1</v>
@@ -4058,10 +4082,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="I51" s="24" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4078,7 +4102,7 @@
         <v>2</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="F52" s="22">
         <v>1</v>
@@ -4088,10 +4112,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="I52" s="24" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4099,16 +4123,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="F53" s="22">
         <v>1</v>
@@ -4121,7 +4145,7 @@
         <v>80</v>
       </c>
       <c r="I53" s="24" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4129,16 +4153,16 @@
         <v>17</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="D54" s="28">
         <v>1</v>
       </c>
       <c r="E54" s="27" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="F54" s="28">
         <v>2</v>
@@ -4151,7 +4175,7 @@
         <v>80</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4159,14 +4183,14 @@
         <v>17</v>
       </c>
       <c r="B55" s="26" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="C55" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D55" s="28"/>
       <c r="E55" s="27" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="F55" s="28">
         <v>2</v>
@@ -4179,7 +4203,7 @@
         <v>80</v>
       </c>
       <c r="I55" s="30" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -4203,12 +4227,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4224,301 +4248,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4569,288 +4593,288 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="B4" s="40">
         <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B5" s="40">
         <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B6" s="40">
         <v>248</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B9" s="40">
         <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B14" s="40">
         <v>14</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B15" s="40">
         <v>0</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -4858,97 +4882,97 @@
         <v>145</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="D31" s="47" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="46" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="C32" s="47" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="D32" s="47" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -4971,24 +4995,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4996,16 +5020,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5013,16 +5037,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5030,16 +5054,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5047,16 +5071,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Thách đấu bạn bè: máy chủ phát đề, bấm giờ và chấm
- 111: bảng thach_dau không policy, bốn RPC (tạo / lấy đề / nộp / danh sách)
- chỉ thách người đang theo dõi, 10 lượt/24 giờ, điểm đối thủ giấu tới khi nộp
- /etudiant/thach-dau + mục menu, i18n vi/fr/en

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -590,13 +590,13 @@
     <t>Đấu dịch thuật PvP trực tiếp</t>
   </si>
   <si>
-    <t>Có game Lộ trình từ 28/09: 12 màn từ bộ flashcard + 4 thử thách, 3 tim, 1–3 sao, mở khoá tuần tự. Chưa có đấu trực tiếp với người khác</t>
-  </si>
-  <si>
-    <t>Đang chạy — chưa ai chơi qua giao diện</t>
-  </si>
-  <si>
-    <t>LoTrinh.jsx + TroChoiMan.jsx; migration 108–110</t>
+    <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Chưa lên 2: chưa có trận nào giữa hai người thật</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa ai đấu qua giao diện</t>
+  </si>
+  <si>
+    <t>ThachDau.jsx; migration 111. Thử trên DB thật rồi huỷ: chưa theo dõi thì bị chặn, nộp hai lần bị chặn, người ngoài không đọc được đề, điểm đối thủ bị giấu tới khi mình nộp</t>
   </si>
   <si>
     <t>XP (điểm kinh nghiệm)</t>

</xml_diff>

<commit_message>
Bảng so sánh: theo dõi bạn học lên 2, lộ trình đã chơi thật, 13 bài nháp chờ duyệt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -443,10 +443,10 @@
     <t>A1 → C2 (6 cấp) + ôn thi cấp 3</t>
   </si>
   <si>
-    <t>Nhận A1 → C1 (C1 thêm 25/09), nhưng nội dung chủ yếu B1 – B2; C1 chưa có bài</t>
-  </si>
-  <si>
-    <t>Có chủ đích — nhắm hẹp</t>
+    <t>Nhận A1 → C1. Bài đã xuất bản: A1 9 · A2 1 · B1 17 · B2 5 · B2+ 1 · C1 0. Đã soạn nháp 3 bài A2, 2 bài B2+, 2 bài C1 (30/09) — xuất bản xong thì mọi cấp đều có bài</t>
+  </si>
+  <si>
+    <t>Chờ duyệt 7 bài nháp A2/B2+/C1</t>
   </si>
   <si>
     <t>docs/roadmap-delf.md; LEVEL_COLORS là nguồn duy nhất cho Builder + dải lọc</t>
@@ -461,7 +461,7 @@
     <t>33 bài (ĐẾM THẬT trên production)</t>
   </si>
   <si>
-    <t>33 bài luyện công khai, đo 26/09/2026; +6 bài nháp B1–B2 chờ duyệt — lên 39 khi xuất bản</t>
+    <t>33 bài luyện công khai, đo 30/09/2026; +13 bài nháp chờ duyệt (6 bài B1–B2, 7 bài A2/B2+/C1, mỗi bài 10 câu có lời giải) — lên 46 khi xuất bản</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -590,10 +590,10 @@
     <t>Đấu dịch thuật PvP trực tiếp</t>
   </si>
   <si>
-    <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Chưa lên 2: chưa có trận nào giữa hai người thật</t>
-  </si>
-  <si>
-    <t>Đang chạy — chưa ai đấu qua giao diện</t>
+    <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Lộ trình đã có người chơi thật (30/09). Chưa lên 2: chưa có trận thách đấu nào giữa hai người thật</t>
+  </si>
+  <si>
+    <t>Lộ trình đang chạy; thách đấu chưa ai thử</t>
   </si>
   <si>
     <t>ThachDau.jsx; migration 111. Thử trên DB thật rồi huỷ: chưa theo dõi thì bị chặn, nộp hai lần bị chặn, người ngoài không đọc được đề, điểm đối thủ bị giấu tới khi mình nộp</t>
@@ -620,10 +620,10 @@
     <t>Có (bạn bè, bảng xếp hạng)</t>
   </si>
   <si>
-    <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa » + bảng xếp hạng XP trong nhóm mình theo dõi (26/09). Chưa lên 2: chưa ai dùng qua giao diện</t>
-  </si>
-  <si>
-    <t>Đang chạy — chưa ai theo dõi qua giao diện</t>
+    <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa » + bảng xếp hạng XP trong nhóm mình theo dõi (26/09). Đã có người theo dõi qua giao diện (28/09)</t>
+  </si>
+  <si>
+    <t>Đang chạy — 1 lượt theo dõi thật</t>
   </si>
   <si>
     <t>RPC follow_user / get_following_streaks; chỉ lộ tên, @username, ảnh và một cờ</t>
@@ -647,7 +647,7 @@
     <t>Bản đồ uốn lượn 4 chương (Nghe/Đọc/Viết/Nói) · 12 màn = 12 bộ flashcard · trắc nghiệm hai chiều + ghép cặp · 3 tim · 1–3 sao · thử thách cuối chương · mở khoá tuần tự. Không cộng XP (chống cày)</t>
   </si>
   <si>
-    <t>Đã dựng 28/09 — chưa ai chơi qua giao diện</t>
+    <t>Đang chạy — 1 màn đã chơi thật 30/09 (2 sao, máy chủ cộng +5 XP)</t>
   </si>
   <si>
     <t>migration 108/109: lo_trinh_ket_qua + RPC ghi_ket_qua_man (giữ sao cao nhất, có biên nhận)</t>
@@ -2105,15 +2105,15 @@
       </c>
       <c r="E10" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>1.6666666666666667</v>
+        <v>1.8333333333333333</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>-0.33333333333333326</v>
+        <v>-0.16666666666666674</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
-        <v>Vivoire</v>
+        <v>ngang nhau</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2221,11 +2221,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>1.3333333333333333</v>
+        <v>1.3636363636363635</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.5454545454545456</v>
+        <v>-0.5151515151515154</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -3461,11 +3461,11 @@
         <v>193</v>
       </c>
       <c r="F30" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" s="23" t="str">
         <f>IF(OR(D30="",F30=""),"chưa rõ",IF(F30&gt;D30,"FRACILE",IF(D30&gt;F30,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
         <v>194</v>

</xml_diff>

<commit_message>
Lô 3 bài nháp (14 bài, A1→C1, 3 bài đọc hiểu) + bảng so sánh: thi đấu lên 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="434">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -443,10 +443,10 @@
     <t>A1 → C2 (6 cấp) + ôn thi cấp 3</t>
   </si>
   <si>
-    <t>Nhận A1 → C1. Bài đã xuất bản: A1 9 · A2 1 · B1 17 · B2 5 · B2+ 1 · C1 0. Đã soạn nháp 3 bài A2, 2 bài B2+, 2 bài C1 (30/09) — xuất bản xong thì mọi cấp đều có bài</t>
-  </si>
-  <si>
-    <t>Chờ duyệt 7 bài nháp A2/B2+/C1</t>
+    <t>Nhận A1 → C1. Bài đã xuất bản (01/10): A1 9 · A2 1 · B1 18 · B2 5 · B2+ 1 · C1 0. Nháp chờ duyệt có đủ mọi cấp (A1 2 · A2 6 · B1 5 · B2 6 · B2+ 3 · C1 4) — xuất bản xong thì mọi cấp đều có bài</t>
+  </si>
+  <si>
+    <t>Chờ duyệt nháp A2/B2+/C1</t>
   </si>
   <si>
     <t>docs/roadmap-delf.md; LEVEL_COLORS là nguồn duy nhất cho Builder + dải lọc</t>
@@ -458,10 +458,13 @@
     <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
   </si>
   <si>
-    <t>33 bài (ĐẾM THẬT trên production)</t>
-  </si>
-  <si>
-    <t>33 bài luyện công khai, đo 30/09/2026; +13 bài nháp chờ duyệt (6 bài B1–B2, 7 bài A2/B2+/C1, mỗi bài 10 câu có lời giải) — lên 46 khi xuất bản</t>
+    <t>34 bài (ĐẾM THẬT trên production, 01/10)</t>
+  </si>
+  <si>
+    <t>Đang chạy — 26 bài nháp chờ duyệt</t>
+  </si>
+  <si>
+    <t>34 bài luyện công khai, đo 01/10/2026; +26 bài nháp chờ duyệt (lô 1–3, mỗi bài 8–10 câu có lời giải, gồm 4 bài đọc hiểu) — lên 60 khi xuất bản hết</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -590,10 +593,10 @@
     <t>Đấu dịch thuật PvP trực tiếp</t>
   </si>
   <si>
-    <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Lộ trình đã có người chơi thật (30/09). Chưa lên 2: chưa có trận thách đấu nào giữa hai người thật</t>
-  </si>
-  <si>
-    <t>Lộ trình đang chạy; thách đấu chưa ai thử</t>
+    <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Đã chạy thật: Lộ trình có người chơi (30/09) và trận thách đấu đầu tiên giữa hai tài khoản thật đã đấu xong (30/09, hoà 2/8 – 2/8 xét giờ). Vẫn kém Vivoire ở chỗ không đấu theo thời gian thực</t>
+  </si>
+  <si>
+    <t>Đang chạy — đã có trận thật</t>
   </si>
   <si>
     <t>ThachDau.jsx; migration 111. Thử trên DB thật rồi huỷ: chưa theo dõi thì bị chặn, nộp hai lần bị chặn, người ngoài không đọc được đề, điểm đối thủ bị giấu tới khi mình nộp</t>
@@ -623,7 +626,7 @@
     <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa » + bảng xếp hạng XP trong nhóm mình theo dõi (26/09). Đã có người theo dõi qua giao diện (28/09)</t>
   </si>
   <si>
-    <t>Đang chạy — 1 lượt theo dõi thật</t>
+    <t>Đang chạy — 1 lượt theo dõi thật. Từ 01/10: người được theo dõi nhận thông báo ở chuông, và có màn « Mạng lưới học tập » (Người theo dõi / Đang theo dõi, theo dõi lại, bỏ theo dõi)</t>
   </si>
   <si>
     <t>RPC follow_user / get_following_streaks; chỉ lộ tên, @username, ảnh và một cờ</t>
@@ -2105,11 +2108,11 @@
       </c>
       <c r="E10" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>1.8333333333333333</v>
+        <v>2</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>-0.16666666666666674</v>
+        <v>0</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2221,11 +2224,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
-        <v>1.3636363636363635</v>
+        <v>1.393939393939394</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.5151515151515154</v>
+        <v>-0.48484848484848486</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -3088,10 +3091,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3099,14 +3102,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3119,7 +3122,7 @@
         <v>80</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3127,16 +3130,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D19" s="22">
         <v>2</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F19" s="22">
         <v>1</v>
@@ -3149,7 +3152,7 @@
         <v>80</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3157,7 +3160,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C20" s="33" t="s">
         <v>124</v>
@@ -3166,7 +3169,7 @@
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3176,10 +3179,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3187,16 +3190,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3209,7 +3212,7 @@
         <v>80</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3217,14 +3220,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C22" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3237,7 +3240,7 @@
         <v>80</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3245,16 +3248,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3264,10 +3267,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3275,14 +3278,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3292,10 +3295,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3303,14 +3306,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C25" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3323,7 +3326,7 @@
         <v>80</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3331,16 +3334,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3353,7 +3356,7 @@
         <v>80</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3361,14 +3364,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C27" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3378,10 +3381,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3389,29 +3392,29 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D28" s="22">
         <v>2</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F28" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28" s="23" t="str">
         <f>IF(OR(D28="",F28=""),"chưa rõ",IF(F28&gt;D28,"FRACILE",IF(D28&gt;F28,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3419,16 +3422,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F29" s="22">
         <v>2</v>
@@ -3438,10 +3441,10 @@
         <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3449,16 +3452,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F30" s="22">
         <v>2</v>
@@ -3468,10 +3471,10 @@
         <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3479,14 +3482,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C31" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3499,7 +3502,7 @@
         <v>80</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3507,16 +3510,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D32" s="22">
         <v>2</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3526,10 +3529,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3537,14 +3540,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C33" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3554,10 +3557,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3565,14 +3568,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C34" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3582,10 +3585,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3593,14 +3596,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C35" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3610,10 +3613,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3621,14 +3624,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C36" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3638,10 +3641,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3649,14 +3652,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C37" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3666,10 +3669,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3677,7 +3680,7 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C38" s="21" t="s">
         <v>124</v>
@@ -3696,10 +3699,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3707,16 +3710,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3726,10 +3729,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3737,7 +3740,7 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C40" s="21" t="s">
         <v>124</v>
@@ -3746,7 +3749,7 @@
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3756,10 +3759,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3767,7 +3770,7 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C41" s="33" t="s">
         <v>124</v>
@@ -3776,7 +3779,7 @@
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3786,10 +3789,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3797,16 +3800,16 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D42" s="22">
         <v>2</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F42" s="22">
         <v>2</v>
@@ -3816,10 +3819,10 @@
         <v>hoà</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3827,14 +3830,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3847,7 +3850,7 @@
         <v>80</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3855,7 +3858,7 @@
         <v>16</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C44" s="21" t="s">
         <v>124</v>
@@ -3877,7 +3880,7 @@
         <v>80</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3885,16 +3888,16 @@
         <v>16</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C45" s="21" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D45" s="22">
         <v>2</v>
       </c>
       <c r="E45" s="21" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F45" s="22">
         <v>1</v>
@@ -3904,10 +3907,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="I45" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3915,16 +3918,16 @@
         <v>16</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F46" s="22">
         <v>1</v>
@@ -3934,10 +3937,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3945,7 +3948,7 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C47" s="21" t="s">
         <v>124</v>
@@ -3954,7 +3957,7 @@
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3967,7 +3970,7 @@
         <v>80</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,16 +3978,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D48" s="28">
         <v>1</v>
       </c>
       <c r="E48" s="27" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F48" s="28">
         <v>2</v>
@@ -3997,7 +4000,7 @@
         <v>80</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4005,14 +4008,14 @@
         <v>16</v>
       </c>
       <c r="B49" s="26" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C49" s="27" t="s">
         <v>105</v>
       </c>
       <c r="D49" s="28"/>
       <c r="E49" s="27" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F49" s="28">
         <v>2</v>
@@ -4025,7 +4028,7 @@
         <v>80</v>
       </c>
       <c r="I49" s="30" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4036,7 @@
         <v>17</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C50" s="21" t="s">
         <v>124</v>
@@ -4042,7 +4045,7 @@
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F50" s="22">
         <v>2</v>
@@ -4055,7 +4058,7 @@
         <v>80</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4063,7 +4066,7 @@
         <v>17</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C51" s="21" t="s">
         <v>124</v>
@@ -4072,7 +4075,7 @@
         <v>2</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F51" s="22">
         <v>1</v>
@@ -4082,10 +4085,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I51" s="24" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4102,7 +4105,7 @@
         <v>2</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F52" s="22">
         <v>1</v>
@@ -4112,10 +4115,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I52" s="24" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4123,16 +4126,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F53" s="22">
         <v>1</v>
@@ -4145,7 +4148,7 @@
         <v>80</v>
       </c>
       <c r="I53" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4153,16 +4156,16 @@
         <v>17</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D54" s="28">
         <v>1</v>
       </c>
       <c r="E54" s="27" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F54" s="28">
         <v>2</v>
@@ -4175,7 +4178,7 @@
         <v>80</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4183,14 +4186,14 @@
         <v>17</v>
       </c>
       <c r="B55" s="26" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C55" s="27" t="s">
         <v>117</v>
       </c>
       <c r="D55" s="28"/>
       <c r="E55" s="27" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F55" s="28">
         <v>2</v>
@@ -4203,7 +4206,7 @@
         <v>80</v>
       </c>
       <c r="I55" s="30" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -4227,12 +4230,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4248,301 +4251,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4593,386 +4596,386 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B4" s="40">
         <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B5" s="40">
         <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B6" s="40">
         <v>248</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
+        <v>359</v>
+      </c>
+      <c r="B8" s="40">
+        <v>2</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>360</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>358</v>
-      </c>
-      <c r="B8" s="40">
-        <v>2</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>359</v>
-      </c>
-      <c r="D8" s="42" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B9" s="40">
         <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B14" s="40">
         <v>14</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B15" s="40">
         <v>0</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
+        <v>395</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>396</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>397</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>394</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>395</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>396</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
+        <v>398</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>396</v>
+      </c>
+      <c r="C29" s="21" t="s">
         <v>397</v>
       </c>
-      <c r="B29" s="21" t="s">
-        <v>395</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>396</v>
-      </c>
       <c r="D29" s="21" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D31" s="47" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="46" t="s">
+        <v>405</v>
+      </c>
+      <c r="B32" s="47" t="s">
+        <v>406</v>
+      </c>
+      <c r="C32" s="47" t="s">
+        <v>407</v>
+      </c>
+      <c r="D32" s="47" t="s">
         <v>404</v>
-      </c>
-      <c r="B32" s="47" t="s">
-        <v>405</v>
-      </c>
-      <c r="C32" s="47" t="s">
-        <v>406</v>
-      </c>
-      <c r="D32" s="47" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>
@@ -4995,24 +4998,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5020,16 +5023,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5037,16 +5040,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5054,16 +5057,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5071,16 +5074,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: 15 tài khoản, 8 trận thách đấu, hai công cụ giáo viên mới
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="442">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -461,7 +461,7 @@
     <t>34 bài (ĐẾM THẬT trên production, 01/10)</t>
   </si>
   <si>
-    <t>Đang chạy — 26 bài nháp chờ duyệt</t>
+    <t>Đang chạy — 26 bài nháp chờ duyệt ở trang « Duyệt nháp » (02/10), xuất bản một cú bấm</t>
   </si>
   <si>
     <t>34 bài luyện công khai, đo 01/10/2026; +26 bài nháp chờ duyệt (lô 1–3, mỗi bài 8–10 câu có lời giải, gồm 3 bài đọc hiểu có ngữ liệu) — lên 60 khi xuất bản hết</t>
@@ -596,7 +596,7 @@
     <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Đã chạy thật: Lộ trình có người chơi (30/09) và trận thách đấu đầu tiên giữa hai tài khoản thật đã đấu xong (30/09, hoà 2/8 – 2/8 xét giờ). Vẫn kém Vivoire ở chỗ không đấu theo thời gian thực</t>
   </si>
   <si>
-    <t>Đang chạy — đã có trận thật</t>
+    <t>Đang chạy — 8 trận thách đấu thật (02/10)</t>
   </si>
   <si>
     <t>ThachDau.jsx; migration 111. Thử trên DB thật rồi huỷ: chưa theo dõi thì bị chặn, nộp hai lần bị chặn, người ngoài không đọc được đề, điểm đối thủ bị giấu tới khi mình nộp</t>
@@ -755,10 +755,34 @@
     <t>Số tài khoản đang có</t>
   </si>
   <si>
-    <t>14 hồ sơ người dùng (gồm cả tài khoản thử)</t>
-  </si>
-  <si>
-    <t>select count(*) from profiles = 14 (auth.users = 19), đo 28/09/2026</t>
+    <t>15 hồ sơ người dùng (gồm cả tài khoản thử)</t>
+  </si>
+  <si>
+    <t>select count(*) from profiles = 15, đo 02/10/2026</t>
+  </si>
+  <si>
+    <t>Giáo viên điều chỉnh lộ trình học</t>
+  </si>
+  <si>
+    <t>Có từ 02/10 (/professeur/lo-trinh): bật/tắt màn, đổi thứ tự, đặt số câu mỗi màn; bảng tiến độ từng học sinh (sao, màn đã qua, thử thách). Chưa giáo viên nào lưu cấu hình qua giao diện</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa ai lưu cấu hình</t>
+  </si>
+  <si>
+    <t>migration 113: lo_trinh_cau_hinh (học sinh đọc, giáo viên ghi) + RPC lo_trinh_tien_do. Claim giả: học sinh ghi → 42501</t>
+  </si>
+  <si>
+    <t>Duyệt và xuất bản bài soạn sẵn</t>
+  </si>
+  <si>
+    <t>Có từ 02/10 (/professeur/duyet-nhap): đọc trọn bài (ngữ liệu, đáp án, lời giải) rồi xuất bản một cú bấm, máy chủ trả biên nhận</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa xuất bản bài nào qua trang này</t>
+  </si>
+  <si>
+    <t>RPC xuat_ban_nhap (113): một lệnh UPDATE, không xoá-chèn lại câu hỏi</t>
   </si>
   <si>
     <t>Web</t>
@@ -2008,19 +2032,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A7)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
@@ -2037,19 +2061,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A8)</f>
         <v>6</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A8)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -2066,19 +2090,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A9)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>0.8</v>
       </c>
       <c r="F9" s="6">
@@ -2095,19 +2119,19 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A10)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A10)</f>
         <v>10</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A10)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F10" s="6">
@@ -2124,19 +2148,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A11)</f>
-        <v>11</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A11)</f>
+        <v>13</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A11)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F11" s="6">
@@ -2153,19 +2177,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A12)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F12" s="6">
@@ -2182,19 +2206,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$55,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$55=$A13)*('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F13" s="6">
@@ -2212,18 +2236,18 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
         <v>33</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$55)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.878787878787879</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$55)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$55&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$55&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
         <v>1.393939393939394</v>
       </c>
       <c r="F14" s="10">
@@ -2588,7 +2612,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3854,63 +3878,59 @@
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B44" s="20" t="s">
+      <c r="A44" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44" s="26" t="s">
         <v>240</v>
       </c>
-      <c r="C44" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D44" s="22">
-        <v>2</v>
-      </c>
-      <c r="E44" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="F44" s="22">
-        <v>2</v>
-      </c>
-      <c r="G44" s="23" t="str">
+      <c r="C44" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="D44" s="28"/>
+      <c r="E44" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="F44" s="28">
+        <v>2</v>
+      </c>
+      <c r="G44" s="29" t="str">
         <f>IF(OR(D44="",F44=""),"chưa rõ",IF(F44&gt;D44,"FRACILE",IF(D44&gt;F44,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H44" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="I44" s="24" t="s">
-        <v>241</v>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H44" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="I44" s="30" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B45" s="20" t="s">
-        <v>242</v>
-      </c>
-      <c r="C45" s="21" t="s">
-        <v>243</v>
-      </c>
-      <c r="D45" s="22">
-        <v>2</v>
-      </c>
-      <c r="E45" s="21" t="s">
+      <c r="A45" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="26" t="s">
         <v>244</v>
       </c>
-      <c r="F45" s="22">
-        <v>1</v>
-      </c>
-      <c r="G45" s="23" t="str">
+      <c r="C45" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="D45" s="28"/>
+      <c r="E45" s="27" t="s">
+        <v>245</v>
+      </c>
+      <c r="F45" s="28">
+        <v>2</v>
+      </c>
+      <c r="G45" s="29" t="str">
         <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H45" s="19" t="s">
-        <v>245</v>
-      </c>
-      <c r="I45" s="24" t="s">
+        <v>chưa rõ</v>
+      </c>
+      <c r="H45" s="25" t="s">
         <v>246</v>
+      </c>
+      <c r="I45" s="30" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3918,29 +3938,29 @@
         <v>16</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>248</v>
+        <v>124</v>
       </c>
       <c r="D46" s="22">
         <v>2</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>249</v>
+        <v>124</v>
       </c>
       <c r="F46" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" s="23" t="str">
         <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>250</v>
+        <v>80</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3948,16 +3968,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>251</v>
+      </c>
+      <c r="D47" s="22">
+        <v>2</v>
+      </c>
+      <c r="E47" s="21" t="s">
         <v>252</v>
-      </c>
-      <c r="C47" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D47" s="22">
-        <v>2</v>
-      </c>
-      <c r="E47" s="21" t="s">
-        <v>253</v>
       </c>
       <c r="F47" s="22">
         <v>1</v>
@@ -3967,128 +3987,128 @@
         <v>Vivoire</v>
       </c>
       <c r="H47" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="I47" s="24" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>256</v>
+      </c>
+      <c r="D48" s="22">
+        <v>2</v>
+      </c>
+      <c r="E48" s="21" t="s">
+        <v>257</v>
+      </c>
+      <c r="F48" s="22">
+        <v>1</v>
+      </c>
+      <c r="G48" s="23" t="str">
+        <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H48" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="I48" s="24" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>260</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D49" s="22">
+        <v>2</v>
+      </c>
+      <c r="E49" s="21" t="s">
+        <v>261</v>
+      </c>
+      <c r="F49" s="22">
+        <v>1</v>
+      </c>
+      <c r="G49" s="23" t="str">
+        <f>IF(OR(D49="",F49=""),"chưa rõ",IF(F49&gt;D49,"FRACILE",IF(D49&gt;F49,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H49" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="I47" s="24" t="s">
+      <c r="I49" s="24" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="25" t="s">
+    <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B48" s="26" t="s">
-        <v>254</v>
-      </c>
-      <c r="C48" s="27" t="s">
-        <v>255</v>
-      </c>
-      <c r="D48" s="28">
+      <c r="B50" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="C50" s="27" t="s">
+        <v>263</v>
+      </c>
+      <c r="D50" s="28">
         <v>1</v>
       </c>
-      <c r="E48" s="27" t="s">
-        <v>256</v>
-      </c>
-      <c r="F48" s="28">
-        <v>2</v>
-      </c>
-      <c r="G48" s="29" t="str">
-        <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
+      <c r="E50" s="27" t="s">
+        <v>264</v>
+      </c>
+      <c r="F50" s="28">
+        <v>2</v>
+      </c>
+      <c r="G50" s="29" t="str">
+        <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H48" s="25" t="s">
+      <c r="H50" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="I48" s="30" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="25" t="s">
+      <c r="I50" s="30" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B49" s="26" t="s">
-        <v>258</v>
-      </c>
-      <c r="C49" s="27" t="s">
+      <c r="B51" s="26" t="s">
+        <v>266</v>
+      </c>
+      <c r="C51" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="D49" s="28"/>
-      <c r="E49" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="F49" s="28">
-        <v>2</v>
-      </c>
-      <c r="G49" s="29" t="str">
-        <f>IF(OR(D49="",F49=""),"chưa rõ",IF(F49&gt;D49,"FRACILE",IF(D49&gt;F49,"Vivoire","hoà")))</f>
+      <c r="D51" s="28"/>
+      <c r="E51" s="27" t="s">
+        <v>267</v>
+      </c>
+      <c r="F51" s="28">
+        <v>2</v>
+      </c>
+      <c r="G51" s="29" t="str">
+        <f>IF(OR(D51="",F51=""),"chưa rõ",IF(F51&gt;D51,"FRACILE",IF(D51&gt;F51,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H49" s="25" t="s">
+      <c r="H51" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="I49" s="30" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B50" s="20" t="s">
-        <v>261</v>
-      </c>
-      <c r="C50" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D50" s="22">
-        <v>2</v>
-      </c>
-      <c r="E50" s="21" t="s">
-        <v>262</v>
-      </c>
-      <c r="F50" s="22">
-        <v>2</v>
-      </c>
-      <c r="G50" s="23" t="str">
-        <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H50" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="I50" s="24" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B51" s="20" t="s">
-        <v>264</v>
-      </c>
-      <c r="C51" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D51" s="22">
-        <v>2</v>
-      </c>
-      <c r="E51" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="F51" s="22">
-        <v>1</v>
-      </c>
-      <c r="G51" s="23" t="str">
-        <f>IF(OR(D51="",F51=""),"chưa rõ",IF(F51&gt;D51,"FRACILE",IF(D51&gt;F51,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
-      </c>
-      <c r="H51" s="19" t="s">
-        <v>266</v>
-      </c>
-      <c r="I51" s="24" t="s">
-        <v>267</v>
+      <c r="I51" s="30" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4096,7 +4116,7 @@
         <v>17</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>37</v>
+        <v>269</v>
       </c>
       <c r="C52" s="21" t="s">
         <v>124</v>
@@ -4105,20 +4125,20 @@
         <v>2</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F52" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G52" s="23" t="str">
         <f>IF(OR(D52="",F52=""),"chưa rõ",IF(F52&gt;D52,"FRACILE",IF(D52&gt;F52,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>266</v>
+        <v>80</v>
       </c>
       <c r="I52" s="24" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4126,16 +4146,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>271</v>
+        <v>124</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F53" s="22">
         <v>1</v>
@@ -4145,68 +4165,128 @@
         <v>Vivoire</v>
       </c>
       <c r="H53" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="I53" s="24" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C54" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D54" s="22">
+        <v>2</v>
+      </c>
+      <c r="E54" s="21" t="s">
+        <v>276</v>
+      </c>
+      <c r="F54" s="22">
+        <v>1</v>
+      </c>
+      <c r="G54" s="23" t="str">
+        <f>IF(OR(D54="",F54=""),"chưa rõ",IF(F54&gt;D54,"FRACILE",IF(D54&gt;F54,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H54" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="I54" s="24" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="C55" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="D55" s="22">
+        <v>2</v>
+      </c>
+      <c r="E55" s="21" t="s">
+        <v>280</v>
+      </c>
+      <c r="F55" s="22">
+        <v>1</v>
+      </c>
+      <c r="G55" s="23" t="str">
+        <f>IF(OR(D55="",F55=""),"chưa rõ",IF(F55&gt;D55,"FRACILE",IF(D55&gt;F55,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H55" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="I53" s="24" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="25" t="s">
+      <c r="I55" s="24" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="56" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B54" s="26" t="s">
-        <v>274</v>
-      </c>
-      <c r="C54" s="27" t="s">
-        <v>275</v>
-      </c>
-      <c r="D54" s="28">
+      <c r="B56" s="26" t="s">
+        <v>282</v>
+      </c>
+      <c r="C56" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="D56" s="28">
         <v>1</v>
       </c>
-      <c r="E54" s="27" t="s">
-        <v>276</v>
-      </c>
-      <c r="F54" s="28">
-        <v>2</v>
-      </c>
-      <c r="G54" s="29" t="str">
-        <f>IF(OR(D54="",F54=""),"chưa rõ",IF(F54&gt;D54,"FRACILE",IF(D54&gt;F54,"Vivoire","hoà")))</f>
+      <c r="E56" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="F56" s="28">
+        <v>2</v>
+      </c>
+      <c r="G56" s="29" t="str">
+        <f>IF(OR(D56="",F56=""),"chưa rõ",IF(F56&gt;D56,"FRACILE",IF(D56&gt;F56,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H54" s="25" t="s">
+      <c r="H56" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="I54" s="30" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="25" t="s">
+      <c r="I56" s="30" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="57" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B55" s="26" t="s">
-        <v>278</v>
-      </c>
-      <c r="C55" s="27" t="s">
+      <c r="B57" s="26" t="s">
+        <v>286</v>
+      </c>
+      <c r="C57" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="D55" s="28"/>
-      <c r="E55" s="27" t="s">
-        <v>279</v>
-      </c>
-      <c r="F55" s="28">
-        <v>2</v>
-      </c>
-      <c r="G55" s="29" t="str">
-        <f>IF(OR(D55="",F55=""),"chưa rõ",IF(F55&gt;D55,"FRACILE",IF(D55&gt;F55,"Vivoire","hoà")))</f>
+      <c r="D57" s="28"/>
+      <c r="E57" s="27" t="s">
+        <v>287</v>
+      </c>
+      <c r="F57" s="28">
+        <v>2</v>
+      </c>
+      <c r="G57" s="29" t="str">
+        <f>IF(OR(D57="",F57=""),"chưa rõ",IF(F57&gt;D57,"FRACILE",IF(D57&gt;F57,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H55" s="25" t="s">
+      <c r="H57" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="I55" s="30" t="s">
-        <v>280</v>
+      <c r="I57" s="30" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -4230,12 +4310,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4251,70 +4331,70 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4322,78 +4402,78 @@
         <v>212</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>80</v>
@@ -4407,145 +4487,145 @@
         <v>218</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4596,288 +4676,288 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="B4" s="40">
         <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B5" s="40">
         <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B6" s="40">
         <v>248</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="B9" s="40">
         <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B14" s="40">
         <v>14</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B15" s="40">
         <v>0</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -4885,97 +4965,97 @@
         <v>146</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="D31" s="47" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="46" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="C32" s="47" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="D32" s="47" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>
@@ -4998,24 +5078,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5023,16 +5103,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5040,16 +5120,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5057,16 +5137,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5074,16 +5154,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: thêm dòng Thống kê lớp + Google Sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="446">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -773,6 +773,18 @@
     <t>migration 113: lo_trinh_cau_hinh (học sinh đọc, giáo viên ghi) + RPC lo_trinh_tien_do. Claim giả: học sinh ghi → 42501</t>
   </si>
   <si>
+    <t>Thống kê lớp + xuất Google Sheets</t>
+  </si>
+  <si>
+    <t>Trang Thống kê: tổng quan 7 ngày (học sinh hoạt động, thời gian học, điểm TB, tỷ lệ hoàn thành — đều so tuần trước), biểu đồ hoạt động, radar kỹ năng, bảng từng học sinh. Nút « Đồng bộ Google Sheets » để máy chủ tự ghi 3 trang tính (30 ngày) vào bảng tính cố định, có biên nhận số dòng</t>
+  </si>
+  <si>
+    <t>Đã dựng 02/10 — chờ chủ dự án nối Google (5 phút, một lần)</t>
+  </si>
+  <si>
+    <t>Edge Function dong-bo-sheets (chỉ giáo viên, số liệu đọc ở máy chủ) + docs/google-sheets/Code.gs. Thử: chưa cấu hình → CHUA_CAU_HINH_SHEETS; CORS đạt. Trang /bao-mat đã ghi Google là bên nhận dữ liệu</t>
+  </si>
+  <si>
     <t>Duyệt và xuất bản bài soạn sẵn</t>
   </si>
   <si>
@@ -1061,7 +1073,7 @@
     <t>GIỮ — DỰNG LẠI</t>
   </si>
   <si>
-    <t>Dựng lại 24/09: KPI, phân bố điểm, TB theo kỹ năng, top học sinh, bảng xu hướng. Màn cũ đọc kho bài giao gần như rỗng nên hiện 0/0; nay đọc lượt làm bài thật.</t>
+    <t>Dựng lại 24/09: KPI, phân bố điểm, TB theo kỹ năng, top học sinh, bảng xu hướng. 02/10: thêm tổng quan 7 ngày (4 thẻ có xu hướng so tuần trước), biểu đồ hoạt động, radar kỹ năng, xuất CSV, và ĐỒNG BỘ GOOGLE SHEETS tự động (máy chủ ghi 3 trang tính qua Apps Script — cần chủ dự án nối một lần theo docs/google-sheets/HUONG-DAN.md).</t>
   </si>
   <si>
     <t>Chấm bài viết của học sinh</t>
@@ -2032,19 +2044,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A7)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
@@ -2061,19 +2073,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A8)</f>
         <v>6</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A8)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -2090,19 +2102,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A9)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>0.8</v>
       </c>
       <c r="F9" s="6">
@@ -2119,19 +2131,19 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A10)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A10)</f>
         <v>10</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A10)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F10" s="6">
@@ -2148,19 +2160,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A11)</f>
-        <v>13</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A11)</f>
+        <v>14</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A11)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F11" s="6">
@@ -2177,19 +2189,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A12)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F12" s="6">
@@ -2206,19 +2218,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$57,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$57=$A13)*('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F13" s="6">
@@ -2236,18 +2248,18 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
         <v>33</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$57)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.878787878787879</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$57)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$57&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$57&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
         <v>1.393939393939394</v>
       </c>
       <c r="F14" s="10">
@@ -2612,7 +2624,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3934,33 +3946,31 @@
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46" s="20" t="s">
+      <c r="A46" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" s="26" t="s">
         <v>248</v>
       </c>
-      <c r="C46" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D46" s="22">
-        <v>2</v>
-      </c>
-      <c r="E46" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="F46" s="22">
-        <v>2</v>
-      </c>
-      <c r="G46" s="23" t="str">
+      <c r="C46" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="D46" s="28"/>
+      <c r="E46" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="F46" s="28">
+        <v>2</v>
+      </c>
+      <c r="G46" s="29" t="str">
         <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H46" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="I46" s="24" t="s">
-        <v>249</v>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H46" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="I46" s="30" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3968,29 +3978,29 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>251</v>
+        <v>124</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>252</v>
+        <v>124</v>
       </c>
       <c r="F47" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G47" s="23" t="str">
         <f>IF(OR(D47="",F47=""),"chưa rõ",IF(F47&gt;D47,"FRACILE",IF(D47&gt;F47,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H47" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="I47" s="24" t="s">
         <v>253</v>
-      </c>
-      <c r="I47" s="24" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3998,16 +4008,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="20" t="s">
+        <v>254</v>
+      </c>
+      <c r="C48" s="21" t="s">
         <v>255</v>
       </c>
-      <c r="C48" s="21" t="s">
+      <c r="D48" s="22">
+        <v>2</v>
+      </c>
+      <c r="E48" s="21" t="s">
         <v>256</v>
-      </c>
-      <c r="D48" s="22">
-        <v>2</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>257</v>
       </c>
       <c r="F48" s="22">
         <v>1</v>
@@ -4017,10 +4027,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="I48" s="24" t="s">
         <v>258</v>
-      </c>
-      <c r="I48" s="24" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4028,10 +4038,10 @@
         <v>16</v>
       </c>
       <c r="B49" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="C49" s="21" t="s">
         <v>260</v>
-      </c>
-      <c r="C49" s="21" t="s">
-        <v>124</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
@@ -4047,40 +4057,40 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
+        <v>262</v>
+      </c>
+      <c r="I49" s="24" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="C50" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D50" s="22">
+        <v>2</v>
+      </c>
+      <c r="E50" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="F50" s="22">
+        <v>1</v>
+      </c>
+      <c r="G50" s="23" t="str">
+        <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
+        <v>Vivoire</v>
+      </c>
+      <c r="H50" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="I49" s="24" t="s">
+      <c r="I50" s="24" t="s">
         <v>153</v>
-      </c>
-    </row>
-    <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B50" s="26" t="s">
-        <v>262</v>
-      </c>
-      <c r="C50" s="27" t="s">
-        <v>263</v>
-      </c>
-      <c r="D50" s="28">
-        <v>1</v>
-      </c>
-      <c r="E50" s="27" t="s">
-        <v>264</v>
-      </c>
-      <c r="F50" s="28">
-        <v>2</v>
-      </c>
-      <c r="G50" s="29" t="str">
-        <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H50" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="I50" s="30" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,54 +4101,54 @@
         <v>266</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="D51" s="28"/>
+        <v>267</v>
+      </c>
+      <c r="D51" s="28">
+        <v>1</v>
+      </c>
       <c r="E51" s="27" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
       </c>
       <c r="G51" s="29" t="str">
         <f>IF(OR(D51="",F51=""),"chưa rõ",IF(F51&gt;D51,"FRACILE",IF(D51&gt;F51,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>FRACILE</v>
       </c>
       <c r="H51" s="25" t="s">
         <v>80</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B52" s="20" t="s">
-        <v>269</v>
-      </c>
-      <c r="C52" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D52" s="22">
-        <v>2</v>
-      </c>
-      <c r="E52" s="21" t="s">
+      <c r="A52" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52" s="26" t="s">
         <v>270</v>
       </c>
-      <c r="F52" s="22">
-        <v>2</v>
-      </c>
-      <c r="G52" s="23" t="str">
+      <c r="C52" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="D52" s="28"/>
+      <c r="E52" s="27" t="s">
+        <v>271</v>
+      </c>
+      <c r="F52" s="28">
+        <v>2</v>
+      </c>
+      <c r="G52" s="29" t="str">
         <f>IF(OR(D52="",F52=""),"chưa rõ",IF(F52&gt;D52,"FRACILE",IF(D52&gt;F52,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H52" s="19" t="s">
+        <v>chưa rõ</v>
+      </c>
+      <c r="H52" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="I52" s="24" t="s">
-        <v>271</v>
+      <c r="I52" s="30" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4146,7 +4156,7 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C53" s="21" t="s">
         <v>124</v>
@@ -4155,17 +4165,17 @@
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F53" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G53" s="23" t="str">
         <f>IF(OR(D53="",F53=""),"chưa rõ",IF(F53&gt;D53,"FRACILE",IF(D53&gt;F53,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H53" s="19" t="s">
-        <v>274</v>
+        <v>80</v>
       </c>
       <c r="I53" s="24" t="s">
         <v>275</v>
@@ -4176,7 +4186,7 @@
         <v>17</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>37</v>
+        <v>276</v>
       </c>
       <c r="C54" s="21" t="s">
         <v>124</v>
@@ -4185,7 +4195,7 @@
         <v>2</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F54" s="22">
         <v>1</v>
@@ -4195,10 +4205,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4206,10 +4216,10 @@
         <v>17</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>278</v>
+        <v>37</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>279</v>
+        <v>124</v>
       </c>
       <c r="D55" s="22">
         <v>2</v>
@@ -4225,39 +4235,39 @@
         <v>Vivoire</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>80</v>
+        <v>278</v>
       </c>
       <c r="I55" s="24" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="56" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="25" t="s">
+      <c r="A56" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B56" s="26" t="s">
+      <c r="B56" s="20" t="s">
         <v>282</v>
       </c>
-      <c r="C56" s="27" t="s">
+      <c r="C56" s="21" t="s">
         <v>283</v>
       </c>
-      <c r="D56" s="28">
+      <c r="D56" s="22">
+        <v>2</v>
+      </c>
+      <c r="E56" s="21" t="s">
+        <v>284</v>
+      </c>
+      <c r="F56" s="22">
         <v>1</v>
       </c>
-      <c r="E56" s="27" t="s">
-        <v>284</v>
-      </c>
-      <c r="F56" s="28">
-        <v>2</v>
-      </c>
-      <c r="G56" s="29" t="str">
+      <c r="G56" s="23" t="str">
         <f>IF(OR(D56="",F56=""),"chưa rõ",IF(F56&gt;D56,"FRACILE",IF(D56&gt;F56,"Vivoire","hoà")))</f>
-        <v>FRACILE</v>
-      </c>
-      <c r="H56" s="25" t="s">
+        <v>Vivoire</v>
+      </c>
+      <c r="H56" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="I56" s="30" t="s">
+      <c r="I56" s="24" t="s">
         <v>285</v>
       </c>
     </row>
@@ -4269,24 +4279,54 @@
         <v>286</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="D57" s="28"/>
+        <v>287</v>
+      </c>
+      <c r="D57" s="28">
+        <v>1</v>
+      </c>
       <c r="E57" s="27" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F57" s="28">
         <v>2</v>
       </c>
       <c r="G57" s="29" t="str">
         <f>IF(OR(D57="",F57=""),"chưa rõ",IF(F57&gt;D57,"FRACILE",IF(D57&gt;F57,"Vivoire","hoà")))</f>
-        <v>chưa rõ</v>
+        <v>FRACILE</v>
       </c>
       <c r="H57" s="25" t="s">
         <v>80</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>288</v>
+        <v>289</v>
+      </c>
+    </row>
+    <row r="58" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B58" s="26" t="s">
+        <v>290</v>
+      </c>
+      <c r="C58" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="D58" s="28"/>
+      <c r="E58" s="27" t="s">
+        <v>291</v>
+      </c>
+      <c r="F58" s="28">
+        <v>2</v>
+      </c>
+      <c r="G58" s="29" t="str">
+        <f>IF(OR(D58="",F58=""),"chưa rõ",IF(F58&gt;D58,"FRACILE",IF(D58&gt;F58,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H58" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I58" s="30" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -4310,12 +4350,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4331,70 +4371,70 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4402,78 +4442,78 @@
         <v>212</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>80</v>
@@ -4487,145 +4527,145 @@
         <v>218</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="B17" s="27" t="s">
+        <v>338</v>
+      </c>
+      <c r="C17" s="25" t="s">
         <v>334</v>
       </c>
-      <c r="C17" s="25" t="s">
-        <v>330</v>
-      </c>
       <c r="D17" s="27" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4676,288 +4716,288 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B4" s="40">
         <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B5" s="40">
         <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B6" s="40">
         <v>248</v>
       </c>
       <c r="C6" s="41" t="s">
+        <v>367</v>
+      </c>
+      <c r="D6" s="42" t="s">
         <v>363</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="B9" s="40">
         <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="B14" s="40">
         <v>14</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B15" s="40">
         <v>0</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -4965,97 +5005,97 @@
         <v>146</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>408</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>409</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>406</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>404</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>405</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D31" s="47" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="46" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="C32" s="47" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="D32" s="47" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>
@@ -5078,24 +5118,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5103,16 +5143,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5120,16 +5160,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5137,16 +5177,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5154,16 +5194,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: đề A2/C1 nháp, 12 bài nghe mới, 44 bài nháp
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="448">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -383,10 +383,13 @@
     <t>DELF/DALF A1–C2</t>
   </si>
   <si>
-    <t>2 đề, đủ 4 phần CO/CE/PE/PO, chỉ B1–B2</t>
-  </si>
-  <si>
-    <t>Bảng exams + exam_sections; migration 026/044/059</t>
+    <t>2 đề B1 đã phát hành. 02/10: thêm 2 đề NHÁP đủ 4 phần — DELF A2 (108') và DALF C1 (270'), có phần Nghe; chờ xuất bản bài + phát hành đề thì lên 2</t>
+  </si>
+  <si>
+    <t>Đang chạy — 2 đề nháp A2/C1 chờ phát hành</t>
+  </si>
+  <si>
+    <t>Bảng exams + exam_sections; migration 026/044/059. Lô scripts/nhap/lo4 + lo6; thang viết C1 phỏng theo thêm vào delfGrille + peBareme</t>
   </si>
   <si>
     <t>Nghe hiểu giới hạn 2 lượt phát</t>
@@ -458,13 +461,13 @@
     <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
   </si>
   <si>
-    <t>34 bài (ĐẾM THẬT trên production, 01/10)</t>
-  </si>
-  <si>
-    <t>Đang chạy — 26 bài nháp chờ duyệt ở trang « Duyệt nháp » (02/10), xuất bản một cú bấm</t>
-  </si>
-  <si>
-    <t>34 bài luyện công khai, đo 01/10/2026; +26 bài nháp chờ duyệt (lô 1–3, mỗi bài 8–10 câu có lời giải, gồm 3 bài đọc hiểu có ngữ liệu) — lên 60 khi xuất bản hết</t>
+    <t>34 bài (ĐẾM THẬT trên production, 02/10)</t>
+  </si>
+  <si>
+    <t>Đang chạy — 44 bài nháp chờ duyệt ở trang « Duyệt nháp », xuất bản một cú bấm</t>
+  </si>
+  <si>
+    <t>34 bài luyện công khai, đo 01/10/2026; +44 bài nháp chờ duyệt (lô 1–6: luyện tập, đọc hiểu, 12 bài nghe, bài viết/nói cho đề A2/C1) — lên 78 khi xuất bản hết</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -509,10 +512,13 @@
     <t>Có (nêu rõ « audio bản xứ »)</t>
   </si>
   <si>
-    <t>Có file nghe cho phần CO, không nêu nguồn giọng đọc</t>
-  </si>
-  <si>
-    <t>Bucket đề bài công khai</t>
+    <t>Có file nghe cho phần CO, không nêu nguồn giọng đọc. 02/10: +9 bài nghe A1–B1 GIỌNG TỔNG HỢP (OpenAI TTS, ghi rõ trong bài) + 3 bài C1 người thật đọc (Wikipédia parlée, CC0/PD/GFDL, ghi nguồn). Chưa có audio người bản xứ thu riêng cho FRACILE</t>
+  </si>
+  <si>
+    <t>Đang chạy — 12 bài nghe mới đang nháp</t>
+  </si>
+  <si>
+    <t>Edge Function tao-audio + kho nghe (114); docs/nghe/kich-ban-nghe.md liệt kê nguồn đã kiểm và đã loại (Audio-Lingua cấm đăng lại, RFI/TV5 có bản quyền)</t>
   </si>
   <si>
     <t>Nhập đề hàng loạt</t>
@@ -2927,10 +2933,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2938,14 +2944,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2958,7 +2964,7 @@
         <v>80</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2966,14 +2972,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2986,7 +2992,7 @@
         <v>80</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2994,14 +3000,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -3014,7 +3020,7 @@
         <v>80</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3022,14 +3028,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -3042,7 +3048,7 @@
         <v>80</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3050,14 +3056,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -3070,7 +3076,7 @@
         <v>80</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3078,16 +3084,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -3097,10 +3103,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3108,16 +3114,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -3127,10 +3133,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3138,14 +3144,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3158,7 +3164,7 @@
         <v>80</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3166,16 +3172,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D19" s="22">
         <v>2</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F19" s="22">
         <v>1</v>
@@ -3188,7 +3194,7 @@
         <v>80</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3196,16 +3202,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3215,10 +3221,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3226,16 +3232,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3245,10 +3251,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>80</v>
+        <v>158</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3256,14 +3262,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3276,7 +3282,7 @@
         <v>80</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3284,16 +3290,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3303,10 +3309,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3314,14 +3320,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3331,10 +3337,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3342,14 +3348,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3362,7 +3368,7 @@
         <v>80</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3370,16 +3376,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3392,7 +3398,7 @@
         <v>80</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3400,14 +3406,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3417,10 +3423,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3428,16 +3434,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D28" s="22">
         <v>2</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F28" s="22">
         <v>2</v>
@@ -3447,10 +3453,10 @@
         <v>hoà</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3458,16 +3464,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F29" s="22">
         <v>2</v>
@@ -3477,10 +3483,10 @@
         <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3488,16 +3494,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F30" s="22">
         <v>2</v>
@@ -3507,10 +3513,10 @@
         <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3518,14 +3524,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3538,7 +3544,7 @@
         <v>80</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3546,16 +3552,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D32" s="22">
         <v>2</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3565,10 +3571,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3576,14 +3582,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3593,10 +3599,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3604,14 +3610,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3621,10 +3627,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3632,14 +3638,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3649,10 +3655,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3660,14 +3666,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3677,10 +3683,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3688,14 +3694,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3705,10 +3711,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3716,16 +3722,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F38" s="22">
         <v>2</v>
@@ -3735,10 +3741,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3746,16 +3752,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3765,10 +3771,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3776,16 +3782,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3795,10 +3801,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3806,16 +3812,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3825,10 +3831,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3836,16 +3842,16 @@
         <v>15</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D42" s="22">
         <v>2</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F42" s="22">
         <v>2</v>
@@ -3855,10 +3861,10 @@
         <v>hoà</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3866,14 +3872,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3886,7 +3892,7 @@
         <v>80</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3894,14 +3900,14 @@
         <v>15</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D44" s="28"/>
       <c r="E44" s="27" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F44" s="28">
         <v>2</v>
@@ -3911,10 +3917,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H44" s="25" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3922,14 +3928,14 @@
         <v>15</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -3939,10 +3945,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3950,14 +3956,14 @@
         <v>15</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D46" s="28"/>
       <c r="E46" s="27" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F46" s="28">
         <v>2</v>
@@ -3967,10 +3973,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H46" s="25" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3978,16 +3984,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F47" s="22">
         <v>2</v>
@@ -4000,7 +4006,7 @@
         <v>80</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4008,16 +4014,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C48" s="21" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D48" s="22">
         <v>2</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F48" s="22">
         <v>1</v>
@@ -4027,10 +4033,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="I48" s="24" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4038,16 +4044,16 @@
         <v>16</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -4057,10 +4063,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4068,16 +4074,16 @@
         <v>16</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -4090,7 +4096,7 @@
         <v>80</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4098,16 +4104,16 @@
         <v>16</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D51" s="28">
         <v>1</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -4120,7 +4126,7 @@
         <v>80</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4128,14 +4134,14 @@
         <v>16</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C52" s="27" t="s">
         <v>105</v>
       </c>
       <c r="D52" s="28"/>
       <c r="E52" s="27" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F52" s="28">
         <v>2</v>
@@ -4148,7 +4154,7 @@
         <v>80</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4156,16 +4162,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F53" s="22">
         <v>2</v>
@@ -4178,7 +4184,7 @@
         <v>80</v>
       </c>
       <c r="I53" s="24" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4186,16 +4192,16 @@
         <v>17</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D54" s="22">
         <v>2</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F54" s="22">
         <v>1</v>
@@ -4205,10 +4211,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4219,13 +4225,13 @@
         <v>37</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D55" s="22">
         <v>2</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F55" s="22">
         <v>1</v>
@@ -4235,10 +4241,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="I55" s="24" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="56" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4246,16 +4252,16 @@
         <v>17</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C56" s="21" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D56" s="22">
         <v>2</v>
       </c>
       <c r="E56" s="21" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F56" s="22">
         <v>1</v>
@@ -4268,7 +4274,7 @@
         <v>80</v>
       </c>
       <c r="I56" s="24" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="57" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4276,16 +4282,16 @@
         <v>17</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D57" s="28">
         <v>1</v>
       </c>
       <c r="E57" s="27" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="F57" s="28">
         <v>2</v>
@@ -4298,7 +4304,7 @@
         <v>80</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="58" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4306,14 +4312,14 @@
         <v>17</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D58" s="28"/>
       <c r="E58" s="27" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F58" s="28">
         <v>2</v>
@@ -4326,7 +4332,7 @@
         <v>80</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -4350,12 +4356,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4371,301 +4377,301 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>307</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>304</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>302</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="B21" s="27" t="s">
         <v>351</v>
       </c>
-      <c r="B21" s="27" t="s">
-        <v>349</v>
-      </c>
       <c r="C21" s="25" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>80</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -4716,386 +4722,386 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B4" s="40">
         <v>40</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B5" s="40">
         <v>413</v>
       </c>
       <c r="C5" s="41" t="s">
+        <v>367</v>
+      </c>
+      <c r="D5" s="42" t="s">
         <v>365</v>
-      </c>
-      <c r="D5" s="42" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B6" s="40">
         <v>248</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B8" s="40">
         <v>2</v>
       </c>
       <c r="C8" s="41" t="s">
+        <v>374</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>372</v>
-      </c>
-      <c r="D8" s="42" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B9" s="40">
         <v>23</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B14" s="40">
         <v>14</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B15" s="40">
         <v>0</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B16" s="40">
         <v>0</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B21" s="43">
         <f>B6/B5</f>
         <v>0.5618279569892473</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B22" s="45">
         <f>B5-B6</f>
         <v>163</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B28" s="21" t="s">
+        <v>410</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>411</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>408</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>409</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
+        <v>412</v>
+      </c>
+      <c r="B29" s="21" t="s">
         <v>410</v>
       </c>
-      <c r="B29" s="21" t="s">
+      <c r="C29" s="21" t="s">
+        <v>411</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>408</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>409</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
+        <v>413</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>414</v>
+      </c>
+      <c r="C30" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="B30" s="21" t="s">
-        <v>412</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>409</v>
-      </c>
       <c r="D30" s="21" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D31" s="47" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="46" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B32" s="47" t="s">
+        <v>420</v>
+      </c>
+      <c r="C32" s="47" t="s">
+        <v>421</v>
+      </c>
+      <c r="D32" s="47" t="s">
         <v>418</v>
-      </c>
-      <c r="C32" s="47" t="s">
-        <v>419</v>
-      </c>
-      <c r="D32" s="47" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -5118,24 +5124,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5143,16 +5149,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5160,16 +5166,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5177,16 +5183,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5194,16 +5200,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
6 bài nghe dài B1/B2 (12–14 câu/bài) + bảng so sánh: 46 bài, 25 bài nghe/196 câu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -446,7 +446,7 @@
     <t>A1 → C2 (6 cấp) + ôn thi cấp 3</t>
   </si>
   <si>
-    <t>Nhận A1 → C1. Bài đã xuất bản (01/10): A1 9 · A2 1 · B1 18 · B2 5 · B2+ 1 · C1 0. Nháp chờ duyệt có đủ mọi cấp (A1 2 · A2 6 · B1 5 · B2 6 · B2+ 3 · C1 4) — xuất bản xong thì mọi cấp đều có bài</t>
+    <t>Nhận A1 → C1. Bài đã xuất bản (02/10): A1 9 · A2 6 · B1 22 · B2 5 · B2+ 4 · C1 0. Nháp chờ duyệt có đủ mọi cấp (A1 2 · A2 6 · B1 5 · B2 6 · B2+ 3 · C1 4) — xuất bản xong thì mọi cấp đều có bài</t>
   </si>
   <si>
     <t>Chờ duyệt nháp A2/B2+/C1</t>
@@ -461,13 +461,13 @@
     <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
   </si>
   <si>
-    <t>34 bài (ĐẾM THẬT trên production, 02/10)</t>
-  </si>
-  <si>
-    <t>Đang chạy — 44 bài nháp chờ duyệt ở trang « Duyệt nháp », xuất bản một cú bấm</t>
-  </si>
-  <si>
-    <t>34 bài luyện công khai, đo 01/10/2026; +44 bài nháp chờ duyệt (lô 1–6: luyện tập, đọc hiểu, 12 bài nghe, bài viết/nói cho đề A2/C1) — lên 78 khi xuất bản hết</t>
+    <t>46 bài (ĐẾM THẬT trên production, 02/10) — trong đó 25 bài nghe (196 câu)</t>
+  </si>
+  <si>
+    <t>Đang chạy — 42 bài nháp chờ duyệt ở trang « Duyệt nháp »</t>
+  </si>
+  <si>
+    <t>34 bài luyện công khai, đo 01/10/2026; +42 bài nháp chờ duyệt (lô 1–8) — lên 88 khi xuất bản hết, đủ ngưỡng 60 để lên 2</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -512,10 +512,10 @@
     <t>Có (nêu rõ « audio bản xứ »)</t>
   </si>
   <si>
-    <t>Có file nghe cho phần CO, không nêu nguồn giọng đọc. 02/10: +9 bài nghe A1–B1 GIỌNG TỔNG HỢP (OpenAI TTS, ghi rõ trong bài) + 3 bài C1 người thật đọc (Wikipédia parlée, CC0/PD/GFDL, ghi nguồn). Chưa có audio người bản xứ thu riêng cho FRACILE</t>
-  </si>
-  <si>
-    <t>Đang chạy — 12 bài nghe mới đang nháp</t>
+    <t>25 bài nghe, 196 câu (02/10): A1 4 bài/23 câu · A2 5/25 · B1 9/71 · B2 4/48 · C1 3/29. Phần lớn là GIỌNG TỔNG HỢP (OpenAI TTS, ghi rõ trong bài); 3 bài C1 người thật đọc (Wikipédia parlée, CC0/PD/GFDL, ghi nguồn); 3 bài cũ không rõ nguồn giọng. Bài B1/B2 mới dài 1'40–2'30, 12–14 câu/bài như đề thật. Chưa có audio người bản xứ thu riêng</t>
+  </si>
+  <si>
+    <t>Đang chạy — 4 bài nghe B1 đã xuất bản; các bài khác đang nháp</t>
   </si>
   <si>
     <t>Edge Function tao-audio + kho nghe (114); docs/nghe/kich-ban-nghe.md liệt kê nguồn đã kiểm và đã loại (Audio-Lingua cấm đăng lại, RFI/TV5 có bản quyền)</t>

</xml_diff>

<commit_message>
Bảng so sánh: 48 bài, 17 tài khoản, 9 trận thách đấu, dọn dấu gạch dài, ảnh mặc định
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -446,7 +446,7 @@
     <t>A1 → C2 (6 cấp) + ôn thi cấp 3</t>
   </si>
   <si>
-    <t>Nhận A1 → C1. Bài đã xuất bản (02/10): A1 9 · A2 6 · B1 22 · B2 5 · B2+ 4 · C1 0. Nháp chờ duyệt có đủ mọi cấp (A1 2 · A2 6 · B1 5 · B2 6 · B2+ 3 · C1 4) — xuất bản xong thì mọi cấp đều có bài</t>
+    <t>Nhận A1 → C1. Bài đã xuất bản (06/10): A1 9 · A2 6 · B1 24 · B2 5 · B2+ 4 · C1 0. Nháp chờ duyệt có đủ mọi cấp (A1 2 · A2 6 · B1 5 · B2 6 · B2+ 3 · C1 4) — xuất bản xong thì mọi cấp đều có bài</t>
   </si>
   <si>
     <t>Chờ duyệt nháp A2/B2+/C1</t>
@@ -461,7 +461,7 @@
     <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
   </si>
   <si>
-    <t>46 bài (ĐẾM THẬT trên production, 02/10) — trong đó 25 bài nghe (196 câu)</t>
+    <t>48 bài (ĐẾM THẬT trên production, 06/10), trong đó 25 bài nghe (196 câu). 06/10: rà toàn bộ nội dung, bỏ dấu gạch dài ở 14 bài, 123 câu, 3 đề, 50 thẻ; thẻ bài không có ảnh dùng ảnh mặc định theo kỹ năng</t>
   </si>
   <si>
     <t>Đang chạy — 42 bài nháp chờ duyệt ở trang « Duyệt nháp »</t>
@@ -602,7 +602,7 @@
     <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Đã chạy thật: Lộ trình có người chơi (30/09) và trận thách đấu đầu tiên giữa hai tài khoản thật đã đấu xong (30/09, hoà 2/8 – 2/8 xét giờ). Vẫn kém Vivoire ở chỗ không đấu theo thời gian thực</t>
   </si>
   <si>
-    <t>Đang chạy — 8 trận thách đấu thật (02/10)</t>
+    <t>Đang chạy — 9 trận thách đấu thật (06/10)</t>
   </si>
   <si>
     <t>ThachDau.jsx; migration 111. Thử trên DB thật rồi huỷ: chưa theo dõi thì bị chặn, nộp hai lần bị chặn, người ngoài không đọc được đề, điểm đối thủ bị giấu tới khi mình nộp</t>
@@ -761,10 +761,10 @@
     <t>Số tài khoản đang có</t>
   </si>
   <si>
-    <t>15 hồ sơ người dùng (gồm cả tài khoản thử)</t>
-  </si>
-  <si>
-    <t>select count(*) from profiles = 15, đo 02/10/2026</t>
+    <t>17 hồ sơ người dùng (gồm cả tài khoản thử)</t>
+  </si>
+  <si>
+    <t>select count(*) from profiles = 17, đo 06/10/2026</t>
   </si>
   <si>
     <t>Giáo viên điều chỉnh lộ trình học</t>

</xml_diff>

<commit_message>
Bỏ nút Làm mới ở trang học sinh; cập nhật bảng so sánh 08/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="485">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -129,7 +129,7 @@
     <t>Chưa kiểm chứng được — KHÔNG tính vào trung bình</t>
   </si>
   <si>
-    <t>ĐÃ ĐỔI GÌ SO VỚI BẢN 09/09 — bản này đo 24/09/2026</t>
+    <t>ĐÃ ĐỔI GÌ SO VỚI BẢN 09/09 — bản này đo 08/10/2026</t>
   </si>
   <si>
     <t>Chấm PE bằng AI</t>
@@ -238,6 +238,12 @@
   </si>
   <si>
     <t>AI chấm PE BẬT (OpenAI gpt-6-luna, chủ dự án chọn vì rẻ nhất; thử qua giao diện: có nhận xét). Bài viết (PE) — AI chấm 1 → 2; Chấm bài cho học sinh 0 → 1. Thêm tour « Nền tối và cài đặt » + nút « Xem lại hướng dẫn »; Chính sách bảo mật ghi OpenAI.</t>
+  </si>
+  <si>
+    <t>07–08/10</t>
+  </si>
+  <si>
+    <t>Đề A1 + A2 Đề 2 theo format 2; nghe kiểu phòng thi (nghỉ 30 s giữa hai lượt); 2 lượt thi/ngày kèm cảnh báo; 3 dạng câu DELF mới; gói VIP + quản lý VIP; thu gọn tài khoản giáo viên (gỡ lời giải, sổ tay, lộ trình, tư vấn, tạo lớp); Flashcard, Neo, Cấp quyền, Thông báo làm lại giao diện; trạng thái online cho người theo dõi nhau. Học sinh: gộp Cần làm + Đã nộp thành « Bài tập được giao », Kết quả thi vào từ màn Thi thử, gỡ nút Làm mới.</t>
   </si>
   <si>
     <t>Số liệu trôi</t>
@@ -359,10 +365,10 @@
     <t>Không thấy nêu trên trang chủ</t>
   </si>
   <si>
-    <t>188/353 câu có lời giải (đo 24/09); có màn xếp ưu tiên theo SỐ HỌC SINH từng sai</t>
-  </si>
-  <si>
-    <t>migration 069/070; /professeur/loi-giai</t>
+    <t>704/881 câu có lời giải (đo 08/10). Màn « Câu cần lời giải » của giáo viên đã gỡ 07/10: AI chấm và giải thích thay</t>
+  </si>
+  <si>
+    <t>select count(*) from questions where explanation is not null = 704</t>
   </si>
   <si>
     <t>Neo đáp án vào ngữ liệu (chỉ ra CHỖ chứa câu trả lời)</t>
@@ -383,13 +389,13 @@
     <t>DELF/DALF A1–C2</t>
   </si>
   <si>
-    <t>2 đề B1 đã phát hành. 02/10: thêm 2 đề NHÁP đủ 4 phần — DELF A2 (108') và DALF C1 (270'), có phần Nghe; chờ xuất bản bài + phát hành đề thì lên 2</t>
-  </si>
-  <si>
-    <t>Đang chạy — 2 đề nháp A2/C1 chờ phát hành</t>
-  </si>
-  <si>
-    <t>Bảng exams + exam_sections; migration 026/044/059. Lô scripts/nhap/lo4 + lo6; thang viết C1 phỏng theo thêm vào delfGrille + peBareme</t>
+    <t>7 đề (3 đã phát hành). Đủ A1 · A2 · B1 · B2 · C1 theo format 2 hiện hành; học sinh chọn đề theo tab trình độ A1–B2. File docs/format-de-thi-DELF-A1-B2.xlsx ghi cấu trúc từng phần. Còn chờ phát hành các đề nháp</t>
+  </si>
+  <si>
+    <t>Đang chạy — đề A1, A2 Đề 2, B2, C1 là nháp</t>
+  </si>
+  <si>
+    <t>lo10 (A1), lo11 (A2 Đề 2), lo9 (B2), lo6 (C1). Chưa lên 2 vì phần lớn đề còn nháp</t>
   </si>
   <si>
     <t>Nghe hiểu giới hạn 2 lượt phát</t>
@@ -398,10 +404,10 @@
     <t>Không thấy nêu</t>
   </si>
   <si>
-    <t>Có, và ĐẾM Ở MÁY CHỦ — không phải ở trình duyệt nên không lách được</t>
-  </si>
-  <si>
-    <t>RPC _exam_play; migration 024 đã thu quyền gọi trực tiếp của học sinh</t>
+    <t>Đếm ở MÁY CHỦ. Từ 07/10 có « nghe kiểu phòng thi »: file chứa sẵn 30 s đọc câu hỏi → lượt 1 → nghỉ 30 s → lượt 2 → 30 s hoàn thành, phát MỘT lần. Sửa lỗi bài 2 trở đi báo hết lượt và lỗi buổi thi mới nhận lượt nghe cũ</t>
+  </si>
+  <si>
+    <t>migration 024, 119, 121; ExamMode AudioGioiHan (key theo bài). Đo bằng silencedetect: 3 khoảng 30 s đúng chỗ</t>
   </si>
   <si>
     <t>Đồng hồ chạy tiếp khi đóng tab</t>
@@ -461,13 +467,13 @@
     <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
   </si>
   <si>
-    <t>48 bài (ĐẾM THẬT trên production, 06/10), trong đó 25 bài nghe (196 câu). 06/10: rà toàn bộ nội dung, bỏ dấu gạch dài ở 14 bài, 123 câu, 3 đề, 50 thẻ; thẻ bài không có ảnh dùng ảnh mặc định theo kỹ năng</t>
-  </si>
-  <si>
-    <t>Đang chạy — 42 bài nháp chờ duyệt ở trang « Duyệt nháp »</t>
-  </si>
-  <si>
-    <t>34 bài luyện công khai, đo 01/10/2026; +42 bài nháp chờ duyệt (lô 1–8) — lên 88 khi xuất bản hết, đủ ngưỡng 60 để lên 2</t>
+    <t>110 bài trong kho (ĐẾM THẬT 08/10), trong đó 62 bài/đề con còn NHÁP chờ duyệt</t>
+  </si>
+  <si>
+    <t>Đang chạy — 62 nháp chờ duyệt</t>
+  </si>
+  <si>
+    <t>select count(*) from exercises = 110; title like '[NHÁP]%' = 62. Lên 2 khi xuất bản đủ ≥ 60 bài công khai</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -476,10 +482,10 @@
     <t>Không công bố</t>
   </si>
   <si>
-    <t>413 câu, 7 dạng (qcm, fill, conj, vf, tableau, order, tự luận) — 60 câu thuộc bài nháp</t>
-  </si>
-  <si>
-    <t>select count(*) from questions = 413, đo 26/09/2026</t>
+    <t>881 câu, 9 dạng: qcm (có thể kèm HÌNH), fill, conj, vf, tableau, ordre, tự luận, GHÉP CẶP, PHIẾU</t>
+  </si>
+  <si>
+    <t>select count(*) from questions = 881, đo 08/10/2026</t>
   </si>
   <si>
     <t>Từ điển Pháp–Việt</t>
@@ -629,13 +635,13 @@
     <t>Có (bạn bè, bảng xếp hạng)</t>
   </si>
   <si>
-    <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa » + bảng xếp hạng XP trong nhóm mình theo dõi (26/09). Đã có người theo dõi qua giao diện (28/09)</t>
-  </si>
-  <si>
-    <t>Đang chạy — 1 lượt theo dõi thật. Từ 01/10: người được theo dõi nhận thông báo ở chuông, và có màn « Mạng lưới học tập » (Người theo dõi / Đang theo dõi, theo dõi lại, bỏ theo dõi)</t>
-  </si>
-  <si>
-    <t>RPC follow_user / get_following_streaks; chỉ lộ tên, @username, ảnh và một cờ</t>
+    <t>Theo dõi một chiều bằng @username; thấy « hôm nay đã học chưa », bảng xếp hạng XP, và từ 08/10 TRẠNG THÁI ONLINE (chấm xanh, « online 12 phút trước ») của người mình theo dõi; có tùy chọn ẩn trạng thái</t>
+  </si>
+  <si>
+    <t>Đang chạy — 4 lượt theo dõi</t>
+  </si>
+  <si>
+    <t>migration 123 (cột profiles.lan_cuoi_online thay blob mcf-presence); thử bằng claim giả: ẩn → người theo dõi không thấy</t>
   </si>
   <si>
     <t>Giờ học đo được</t>
@@ -665,21 +671,21 @@
     <t>Kiểm soát ai được học bài nào</t>
   </si>
   <si>
-    <t>Hai tầng: trọn gói (profiles.has_premium_access) + từng bài (exercise_access)</t>
+    <t>Ba tầng: gói VIP 99.000 đ/30 ngày (tự gia hạn qua SePay), trọn gói, từng bài. Màn cấp quyền làm lại 08/10: xem theo bài hoặc theo học sinh, cấp cho cả nhóm; giáo viên tự gia hạn/thu hồi VIP</t>
+  </si>
+  <si>
+    <t>QuyenBaiTap.jsx, QuanLyVip.jsx; migration 118, 122. vip_giao_dich = 2 dòng</t>
+  </si>
+  <si>
+    <t>Học sinh KHÔNG tự mở khoá được cho mình</t>
+  </si>
+  <si>
+    <t>exercise_access chặn mọi lệnh ghi từ trình duyệt; phải qua Edge Function</t>
   </si>
   <si>
     <t>Đang chạy — GIỮ</t>
   </si>
   <si>
-    <t>Đây chính là « kiểm soát số lượng học sinh ». AccessPanel.jsx</t>
-  </si>
-  <si>
-    <t>Học sinh KHÔNG tự mở khoá được cho mình</t>
-  </si>
-  <si>
-    <t>exercise_access chặn mọi lệnh ghi từ trình duyệt; phải qua Edge Function</t>
-  </si>
-  <si>
     <t>migration 001; grant-access giữ service_role</t>
   </si>
   <si>
@@ -749,13 +755,10 @@
     <t>Có form thu thông tin</t>
   </si>
   <si>
-    <t>Có lại từ 25/09: nút « Gửi câu hỏi » mở ngăn kéo form (tên, SĐT, năm sinh, email, vai, mục tiêu, nội dung), gửi thật vào bảng leads</t>
-  </si>
-  <si>
-    <t>Đang chạy — chưa ai gửi qua giao diện</t>
-  </si>
-  <si>
-    <t>migration 077–080; /professeur/lien-he. Thử bằng vai anon trong khối rollback: lưu đúng. RỦI RO: thu dữ liệu cá nhân (có thể của trẻ vị thành niên) khi chưa có Chính sách bảo mật</t>
+    <t>ĐÃ GỠ khỏi tài khoản giáo viên 07/10 theo chủ dự án; bảng leads còn nguyên</t>
+  </si>
+  <si>
+    <t>Lấy lại XemLienHe.jsx từ git trước commit 35759f3</t>
   </si>
   <si>
     <t>Số tài khoản đang có</t>
@@ -770,13 +773,10 @@
     <t>Giáo viên điều chỉnh lộ trình học</t>
   </si>
   <si>
-    <t>Có từ 02/10 (/professeur/lo-trinh): bật/tắt màn, đổi thứ tự, đặt số câu mỗi màn; bảng tiến độ từng học sinh (sao, màn đã qua, thử thách). Chưa giáo viên nào lưu cấu hình qua giao diện</t>
-  </si>
-  <si>
-    <t>Đang chạy — chưa ai lưu cấu hình</t>
-  </si>
-  <si>
-    <t>migration 113: lo_trinh_cau_hinh (học sinh đọc, giáo viên ghi) + RPC lo_trinh_tien_do. Claim giả: học sinh ghi → 42501</t>
+    <t>ĐÃ GỠ màn giáo viên 07/10; lộ trình chạy theo cấu hình mặc định (bảng lo_trinh_cau_hinh còn nguyên)</t>
+  </si>
+  <si>
+    <t>Lấy lại LoTrinhGiaoVien.jsx từ git</t>
   </si>
   <si>
     <t>Thống kê lớp + xuất Google Sheets</t>
@@ -926,6 +926,54 @@
     <t>migration 057/058 — giọng trẻ vị thành niên ở URL đoán được là chuyện pháp lý</t>
   </si>
   <si>
+    <t>Giới hạn lượt thi + cảnh báo</t>
+  </si>
+  <si>
+    <t>2 lượt thi/ngày (giờ VN, đếm ở máy chủ). Hộp cảnh báo « mô phỏng phòng thi DELF thật » trước khi vào; thoát giữa chừng (nút Thoát, Back, đóng tab) có cảnh báo và mất lượt</t>
+  </si>
+  <si>
+    <t>migration 120 (luot_thi); thử claim giả: lượt 3 → HET_LUOT</t>
+  </si>
+  <si>
+    <t>Dạng câu riêng của DELF (ghép cặp, phiếu, chọn hình)</t>
+  </si>
+  <si>
+    <t>Có từ 07/10: Appariement (chấm từng mục), Formulaire (điền phiếu A1), QCM có hình; soạn được ở Builder và nhập JSON</t>
+  </si>
+  <si>
+    <t>Đang chạy — 5 câu dạng mới</t>
+  </si>
+  <si>
+    <t>dangMoi.jsx, SoanDangMoi.jsx; hàm grade chấm 3/4 đúng khi thử thật</t>
+  </si>
+  <si>
+    <t>Gửi thông báo tới học sinh</t>
+  </si>
+  <si>
+    <t>Trang riêng (08/10): mẫu nhanh, chọn tất cả hoặc từng em (có chấm online), xem trước như chuông học sinh, lịch sử kèm số đã đọc</t>
+  </si>
+  <si>
+    <t>Đang chạy — 7 thông báo đã gửi</t>
+  </si>
+  <si>
+    <t>GuiThongBao.jsx; RPC send_announcement_to_students trả số người nhận</t>
+  </si>
+  <si>
+    <t>Gói VIP</t>
+  </si>
+  <si>
+    <t>Không thấy nêu giá gói</t>
+  </si>
+  <si>
+    <t>99.000 đ / 30 ngày, mở mọi bài trả phí và đề thi; thanh toán SePay tự kích hoạt, gia hạn nối tiếp không mất ngày</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa thử chuyển khoản thật</t>
+  </si>
+  <si>
+    <t>migration 118; sepay-webhook mã VIP1TH</t>
+  </si>
+  <si>
     <t>TÀI KHOẢN GIÁO VIÊN — giữ để KIỂM SOÁT, không để CHẤM BÀI</t>
   </si>
   <si>
@@ -953,18 +1001,24 @@
     <t>AccessPanel (trong dashboard)</t>
   </si>
   <si>
+    <t>GIỮ — DỰNG LẠI</t>
+  </si>
+  <si>
+    <t>Đang chạy — giao diện mới 08/10</t>
+  </si>
+  <si>
+    <t>QuyenBaiTap.jsx: theo bài / theo học sinh, cấp theo nhóm. Quyền học sinh tự mua không gỡ được.</t>
+  </si>
+  <si>
+    <t>Bật/tắt trọn gói cho một học sinh</t>
+  </si>
+  <si>
+    <t>AccessPanel</t>
+  </si>
+  <si>
     <t>GIỮ</t>
   </si>
   <si>
-    <t>Đây chính là « kiểm soát số lượng học sinh ». Ghi qua Edge Function grant-access.</t>
-  </si>
-  <si>
-    <t>Bật/tắt trọn gói cho một học sinh</t>
-  </si>
-  <si>
-    <t>AccessPanel</t>
-  </si>
-  <si>
     <t>profiles.has_premium_access — mở cả những bài chưa tồn tại lúc bật.</t>
   </si>
   <si>
@@ -1001,7 +1055,13 @@
     <t>/professeur/loi-giai</t>
   </si>
   <si>
-    <t>Thay thế trực tiếp cho chấm tay: dạy một lần cho tất cả, thay vì nhận xét từng bài.</t>
+    <t>ĐÃ GỠ</t>
+  </si>
+  <si>
+    <t>Không còn trong menu</t>
+  </si>
+  <si>
+    <t>Gỡ 07/10: AI chấm và giải thích thay. Dữ liệu lời giải giữ nguyên.</t>
   </si>
   <si>
     <t>Đặt neo đáp án vào ngữ liệu</t>
@@ -1010,10 +1070,10 @@
     <t>/professeur/neo</t>
   </si>
   <si>
-    <t>Đang chạy — 22 neo</t>
-  </si>
-  <si>
-    <t>Chủ dự án đã đặt neo qua giao diện 23/09. Lưu bài trong Builder từng xoá sạch neo — sửa 23/09 (093/094).</t>
+    <t>Đang chạy — giao diện mới 07/10</t>
+  </si>
+  <si>
+    <t>Lưới bài + màn 3 cột (danh sách câu · đoạn văn · neo và xem trước).</t>
   </si>
   <si>
     <t>Sổ tay / mẹo</t>
@@ -1022,13 +1082,13 @@
     <t>/professeur/carnet</t>
   </si>
   <si>
+    <t>Gỡ 07/10 theo chủ dự án; mẹo cũ vẫn hiện cho học sinh.</t>
+  </si>
+  <si>
     <t>/professeur/bo-the</t>
   </si>
   <si>
-    <t>Đang chạy — chạy thật 21/09</t>
-  </si>
-  <si>
-    <t>Dựng 09/09. Học sinh không còn tự tạo thẻ — chỉ giáo viên soạn, chặn ở database bằng RLS chứ không chỉ ẩn nút.</t>
+    <t>Lưới bộ lọc theo kỹ năng; thêm từng thẻ hoặc dán nhiều dòng; sửa thẻ tại chỗ.</t>
   </si>
   <si>
     <t>Xem câu hỏi / đăng ký tư vấn</t>
@@ -1037,10 +1097,7 @@
     <t>/professeur/lien-he</t>
   </si>
   <si>
-    <t>Đang chạy — có nguồn vào từ 25/09</t>
-  </si>
-  <si>
-    <t>Nguồn: nút « Gửi câu hỏi » trên trang giới thiệu. Năm sinh nằm ở dòng đầu phần nội dung.</t>
+    <t>Gỡ 07/10; bảng leads còn nguyên.</t>
   </si>
   <si>
     <t>Nghe bản ghi âm bài nói của học sinh</t>
@@ -1049,9 +1106,6 @@
     <t>/professeur/oral</t>
   </si>
   <si>
-    <t>ĐÃ GỠ</t>
-  </si>
-  <si>
     <t>Không còn trong mã</t>
   </si>
   <si>
@@ -1076,9 +1130,6 @@
     <t>/professeur (Thống kê)</t>
   </si>
   <si>
-    <t>GIỮ — DỰNG LẠI</t>
-  </si>
-  <si>
     <t>Dựng lại 24/09: KPI, phân bố điểm, TB theo kỹ năng, top học sinh, bảng xu hướng. 02/10: thêm tổng quan 7 ngày (4 thẻ có xu hướng so tuần trước), biểu đồ hoạt động, radar kỹ năng, xuất CSV, và ĐỒNG BỘ GOOGLE SHEETS tự động (máy chủ ghi 3 trang tính qua Apps Script — cần chủ dự án nối một lần theo docs/google-sheets/HUONG-DAN.md).</t>
   </si>
   <si>
@@ -1107,6 +1158,45 @@
   </si>
   <si>
     <t>« Chờ chấm » → « Chưa chấm » (Non noté / Not marked): mô tả trạng thái thay vì hứa một hành động sẽ không xảy ra.</t>
+  </si>
+  <si>
+    <t>Quản lý gói VIP</t>
+  </si>
+  <si>
+    <t>/professeur/eleves</t>
+  </si>
+  <si>
+    <t>Đang chạy — mới 07/10</t>
+  </si>
+  <si>
+    <t>Xem ai đang VIP, +30 ngày, thu hồi; ghi vào vip_giao_dich (122).</t>
+  </si>
+  <si>
+    <t>Gửi thông báo</t>
+  </si>
+  <si>
+    <t>/professeur/thong-bao</t>
+  </si>
+  <si>
+    <t>Đang chạy — trang mới 08/10</t>
+  </si>
+  <si>
+    <t>Thay hộp nổi cũ; có lịch sử và số đã đọc.</t>
+  </si>
+  <si>
+    <t>Tạo lớp / xếp lớp</t>
+  </si>
+  <si>
+    <t>Gỡ 07/10 theo chủ dự án; dữ liệu mcf-classes còn nguyên.</t>
+  </si>
+  <si>
+    <t>Thư viện luyện tập (mục riêng)</t>
+  </si>
+  <si>
+    <t>/professeur/exercices</t>
+  </si>
+  <si>
+    <t>Gộp thành tab thứ hai trong « Bài tập » 07/10.</t>
   </si>
   <si>
     <t>MỘT CÂU PHẢI NÓI THẲNG</t>
@@ -1135,63 +1225,66 @@
     <t>Bài tập</t>
   </si>
   <si>
-    <t>select count(*) from exercises — 33 luyện tập + 1 bài giao + 6 NHÁP chờ duyệt</t>
+    <t>select count(*) from exercises — 62 bài/đề con NHÁP chờ duyệt</t>
+  </si>
+  <si>
+    <t>08/10/2026</t>
+  </si>
+  <si>
+    <t>Câu hỏi</t>
+  </si>
+  <si>
+    <t>select count(*) from questions — 9 dạng câu</t>
+  </si>
+  <si>
+    <t>Câu có lời giải thích</t>
+  </si>
+  <si>
+    <t>questions where explanation is not null</t>
+  </si>
+  <si>
+    <t>Câu có neo ngữ liệu</t>
+  </si>
+  <si>
+    <t>questions where evidence is not null</t>
+  </si>
+  <si>
+    <t>Đề thi thử</t>
+  </si>
+  <si>
+    <t>select count(*) from exams — 3 đã phát hành</t>
+  </si>
+  <si>
+    <t>Lượt làm bài đã chấm</t>
+  </si>
+  <si>
+    <t>attempts where finished_at is not null</t>
+  </si>
+  <si>
+    <t>Bộ Flashcard (cả 12 công khai)</t>
+  </si>
+  <si>
+    <t>select count(*) from the_bo where cong_khai</t>
   </si>
   <si>
     <t>26/09/2026</t>
   </si>
   <si>
-    <t>Câu hỏi</t>
-  </si>
-  <si>
-    <t>select count(*) from questions — gồm 60 câu của 6 bài nháp</t>
-  </si>
-  <si>
-    <t>Câu có lời giải thích</t>
-  </si>
-  <si>
-    <t>questions where explanation is not null — gồm 60 câu nháp</t>
-  </si>
-  <si>
-    <t>Câu có neo ngữ liệu</t>
-  </si>
-  <si>
-    <t>questions where evidence is not null — trên 2 bài</t>
+    <t>Thẻ trong các bộ</t>
+  </si>
+  <si>
+    <t>select count(*) from the_bo_the</t>
+  </si>
+  <si>
+    <t>Thẻ trong bảng cards</t>
+  </si>
+  <si>
+    <t>select count(*) from cards — 36 thẻ đi theo hai tài khoản thử đã xoá</t>
   </si>
   <si>
     <t>24/09/2026</t>
   </si>
   <si>
-    <t>Đề thi thử</t>
-  </si>
-  <si>
-    <t>select count(*) from exams</t>
-  </si>
-  <si>
-    <t>Lượt làm bài đã chấm</t>
-  </si>
-  <si>
-    <t>attempts where finished_at is not null</t>
-  </si>
-  <si>
-    <t>Bộ Flashcard (cả 12 công khai)</t>
-  </si>
-  <si>
-    <t>select count(*) from the_bo where cong_khai</t>
-  </si>
-  <si>
-    <t>Thẻ trong các bộ</t>
-  </si>
-  <si>
-    <t>select count(*) from the_bo_the</t>
-  </si>
-  <si>
-    <t>Thẻ trong bảng cards</t>
-  </si>
-  <si>
-    <t>select count(*) from cards — 36 thẻ đi theo hai tài khoản thử đã xoá</t>
-  </si>
-  <si>
     <t>Lượt trả lời đã ghi</t>
   </si>
   <si>
@@ -1204,40 +1297,58 @@
     <t>select count(*) from profiles</t>
   </si>
   <si>
+    <t>Lượt đổi XP lấy bài</t>
+  </si>
+  <si>
+    <t>exercise_access where status='XP'</t>
+  </si>
+  <si>
+    <t>Lượt theo dõi bạn học</t>
+  </si>
+  <si>
+    <t>select count(*) from follows</t>
+  </si>
+  <si>
+    <t>Bài tự luận CHƯA có điểm nào</t>
+  </si>
+  <si>
+    <t>câu open, không điểm GV lẫn tự chấm. 7/8 thuộc 2 tài khoản thử của chủ dự án; 1 bài của học sinh thật, dài 12 ký tự</t>
+  </si>
+  <si>
+    <t>21/09/2026</t>
+  </si>
+  <si>
+    <t>Lượt ôn Flashcard đã ghi</t>
+  </si>
+  <si>
+    <t>reviews có reps &gt; 0 trên thẻ bo_giao_vien — 2 lượt cũ thuộc tài khoản thử đã xoá</t>
+  </si>
+  <si>
+    <t>Gợi ý chấm AI đã sinh</t>
+  </si>
+  <si>
+    <t>select count(*) from pe_ai_goi_y — gpt-6-luna, bật 27/09</t>
+  </si>
+  <si>
     <t>27/09/2026</t>
   </si>
   <si>
-    <t>Lượt đổi XP lấy bài</t>
-  </si>
-  <si>
-    <t>exercise_access where status='XP' — chưa bài nào đặt giá XP</t>
-  </si>
-  <si>
-    <t>Lượt theo dõi bạn học</t>
-  </si>
-  <si>
-    <t>select count(*) from follows</t>
-  </si>
-  <si>
-    <t>Bài tự luận CHƯA có điểm nào</t>
-  </si>
-  <si>
-    <t>câu open, không điểm GV lẫn tự chấm. 7/8 thuộc 2 tài khoản thử của chủ dự án; 1 bài của học sinh thật, dài 12 ký tự</t>
-  </si>
-  <si>
-    <t>21/09/2026</t>
-  </si>
-  <si>
-    <t>Lượt ôn Flashcard đã ghi</t>
-  </si>
-  <si>
-    <t>reviews có reps &gt; 0 trên thẻ bo_giao_vien — 2 lượt cũ thuộc tài khoản thử đã xoá</t>
-  </si>
-  <si>
-    <t>Gợi ý chấm AI đã sinh</t>
-  </si>
-  <si>
-    <t>select count(*) from pe_ai_goi_y — gpt-6-luna, bật 27/09</t>
+    <t>Giao dịch VIP</t>
+  </si>
+  <si>
+    <t>select count(*) from vip_giao_dich</t>
+  </si>
+  <si>
+    <t>Lượt thi thử đã mở (từ 07/10)</t>
+  </si>
+  <si>
+    <t>select count(*) from luot_thi</t>
+  </si>
+  <si>
+    <t>Thông báo đã gửi (dòng người nhận)</t>
+  </si>
+  <si>
+    <t>notifications where type='announcement'</t>
   </si>
   <si>
     <t>Tỷ lệ câu có lời giải</t>
@@ -1993,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2050,19 +2161,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A7)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
@@ -2079,19 +2190,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A8)</f>
-        <v>6</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A8)</f>
+        <v>7</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A8)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F8" s="6">
@@ -2108,19 +2219,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A9)</f>
-        <v>7</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A9)</f>
+        <v>8</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A9)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>0.8</v>
       </c>
       <c r="F9" s="6">
@@ -2137,19 +2248,19 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A10)</f>
-        <v>10</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A10)</f>
+        <v>11</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A10)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F10" s="6">
@@ -2166,24 +2277,24 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A11)</f>
-        <v>14</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A11)</f>
+        <v>15</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A11)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
-        <v>1.4</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <v>1</v>
       </c>
       <c r="F11" s="6">
         <f>IFERROR(E11-D11,"")</f>
-        <v>-0.6000000000000001</v>
+        <v>-1</v>
       </c>
       <c r="G11" s="7" t="str">
         <f>IF(OR(C11&lt;3,F11=""),"quá ít mục",IF(F11&gt;0.25,"FRACILE",IF(F11&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2195,19 +2306,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A12)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F12" s="6">
@@ -2224,19 +2335,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$58,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$58=$A13)*('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F13" s="6">
@@ -2254,23 +2365,23 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
         <v>33</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$58)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
         <v>1.878787878787879</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$58)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$58&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$58&lt;&gt;"")),"")</f>
-        <v>1.393939393939394</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <v>1.3333333333333333</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.48484848484848486</v>
+        <v>-0.5454545454545456</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2600,8 +2711,21 @@
       <c r="F46" s="18"/>
       <c r="G46" s="18"/>
     </row>
+    <row r="47" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2622,6 +2746,7 @@
     <mergeCell ref="B44:G44"/>
     <mergeCell ref="B45:G45"/>
     <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B47:G47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2630,7 +2755,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2649,28 +2774,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2678,16 +2803,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2697,10 +2822,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2708,14 +2833,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2725,10 +2850,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2736,16 +2861,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F4" s="22">
         <v>2</v>
@@ -2755,10 +2880,10 @@
         <v>hoà</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2766,16 +2891,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2785,10 +2910,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2796,16 +2921,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D6" s="22">
         <v>2</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F6" s="22">
         <v>1</v>
@@ -2815,10 +2940,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2826,16 +2951,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2845,10 +2970,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2856,14 +2981,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -2873,10 +2998,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2884,7 +3009,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -2893,7 +3018,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -2903,10 +3028,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2914,16 +3039,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F10" s="22">
         <v>1</v>
@@ -2933,10 +3058,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2944,14 +3069,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -2961,10 +3086,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2972,14 +3097,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -2989,10 +3114,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3000,14 +3125,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -3017,10 +3142,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3028,14 +3153,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -3045,10 +3170,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3056,14 +3181,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -3073,10 +3198,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3084,16 +3209,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -3103,10 +3228,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3114,16 +3239,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F17" s="22">
         <v>1</v>
@@ -3133,10 +3258,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3144,14 +3269,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3161,10 +3286,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3172,16 +3297,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D19" s="22">
         <v>2</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F19" s="22">
         <v>1</v>
@@ -3191,10 +3316,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3202,16 +3327,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3221,10 +3346,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3232,16 +3357,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3251,10 +3376,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3262,14 +3387,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3279,10 +3404,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3290,16 +3415,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3309,10 +3434,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3320,14 +3445,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3337,10 +3462,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3348,14 +3473,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3365,10 +3490,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3376,16 +3501,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3395,10 +3520,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3406,14 +3531,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3423,10 +3548,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3434,16 +3559,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D28" s="22">
         <v>2</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F28" s="22">
         <v>2</v>
@@ -3453,10 +3578,10 @@
         <v>hoà</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3464,16 +3589,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F29" s="22">
         <v>2</v>
@@ -3483,10 +3608,10 @@
         <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3494,16 +3619,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F30" s="22">
         <v>2</v>
@@ -3513,10 +3638,10 @@
         <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3524,14 +3649,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3541,10 +3666,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3552,16 +3677,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D32" s="22">
         <v>2</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3571,10 +3696,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3582,14 +3707,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3599,10 +3724,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>209</v>
+        <v>82</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3610,14 +3735,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3627,10 +3752,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3638,14 +3763,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3655,10 +3780,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3666,14 +3791,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3683,10 +3808,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3694,14 +3819,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3711,10 +3836,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3722,16 +3847,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F38" s="22">
         <v>2</v>
@@ -3741,10 +3866,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3752,16 +3877,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3771,10 +3896,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3782,16 +3907,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3801,10 +3926,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3812,16 +3937,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3831,40 +3956,40 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="19" t="s">
+      <c r="A42" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B42" s="20" t="s">
-        <v>234</v>
-      </c>
-      <c r="C42" s="21" t="s">
-        <v>235</v>
-      </c>
-      <c r="D42" s="22">
-        <v>2</v>
-      </c>
-      <c r="E42" s="21" t="s">
+      <c r="B42" s="32" t="s">
         <v>236</v>
       </c>
-      <c r="F42" s="22">
-        <v>2</v>
-      </c>
-      <c r="G42" s="23" t="str">
+      <c r="C42" s="33" t="s">
+        <v>237</v>
+      </c>
+      <c r="D42" s="34">
+        <v>2</v>
+      </c>
+      <c r="E42" s="33" t="s">
+        <v>238</v>
+      </c>
+      <c r="F42" s="34">
+        <v>0</v>
+      </c>
+      <c r="G42" s="35" t="str">
         <f>IF(OR(D42="",F42=""),"chưa rõ",IF(F42&gt;D42,"FRACILE",IF(D42&gt;F42,"Vivoire","hoà")))</f>
-        <v>hoà</v>
-      </c>
-      <c r="H42" s="19" t="s">
-        <v>237</v>
-      </c>
-      <c r="I42" s="24" t="s">
-        <v>238</v>
+        <v>Vivoire</v>
+      </c>
+      <c r="H42" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="I42" s="36" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3872,14 +3997,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -3889,37 +4014,37 @@
         <v>chưa rõ</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="25" t="s">
+      <c r="A44" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="26" t="s">
-        <v>242</v>
-      </c>
-      <c r="C44" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="D44" s="28"/>
-      <c r="E44" s="27" t="s">
+      <c r="B44" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="F44" s="28">
-        <v>2</v>
-      </c>
-      <c r="G44" s="29" t="str">
+      <c r="C44" s="33" t="s">
+        <v>120</v>
+      </c>
+      <c r="D44" s="34"/>
+      <c r="E44" s="33" t="s">
+        <v>244</v>
+      </c>
+      <c r="F44" s="34">
+        <v>0</v>
+      </c>
+      <c r="G44" s="35" t="str">
         <f>IF(OR(D44="",F44=""),"chưa rõ",IF(F44&gt;D44,"FRACILE",IF(D44&gt;F44,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H44" s="25" t="s">
-        <v>244</v>
-      </c>
-      <c r="I44" s="30" t="s">
+      <c r="H44" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="I44" s="36" t="s">
         <v>245</v>
       </c>
     </row>
@@ -3931,7 +4056,7 @@
         <v>246</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
@@ -3959,7 +4084,7 @@
         <v>250</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D46" s="28"/>
       <c r="E46" s="27" t="s">
@@ -3987,13 +4112,13 @@
         <v>254</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F47" s="22">
         <v>2</v>
@@ -4003,7 +4128,7 @@
         <v>hoà</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I47" s="24" t="s">
         <v>255</v>
@@ -4077,7 +4202,7 @@
         <v>266</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
@@ -4093,10 +4218,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4123,7 +4248,7 @@
         <v>FRACILE</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I51" s="30" t="s">
         <v>271</v>
@@ -4137,7 +4262,7 @@
         <v>272</v>
       </c>
       <c r="C52" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D52" s="28"/>
       <c r="E52" s="27" t="s">
@@ -4151,7 +4276,7 @@
         <v>chưa rõ</v>
       </c>
       <c r="H52" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I52" s="30" t="s">
         <v>274</v>
@@ -4165,7 +4290,7 @@
         <v>275</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
@@ -4181,7 +4306,7 @@
         <v>hoà</v>
       </c>
       <c r="H53" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I53" s="24" t="s">
         <v>277</v>
@@ -4195,7 +4320,7 @@
         <v>278</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D54" s="22">
         <v>2</v>
@@ -4225,7 +4350,7 @@
         <v>37</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D55" s="22">
         <v>2</v>
@@ -4271,7 +4396,7 @@
         <v>Vivoire</v>
       </c>
       <c r="H56" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I56" s="24" t="s">
         <v>287</v>
@@ -4301,7 +4426,7 @@
         <v>FRACILE</v>
       </c>
       <c r="H57" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I57" s="30" t="s">
         <v>291</v>
@@ -4315,7 +4440,7 @@
         <v>292</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D58" s="28"/>
       <c r="E58" s="27" t="s">
@@ -4329,10 +4454,122 @@
         <v>chưa rõ</v>
       </c>
       <c r="H58" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I58" s="30" t="s">
         <v>294</v>
+      </c>
+    </row>
+    <row r="59" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59" s="26" t="s">
+        <v>295</v>
+      </c>
+      <c r="C59" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="D59" s="28"/>
+      <c r="E59" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="F59" s="28">
+        <v>2</v>
+      </c>
+      <c r="G59" s="29" t="str">
+        <f>IF(OR(D59="",F59=""),"chưa rõ",IF(F59&gt;D59,"FRACILE",IF(D59&gt;F59,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H59" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="I59" s="30" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="60" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60" s="26" t="s">
+        <v>298</v>
+      </c>
+      <c r="C60" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="D60" s="28"/>
+      <c r="E60" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="F60" s="28">
+        <v>2</v>
+      </c>
+      <c r="G60" s="29" t="str">
+        <f>IF(OR(D60="",F60=""),"chưa rõ",IF(F60&gt;D60,"FRACILE",IF(D60&gt;F60,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H60" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="I60" s="30" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="61" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B61" s="26" t="s">
+        <v>302</v>
+      </c>
+      <c r="C61" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="D61" s="28"/>
+      <c r="E61" s="27" t="s">
+        <v>303</v>
+      </c>
+      <c r="F61" s="28">
+        <v>2</v>
+      </c>
+      <c r="G61" s="29" t="str">
+        <f>IF(OR(D61="",F61=""),"chưa rõ",IF(F61&gt;D61,"FRACILE",IF(D61&gt;F61,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H61" s="25" t="s">
+        <v>304</v>
+      </c>
+      <c r="I61" s="30" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="62" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B62" s="26" t="s">
+        <v>306</v>
+      </c>
+      <c r="C62" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="D62" s="28"/>
+      <c r="E62" s="27" t="s">
+        <v>308</v>
+      </c>
+      <c r="F62" s="28">
+        <v>2</v>
+      </c>
+      <c r="G62" s="29" t="str">
+        <f>IF(OR(D62="",F62=""),"chưa rõ",IF(F62&gt;D62,"FRACILE",IF(D62&gt;F62,"Vivoire","hoà")))</f>
+        <v>chưa rõ</v>
+      </c>
+      <c r="H62" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="I62" s="30" t="s">
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -4344,7 +4581,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -4356,12 +4593,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>295</v>
+        <v>311</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>296</v>
+        <v>312</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4377,332 +4614,400 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>297</v>
+        <v>313</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>299</v>
+        <v>315</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>300</v>
+        <v>316</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>302</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>303</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>305</v>
+      <c r="A6" s="27" t="s">
+        <v>318</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>319</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>321</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>306</v>
+        <v>323</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>307</v>
+        <v>324</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>316</v>
+        <v>334</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
-        <v>318</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>319</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" s="21" t="s">
+      <c r="A11" s="27" t="s">
+        <v>336</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>337</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>339</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="27" t="s">
+        <v>341</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>342</v>
+      </c>
+      <c r="C12" s="25" t="s">
         <v>320</v>
       </c>
-    </row>
-    <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
-        <v>321</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>322</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>324</v>
+      <c r="D12" s="27" t="s">
+        <v>343</v>
+      </c>
+      <c r="E12" s="27" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
-        <v>325</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>326</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>154</v>
+      <c r="A13" s="27" t="s">
+        <v>345</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>346</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>339</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
-        <v>220</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>327</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>328</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>329</v>
+      <c r="A14" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>348</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>343</v>
+      </c>
+      <c r="E14" s="27" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>331</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>332</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>333</v>
+      <c r="A15" s="27" t="s">
+        <v>350</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>351</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>339</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>345</v>
+        <v>320</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>346</v>
+        <v>363</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>347</v>
+        <v>364</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>348</v>
+        <v>365</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>349</v>
+        <v>366</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>350</v>
+        <v>367</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>351</v>
+        <v>368</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>352</v>
+        <v>369</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>353</v>
+        <v>370</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>351</v>
+        <v>368</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>354</v>
+        <v>371</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="38" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
-        <v>357</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="18"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="18"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="18"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
+        <v>372</v>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="27" t="s">
+        <v>373</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>374</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="D22" s="27" t="s">
+        <v>375</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="27" t="s">
+        <v>377</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>378</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>379</v>
+      </c>
+      <c r="E23" s="27" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="27" t="s">
+        <v>381</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>374</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="D24" s="27" t="s">
+        <v>359</v>
+      </c>
+      <c r="E24" s="27" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="27" t="s">
+        <v>383</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>384</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>371</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25" s="27" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="38" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="18" t="s">
+        <v>387</v>
+      </c>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="18"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="18"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="18"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E3"/>
-    <mergeCell ref="A25:E28"/>
+    <mergeCell ref="A29:E32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4711,7 +5016,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -4722,386 +5027,428 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>358</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>360</v>
+        <v>390</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>361</v>
+        <v>391</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>363</v>
+        <v>393</v>
       </c>
       <c r="B4" s="40">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>364</v>
+        <v>394</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>365</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>366</v>
+        <v>396</v>
       </c>
       <c r="B5" s="40">
-        <v>413</v>
+        <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>367</v>
+        <v>397</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>365</v>
+        <v>395</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>368</v>
+        <v>398</v>
       </c>
       <c r="B6" s="40">
-        <v>248</v>
+        <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>365</v>
+        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>370</v>
+        <v>400</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>371</v>
+        <v>401</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>372</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>373</v>
+        <v>402</v>
       </c>
       <c r="B8" s="40">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>374</v>
+        <v>403</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>372</v>
+        <v>395</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>375</v>
+        <v>404</v>
       </c>
       <c r="B9" s="40">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>376</v>
+        <v>405</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>365</v>
+        <v>395</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>377</v>
+        <v>406</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>378</v>
+        <v>407</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>365</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>379</v>
+        <v>409</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>380</v>
+        <v>410</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>365</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>381</v>
+        <v>411</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>382</v>
+        <v>412</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>372</v>
+        <v>413</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>383</v>
+        <v>414</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>384</v>
+        <v>415</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>372</v>
+        <v>413</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>385</v>
+        <v>416</v>
       </c>
       <c r="B14" s="40">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>386</v>
+        <v>417</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="B15" s="40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>389</v>
+        <v>419</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>365</v>
+        <v>395</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>390</v>
+        <v>420</v>
       </c>
       <c r="B16" s="40">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>391</v>
+        <v>421</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>365</v>
+        <v>395</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>392</v>
+        <v>422</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>393</v>
+        <v>423</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>394</v>
+        <v>424</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>395</v>
+        <v>425</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>396</v>
+        <v>426</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>372</v>
+        <v>413</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>397</v>
+        <v>427</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>398</v>
+        <v>428</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
-        <v>399</v>
-      </c>
-      <c r="B21" s="43">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="39" t="s">
+        <v>430</v>
+      </c>
+      <c r="B20" s="40">
+        <v>2</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>431</v>
+      </c>
+      <c r="D20" s="42" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="39" t="s">
+        <v>432</v>
+      </c>
+      <c r="B21" s="40">
+        <v>2</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>433</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="39" t="s">
+        <v>434</v>
+      </c>
+      <c r="B22" s="40">
+        <v>7</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>435</v>
+      </c>
+      <c r="D22" s="42" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>436</v>
+      </c>
+      <c r="B24" s="43">
         <f>B6/B5</f>
-        <v>0.5618279569892473</v>
-      </c>
-      <c r="C21" s="44" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
-        <v>401</v>
-      </c>
-      <c r="B22" s="45">
+        <v>0.7990919409761634</v>
+      </c>
+      <c r="C24" s="44" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>438</v>
+      </c>
+      <c r="B25" s="45">
         <f>B5-B6</f>
-        <v>163</v>
-      </c>
-      <c r="C22" s="44" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="38" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>406</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>407</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
-        <v>409</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>410</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>411</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="19" t="s">
-        <v>412</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>410</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>411</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>408</v>
+        <v>177</v>
+      </c>
+      <c r="C25" s="44" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="38" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>413</v>
+        <v>149</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>414</v>
+        <v>443</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>411</v>
+        <v>444</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>408</v>
+        <v>445</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="46" t="s">
-        <v>415</v>
-      </c>
-      <c r="B31" s="47" t="s">
-        <v>416</v>
-      </c>
-      <c r="C31" s="47" t="s">
-        <v>417</v>
-      </c>
-      <c r="D31" s="47" t="s">
-        <v>418</v>
+      <c r="A31" s="19" t="s">
+        <v>446</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>447</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>448</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="46" t="s">
-        <v>419</v>
-      </c>
-      <c r="B32" s="47" t="s">
-        <v>420</v>
-      </c>
-      <c r="C32" s="47" t="s">
-        <v>421</v>
-      </c>
-      <c r="D32" s="47" t="s">
-        <v>418</v>
+      <c r="A32" s="19" t="s">
+        <v>449</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>447</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>448</v>
+      </c>
+      <c r="D32" s="21" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>422</v>
+        <v>450</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>423</v>
+        <v>451</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>424</v>
+        <v>448</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>425</v>
+        <v>445</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="46" t="s">
+        <v>452</v>
+      </c>
+      <c r="B34" s="47" t="s">
+        <v>453</v>
+      </c>
+      <c r="C34" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="D34" s="47" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="46" t="s">
+        <v>456</v>
+      </c>
+      <c r="B35" s="47" t="s">
+        <v>457</v>
+      </c>
+      <c r="C35" s="47" t="s">
+        <v>458</v>
+      </c>
+      <c r="D35" s="47" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
+        <v>459</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>460</v>
+      </c>
+      <c r="C36" s="21" t="s">
+        <v>461</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>462</v>
       </c>
     </row>
   </sheetData>
@@ -5124,24 +5471,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>426</v>
+        <v>463</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>427</v>
+        <v>464</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>428</v>
+        <v>465</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>429</v>
+        <v>466</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>430</v>
+        <v>467</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>431</v>
+        <v>468</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5149,16 +5496,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>432</v>
+        <v>469</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>433</v>
+        <v>470</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>434</v>
+        <v>471</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>435</v>
+        <v>472</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5166,16 +5513,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>436</v>
+        <v>473</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>437</v>
+        <v>474</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>438</v>
+        <v>475</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>439</v>
+        <v>476</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5183,16 +5530,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>440</v>
+        <v>477</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>441</v>
+        <v>478</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>442</v>
+        <v>479</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>443</v>
+        <v>480</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5200,16 +5547,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>444</v>
+        <v>481</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>445</v>
+        <v>482</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>446</v>
+        <v>483</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>447</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: đã xuất bản 62 bài nháp + 7 đề; cập nhật Việc cần làm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="487">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -389,13 +389,10 @@
     <t>DELF/DALF A1–C2</t>
   </si>
   <si>
-    <t>7 đề (3 đã phát hành). Đủ A1 · A2 · B1 · B2 · C1 theo format 2 hiện hành; học sinh chọn đề theo tab trình độ A1–B2. File docs/format-de-thi-DELF-A1-B2.xlsx ghi cấu trúc từng phần. Còn chờ phát hành các đề nháp</t>
-  </si>
-  <si>
-    <t>Đang chạy — đề A1, A2 Đề 2, B2, C1 là nháp</t>
-  </si>
-  <si>
-    <t>lo10 (A1), lo11 (A2 Đề 2), lo9 (B2), lo6 (C1). Chưa lên 2 vì phần lớn đề còn nháp</t>
+    <t>7 đề, CẢ 7 ĐÃ PHÁT HÀNH (08/10): DELF A1 · A2 (2 đề) · B1 (2 đề) · B2 · DALF C1, đủ 4 phần theo format 2; học sinh chọn đề theo tab trình độ. Cấu trúc từng phần ghi ở docs/format-de-thi-DELF-A1-B2.xlsx</t>
+  </si>
+  <si>
+    <t>select count(*) from exams where is_published = 7, đo 08/10. Lô lo4, lo6, lo9, lo10, lo11</t>
   </si>
   <si>
     <t>Nghe hiểu giới hạn 2 lượt phát</t>
@@ -467,13 +464,10 @@
     <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
   </si>
   <si>
-    <t>110 bài trong kho (ĐẾM THẬT 08/10), trong đó 62 bài/đề con còn NHÁP chờ duyệt</t>
-  </si>
-  <si>
-    <t>Đang chạy — 62 nháp chờ duyệt</t>
-  </si>
-  <si>
-    <t>select count(*) from exercises = 110; title like '[NHÁP]%' = 62. Lên 2 khi xuất bản đủ ≥ 60 bài công khai</t>
+    <t>110 bài, TẤT CẢ đã xuất bản (08/10): 90 bài luyện tập riêng + 20 bài thuộc đề thi thử, A1 → C1, trong đó các bài nghe giọng tổng hợp và 3 bài cắt từ Wikipédia parlée</t>
+  </si>
+  <si>
+    <t>select count(*) from exercises = 110, nháp = 0, đo 08/10/2026. Vẫn ít hơn 400 bài Vivoire công bố, nhưng vượt ngưỡng 60 để chấm 2</t>
   </si>
   <si>
     <t>Số câu hỏi</t>
@@ -1225,7 +1219,7 @@
     <t>Bài tập</t>
   </si>
   <si>
-    <t>select count(*) from exercises — 62 bài/đề con NHÁP chờ duyệt</t>
+    <t>select count(*) from exercises — đã xuất bản hết, 0 nháp</t>
   </si>
   <si>
     <t>08/10/2026</t>
@@ -1252,7 +1246,7 @@
     <t>Đề thi thử</t>
   </si>
   <si>
-    <t>select count(*) from exams — 3 đã phát hành</t>
+    <t>select count(*) from exams — cả 7 đã phát hành</t>
   </si>
   <si>
     <t>Lượt làm bài đã chấm</t>
@@ -1450,46 +1444,58 @@
     <t>Công sức</t>
   </si>
   <si>
-    <t>Đặt khoá API để bật chấm PE bằng AI</t>
-  </si>
-  <si>
-    <t>Chủ dự án tạm gác 23/09. Mọi thứ đã dựng và kiểm; thiếu khoá thì nút « Xin gợi ý » báo tính năng chưa bật, không lỗi.</t>
-  </si>
-  <si>
-    <t>npx supabase secrets set ANTHROPIC_API_KEY=sk-ant-…</t>
+    <t>Quyết định số phận 5 tài khoản không có hồ sơ</t>
+  </si>
+  <si>
+    <t>Đăng nhập được nhưng không có dòng profiles (không vai, không tên), nên vào app sẽ hỏng. Hai tài khoản vẫn đăng nhập ngày 27/09. Xoá hay tạo hồ sơ là việc xoá/sửa dữ liệu người dùng — cần chủ dự án quyết.</t>
+  </si>
+  <si>
+    <t>auth.users trái join profiles; tạo hồ sơ hoặc xoá tài khoản</t>
+  </si>
+  <si>
+    <t>10 phút</t>
+  </si>
+  <si>
+    <t>Thử một lần chuyển khoản VIP thật</t>
+  </si>
+  <si>
+    <t>Gói VIP đã kiểm trên database và webhook, nhưng chưa có giao dịch thật đi hết đường SePay → gia hạn.</t>
+  </si>
+  <si>
+    <t>Chuyển 99.000 đ với nội dung trên màn thanh toán</t>
   </si>
   <si>
     <t>5 phút</t>
   </si>
   <si>
-    <t>Xem 5 tài khoản không có hồ sơ</t>
-  </si>
-  <si>
-    <t>14 tài khoản đăng nhập nhưng chỉ 9 hồ sơ. Có thể là tài khoản thử khác, hoặc người đăng ký dở — chưa ai xem.</t>
-  </si>
-  <si>
-    <t>Quyết định sau khi xem danh sách</t>
-  </si>
-  <si>
-    <t>10 phút</t>
-  </si>
-  <si>
-    <t>Cân nhắc dựng lại Chính sách bảo mật trước khi thu tiền nhiều</t>
-  </si>
-  <si>
-    <t>Đã gỡ theo quyết định 21/09; nội dung còn trong git.</t>
-  </si>
-  <si>
-    <t>Lấy TrangBaoMat từ commit cũ + route /bao-mat</t>
+    <t>Nghe thử đề A1 và A2 Đề 2 trên giao diện thi</t>
+  </si>
+  <si>
+    <t>Đề vừa phát hành 08/10; file nghe kiểu phòng thi mới đo bằng máy, chưa ai nghe từ đầu tới cuối trong màn thi.</t>
+  </si>
+  <si>
+    <t>Tài khoản học sinh → Thi thử (dùng 1 trong 2 lượt/ngày)</t>
   </si>
   <si>
     <t>30 phút</t>
   </si>
   <si>
-    <t>Cân nhắc KHÔNG đuổi theo: từ điển, podcast, PvP, app mobile</t>
-  </si>
-  <si>
-    <t>Bốn ô Vivoire hơn tuyệt đối. Đuổi theo cả bốn với một người là cách chắc chắn để không ô nào xong.</t>
+    <t>Đối chiếu số câu và điểm từng bài A1/A2 với đề mẫu chính thức</t>
+  </si>
+  <si>
+    <t>Phần A1/A2 của file format đề dựa trên nguồn thứ cấp vì trang FEI chặn truy cập tự động.</t>
+  </si>
+  <si>
+    <t>docs/format-de-thi-DELF-A1-B2.xlsx</t>
+  </si>
+  <si>
+    <t>1 giờ</t>
+  </si>
+  <si>
+    <t>Cân nhắc KHÔNG đuổi theo: từ điển 56.000 từ, podcast, lớp video, app trên store</t>
+  </si>
+  <si>
+    <t>Các ô Vivoire hơn tuyệt đối. Đuổi theo cả bốn với một người là cách chắc chắn để không ô nào xong.</t>
   </si>
   <si>
     <t>—</t>
@@ -2203,11 +2209,11 @@
       </c>
       <c r="E8" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="6">
         <f>IFERROR(E8-D8,"")</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="7" t="str">
         <f>IF(OR(C8&lt;3,F8=""),"quá ít mục",IF(F8&gt;0.25,"FRACILE",IF(F8&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2232,11 +2238,11 @@
       </c>
       <c r="E9" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F9" s="6">
         <f>IFERROR(E9-D9,"")</f>
-        <v>-1.2</v>
+        <v>-1</v>
       </c>
       <c r="G9" s="7" t="str">
         <f>IF(OR(C9&lt;3,F9=""),"quá ít mục",IF(F9&gt;0.25,"FRACILE",IF(F9&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2377,11 +2383,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>1.3333333333333333</v>
+        <v>1.393939393939394</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.5454545454545456</v>
+        <v>-0.48484848484848486</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -3051,17 +3057,17 @@
         <v>116</v>
       </c>
       <c r="F10" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" s="23" t="str">
         <f>IF(OR(D10="",F10=""),"chưa rõ",IF(F10&gt;D10,"FRACILE",IF(D10&gt;F10,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H10" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" s="24" t="s">
         <v>117</v>
-      </c>
-      <c r="I10" s="24" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3069,14 +3075,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="27" t="s">
         <v>119</v>
-      </c>
-      <c r="C11" s="27" t="s">
-        <v>120</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -3089,7 +3095,7 @@
         <v>82</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3097,14 +3103,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -3117,7 +3123,7 @@
         <v>82</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3125,14 +3131,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -3145,7 +3151,7 @@
         <v>82</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3153,14 +3159,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -3173,7 +3179,7 @@
         <v>82</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3181,14 +3187,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -3201,7 +3207,7 @@
         <v>82</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3209,16 +3215,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="D16" s="22">
+        <v>2</v>
+      </c>
+      <c r="E16" s="21" t="s">
         <v>136</v>
-      </c>
-      <c r="D16" s="22">
-        <v>2</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>137</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -3228,10 +3234,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="I16" s="24" t="s">
         <v>138</v>
-      </c>
-      <c r="I16" s="24" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3239,29 +3245,29 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="C17" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="D17" s="22">
+        <v>2</v>
+      </c>
+      <c r="E17" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="D17" s="22">
-        <v>2</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>142</v>
-      </c>
       <c r="F17" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" s="23" t="str">
         <f>IF(OR(D17="",F17=""),"chưa rõ",IF(F17&gt;D17,"FRACILE",IF(D17&gt;F17,"Vivoire","hoà")))</f>
-        <v>Vivoire</v>
+        <v>hoà</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>143</v>
+        <v>82</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3269,14 +3275,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3289,7 +3295,7 @@
         <v>82</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3297,16 +3303,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="D19" s="22">
+        <v>2</v>
+      </c>
+      <c r="E19" s="21" t="s">
         <v>149</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>150</v>
-      </c>
-      <c r="D19" s="22">
-        <v>2</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>151</v>
       </c>
       <c r="F19" s="22">
         <v>1</v>
@@ -3319,7 +3325,7 @@
         <v>82</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3327,16 +3333,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3346,10 +3352,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3357,16 +3363,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="D21" s="22">
+        <v>2</v>
+      </c>
+      <c r="E21" s="21" t="s">
         <v>157</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>158</v>
-      </c>
-      <c r="D21" s="22">
-        <v>2</v>
-      </c>
-      <c r="E21" s="21" t="s">
-        <v>159</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3376,10 +3382,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3387,14 +3393,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3407,7 +3413,7 @@
         <v>82</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3415,16 +3421,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="D23" s="22">
+        <v>2</v>
+      </c>
+      <c r="E23" s="21" t="s">
         <v>165</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>166</v>
-      </c>
-      <c r="D23" s="22">
-        <v>2</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>167</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3434,10 +3440,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3445,14 +3451,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3462,10 +3468,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3473,14 +3479,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3493,7 +3499,7 @@
         <v>82</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3501,16 +3507,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="D26" s="22">
+        <v>2</v>
+      </c>
+      <c r="E26" s="21" t="s">
         <v>178</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>179</v>
-      </c>
-      <c r="D26" s="22">
-        <v>2</v>
-      </c>
-      <c r="E26" s="21" t="s">
-        <v>180</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3523,7 +3529,7 @@
         <v>82</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3531,14 +3537,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3548,10 +3554,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3559,16 +3565,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="D28" s="22">
+        <v>2</v>
+      </c>
+      <c r="E28" s="21" t="s">
         <v>186</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="D28" s="22">
-        <v>2</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>188</v>
       </c>
       <c r="F28" s="22">
         <v>2</v>
@@ -3578,10 +3584,10 @@
         <v>hoà</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3589,16 +3595,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>190</v>
+      </c>
+      <c r="D29" s="22">
+        <v>2</v>
+      </c>
+      <c r="E29" s="21" t="s">
         <v>191</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="D29" s="22">
-        <v>2</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>193</v>
       </c>
       <c r="F29" s="22">
         <v>2</v>
@@ -3608,10 +3614,10 @@
         <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3619,16 +3625,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="D30" s="22">
+        <v>2</v>
+      </c>
+      <c r="E30" s="21" t="s">
         <v>196</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="D30" s="22">
-        <v>2</v>
-      </c>
-      <c r="E30" s="21" t="s">
-        <v>198</v>
       </c>
       <c r="F30" s="22">
         <v>2</v>
@@ -3638,10 +3644,10 @@
         <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3649,14 +3655,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3669,7 +3675,7 @@
         <v>82</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3677,16 +3683,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="D32" s="22">
+        <v>2</v>
+      </c>
+      <c r="E32" s="21" t="s">
         <v>204</v>
-      </c>
-      <c r="C32" s="21" t="s">
-        <v>205</v>
-      </c>
-      <c r="D32" s="22">
-        <v>2</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>206</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3696,10 +3702,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3707,14 +3713,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3727,7 +3733,7 @@
         <v>82</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3735,14 +3741,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3752,10 +3758,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3763,14 +3769,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3780,10 +3786,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3791,14 +3797,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3808,10 +3814,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3819,14 +3825,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3836,10 +3842,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3847,16 +3853,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F38" s="22">
         <v>2</v>
@@ -3866,10 +3872,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3877,16 +3883,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="D39" s="22">
+        <v>2</v>
+      </c>
+      <c r="E39" s="21" t="s">
         <v>227</v>
-      </c>
-      <c r="C39" s="21" t="s">
-        <v>228</v>
-      </c>
-      <c r="D39" s="22">
-        <v>2</v>
-      </c>
-      <c r="E39" s="21" t="s">
-        <v>229</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3896,10 +3902,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3907,16 +3913,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3926,10 +3932,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3937,16 +3943,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3956,10 +3962,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3967,16 +3973,16 @@
         <v>15</v>
       </c>
       <c r="B42" s="32" t="s">
+        <v>234</v>
+      </c>
+      <c r="C42" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="D42" s="34">
+        <v>2</v>
+      </c>
+      <c r="E42" s="33" t="s">
         <v>236</v>
-      </c>
-      <c r="C42" s="33" t="s">
-        <v>237</v>
-      </c>
-      <c r="D42" s="34">
-        <v>2</v>
-      </c>
-      <c r="E42" s="33" t="s">
-        <v>238</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3989,7 +3995,7 @@
         <v>104</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3997,14 +4003,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -4017,7 +4023,7 @@
         <v>82</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4025,14 +4031,14 @@
         <v>15</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D44" s="34"/>
       <c r="E44" s="33" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -4045,7 +4051,7 @@
         <v>104</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4053,14 +4059,14 @@
         <v>15</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -4070,10 +4076,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4081,14 +4087,14 @@
         <v>15</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D46" s="28"/>
       <c r="E46" s="27" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F46" s="28">
         <v>2</v>
@@ -4098,10 +4104,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H46" s="25" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4109,16 +4115,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F47" s="22">
         <v>2</v>
@@ -4131,7 +4137,7 @@
         <v>82</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4139,16 +4145,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="20" t="s">
+        <v>254</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>255</v>
+      </c>
+      <c r="D48" s="22">
+        <v>2</v>
+      </c>
+      <c r="E48" s="21" t="s">
         <v>256</v>
-      </c>
-      <c r="C48" s="21" t="s">
-        <v>257</v>
-      </c>
-      <c r="D48" s="22">
-        <v>2</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>258</v>
       </c>
       <c r="F48" s="22">
         <v>1</v>
@@ -4158,10 +4164,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I48" s="24" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4169,16 +4175,16 @@
         <v>16</v>
       </c>
       <c r="B49" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>260</v>
+      </c>
+      <c r="D49" s="22">
+        <v>2</v>
+      </c>
+      <c r="E49" s="21" t="s">
         <v>261</v>
-      </c>
-      <c r="C49" s="21" t="s">
-        <v>262</v>
-      </c>
-      <c r="D49" s="22">
-        <v>2</v>
-      </c>
-      <c r="E49" s="21" t="s">
-        <v>263</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -4188,10 +4194,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4199,16 +4205,16 @@
         <v>16</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -4221,7 +4227,7 @@
         <v>82</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4229,16 +4235,16 @@
         <v>16</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D51" s="28">
         <v>1</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -4251,7 +4257,7 @@
         <v>82</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4259,14 +4265,14 @@
         <v>16</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C52" s="27" t="s">
         <v>107</v>
       </c>
       <c r="D52" s="28"/>
       <c r="E52" s="27" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F52" s="28">
         <v>2</v>
@@ -4279,7 +4285,7 @@
         <v>82</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4287,16 +4293,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F53" s="22">
         <v>2</v>
@@ -4309,7 +4315,7 @@
         <v>82</v>
       </c>
       <c r="I53" s="24" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4317,16 +4323,16 @@
         <v>17</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D54" s="22">
         <v>2</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="F54" s="22">
         <v>1</v>
@@ -4336,10 +4342,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4350,13 +4356,13 @@
         <v>37</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D55" s="22">
         <v>2</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="F55" s="22">
         <v>1</v>
@@ -4366,10 +4372,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="I55" s="24" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="56" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4377,16 +4383,16 @@
         <v>17</v>
       </c>
       <c r="B56" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="C56" s="21" t="s">
+        <v>283</v>
+      </c>
+      <c r="D56" s="22">
+        <v>2</v>
+      </c>
+      <c r="E56" s="21" t="s">
         <v>284</v>
-      </c>
-      <c r="C56" s="21" t="s">
-        <v>285</v>
-      </c>
-      <c r="D56" s="22">
-        <v>2</v>
-      </c>
-      <c r="E56" s="21" t="s">
-        <v>286</v>
       </c>
       <c r="F56" s="22">
         <v>1</v>
@@ -4399,7 +4405,7 @@
         <v>82</v>
       </c>
       <c r="I56" s="24" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="57" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4407,16 +4413,16 @@
         <v>17</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D57" s="28">
         <v>1</v>
       </c>
       <c r="E57" s="27" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="F57" s="28">
         <v>2</v>
@@ -4429,7 +4435,7 @@
         <v>82</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="58" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4437,14 +4443,14 @@
         <v>17</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D58" s="28"/>
       <c r="E58" s="27" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="F58" s="28">
         <v>2</v>
@@ -4457,7 +4463,7 @@
         <v>82</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="59" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4465,14 +4471,14 @@
         <v>12</v>
       </c>
       <c r="B59" s="26" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D59" s="28"/>
       <c r="E59" s="27" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="F59" s="28">
         <v>2</v>
@@ -4485,7 +4491,7 @@
         <v>82</v>
       </c>
       <c r="I59" s="30" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="60" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4493,14 +4499,14 @@
         <v>13</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C60" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D60" s="28"/>
       <c r="E60" s="27" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="F60" s="28">
         <v>2</v>
@@ -4510,10 +4516,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H60" s="25" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="61" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4521,14 +4527,14 @@
         <v>15</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C61" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D61" s="28"/>
       <c r="E61" s="27" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="F61" s="28">
         <v>2</v>
@@ -4538,10 +4544,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H61" s="25" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="62" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4549,14 +4555,14 @@
         <v>14</v>
       </c>
       <c r="B62" s="26" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C62" s="27" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D62" s="28"/>
       <c r="E62" s="27" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="F62" s="28">
         <v>2</v>
@@ -4566,10 +4572,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H62" s="25" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>
@@ -4593,12 +4599,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4614,369 +4620,369 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>315</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
+        <v>316</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>317</v>
+      </c>
+      <c r="C6" s="25" t="s">
         <v>318</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="D6" s="27" t="s">
         <v>319</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="E6" s="27" t="s">
         <v>320</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>321</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
+        <v>321</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>322</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>323</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>324</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>325</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>82</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
+        <v>325</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>326</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="D8" s="21" t="s">
         <v>327</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="E8" s="21" t="s">
         <v>328</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>325</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>329</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>82</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>82</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
+        <v>334</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>335</v>
+      </c>
+      <c r="C11" s="25" t="s">
         <v>336</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="D11" s="27" t="s">
         <v>337</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="E11" s="27" t="s">
         <v>338</v>
-      </c>
-      <c r="D11" s="27" t="s">
-        <v>339</v>
-      </c>
-      <c r="E11" s="27" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
+        <v>339</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>340</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="D12" s="27" t="s">
         <v>341</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="E12" s="27" t="s">
         <v>342</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>320</v>
-      </c>
-      <c r="D12" s="27" t="s">
-        <v>343</v>
-      </c>
-      <c r="E12" s="27" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
+        <v>343</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>344</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>337</v>
+      </c>
+      <c r="E13" s="27" t="s">
         <v>345</v>
-      </c>
-      <c r="B13" s="27" t="s">
-        <v>346</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="D13" s="27" t="s">
-        <v>339</v>
-      </c>
-      <c r="E13" s="27" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
+        <v>348</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>349</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>337</v>
+      </c>
+      <c r="E15" s="27" t="s">
         <v>350</v>
-      </c>
-      <c r="B15" s="27" t="s">
-        <v>351</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="D15" s="27" t="s">
-        <v>339</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
+        <v>351</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="D16" s="27" t="s">
         <v>353</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="E16" s="27" t="s">
         <v>354</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>355</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
+        <v>355</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>356</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="D17" s="27" t="s">
         <v>357</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="E17" s="27" t="s">
         <v>358</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>359</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>82</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
+        <v>362</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>363</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="E19" s="27" t="s">
         <v>364</v>
-      </c>
-      <c r="B19" s="27" t="s">
-        <v>365</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="D19" s="27" t="s">
-        <v>355</v>
-      </c>
-      <c r="E19" s="27" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
+        <v>365</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>366</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="E20" s="27" t="s">
         <v>367</v>
-      </c>
-      <c r="B20" s="27" t="s">
-        <v>368</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>355</v>
-      </c>
-      <c r="E20" s="27" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>82</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
+        <v>371</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>372</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="D22" s="27" t="s">
         <v>373</v>
       </c>
-      <c r="B22" s="27" t="s">
+      <c r="E22" s="27" t="s">
         <v>374</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>320</v>
-      </c>
-      <c r="D22" s="27" t="s">
-        <v>375</v>
-      </c>
-      <c r="E22" s="27" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
+        <v>375</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>376</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="D23" s="27" t="s">
         <v>377</v>
       </c>
-      <c r="B23" s="27" t="s">
+      <c r="E23" s="27" t="s">
         <v>378</v>
-      </c>
-      <c r="C23" s="25" t="s">
-        <v>320</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>379</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D25" s="27" t="s">
         <v>82</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5027,428 +5033,428 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>390</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B4" s="40">
         <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B5" s="40">
         <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B6" s="40">
         <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B8" s="40">
         <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B9" s="40">
         <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B14" s="40">
         <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B16" s="40">
         <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B20" s="40">
         <v>2</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B21" s="40">
         <v>2</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B22" s="40">
         <v>7</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B24" s="43">
         <f>B6/B5</f>
         <v>0.7990919409761634</v>
       </c>
       <c r="C24" s="44" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B25" s="45">
         <f>B5-B6</f>
         <v>177</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B30" s="21" t="s">
+        <v>441</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>442</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>443</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>444</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
+        <v>444</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>445</v>
+      </c>
+      <c r="C31" s="21" t="s">
         <v>446</v>
       </c>
-      <c r="B31" s="21" t="s">
-        <v>447</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>448</v>
-      </c>
       <c r="D31" s="21" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
+        <v>450</v>
+      </c>
+      <c r="B34" s="47" t="s">
+        <v>451</v>
+      </c>
+      <c r="C34" s="47" t="s">
         <v>452</v>
       </c>
-      <c r="B34" s="47" t="s">
+      <c r="D34" s="47" t="s">
         <v>453</v>
-      </c>
-      <c r="C34" s="47" t="s">
-        <v>454</v>
-      </c>
-      <c r="D34" s="47" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
+        <v>454</v>
+      </c>
+      <c r="B35" s="47" t="s">
+        <v>455</v>
+      </c>
+      <c r="C35" s="47" t="s">
         <v>456</v>
       </c>
-      <c r="B35" s="47" t="s">
-        <v>457</v>
-      </c>
-      <c r="C35" s="47" t="s">
-        <v>458</v>
-      </c>
       <c r="D35" s="47" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
+        <v>457</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>458</v>
+      </c>
+      <c r="C36" s="21" t="s">
         <v>459</v>
       </c>
-      <c r="B36" s="21" t="s">
+      <c r="D36" s="21" t="s">
         <v>460</v>
-      </c>
-      <c r="C36" s="21" t="s">
-        <v>461</v>
-      </c>
-      <c r="D36" s="21" t="s">
-        <v>462</v>
       </c>
     </row>
   </sheetData>
@@ -5459,7 +5465,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5471,24 +5477,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>465</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>466</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>467</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5496,16 +5502,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
+        <v>467</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>468</v>
+      </c>
+      <c r="D4" s="21" t="s">
         <v>469</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="E4" s="21" t="s">
         <v>470</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>471</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5513,16 +5519,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
+        <v>471</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>472</v>
+      </c>
+      <c r="D5" s="21" t="s">
         <v>473</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="E5" s="21" t="s">
         <v>474</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>475</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5530,16 +5536,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
+        <v>475</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>476</v>
+      </c>
+      <c r="D6" s="21" t="s">
         <v>477</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="E6" s="21" t="s">
         <v>478</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5547,16 +5553,33 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
+        <v>479</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>480</v>
+      </c>
+      <c r="D7" s="21" t="s">
         <v>481</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="E7" s="21" t="s">
         <v>482</v>
       </c>
-      <c r="D7" s="21" t="s">
+    </row>
+    <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="22">
+        <v>5</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>483</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="C8" s="21" t="s">
         <v>484</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>485</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: AI chấm PE thi thử, VIP không giới hạn, cảnh báo câu chưa làm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="490">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -246,6 +246,12 @@
     <t>Đề A1 + A2 Đề 2 theo format 2; nghe kiểu phòng thi (nghỉ 30 s giữa hai lượt); 2 lượt thi/ngày kèm cảnh báo; 3 dạng câu DELF mới; gói VIP + quản lý VIP; thu gọn tài khoản giáo viên (gỡ lời giải, sổ tay, lộ trình, tư vấn, tạo lớp); Flashcard, Neo, Cấp quyền, Thông báo làm lại giao diện; trạng thái online cho người theo dõi nhau. Học sinh: gộp Cần làm + Đã nộp thành « Bài tập được giao », Kết quả thi vào từ màn Thi thử, gỡ nút Làm mới.</t>
   </si>
   <si>
+    <t>08/10 chiều</t>
+  </si>
+  <si>
+    <t>AI tự chấm phần viết bài thi thử (thay « giáo viên đang chấm »); thanh chuyển bài + cảnh báo câu chưa làm trong thi thử; VIP không giới hạn lượt thi và lượt AI, có huy hiệu trên ảnh đại diện; xoá 5 tài khoản không có hồ sơ (đã sao lưu); xuất bản 62 bài nháp + 7 đề.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -311,10 +317,13 @@
     <t>AI chấm ngữ pháp và cách diễn đạt</t>
   </si>
   <si>
-    <t>ĐÃ BẬT 27/09 — OpenAI gpt-6-luna. Gợi ý điểm + nhận xét tiếng Việt theo từng tiêu chí grille; không tự điền, học sinh bấm « dùng số này » mới nhận. 6 lượt / 24 giờ</t>
-  </si>
-  <si>
-    <t>Edge Function cham-pe; chủ dự án thử qua giao diện 27/09, pe_ai_goi_y = 1 dòng (model gpt-6-luna). Đổi model: secrets set PE_AI_MODEL=…</t>
+    <t>Thi thử: AI TỰ CHẤM phần viết ngay khi mở trang Kết quả thi (thang DELF đúng trình độ, phiếu A1 gộp vào), điểm AI là điểm phần viết, kèm nhận xét từng tiêu chí. Luyện tập: học sinh tự chấm, xin gợi ý AI (6 lượt/24 giờ, VIP không giới hạn)</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa có bài thi nào chấm đầu-cuối qua giao diện</t>
+  </si>
+  <si>
+    <t>Edge Function cham-pe chế độ chinhThuc (08/10): ghi answers.score + feedback, chỉ câu chưa có điểm; AI thiếu tiêu chí thì không ghi. FAQ + /bao-mat đã sửa: phần viết thi thử gửi AI tự động</t>
   </si>
   <si>
     <t>Bài nói (PO) — ghi âm và nghe lại</t>
@@ -923,10 +932,10 @@
     <t>Giới hạn lượt thi + cảnh báo</t>
   </si>
   <si>
-    <t>2 lượt thi/ngày (giờ VN, đếm ở máy chủ). Hộp cảnh báo « mô phỏng phòng thi DELF thật » trước khi vào; thoát giữa chừng (nút Thoát, Back, đóng tab) có cảnh báo và mất lượt</t>
-  </si>
-  <si>
-    <t>migration 120 (luot_thi); thử claim giả: lượt 3 → HET_LUOT</t>
+    <t>2 lượt thi/ngày (giờ VN, đếm ở máy chủ), VIP không giới hạn. Cảnh báo trước khi vào thi và khi thoát; cảnh báo còn câu chưa làm trước khi nộp từng phần; thanh chuyển bài trong phần (số câu đã làm, bài trước/tiếp)</t>
+  </si>
+  <si>
+    <t>migration 120, 121, 124; claim giả: học sinh thường lượt 3 → HET_LUOT, VIP lượt 3 → được</t>
   </si>
   <si>
     <t>Dạng câu riêng của DELF (ghép cặp, phiếu, chọn hình)</t>
@@ -959,13 +968,13 @@
     <t>Không thấy nêu giá gói</t>
   </si>
   <si>
-    <t>99.000 đ / 30 ngày, mở mọi bài trả phí và đề thi; thanh toán SePay tự kích hoạt, gia hạn nối tiếp không mất ngày</t>
+    <t>99.000 đ / 30 ngày: mở mọi bài trả phí và đề thi, KHÔNG GIỚI HẠN lượt thi thử và lượt AI (gợi ý chấm viết, nhận xét bài nói), huy hiệu vương miện trên ảnh đại diện. SePay tự kích hoạt, gia hạn nối tiếp</t>
   </si>
   <si>
     <t>Đang chạy — chưa thử chuyển khoản thật</t>
   </si>
   <si>
-    <t>migration 118; sepay-webhook mã VIP1TH</t>
+    <t>migration 118, 122, 124; AvatarMenu.jsx (RPC toi_la_vip)</t>
   </si>
   <si>
     <t>TÀI KHOẢN GIÁO VIÊN — giữ để KIỂM SOÁT, không để CHẤM BÀI</t>
@@ -1444,16 +1453,16 @@
     <t>Công sức</t>
   </si>
   <si>
-    <t>Quyết định số phận 5 tài khoản không có hồ sơ</t>
-  </si>
-  <si>
-    <t>Đăng nhập được nhưng không có dòng profiles (không vai, không tên), nên vào app sẽ hỏng. Hai tài khoản vẫn đăng nhập ngày 27/09. Xoá hay tạo hồ sơ là việc xoá/sửa dữ liệu người dùng — cần chủ dự án quyết.</t>
-  </si>
-  <si>
-    <t>auth.users trái join profiles; tạo hồ sơ hoặc xoá tài khoản</t>
-  </si>
-  <si>
-    <t>10 phút</t>
+    <t>Mở trang Kết quả thi để AI chấm phần viết bài thi A1</t>
+  </si>
+  <si>
+    <t>Chế độ AI chấm chính thức vừa bật 08/10, chưa có bài nào đi hết đường qua giao diện.</t>
+  </si>
+  <si>
+    <t>Thi thử → « Kết quả thi của tôi »</t>
+  </si>
+  <si>
+    <t>2 phút</t>
   </si>
   <si>
     <t>Thử một lần chuyển khoản VIP thật</t>
@@ -2110,7 +2119,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2730,8 +2739,21 @@
       <c r="F47" s="18"/>
       <c r="G47" s="18"/>
     </row>
+    <row r="48" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2753,6 +2775,7 @@
     <mergeCell ref="B45:G45"/>
     <mergeCell ref="B46:G46"/>
     <mergeCell ref="B47:G47"/>
+    <mergeCell ref="B48:G48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2780,28 +2803,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2809,16 +2832,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2828,10 +2851,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2839,14 +2862,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2856,10 +2879,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2867,16 +2890,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F4" s="22">
         <v>2</v>
@@ -2886,10 +2909,10 @@
         <v>hoà</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2897,16 +2920,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2916,10 +2939,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2927,16 +2950,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D6" s="22">
         <v>2</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F6" s="22">
         <v>1</v>
@@ -2946,10 +2969,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2957,16 +2980,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2976,10 +2999,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2987,14 +3010,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -3004,10 +3027,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3015,7 +3038,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -3024,7 +3047,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -3034,10 +3057,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3045,16 +3068,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F10" s="22">
         <v>2</v>
@@ -3064,10 +3087,10 @@
         <v>hoà</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3075,14 +3098,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -3092,10 +3115,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3103,14 +3126,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="27" t="s">
         <v>122</v>
-      </c>
-      <c r="C12" s="27" t="s">
-        <v>119</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -3120,10 +3143,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3131,14 +3154,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -3148,10 +3171,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3159,14 +3182,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -3176,10 +3199,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3187,14 +3210,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -3204,10 +3227,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3215,16 +3238,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -3234,10 +3257,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3245,16 +3268,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F17" s="22">
         <v>2</v>
@@ -3264,10 +3287,10 @@
         <v>hoà</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3275,14 +3298,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3292,10 +3315,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3303,16 +3326,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D19" s="22">
         <v>2</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F19" s="22">
         <v>1</v>
@@ -3322,10 +3345,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3333,16 +3356,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3352,10 +3375,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3363,16 +3386,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3382,10 +3405,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3393,14 +3416,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3410,10 +3433,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3421,16 +3444,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3440,10 +3463,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3451,14 +3474,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3468,10 +3491,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3479,14 +3502,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3496,10 +3519,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3507,16 +3530,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3526,10 +3549,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3537,14 +3560,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3554,10 +3577,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3565,16 +3588,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D28" s="22">
         <v>2</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F28" s="22">
         <v>2</v>
@@ -3584,10 +3607,10 @@
         <v>hoà</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3595,16 +3618,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F29" s="22">
         <v>2</v>
@@ -3614,10 +3637,10 @@
         <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3625,16 +3648,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F30" s="22">
         <v>2</v>
@@ -3644,10 +3667,10 @@
         <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3655,14 +3678,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3672,10 +3695,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3683,16 +3706,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D32" s="22">
         <v>2</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3702,10 +3725,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3713,14 +3736,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3730,10 +3753,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3741,14 +3764,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3758,10 +3781,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3769,14 +3792,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3786,10 +3809,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3797,14 +3820,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3814,10 +3837,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3825,14 +3848,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3842,10 +3865,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3853,16 +3876,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F38" s="22">
         <v>2</v>
@@ -3872,10 +3895,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3883,16 +3906,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3902,10 +3925,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3913,16 +3936,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3932,10 +3955,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3943,16 +3966,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3962,10 +3985,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3973,16 +3996,16 @@
         <v>15</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -3992,10 +4015,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4003,14 +4026,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -4020,10 +4043,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4031,14 +4054,14 @@
         <v>15</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D44" s="34"/>
       <c r="E44" s="33" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -4048,10 +4071,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4059,14 +4082,14 @@
         <v>15</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -4076,10 +4099,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4087,14 +4110,14 @@
         <v>15</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D46" s="28"/>
       <c r="E46" s="27" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="F46" s="28">
         <v>2</v>
@@ -4104,10 +4127,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H46" s="25" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4115,16 +4138,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F47" s="22">
         <v>2</v>
@@ -4134,10 +4157,10 @@
         <v>hoà</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4145,16 +4168,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C48" s="21" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D48" s="22">
         <v>2</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F48" s="22">
         <v>1</v>
@@ -4164,10 +4187,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="I48" s="24" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4175,16 +4198,16 @@
         <v>16</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -4194,10 +4217,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4205,16 +4228,16 @@
         <v>16</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -4224,10 +4247,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4235,16 +4258,16 @@
         <v>16</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D51" s="28">
         <v>1</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -4254,10 +4277,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,14 +4288,14 @@
         <v>16</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C52" s="27" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D52" s="28"/>
       <c r="E52" s="27" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F52" s="28">
         <v>2</v>
@@ -4282,10 +4305,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H52" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4293,16 +4316,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F53" s="22">
         <v>2</v>
@@ -4312,10 +4335,10 @@
         <v>hoà</v>
       </c>
       <c r="H53" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I53" s="24" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,16 +4346,16 @@
         <v>17</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D54" s="22">
         <v>2</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F54" s="22">
         <v>1</v>
@@ -4342,10 +4365,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4356,13 +4379,13 @@
         <v>37</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D55" s="22">
         <v>2</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F55" s="22">
         <v>1</v>
@@ -4372,10 +4395,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="I55" s="24" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="56" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4383,16 +4406,16 @@
         <v>17</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C56" s="21" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D56" s="22">
         <v>2</v>
       </c>
       <c r="E56" s="21" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F56" s="22">
         <v>1</v>
@@ -4402,10 +4425,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H56" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I56" s="24" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="57" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4413,16 +4436,16 @@
         <v>17</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D57" s="28">
         <v>1</v>
       </c>
       <c r="E57" s="27" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="F57" s="28">
         <v>2</v>
@@ -4432,10 +4455,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H57" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="58" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4443,14 +4466,14 @@
         <v>17</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D58" s="28"/>
       <c r="E58" s="27" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F58" s="28">
         <v>2</v>
@@ -4460,10 +4483,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H58" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="59" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4471,14 +4494,14 @@
         <v>12</v>
       </c>
       <c r="B59" s="26" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D59" s="28"/>
       <c r="E59" s="27" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F59" s="28">
         <v>2</v>
@@ -4488,10 +4511,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H59" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I59" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="60" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4499,14 +4522,14 @@
         <v>13</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C60" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D60" s="28"/>
       <c r="E60" s="27" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F60" s="28">
         <v>2</v>
@@ -4516,10 +4539,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H60" s="25" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="61" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4527,14 +4550,14 @@
         <v>15</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C61" s="27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D61" s="28"/>
       <c r="E61" s="27" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F61" s="28">
         <v>2</v>
@@ -4544,10 +4567,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H61" s="25" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="62" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,14 +4578,14 @@
         <v>14</v>
       </c>
       <c r="B62" s="26" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C62" s="27" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="D62" s="28"/>
       <c r="E62" s="27" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F62" s="28">
         <v>2</v>
@@ -4572,10 +4595,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H62" s="25" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>
@@ -4599,12 +4622,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4620,369 +4643,369 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B8" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>326</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>323</v>
-      </c>
       <c r="D8" s="21" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5033,428 +5056,428 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B4" s="40">
         <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B5" s="40">
         <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B6" s="40">
         <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B8" s="40">
         <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B9" s="40">
         <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B14" s="40">
         <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B16" s="40">
         <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B20" s="40">
         <v>2</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B21" s="40">
         <v>2</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B22" s="40">
         <v>7</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B24" s="43">
         <f>B6/B5</f>
         <v>0.7990919409761634</v>
       </c>
       <c r="C24" s="44" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B25" s="45">
         <f>B5-B6</f>
         <v>177</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="C31" s="21" t="s">
+        <v>449</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>446</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="C32" s="21" t="s">
+        <v>449</v>
+      </c>
+      <c r="D32" s="21" t="s">
         <v>446</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B33" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>449</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="D33" s="21" t="s">
         <v>446</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="C34" s="47" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="D34" s="47" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="C35" s="47" t="s">
+        <v>459</v>
+      </c>
+      <c r="D35" s="47" t="s">
         <v>456</v>
-      </c>
-      <c r="D35" s="47" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
     </row>
   </sheetData>
@@ -5477,24 +5500,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5502,16 +5525,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5519,16 +5542,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5536,16 +5559,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5553,16 +5576,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5570,16 +5593,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: ba ngôn ngữ, AI chấm mới, nghe kiểu thi mọi đề, gỡ từ điển
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="493">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -252,6 +252,12 @@
     <t>AI tự chấm phần viết bài thi thử (thay « giáo viên đang chấm »); thanh chuyển bài + cảnh báo câu chưa làm trong thi thử; VIP không giới hạn lượt thi và lượt AI, có huy hiệu trên ảnh đại diện; xoá 5 tài khoản không có hồ sơ (đã sao lưu); xuất bản 62 bài nháp + 7 đề.</t>
   </si>
   <si>
+    <t>08/10 tối</t>
+  </si>
+  <si>
+    <t>Ba ngôn ngữ làm lại (~650 chuỗi, ~40 màn); FAQ/Điều khoản/Bảo mật viết lại ba thứ tiếng; AI chấm viết làm lại (phiếu nhận xét theo grille + mốc điểm DELF, 3 lượt/ngày, VIP không giới hạn); nghe kiểu phòng thi cho MỌI đề; bài nghe 5 cho đề A1 theo đề mẫu chính thức; gỡ Từ điển; ô tick chuỗi ngày màu cam.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -317,13 +323,13 @@
     <t>AI chấm ngữ pháp và cách diễn đạt</t>
   </si>
   <si>
-    <t>Thi thử: AI TỰ CHẤM phần viết ngay khi mở trang Kết quả thi (thang DELF đúng trình độ, phiếu A1 gộp vào), điểm AI là điểm phần viết, kèm nhận xét từng tiêu chí. Luyện tập: học sinh tự chấm, xin gợi ý AI (6 lượt/24 giờ, VIP không giới hạn)</t>
-  </si>
-  <si>
-    <t>Đang chạy — chưa có bài thi nào chấm đầu-cuối qua giao diện</t>
-  </si>
-  <si>
-    <t>Edge Function cham-pe chế độ chinhThuc (08/10): ghi answers.score + feedback, chỉ câu chưa có điểm; AI thiếu tiêu chí thì không ghi. FAQ + /bao-mat đã sửa: phần viết thi thử gửi AI tự động</t>
+    <t>Làm lại 08/10: AI đóng vai giám khảo DELF, chấm theo grille + MỐC ĐIỂM của đúng trình độ; phiếu nhận xét có cấu trúc (điểm từng tiêu chí, điểm mạnh, cần cải thiện, trích dẫn, 3 ưu tiên sửa, câu viết lại). Thi thử: AI tự chấm khi mở Kết quả thi. 3 lượt AI/ngày (giờ VN), VIP không giới hạn</t>
+  </si>
+  <si>
+    <t>Đang chạy — phiếu kiểu mới chưa chạy đầu-cuối với AI thật</t>
+  </si>
+  <si>
+    <t>cham-pe (chinhThuc + prompt mới), _shared/goiYPE.js mở rộng, NhanXetAI.jsx; check:champe 38 ca</t>
   </si>
   <si>
     <t>Bài nói (PO) — ghi âm và nghe lại</t>
@@ -410,10 +416,10 @@
     <t>Không thấy nêu</t>
   </si>
   <si>
-    <t>Đếm ở MÁY CHỦ. Từ 07/10 có « nghe kiểu phòng thi »: file chứa sẵn 30 s đọc câu hỏi → lượt 1 → nghỉ 30 s → lượt 2 → 30 s hoàn thành, phát MỘT lần. Sửa lỗi bài 2 trở đi báo hết lượt và lỗi buổi thi mới nhận lượt nghe cũ</t>
-  </si>
-  <si>
-    <t>migration 024, 119, 121; ExamMode AudioGioiHan (key theo bài). Đo bằng silencedetect: 3 khoảng 30 s đúng chỗ</t>
+    <t>Đếm ở MÁY CHỦ. Từ 08/10 MỌI đề thi thử (21 bài nghe) dùng « nghe kiểu phòng thi »: 30 s đọc câu hỏi, lượt 1, nghỉ 30 s, lượt 2, 30 s hoàn thành, phát một lần; luyện tập vẫn phát file gốc</t>
+  </si>
+  <si>
+    <t>migration 119, 121; lô 11 + 13; meta.audioLuyen giữ file gốc; đo silencedetect 3 khoảng 30 s</t>
   </si>
   <si>
     <t>Đồng hồ chạy tiếp khi đóng tab</t>
@@ -497,10 +503,10 @@
     <t>56.000+ từ · IPA · nghĩa Việt · cấp CEFR · chia động từ · tra ngay trong bài</t>
   </si>
   <si>
-    <t>Có từ 29/09 (/etudiant/tu-dien): 131 mục Pháp–Việt lấy từ flashcard giáo viên công khai, tra hai chiều, không cần gõ dấu, kèm câu ví dụ. Nhỏ hơn Vivoire hàng trăm lần — không IPA, không chia động từ</t>
-  </si>
-  <si>
-    <t>TuDien.jsx; nguồn duy nhất là the_bo_the, không nhúng từ điển ngoài hay AI. Claim giả học sinh đọc được 131 thẻ</t>
+    <t>ĐÃ GỠ 08/10 theo chủ dự án: chỉ tra lại ~130 thẻ Flashcard công khai, trùng với mục Flashcard</t>
+  </si>
+  <si>
+    <t>Lấy lại TuDien.jsx từ git trước commit a2d5176</t>
   </si>
   <si>
     <t>Podcast / học theo video</t>
@@ -854,10 +860,13 @@
     <t>Việt (giao diện) + Pháp (nội dung)</t>
   </si>
   <si>
-    <t>Việt · Pháp · Anh</t>
-  </si>
-  <si>
-    <t>shared/i18n.jsx; check:nav 74 ca. 26/09: form soạn bài (60 chuỗi), chuông thông báo, theo dõi luyện tập đã dịch — còn một số màn giáo viên cũ viết cứng tiếng Pháp</t>
+    <t>Việt · Pháp · Anh, LÀM LẠI 08/10: ~650 chuỗi viết cứng trong ~40 màn (thi thử, chấm bài, luyện tập, giáo viên, trang giới thiệu, pháp lý) đưa qua bộ dịch, không còn lẫn ngôn ngữ. Nội dung học (đề tiếng Pháp) giữ nguyên</t>
+  </si>
+  <si>
+    <t>Đang chạy — còn nút định dạng trong trình soạn của giáo viên</t>
+  </si>
+  <si>
+    <t>Hàm tr(vi, fr, en) trong shared/i18n.jsx; công cụ scripts/i18n/trich.cjs + ap.cjs; quy tắc 6b trong CLAUDE.md. Xem trước ở /preview.html bằng fr/en</t>
   </si>
   <si>
     <t>Thanh toán</t>
@@ -872,7 +881,7 @@
     <t>Câu hỏi thường gặp (FAQ)</t>
   </si>
   <si>
-    <t>15 câu (cập nhật 26/09): XP, chuỗi ngày, theo dõi bạn học, mở bài bằng XP, quên mật khẩu, liên hệ. Mỗi câu đối chiếu mã nguồn; câu AI chấm ghi rõ « chưa bật ». Có email liên hệ</t>
+    <t>16 câu, ĐỦ BA THỨ TIẾNG (08/10), cập nhật theo hiện trạng: AI chấm, nghe kiểu phòng thi, lượt thi/ngày, VIP, trạng thái online. Có email liên hệ</t>
   </si>
   <si>
     <t>/faq; contact.fracile@gmail.com</t>
@@ -881,7 +890,7 @@
     <t>Điều khoản sử dụng</t>
   </si>
   <si>
-    <t>Có từ 21/09 — ghi rõ điểm thi thử không phải điểm DELF chính thức; không tự đặt chính sách hoàn tiền</t>
+    <t>Đủ ba thứ tiếng (08/10); ghi rõ điểm thi thử và điểm AI không phải điểm DELF chính thức, thanh toán chuyển khoản + VIP</t>
   </si>
   <si>
     <t>Có — bản nháp, chưa qua luật sư</t>
@@ -890,10 +899,10 @@
     <t>/dieu-khoan</t>
   </si>
   <si>
-    <t>Có từ 25/09 (/bao-mat) — có mục riêng cho dữ liệu form « Gửi câu hỏi »; gỡ 21/09 rồi dựng lại</t>
-  </si>
-  <si>
-    <t>Điểm 0 → 1. Chưa lên 2 vì chưa qua luật sư, giống Điều khoản</t>
+    <t>Đủ ba thứ tiếng (08/10); ghi việc gửi bài viết thi thử cho AI tự động, thời điểm online, Google Sheets, SePay</t>
+  </si>
+  <si>
+    <t>/bao-mat</t>
   </si>
   <si>
     <t>Đội ngũ công khai</t>
@@ -2119,7 +2128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2247,11 +2256,11 @@
       </c>
       <c r="E9" s="6">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F9" s="6">
         <f>IFERROR(E9-D9,"")</f>
-        <v>-1</v>
+        <v>-1.2</v>
       </c>
       <c r="G9" s="7" t="str">
         <f>IF(OR(C9&lt;3,F9=""),"quá ít mục",IF(F9&gt;0.25,"FRACILE",IF(F9&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2392,11 +2401,11 @@
       </c>
       <c r="E14" s="10">
         <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>1.393939393939394</v>
+        <v>1.3636363636363635</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.48484848484848486</v>
+        <v>-0.5151515151515154</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2752,8 +2761,21 @@
       <c r="F48" s="18"/>
       <c r="G48" s="18"/>
     </row>
+    <row r="49" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2776,6 +2798,7 @@
     <mergeCell ref="B46:G46"/>
     <mergeCell ref="B47:G47"/>
     <mergeCell ref="B48:G48"/>
+    <mergeCell ref="B49:G49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2803,28 +2826,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2832,16 +2855,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2851,10 +2874,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2862,14 +2885,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2879,10 +2902,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2890,16 +2913,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F4" s="22">
         <v>2</v>
@@ -2909,10 +2932,10 @@
         <v>hoà</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2920,16 +2943,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2939,10 +2962,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2950,16 +2973,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D6" s="22">
         <v>2</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F6" s="22">
         <v>1</v>
@@ -2969,10 +2992,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2980,16 +3003,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -2999,10 +3022,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3010,14 +3033,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -3027,10 +3050,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3038,7 +3061,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -3047,7 +3070,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -3057,10 +3080,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3068,16 +3091,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F10" s="22">
         <v>2</v>
@@ -3087,10 +3110,10 @@
         <v>hoà</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3098,14 +3121,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -3115,10 +3138,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3126,14 +3149,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -3143,10 +3166,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3154,14 +3177,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -3171,10 +3194,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3182,14 +3205,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -3199,10 +3222,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3210,14 +3233,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -3227,10 +3250,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3238,16 +3261,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -3257,10 +3280,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3268,16 +3291,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F17" s="22">
         <v>2</v>
@@ -3287,10 +3310,10 @@
         <v>hoà</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3298,14 +3321,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3315,40 +3338,40 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>151</v>
-      </c>
-      <c r="D19" s="22">
-        <v>2</v>
-      </c>
-      <c r="E19" s="21" t="s">
+      <c r="B19" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="F19" s="22">
-        <v>1</v>
-      </c>
-      <c r="G19" s="23" t="str">
+      <c r="C19" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="D19" s="34">
+        <v>2</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="F19" s="34">
+        <v>0</v>
+      </c>
+      <c r="G19" s="35" t="str">
         <f>IF(OR(D19="",F19=""),"chưa rõ",IF(F19&gt;D19,"FRACILE",IF(D19&gt;F19,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H19" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>153</v>
+      <c r="H19" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="I19" s="36" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3356,16 +3379,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3375,10 +3398,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3386,16 +3409,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3405,10 +3428,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3416,14 +3439,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3433,10 +3456,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3444,16 +3467,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3463,10 +3486,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3474,14 +3497,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3491,10 +3514,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3502,14 +3525,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3519,10 +3542,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3530,16 +3553,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3549,10 +3572,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3560,14 +3583,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3577,10 +3600,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3588,16 +3611,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D28" s="22">
         <v>2</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F28" s="22">
         <v>2</v>
@@ -3607,10 +3630,10 @@
         <v>hoà</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3618,16 +3641,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F29" s="22">
         <v>2</v>
@@ -3637,10 +3660,10 @@
         <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3648,16 +3671,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F30" s="22">
         <v>2</v>
@@ -3667,10 +3690,10 @@
         <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3678,14 +3701,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3695,10 +3718,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3706,16 +3729,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D32" s="22">
         <v>2</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3725,10 +3748,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3736,14 +3759,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3753,10 +3776,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3764,14 +3787,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3781,10 +3804,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3792,14 +3815,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3809,10 +3832,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3820,14 +3843,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3837,10 +3860,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3848,14 +3871,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3865,10 +3888,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3876,16 +3899,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F38" s="22">
         <v>2</v>
@@ -3895,10 +3918,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3906,16 +3929,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3925,10 +3948,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3936,16 +3959,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3955,10 +3978,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3966,16 +3989,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -3985,10 +4008,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3996,16 +4019,16 @@
         <v>15</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -4015,10 +4038,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4026,14 +4049,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -4043,10 +4066,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4054,14 +4077,14 @@
         <v>15</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D44" s="34"/>
       <c r="E44" s="33" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -4071,10 +4094,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4082,14 +4105,14 @@
         <v>15</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -4099,10 +4122,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4110,14 +4133,14 @@
         <v>15</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D46" s="28"/>
       <c r="E46" s="27" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F46" s="28">
         <v>2</v>
@@ -4127,10 +4150,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H46" s="25" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4138,16 +4161,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F47" s="22">
         <v>2</v>
@@ -4157,10 +4180,10 @@
         <v>hoà</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4168,16 +4191,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C48" s="21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D48" s="22">
         <v>2</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F48" s="22">
         <v>1</v>
@@ -4187,10 +4210,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="I48" s="24" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4198,16 +4221,16 @@
         <v>16</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -4217,10 +4240,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4228,16 +4251,16 @@
         <v>16</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -4247,10 +4270,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4258,16 +4281,16 @@
         <v>16</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D51" s="28">
         <v>1</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -4277,10 +4300,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>84</v>
+        <v>274</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4288,14 +4311,14 @@
         <v>16</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C52" s="27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D52" s="28"/>
       <c r="E52" s="27" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F52" s="28">
         <v>2</v>
@@ -4305,10 +4328,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H52" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4316,16 +4339,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F53" s="22">
         <v>2</v>
@@ -4335,10 +4358,10 @@
         <v>hoà</v>
       </c>
       <c r="H53" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I53" s="24" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4346,16 +4369,16 @@
         <v>17</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D54" s="22">
         <v>2</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F54" s="22">
         <v>1</v>
@@ -4365,10 +4388,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4379,13 +4402,13 @@
         <v>37</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D55" s="22">
         <v>2</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F55" s="22">
         <v>1</v>
@@ -4395,10 +4418,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="I55" s="24" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="56" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4406,16 +4429,16 @@
         <v>17</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C56" s="21" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D56" s="22">
         <v>2</v>
       </c>
       <c r="E56" s="21" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F56" s="22">
         <v>1</v>
@@ -4425,10 +4448,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H56" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I56" s="24" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="57" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4436,16 +4459,16 @@
         <v>17</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="D57" s="28">
         <v>1</v>
       </c>
       <c r="E57" s="27" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F57" s="28">
         <v>2</v>
@@ -4455,10 +4478,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H57" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="58" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4466,14 +4489,14 @@
         <v>17</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D58" s="28"/>
       <c r="E58" s="27" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F58" s="28">
         <v>2</v>
@@ -4483,10 +4506,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H58" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="59" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4494,14 +4517,14 @@
         <v>12</v>
       </c>
       <c r="B59" s="26" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D59" s="28"/>
       <c r="E59" s="27" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F59" s="28">
         <v>2</v>
@@ -4511,10 +4534,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H59" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I59" s="30" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="60" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4522,14 +4545,14 @@
         <v>13</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C60" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D60" s="28"/>
       <c r="E60" s="27" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="F60" s="28">
         <v>2</v>
@@ -4539,10 +4562,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H60" s="25" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="61" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4550,14 +4573,14 @@
         <v>15</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C61" s="27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D61" s="28"/>
       <c r="E61" s="27" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="F61" s="28">
         <v>2</v>
@@ -4567,10 +4590,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H61" s="25" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="62" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4578,14 +4601,14 @@
         <v>14</v>
       </c>
       <c r="B62" s="26" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C62" s="27" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D62" s="28"/>
       <c r="E62" s="27" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="F62" s="28">
         <v>2</v>
@@ -4595,10 +4618,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H62" s="25" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -4622,12 +4645,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4643,369 +4666,369 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B8" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>329</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>326</v>
-      </c>
       <c r="D8" s="21" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5056,428 +5079,428 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B4" s="40">
         <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B5" s="40">
         <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B6" s="40">
         <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B8" s="40">
         <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B9" s="40">
         <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B14" s="40">
         <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B16" s="40">
         <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B20" s="40">
         <v>2</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B21" s="40">
         <v>2</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B22" s="40">
         <v>7</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B24" s="43">
         <f>B6/B5</f>
         <v>0.7990919409761634</v>
       </c>
       <c r="C24" s="44" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B25" s="45">
         <f>B5-B6</f>
         <v>177</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="C31" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>449</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="C32" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="D32" s="21" t="s">
         <v>449</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B33" s="21" t="s">
+        <v>455</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>452</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="D33" s="21" t="s">
         <v>449</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="C34" s="47" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="D34" s="47" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C35" s="47" t="s">
+        <v>462</v>
+      </c>
+      <c r="D35" s="47" t="s">
         <v>459</v>
-      </c>
-      <c r="D35" s="47" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
   </sheetData>
@@ -5500,24 +5523,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5525,16 +5548,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5542,16 +5565,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5559,16 +5582,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5576,16 +5599,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5593,16 +5616,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật bảng so sánh Vivoire–FRACILE tới 10/10 (Thách đấu theo chủ đề, Flashcard trả phí + mua chuyển khoản, giao diện mới, Leon, Hỏi Leon, tài liệu 111 bài, chính sách bảo mật rút gọn)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="497">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -258,6 +258,12 @@
     <t>Ba ngôn ngữ làm lại (~650 chuỗi, ~40 màn); FAQ/Điều khoản/Bảo mật viết lại ba thứ tiếng; AI chấm viết làm lại (phiếu nhận xét theo grille + mốc điểm DELF, 3 lượt/ngày, VIP không giới hạn); nghe kiểu phòng thi cho MỌI đề; bài nghe 5 cho đề A1 theo đề mẫu chính thức; gỡ Từ điển; ô tick chuỗi ngày màu cam.</t>
   </si>
   <si>
+    <t>09–10/10</t>
+  </si>
+  <si>
+    <t>Linh vật Leon (logo, favicon, 24 sticker, có mặt ở mọi thẻ, phần hướng dẫn, trang đăng nhập); trợ lý « Hỏi Leon » (AI hỏi đáp tiếng Pháp, 10 câu/ngày, VIP không giới hạn); trang giới thiệu làm lại; giao diện mới cho Lộ trình, Thách đấu, Flashcard, Thi thử, Kết quả thi, Bài tập được giao; hiệu ứng âm thanh (có nút tắt); Thách đấu theo chủ đề 10 câu; Flashcard trả phí, cấp quyền, mua bằng chuyển khoản; tài liệu Từ vựng + Giải thích cho 111 bài; sửa lỗi nhiều lúc không cuộn được trang.</t>
+  </si>
+  <si>
     <t>Số liệu trôi</t>
   </si>
   <si>
@@ -380,10 +386,13 @@
     <t>Không thấy nêu trên trang chủ</t>
   </si>
   <si>
-    <t>704/881 câu có lời giải (đo 08/10). Màn « Câu cần lời giải » của giáo viên đã gỡ 07/10: AI chấm và giải thích thay</t>
-  </si>
-  <si>
-    <t>select count(*) from questions where explanation is not null = 704</t>
+    <t>704/881 câu có lời giải. Thêm 09/10: đủ 111/111 bài luyện tập có « Từ vựng » + « Giải thích » (AI soạn, không lộ đáp án, không dấu gạch dài); « Đề và đáp án » mở cho học sinh SAU khi đã nộp bài</t>
+  </si>
+  <si>
+    <t>Đang chạy — nội dung AI soạn, giáo viên sửa được</t>
+  </si>
+  <si>
+    <t>Edge Function soan-tai-lieu; migration 126 (corrige_bai)</t>
   </si>
   <si>
     <t>Neo đáp án vào ngữ liệu (chỉ ra CHỖ chứa câu trả lời)</t>
@@ -404,10 +413,10 @@
     <t>DELF/DALF A1–C2</t>
   </si>
   <si>
-    <t>7 đề, CẢ 7 ĐÃ PHÁT HÀNH (08/10): DELF A1 · A2 (2 đề) · B1 (2 đề) · B2 · DALF C1, đủ 4 phần theo format 2; học sinh chọn đề theo tab trình độ. Cấu trúc từng phần ghi ở docs/format-de-thi-DELF-A1-B2.xlsx</t>
-  </si>
-  <si>
-    <t>select count(*) from exams where is_published = 7, đo 08/10. Lô lo4, lo6, lo9, lo10, lo11</t>
+    <t>7 đề đã phát hành (A1 · A2 ×2 · B1 ×2 · B2 · C1), đủ 4 phần. Màn chọn đề và màn kết quả làm lại 09/10 (thẻ trình độ, cấu trúc 4 phần có biểu tượng, vòng điểm, vạch ngưỡng 5/25), âm thanh nhắc còn 5 phút / 1 phút / hết giờ. Sửa lỗi đổi tab hiện « chưa có bài »</t>
+  </si>
+  <si>
+    <t>ExamMode.jsx, ExamResults.jsx, exam/KetQuaVisual.jsx; check:exam 114 ca</t>
   </si>
   <si>
     <t>Nghe hiểu giới hạn 2 lượt phát</t>
@@ -551,13 +560,13 @@
     <t>Flashcard + 3 game mỗi ngày, « ôn từ đúng lúc sắp quên »</t>
   </si>
   <si>
-    <t>Bộ do GIÁO VIÊN soạn, chia theo kỹ năng, thẻ lật 3D, CÓ lịch ôn SM-2 từ 21/09 (chỉ hiện thẻ đến hạn, bốn mức nhớ). Từ 28/09 có game Lộ trình dựng từ chính các bộ này</t>
-  </si>
-  <si>
-    <t>Đang chạy — lưu thật 22/09</t>
-  </si>
-  <si>
-    <t>migration 085–091; tài khoản thật bấm Tốt → 2 thẻ reps=1, hẹn 23/09. Mỗi lần chấm có biên nhận, hỏng thì hiện chữ đỏ</t>
+    <t>Bộ do GIÁO VIÊN soạn, lịch ôn SM-2, thẻ lật 3D. Giao diện làm lại 09/10: Leon phản ứng theo lần chấm, nút chấm có phím 1–4, phím cách để lật, âm thanh. Từ 10/10 có BỘ TRẢ PHÍ: học sinh thấy ổ khoá + giá, mua bằng chuyển khoản (tự mở khoá khi tiền về), VIP mở hết</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa có giao dịch mua bộ thật</t>
+  </si>
+  <si>
+    <t>LuyenBoThe.jsx, BoTheApp.jsx; migration 128 (co_quyen_bo, RLS thẻ theo quyền), 130 (mua_bo_the); webhook SePay nhận mã BO&lt;4 ký tự&gt;</t>
   </si>
   <si>
     <t>Flashcard — quy mô</t>
@@ -614,13 +623,13 @@
     <t>Đấu dịch thuật PvP trực tiếp</t>
   </si>
   <si>
-    <t>Game Lộ trình (28/09) + Thách đấu bạn bè (30/09): hai người làm cùng một đề 8 câu, máy chủ phát đề, bấm giờ và chấm; đúng nhiều hơn thắng, hoà thì ai nhanh hơn. Không theo thời gian thực. Đã chạy thật: Lộ trình có người chơi (30/09) và trận thách đấu đầu tiên giữa hai tài khoản thật đã đấu xong (30/09, hoà 2/8 – 2/8 xét giờ). Vẫn kém Vivoire ở chỗ không đấu theo thời gian thực</t>
-  </si>
-  <si>
-    <t>Đang chạy — 9 trận thách đấu thật (06/10)</t>
-  </si>
-  <si>
-    <t>ThachDau.jsx; migration 111. Thử trên DB thật rồi huỷ: chưa theo dõi thì bị chặn, nộp hai lần bị chặn, người ngoài không đọc được đề, điểm đối thủ bị giấu tới khi mình nộp</t>
+    <t>Game Lộ trình + Thách đấu bạn bè. Từ 10/10 thách đấu theo CHỦ ĐỀ (3 chủ đề từ vựng, 4 chủ đề ngữ pháp và diễn đạt): gộp thẻ mọi bộ cùng chủ đề, rút ngẫu nhiên 10 câu; phương án cùng DẠNG, ưu tiên cùng chủ đề, bỏ phần giải thích trong ngoặc; giáo viên soạn được 3 nghĩa sai cho từng thẻ. Giao diện đấu trường mới: đếm ngược 3-2-1, phím 1–4, hiệu ứng và âm thanh</t>
+  </si>
+  <si>
+    <t>Đang chạy — trận theo chủ đề chưa chơi thật trên giao diện</t>
+  </si>
+  <si>
+    <t>migration 127–129 (chu_de_the, the_bo.chu_de, the_bo_the.loai/nhieu, sach_pa). Thử trên DB: 7 chủ đề đều ra 10 câu, 0 dấu ngoặc</t>
   </si>
   <si>
     <t>XP (điểm kinh nghiệm)</t>
@@ -668,22 +677,19 @@
     <t>Lộ trình theo cấp độ</t>
   </si>
   <si>
-    <t>Bản đồ uốn lượn 4 chương (Nghe/Đọc/Viết/Nói) · 12 màn = 12 bộ flashcard · trắc nghiệm hai chiều + ghép cặp · 3 tim · 1–3 sao · thử thách cuối chương · mở khoá tuần tự. Không cộng XP (chống cày)</t>
-  </si>
-  <si>
-    <t>Đang chạy — 1 màn đã chơi thật 30/09 (2 sao, máy chủ cộng +5 XP)</t>
-  </si>
-  <si>
-    <t>migration 108/109: lo_trinh_ket_qua + RPC ghi_ket_qua_man (giữ sao cao nhất, có biên nhận)</t>
+    <t>16 chủ đề xã hội, 100 màn, 800 mục từ có loại từ; nhiễu cùng loại từ. Giao diện làm lại 09/10: khung đầu có Leon + thanh sao, đường tự vẽ, màn hiện tại có vòng sáng và Leon đứng cạnh; màn chơi có Leon phản ứng, pháo giấy, rung khi sai, âm thanh, phím 1–4</t>
+  </si>
+  <si>
+    <t>LoTrinh.jsx, TroChoiMan.jsx, shared/amThanh.js (Web Audio, không file)</t>
   </si>
   <si>
     <t>Kiểm soát ai được học bài nào</t>
   </si>
   <si>
-    <t>Ba tầng: gói VIP 99.000 đ/30 ngày (tự gia hạn qua SePay), trọn gói, từng bài. Màn cấp quyền làm lại 08/10: xem theo bài hoặc theo học sinh, cấp cho cả nhóm; giáo viên tự gia hạn/thu hồi VIP</t>
-  </si>
-  <si>
-    <t>QuyenBaiTap.jsx, QuanLyVip.jsx; migration 118, 122. vip_giao_dich = 2 dòng</t>
+    <t>Ba tầng cho bài tập (VIP 99.000 đ/30 ngày, trọn gói, từng bài) và từ 10/10 cho cả BỘ FLASHCARD: giáo viên đặt bộ trả phí + giá, cấp/thu quyền từng học sinh; học sinh tự mua bằng chuyển khoản</t>
+  </si>
+  <si>
+    <t>QuyenBaiTap.jsx, QuanLyVip.jsx, SoanBoThe.jsx; migration 118, 122, 128, 130</t>
   </si>
   <si>
     <t>Học sinh KHÔNG tự mở khoá được cho mình</t>
@@ -719,10 +725,13 @@
     <t>Soạn Flashcard</t>
   </si>
   <si>
-    <t>Có — /professeur/bo-the: tạo bộ, nhập hàng loạt, nháp ↔ công khai, xoá (thẻ đi theo)</t>
-  </si>
-  <si>
-    <t>RLS chỉ giáo viên ghi; đo bằng claim giả: HS thấy 8 thẻ, sửa 0, xoá 0</t>
+    <t>Lưới bộ lọc theo kỹ năng; thêm từng thẻ hoặc dán nhiều dòng; sửa tại chỗ. Từ 10/10: chọn chủ đề thách đấu cho bộ, dạng cho từng thẻ, 3 nghĩa sai tự soạn, bộ trả phí + giá, bảng cấp quyền học sinh</t>
+  </si>
+  <si>
+    <t>Đang chạy — giao diện mới chưa ai bấm thử</t>
+  </si>
+  <si>
+    <t>SoanBoThe.jsx, boTheGiaoVien.js</t>
   </si>
   <si>
     <t>Giao bài theo kỹ năng và cấp độ</t>
@@ -872,10 +881,13 @@
     <t>Thanh toán</t>
   </si>
   <si>
-    <t>Webhook SePay đã ghim công thức ký (ts.raw kiểu Stripe)</t>
-  </si>
-  <si>
-    <t>check:hmac 45 ca; giao dịch #76732769 xác nhận</t>
+    <t>Webhook SePay đã ghim công thức ký; mua bài lẻ, gói VIP và (từ 10/10) bộ Flashcard trả phí qua cùng một mã nội dung chuyển khoản</t>
+  </si>
+  <si>
+    <t>Đang chạy — mua bộ Flashcard chưa có giao dịch thật</t>
+  </si>
+  <si>
+    <t>check:hmac 45 ca; mua_bo_the thử trên DB: thiếu tiền bị từ chối, giao dịch gửi lại không ghi hai lần</t>
   </si>
   <si>
     <t>Câu hỏi thường gặp (FAQ)</t>
@@ -899,7 +911,7 @@
     <t>/dieu-khoan</t>
   </si>
   <si>
-    <t>Đủ ba thứ tiếng (08/10); ghi việc gửi bài viết thi thử cho AI tự động, thời điểm online, Google Sheets, SePay</t>
+    <t>Đủ ba thứ tiếng. Rút gọn 10/10 theo chủ dự án: còn Tóm tắt, Thu gì, Dùng làm gì, Quyền của bạn; nhà xử lý (Supabase, Vercel, OpenAI), nơi lưu và thời hạn gộp thành một ý trong Tóm tắt</t>
   </si>
   <si>
     <t>/bao-mat</t>
@@ -2128,7 +2140,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2774,8 +2786,21 @@
       <c r="F49" s="18"/>
       <c r="G49" s="18"/>
     </row>
+    <row r="50" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="A17:G19"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
@@ -2799,6 +2824,7 @@
     <mergeCell ref="B47:G47"/>
     <mergeCell ref="B48:G48"/>
     <mergeCell ref="B49:G49"/>
+    <mergeCell ref="B50:G50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2826,28 +2852,28 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2855,16 +2881,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D2" s="22">
         <v>2</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F2" s="22">
         <v>2</v>
@@ -2874,10 +2900,10 @@
         <v>hoà</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2885,14 +2911,14 @@
         <v>11</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3" s="28"/>
       <c r="E3" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F3" s="28">
         <v>2</v>
@@ -2902,10 +2928,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2913,16 +2939,16 @@
         <v>11</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D4" s="22">
         <v>2</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F4" s="22">
         <v>2</v>
@@ -2932,10 +2958,10 @@
         <v>hoà</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2943,16 +2969,16 @@
         <v>11</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F5" s="22">
         <v>1</v>
@@ -2962,10 +2988,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2973,16 +2999,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D6" s="22">
         <v>2</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F6" s="22">
         <v>1</v>
@@ -2992,10 +3018,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3003,16 +3029,16 @@
         <v>11</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D7" s="34">
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F7" s="34">
         <v>0</v>
@@ -3022,10 +3048,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3033,14 +3059,14 @@
         <v>11</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="27" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F8" s="28">
         <v>2</v>
@@ -3050,10 +3076,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3061,7 +3087,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>23</v>
@@ -3070,7 +3096,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F9" s="28">
         <v>2</v>
@@ -3080,10 +3106,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3091,16 +3117,16 @@
         <v>12</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D10" s="22">
         <v>2</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F10" s="22">
         <v>2</v>
@@ -3110,10 +3136,10 @@
         <v>hoà</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3121,14 +3147,14 @@
         <v>12</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D11" s="28"/>
       <c r="E11" s="27" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F11" s="28">
         <v>2</v>
@@ -3138,10 +3164,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3149,14 +3175,14 @@
         <v>12</v>
       </c>
       <c r="B12" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12" s="27" t="s">
         <v>127</v>
-      </c>
-      <c r="C12" s="27" t="s">
-        <v>124</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="27" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F12" s="28">
         <v>2</v>
@@ -3166,10 +3192,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3177,14 +3203,14 @@
         <v>12</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="27" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F13" s="28">
         <v>2</v>
@@ -3194,10 +3220,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3205,14 +3231,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D14" s="28"/>
       <c r="E14" s="27" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F14" s="28">
         <v>2</v>
@@ -3222,10 +3248,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3233,14 +3259,14 @@
         <v>12</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="27" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F15" s="28">
         <v>2</v>
@@ -3250,10 +3276,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3261,16 +3287,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D16" s="22">
         <v>2</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F16" s="22">
         <v>1</v>
@@ -3280,10 +3306,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3291,16 +3317,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D17" s="22">
         <v>2</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F17" s="22">
         <v>2</v>
@@ -3310,10 +3336,10 @@
         <v>hoà</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3321,14 +3347,14 @@
         <v>13</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="27" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F18" s="28">
         <v>2</v>
@@ -3338,10 +3364,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3349,16 +3375,16 @@
         <v>13</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D19" s="34">
         <v>2</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F19" s="34">
         <v>0</v>
@@ -3368,10 +3394,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3379,16 +3405,16 @@
         <v>13</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D20" s="34">
         <v>2</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F20" s="34">
         <v>0</v>
@@ -3398,10 +3424,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="I20" s="36" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3409,16 +3435,16 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D21" s="22">
         <v>2</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F21" s="22">
         <v>1</v>
@@ -3428,10 +3454,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3439,14 +3465,14 @@
         <v>13</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="27" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F22" s="28">
         <v>2</v>
@@ -3456,10 +3482,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3467,16 +3493,16 @@
         <v>14</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D23" s="22">
         <v>2</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F23" s="22">
         <v>2</v>
@@ -3486,10 +3512,10 @@
         <v>hoà</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3497,14 +3523,14 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="27" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F24" s="28">
         <v>2</v>
@@ -3514,10 +3540,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3525,14 +3551,14 @@
         <v>14</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="27" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F25" s="28">
         <v>2</v>
@@ -3542,10 +3568,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3553,16 +3579,16 @@
         <v>14</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D26" s="22">
         <v>2</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="F26" s="22">
         <v>2</v>
@@ -3572,10 +3598,10 @@
         <v>hoà</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3583,14 +3609,14 @@
         <v>14</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D27" s="28"/>
       <c r="E27" s="27" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F27" s="28">
         <v>2</v>
@@ -3600,10 +3626,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3611,16 +3637,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D28" s="22">
         <v>2</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F28" s="22">
         <v>2</v>
@@ -3630,10 +3656,10 @@
         <v>hoà</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3641,16 +3667,16 @@
         <v>14</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D29" s="22">
         <v>2</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F29" s="22">
         <v>2</v>
@@ -3660,10 +3686,10 @@
         <v>hoà</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3671,16 +3697,16 @@
         <v>14</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D30" s="22">
         <v>2</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F30" s="22">
         <v>2</v>
@@ -3690,10 +3716,10 @@
         <v>hoà</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3701,14 +3727,14 @@
         <v>14</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="27" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F31" s="28">
         <v>2</v>
@@ -3718,10 +3744,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3729,16 +3755,16 @@
         <v>14</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D32" s="22">
         <v>2</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F32" s="22">
         <v>2</v>
@@ -3748,10 +3774,10 @@
         <v>hoà</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>210</v>
+        <v>88</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3759,14 +3785,14 @@
         <v>15</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D33" s="28"/>
       <c r="E33" s="27" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F33" s="28">
         <v>2</v>
@@ -3776,10 +3802,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3787,14 +3813,14 @@
         <v>15</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D34" s="28"/>
       <c r="E34" s="27" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F34" s="28">
         <v>2</v>
@@ -3804,10 +3830,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3815,14 +3841,14 @@
         <v>15</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D35" s="28"/>
       <c r="E35" s="27" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F35" s="28">
         <v>2</v>
@@ -3832,10 +3858,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H35" s="25" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3843,14 +3869,14 @@
         <v>15</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="27" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F36" s="28">
         <v>2</v>
@@ -3860,10 +3886,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3871,14 +3897,14 @@
         <v>15</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D37" s="28"/>
       <c r="E37" s="27" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F37" s="28">
         <v>2</v>
@@ -3888,10 +3914,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3899,16 +3925,16 @@
         <v>15</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D38" s="22">
         <v>2</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F38" s="22">
         <v>2</v>
@@ -3918,10 +3944,10 @@
         <v>hoà</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3929,16 +3955,16 @@
         <v>15</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D39" s="22">
         <v>2</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F39" s="22">
         <v>1</v>
@@ -3948,10 +3974,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3959,16 +3985,16 @@
         <v>15</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D40" s="22">
         <v>2</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F40" s="22">
         <v>2</v>
@@ -3978,10 +4004,10 @@
         <v>hoà</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3989,16 +4015,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D41" s="34">
         <v>2</v>
       </c>
       <c r="E41" s="33" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F41" s="34">
         <v>0</v>
@@ -4008,10 +4034,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4019,16 +4045,16 @@
         <v>15</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D42" s="34">
         <v>2</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="F42" s="34">
         <v>0</v>
@@ -4038,10 +4064,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H42" s="31" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I42" s="36" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4049,14 +4075,14 @@
         <v>15</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D43" s="22"/>
       <c r="E43" s="21" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F43" s="22">
         <v>1</v>
@@ -4066,10 +4092,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4077,14 +4103,14 @@
         <v>15</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D44" s="34"/>
       <c r="E44" s="33" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F44" s="34">
         <v>0</v>
@@ -4094,10 +4120,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I44" s="36" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4105,14 +4131,14 @@
         <v>15</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D45" s="28"/>
       <c r="E45" s="27" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="F45" s="28">
         <v>2</v>
@@ -4122,10 +4148,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H45" s="25" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4133,14 +4159,14 @@
         <v>15</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D46" s="28"/>
       <c r="E46" s="27" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="F46" s="28">
         <v>2</v>
@@ -4150,10 +4176,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H46" s="25" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4161,16 +4187,16 @@
         <v>16</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D47" s="22">
         <v>2</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F47" s="22">
         <v>2</v>
@@ -4180,10 +4206,10 @@
         <v>hoà</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I47" s="24" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4191,16 +4217,16 @@
         <v>16</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C48" s="21" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D48" s="22">
         <v>2</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="F48" s="22">
         <v>1</v>
@@ -4210,10 +4236,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="I48" s="24" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4221,16 +4247,16 @@
         <v>16</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D49" s="22">
         <v>2</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F49" s="22">
         <v>1</v>
@@ -4240,10 +4266,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="I49" s="24" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4251,16 +4277,16 @@
         <v>16</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D50" s="22">
         <v>2</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="F50" s="22">
         <v>1</v>
@@ -4270,10 +4296,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4281,16 +4307,16 @@
         <v>16</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D51" s="28">
         <v>1</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="F51" s="28">
         <v>2</v>
@@ -4300,10 +4326,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H51" s="25" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="52" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4311,14 +4337,14 @@
         <v>16</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C52" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D52" s="28"/>
       <c r="E52" s="27" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F52" s="28">
         <v>2</v>
@@ -4328,10 +4354,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H52" s="25" t="s">
-        <v>86</v>
+        <v>281</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4339,16 +4365,16 @@
         <v>17</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D53" s="22">
         <v>2</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="F53" s="22">
         <v>2</v>
@@ -4358,10 +4384,10 @@
         <v>hoà</v>
       </c>
       <c r="H53" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I53" s="24" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="54" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4369,16 +4395,16 @@
         <v>17</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D54" s="22">
         <v>2</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="F54" s="22">
         <v>1</v>
@@ -4388,10 +4414,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4402,13 +4428,13 @@
         <v>37</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D55" s="22">
         <v>2</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="F55" s="22">
         <v>1</v>
@@ -4418,10 +4444,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="I55" s="24" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="56" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4429,16 +4455,16 @@
         <v>17</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C56" s="21" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D56" s="22">
         <v>2</v>
       </c>
       <c r="E56" s="21" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="F56" s="22">
         <v>1</v>
@@ -4448,10 +4474,10 @@
         <v>Vivoire</v>
       </c>
       <c r="H56" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I56" s="24" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
     </row>
     <row r="57" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4459,16 +4485,16 @@
         <v>17</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="D57" s="28">
         <v>1</v>
       </c>
       <c r="E57" s="27" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="F57" s="28">
         <v>2</v>
@@ -4478,10 +4504,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H57" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="58" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4489,14 +4515,14 @@
         <v>17</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D58" s="28"/>
       <c r="E58" s="27" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F58" s="28">
         <v>2</v>
@@ -4506,10 +4532,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H58" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
     </row>
     <row r="59" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4517,14 +4543,14 @@
         <v>12</v>
       </c>
       <c r="B59" s="26" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D59" s="28"/>
       <c r="E59" s="27" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="F59" s="28">
         <v>2</v>
@@ -4534,10 +4560,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H59" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I59" s="30" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
     <row r="60" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4545,14 +4571,14 @@
         <v>13</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C60" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D60" s="28"/>
       <c r="E60" s="27" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F60" s="28">
         <v>2</v>
@@ -4562,10 +4588,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H60" s="25" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
     <row r="61" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4573,14 +4599,14 @@
         <v>15</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="C61" s="27" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D61" s="28"/>
       <c r="E61" s="27" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="F61" s="28">
         <v>2</v>
@@ -4590,10 +4616,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H61" s="25" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="62" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4601,14 +4627,14 @@
         <v>14</v>
       </c>
       <c r="B62" s="26" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C62" s="27" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="D62" s="28"/>
       <c r="E62" s="27" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="F62" s="28">
         <v>2</v>
@@ -4618,10 +4644,10 @@
         <v>chưa rõ</v>
       </c>
       <c r="H62" s="25" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
   </sheetData>
@@ -4645,12 +4671,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4666,369 +4692,369 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5079,428 +5105,428 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B4" s="40">
         <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="B5" s="40">
         <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B6" s="40">
         <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
+        <v>407</v>
+      </c>
+      <c r="D6" s="42" t="s">
         <v>403</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B8" s="40">
         <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="B9" s="40">
         <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="B14" s="40">
         <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="B16" s="40">
         <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="B20" s="40">
         <v>2</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="B21" s="40">
         <v>2</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="B22" s="40">
         <v>7</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="B24" s="43">
         <f>B6/B5</f>
         <v>0.7990919409761634</v>
       </c>
       <c r="C24" s="44" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="B25" s="45">
         <f>B5-B6</f>
         <v>177</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
+        <v>457</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>455</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>456</v>
+      </c>
+      <c r="D32" s="21" t="s">
         <v>453</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>451</v>
-      </c>
-      <c r="C32" s="21" t="s">
-        <v>452</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="C34" s="47" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="D34" s="47" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="C35" s="47" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="D35" s="47" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -5523,24 +5549,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5548,16 +5574,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5565,16 +5591,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5582,16 +5608,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5599,16 +5625,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5616,16 +5642,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: thêm dòng « Trợ lý AI hỏi đáp » (Vivoire không có, FRACILE có Hỏi Leon)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="502">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -996,6 +996,21 @@
   </si>
   <si>
     <t>migration 118, 122, 124; AvatarMenu.jsx (RPC toi_la_vip)</t>
+  </si>
+  <si>
+    <t>Trợ lý AI hỏi đáp</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ (chủ dự án xác nhận 10/10)</t>
+  </si>
+  <si>
+    <t>« Hỏi Leon »: trợ lý AI ngay trong web, giải thích ngữ pháp và từ vựng, sửa câu tiếng Pháp, trả lời theo ngôn ngữ giao diện, nhớ 6 lượt gần nhất; không giải hộ bài đang làm; ẩn khi thi thử. 10 câu/ngày, VIP không giới hạn</t>
+  </si>
+  <si>
+    <t>Đang chạy — 11 câu hỏi thật đã được trả lời (đo 10/10)</t>
+  </si>
+  <si>
+    <t>Edge Function hoi-leon, bảng leon_hoi (migration 125), shared/HoiLeon.jsx</t>
   </si>
   <si>
     <t>TÀI KHOẢN GIÁO VIÊN — giữ để KIỂM SOÁT, không để CHẤM BÀI</t>
@@ -2197,19 +2212,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A7)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
@@ -2226,19 +2241,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A8)</f>
         <v>7</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A8)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F8" s="6">
@@ -2255,19 +2270,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A9)</f>
         <v>8</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A9)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>0.8</v>
       </c>
       <c r="F9" s="6">
@@ -2284,28 +2299,28 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A10)</f>
-        <v>11</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A10)</f>
+        <v>12</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
-        <v>6</v>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
+        <v>7</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>2</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <v>1.7142857142857142</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A10)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>0</v>
+        <v>0.2857142857142858</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
-        <v>ngang nhau</v>
+        <v>FRACILE</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2313,19 +2328,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A11)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A11)</f>
         <v>15</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A11)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F11" s="6">
@@ -2342,19 +2357,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A12)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F12" s="6">
@@ -2371,19 +2386,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$62,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$62=$A13)*('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F13" s="6">
@@ -2401,23 +2416,23 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$62)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>1.878787878787879</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <v>1.8235294117647058</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$62)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$62&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$62&lt;&gt;"")),"")</f>
-        <v>1.3636363636363635</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <v>1.3823529411764706</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.5151515151515154</v>
+        <v>-0.4411764705882353</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2833,7 +2848,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4648,6 +4663,36 @@
       </c>
       <c r="I62" s="30" t="s">
         <v>318</v>
+      </c>
+    </row>
+    <row r="63" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B63" s="26" t="s">
+        <v>319</v>
+      </c>
+      <c r="C63" s="27" t="s">
+        <v>320</v>
+      </c>
+      <c r="D63" s="28">
+        <v>0</v>
+      </c>
+      <c r="E63" s="27" t="s">
+        <v>321</v>
+      </c>
+      <c r="F63" s="28">
+        <v>2</v>
+      </c>
+      <c r="G63" s="29" t="str">
+        <f>IF(OR(D63="",F63=""),"chưa rõ",IF(F63&gt;D63,"FRACILE",IF(D63&gt;F63,"Vivoire","hoà")))</f>
+        <v>FRACILE</v>
+      </c>
+      <c r="H63" s="25" t="s">
+        <v>322</v>
+      </c>
+      <c r="I63" s="30" t="s">
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -4671,12 +4716,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4692,70 +4737,70 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4763,84 +4808,84 @@
         <v>221</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4848,213 +4893,213 @@
         <v>227</v>
       </c>
       <c r="B14" s="27" t="s">
+        <v>361</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>333</v>
+      </c>
+      <c r="D14" s="27" t="s">
         <v>356</v>
       </c>
-      <c r="C14" s="25" t="s">
-        <v>328</v>
-      </c>
-      <c r="D14" s="27" t="s">
-        <v>351</v>
-      </c>
       <c r="E14" s="27" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="D25" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5105,330 +5150,330 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="B4" s="40">
         <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="B5" s="40">
         <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="B6" s="40">
         <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="B8" s="40">
         <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="B9" s="40">
         <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B14" s="40">
         <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="B16" s="40">
         <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="B20" s="40">
         <v>2</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="B21" s="40">
         <v>2</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="B22" s="40">
         <v>7</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="B24" s="43">
         <f>B6/B5</f>
         <v>0.7990919409761634</v>
       </c>
       <c r="C24" s="44" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="B25" s="45">
         <f>B5-B6</f>
         <v>177</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -5436,97 +5481,97 @@
         <v>155</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
+        <v>463</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>464</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>461</v>
+      </c>
+      <c r="D33" s="21" t="s">
         <v>458</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>459</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>456</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="C34" s="47" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="D34" s="47" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="C35" s="47" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="D35" s="47" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
     </row>
   </sheetData>
@@ -5549,24 +5594,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5574,16 +5619,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5591,16 +5636,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5608,16 +5653,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5625,16 +5670,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5642,16 +5687,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: thêm « Linh vật đồng hành » và « Hiệu ứng âm thanh khi học » (Vivoire không có)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="509">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -998,10 +998,31 @@
     <t>migration 118, 122, 124; AvatarMenu.jsx (RPC toi_la_vip)</t>
   </si>
   <si>
+    <t>Linh vật đồng hành</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ (chủ dự án xác nhận 10/10)</t>
+  </si>
+  <si>
+    <t>Leon (bulldog Pháp áo sọc): logo, favicon, 24 sticker cảm xúc; có mặt ở mọi thẻ, phần hướng dẫn lần đầu, trang giới thiệu, đăng nhập; phản ứng theo đúng/sai trong Lộ trình, Thách đấu, Flashcard; lời động viên trong phiếu AI chấm; sticker trong nhận xét giáo viên</t>
+  </si>
+  <si>
+    <t>shared/leon.jsx, public/leon/*.webp</t>
+  </si>
+  <si>
+    <t>Hiệu ứng âm thanh khi học</t>
+  </si>
+  <si>
+    <t>Âm thanh cho Lộ trình, Thách đấu, Flashcard, Luyện tập, Thi thử (nhắc còn 5 phút, 1 phút, hết giờ) và kết quả; tổng hợp bằng Web Audio nên không tải thêm file; nút tắt/bật dùng chung, trình duyệt nhớ lựa chọn</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa nghe thử trên máy thật</t>
+  </si>
+  <si>
+    <t>shared/amThanh.js, shared/NutTieng.jsx</t>
+  </si>
+  <si>
     <t>Trợ lý AI hỏi đáp</t>
-  </si>
-  <si>
-    <t>KHÔNG CÓ (chủ dự án xác nhận 10/10)</t>
   </si>
   <si>
     <t>« Hỏi Leon »: trợ lý AI ngay trong web, giải thích ngữ pháp và từ vựng, sửa câu tiếng Pháp, trả lời theo ngôn ngữ giao diện, nhớ 6 lượt gần nhất; không giải hộ bài đang làm; ẩn khi thi thử. 10 câu/ngày, VIP không giới hạn</t>
@@ -2212,19 +2233,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A7)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
@@ -2241,19 +2262,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A8)</f>
         <v>7</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A8)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F8" s="6">
@@ -2270,19 +2291,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A9)</f>
         <v>8</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A9)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>0.8</v>
       </c>
       <c r="F9" s="6">
@@ -2299,24 +2320,24 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A10)</f>
-        <v>12</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A10)</f>
+        <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
-        <v>7</v>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
+        <v>9</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
-        <v>1.7142857142857142</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <v>1.3333333333333333</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A10)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>0.2857142857142858</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2328,19 +2349,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A11)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A11)</f>
         <v>15</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A11)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F11" s="6">
@@ -2357,19 +2378,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A12)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F12" s="6">
@@ -2386,19 +2407,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$63,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$63=$A13)*('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F13" s="6">
@@ -2416,23 +2437,23 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$63)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
-        <v>1.8235294117647058</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <v>1.7222222222222223</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$63)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$63&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$63&lt;&gt;"")),"")</f>
-        <v>1.3823529411764706</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <v>1.4166666666666667</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.4411764705882353</v>
+        <v>-0.3055555555555556</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
@@ -2848,7 +2869,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4689,10 +4710,70 @@
         <v>FRACILE</v>
       </c>
       <c r="H63" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="I63" s="30" t="s">
         <v>322</v>
       </c>
-      <c r="I63" s="30" t="s">
+    </row>
+    <row r="64" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B64" s="26" t="s">
         <v>323</v>
+      </c>
+      <c r="C64" s="27" t="s">
+        <v>320</v>
+      </c>
+      <c r="D64" s="28">
+        <v>0</v>
+      </c>
+      <c r="E64" s="27" t="s">
+        <v>324</v>
+      </c>
+      <c r="F64" s="28">
+        <v>2</v>
+      </c>
+      <c r="G64" s="29" t="str">
+        <f>IF(OR(D64="",F64=""),"chưa rõ",IF(F64&gt;D64,"FRACILE",IF(D64&gt;F64,"Vivoire","hoà")))</f>
+        <v>FRACILE</v>
+      </c>
+      <c r="H64" s="25" t="s">
+        <v>325</v>
+      </c>
+      <c r="I64" s="30" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="65" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B65" s="26" t="s">
+        <v>327</v>
+      </c>
+      <c r="C65" s="27" t="s">
+        <v>320</v>
+      </c>
+      <c r="D65" s="28">
+        <v>0</v>
+      </c>
+      <c r="E65" s="27" t="s">
+        <v>328</v>
+      </c>
+      <c r="F65" s="28">
+        <v>2</v>
+      </c>
+      <c r="G65" s="29" t="str">
+        <f>IF(OR(D65="",F65=""),"chưa rõ",IF(F65&gt;D65,"FRACILE",IF(D65&gt;F65,"Vivoire","hoà")))</f>
+        <v>FRACILE</v>
+      </c>
+      <c r="H65" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="I65" s="30" t="s">
+        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -4716,12 +4797,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4737,70 +4818,70 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4808,84 +4889,84 @@
         <v>221</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
+        <v>365</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>366</v>
+      </c>
+      <c r="C13" s="25" t="s">
         <v>358</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="D13" s="27" t="s">
         <v>359</v>
       </c>
-      <c r="C13" s="25" t="s">
-        <v>351</v>
-      </c>
-      <c r="D13" s="27" t="s">
-        <v>352</v>
-      </c>
       <c r="E13" s="27" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4893,213 +4974,213 @@
         <v>227</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
+        <v>401</v>
+      </c>
+      <c r="B24" s="27" t="s">
         <v>394</v>
       </c>
-      <c r="B24" s="27" t="s">
-        <v>387</v>
-      </c>
       <c r="C24" s="25" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D25" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5150,330 +5231,330 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="B4" s="40">
         <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="B5" s="40">
         <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="B6" s="40">
         <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="B8" s="40">
         <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="B9" s="40">
         <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="B14" s="40">
         <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B16" s="40">
         <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="B20" s="40">
         <v>2</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="B21" s="40">
         <v>2</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="B22" s="40">
         <v>7</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="B24" s="43">
         <f>B6/B5</f>
         <v>0.7990919409761634</v>
       </c>
       <c r="C24" s="44" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="B25" s="45">
         <f>B5-B6</f>
         <v>177</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -5481,97 +5562,97 @@
         <v>155</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C34" s="47" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="D34" s="47" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="C35" s="47" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="D35" s="47" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
     </row>
   </sheetData>
@@ -5594,24 +5675,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5619,16 +5700,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5636,16 +5717,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5653,16 +5734,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5670,16 +5751,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5687,16 +5768,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: thêm « Thách đấu theo chủ đề từ vựng / ngữ pháp » (Vivoire không có)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="514">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -996,6 +996,21 @@
   </si>
   <si>
     <t>migration 118, 122, 124; AvatarMenu.jsx (RPC toi_la_vip)</t>
+  </si>
+  <si>
+    <t>Thách đấu theo chủ đề từ vựng / ngữ pháp</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ (chủ dự án xác nhận 10/10; Vivoire chỉ có đấu dịch thuật)</t>
+  </si>
+  <si>
+    <t>Chọn 1 trong 7 chủ đề (3 từ vựng, 4 ngữ pháp và diễn đạt); máy chủ gộp thẻ mọi bộ cùng chủ đề, rút ngẫu nhiên 10 câu, phương án cùng dạng; giáo viên xếp bộ vào chủ đề và soạn nghĩa sai</t>
+  </si>
+  <si>
+    <t>Đang chạy — chưa có trận theo chủ đề nào chơi thật</t>
+  </si>
+  <si>
+    <t>migration 127–129; tao_thach_dau_chu_de</t>
   </si>
   <si>
     <t>Linh vật đồng hành</t>
@@ -2233,19 +2248,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A7)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
@@ -2262,19 +2277,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A8)</f>
         <v>7</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A8)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F8" s="6">
@@ -2291,19 +2306,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A9)</f>
         <v>8</v>
       </c>
       <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A9)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>0.8</v>
       </c>
       <c r="F9" s="6">
@@ -2320,24 +2335,24 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A10)</f>
-        <v>14</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A10)</f>
+        <v>15</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
-        <v>9</v>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A10)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
+        <v>10</v>
       </c>
       <c r="D10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
-        <v>1.3333333333333333</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A10)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A10)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <v>1.2</v>
       </c>
       <c r="E10" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A10)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A10)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A10)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F10" s="6">
         <f>IFERROR(E10-D10,"")</f>
-        <v>0.6666666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="G10" s="7" t="str">
         <f>IF(OR(C10&lt;3,F10=""),"quá ít mục",IF(F10&gt;0.25,"FRACILE",IF(F10&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2349,19 +2364,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A11)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A11)</f>
         <v>15</v>
       </c>
       <c r="C11" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A11)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A11)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A11)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E11" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A11)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A11)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A11)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>1</v>
       </c>
       <c r="F11" s="6">
@@ -2378,19 +2393,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A12)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A12)</f>
         <v>6</v>
       </c>
       <c r="C12" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A12)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A12)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A12)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E12" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A12)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A12)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A12)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F12" s="6">
@@ -2407,19 +2422,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$65,$A13)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A13)</f>
         <v>6</v>
       </c>
       <c r="C13" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A13)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A13)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A13)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>1.8</v>
       </c>
       <c r="E13" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$65=$A13)*('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A13)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A13)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
         <v>1.4</v>
       </c>
       <c r="F13" s="6">
@@ -2437,27 +2452,27 @@
       </c>
       <c r="B14" s="9">
         <f>SUM(B7:B13)</f>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(C7:C13)</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$65)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
-        <v>1.7222222222222223</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <v>1.6756756756756757</v>
       </c>
       <c r="E14" s="10">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$65)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$65&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$65&lt;&gt;"")),"")</f>
-        <v>1.4166666666666667</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <v>1.4324324324324325</v>
       </c>
       <c r="F14" s="10">
         <f>E14-D14</f>
-        <v>-0.3055555555555556</v>
+        <v>-0.2432432432432432</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(F14&gt;0.25,"FRACILE",IF(F14&lt;-0.25,"Vivoire","ngang nhau"))</f>
-        <v>Vivoire</v>
+        <v>ngang nhau</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -2869,7 +2884,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4710,10 +4725,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H63" s="25" t="s">
-        <v>88</v>
+        <v>322</v>
       </c>
       <c r="I63" s="30" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="64" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4721,16 +4736,16 @@
         <v>14</v>
       </c>
       <c r="B64" s="26" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C64" s="27" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D64" s="28">
         <v>0</v>
       </c>
       <c r="E64" s="27" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="F64" s="28">
         <v>2</v>
@@ -4740,10 +4755,10 @@
         <v>FRACILE</v>
       </c>
       <c r="H64" s="25" t="s">
-        <v>325</v>
+        <v>88</v>
       </c>
       <c r="I64" s="30" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="65" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -4751,16 +4766,16 @@
         <v>14</v>
       </c>
       <c r="B65" s="26" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C65" s="27" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D65" s="28">
         <v>0</v>
       </c>
       <c r="E65" s="27" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F65" s="28">
         <v>2</v>
@@ -4770,10 +4785,40 @@
         <v>FRACILE</v>
       </c>
       <c r="H65" s="25" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I65" s="30" t="s">
-        <v>330</v>
+        <v>331</v>
+      </c>
+    </row>
+    <row r="66" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B66" s="26" t="s">
+        <v>332</v>
+      </c>
+      <c r="C66" s="27" t="s">
+        <v>325</v>
+      </c>
+      <c r="D66" s="28">
+        <v>0</v>
+      </c>
+      <c r="E66" s="27" t="s">
+        <v>333</v>
+      </c>
+      <c r="F66" s="28">
+        <v>2</v>
+      </c>
+      <c r="G66" s="29" t="str">
+        <f>IF(OR(D66="",F66=""),"chưa rõ",IF(F66&gt;D66,"FRACILE",IF(D66&gt;F66,"Vivoire","hoà")))</f>
+        <v>FRACILE</v>
+      </c>
+      <c r="H66" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="I66" s="30" t="s">
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4797,12 +4842,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4818,70 +4863,70 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4889,84 +4934,84 @@
         <v>221</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>88</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4974,213 +5019,213 @@
         <v>227</v>
       </c>
       <c r="B14" s="27" t="s">
+        <v>373</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>345</v>
+      </c>
+      <c r="D14" s="27" t="s">
         <v>368</v>
       </c>
-      <c r="C14" s="25" t="s">
-        <v>340</v>
-      </c>
-      <c r="D14" s="27" t="s">
-        <v>363</v>
-      </c>
       <c r="E14" s="27" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="D25" s="27" t="s">
         <v>88</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5231,330 +5276,330 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="B4" s="40">
         <v>110</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="B5" s="40">
         <v>881</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B6" s="40">
         <v>704</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="B7" s="40">
         <v>22</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="B8" s="40">
         <v>7</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B9" s="40">
         <v>56</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="D9" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="B10" s="40">
         <v>12</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="B11" s="40">
         <v>131</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="B12" s="40">
         <v>18</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="B13" s="40">
         <v>57</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="39" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="B14" s="40">
         <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="39" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="B16" s="40">
         <v>4</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="39" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="B17" s="40">
         <v>8</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="39" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="B19" s="40">
         <v>1</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="B20" s="40">
         <v>2</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="B21" s="40">
         <v>2</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="39" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="B22" s="40">
         <v>7</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="B24" s="43">
         <f>B6/B5</f>
         <v>0.7990919409761634</v>
       </c>
       <c r="C24" s="44" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="B25" s="45">
         <f>B5-B6</f>
         <v>177</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -5562,97 +5607,97 @@
         <v>155</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
+        <v>475</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>476</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>473</v>
+      </c>
+      <c r="D33" s="21" t="s">
         <v>470</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>471</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>468</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="C34" s="47" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="D34" s="47" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="C35" s="47" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="D35" s="47" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
     </row>
   </sheetData>
@@ -5675,24 +5720,24 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5700,16 +5745,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5717,16 +5762,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5734,16 +5779,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5751,16 +5796,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5768,16 +5813,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bảng so sánh: đối chiếu lại vivoire.app 10/10 (thi thử A1–B2, 400 bài phát âm, miễn phí, đánh giá 4,9/5), thêm 5 dòng: Bộ Flashcard trả phí, Bài luyện phát âm có AI, Chép chính tả, Bài học ngữ pháp công khai, Đánh giá trên kho ứng dụng
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="535">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -410,7 +410,7 @@
     <t>Đề thi thử đúng cấu trúc DELF</t>
   </si>
   <si>
-    <t>DELF/DALF A1–C2</t>
+    <t>Đề thi thử DELF A1–B2 « đúng cấu trúc » (FAQ 10/10); viết có AI chấm, nói luyện riêng qua bài phát âm. Không thấy DALF C1/C2</t>
   </si>
   <si>
     <t>7 đề đã phát hành (A1 · A2 ×2 · B1 ×2 · B2 · C1), đủ 4 phần. Màn chọn đề và màn kết quả làm lại 09/10 (thẻ trình độ, cấu trúc 4 phần có biểu tượng, vòng điểm, vạch ngưỡng 5/25), âm thanh nhắc còn 5 phút / 1 phút / hết giờ. Sửa lỗi đổi tab hiện « chưa có bài »</t>
@@ -470,7 +470,7 @@
     <t>Dải cấp độ</t>
   </si>
   <si>
-    <t>A1 → C2 (6 cấp) + ôn thi cấp 3</t>
+    <t>A1 → C2 (6 cấp) cho luyện kỹ năng + ôn thi cấp 3; thi thử chỉ A1–B2</t>
   </si>
   <si>
     <t>Nhận A1 → C1. Bài đã xuất bản (06/10): A1 9 · A2 6 · B1 24 · B2 5 · B2+ 4 · C1 0. Nháp chờ duyệt có đủ mọi cấp (A1 2 · A2 6 · B1 5 · B2 6 · B2+ 3 · C1 4) — xuất bản xong thì mọi cấp đều có bài</t>
@@ -485,7 +485,7 @@
     <t>Số bài luyện</t>
   </si>
   <si>
-    <t>200 chép chính tả + 200 nghe điền từ (họ công bố)</t>
+    <t>200 chép chính tả + 200 nghe điền từ + 400 bài luyện phát âm (công bố 10/10)</t>
   </si>
   <si>
     <t>110 bài, TẤT CẢ đã xuất bản (08/10): 90 bài luyện tập riêng + 20 bài thuộc đề thi thử, A1 → C1, trong đó các bài nghe giọng tổng hợp và 3 bài cắt từ Wikipédia parlée</t>
@@ -881,6 +881,9 @@
     <t>Thanh toán</t>
   </si>
   <si>
+    <t>Không có — FAQ 10/10: « mọi tính năng học đều miễn phí »; có trang « Ủng hộ »</t>
+  </si>
+  <si>
     <t>Webhook SePay đã ghim công thức ký; mua bài lẻ, gói VIP và (từ 10/10) bộ Flashcard trả phí qua cùng một mã nội dung chuyển khoản</t>
   </si>
   <si>
@@ -932,7 +935,7 @@
     <t>Số liệu trên trang bán hàng</t>
   </si>
   <si>
-    <t>« 56.000+ từ », « 200+200 bài » — không nói nguồn</t>
+    <t>« 56.000+ từ », « 400 bài phát âm », « 200+200 bài », 4,9/5 (32 lượt App Store, 12 lượt Google Play) — số đánh giá có nguồn, số bài không nói nguồn</t>
   </si>
   <si>
     <t>ĐẾM THẬT từ máy chủ lúc tải trang; hỏng thì hiện dấu gạch chứ không hiện 0</t>
@@ -996,6 +999,66 @@
   </si>
   <si>
     <t>migration 118, 122, 124; AvatarMenu.jsx (RPC toi_la_vip)</t>
+  </si>
+  <si>
+    <t>Bài luyện phát âm có AI chấm</t>
+  </si>
+  <si>
+    <t>400 bài, AI chấm phát âm và trôi chảy (công bố 10/10)</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ bài luyện phát âm riêng. Bài nói ghi âm được AI nhận xét qua bản chép lời, không chấm phát âm</t>
+  </si>
+  <si>
+    <t>Chưa có</t>
+  </si>
+  <si>
+    <t>nhan-xet-noi chỉ nhận xét nội dung, không đo phát âm</t>
+  </si>
+  <si>
+    <t>Chép chính tả / nghe điền từ</t>
+  </si>
+  <si>
+    <t>200 + 200 bài, audio bản xứ</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ dạng chép chính tả. Có câu điền từ trong bài nghe nhưng không phải bài chép chính tả</t>
+  </si>
+  <si>
+    <t>Bài học ngữ pháp công khai</t>
+  </si>
+  <si>
+    <t>Có trang « Ngữ pháp tiếng Pháp », đọc không cần đăng nhập (FAQ 10/10)</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ trang bài học ngữ pháp. Ngữ pháp nằm trong lời giải và mục « Giải thích » của từng bài</t>
+  </si>
+  <si>
+    <t>Chưa có trang riêng</t>
+  </si>
+  <si>
+    <t>Mục Giải thích: 111/111 bài luyện tập</t>
+  </si>
+  <si>
+    <t>Đánh giá trên kho ứng dụng</t>
+  </si>
+  <si>
+    <t>4,9/5 App Store (32 lượt) · 4,9/5 Google Play (12 lượt)</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ — chưa lên App Store / Google Play (chỉ cài được từ web dạng PWA)</t>
+  </si>
+  <si>
+    <t>Bộ Flashcard trả phí</t>
+  </si>
+  <si>
+    <t>KHÔNG CÓ (chủ dự án xác nhận 10/10; mọi tính năng Vivoire miễn phí)</t>
+  </si>
+  <si>
+    <t>Giáo viên đặt bộ trả phí + giá; học sinh mua bằng chuyển khoản (tự mở khoá khi tiền về), VIP mở hết, giáo viên cấp/thu quyền từng học sinh; thẻ khoá ở database</t>
+  </si>
+  <si>
+    <t>migration 128, 130; webhook SePay mã BO&lt;4&gt;</t>
   </si>
   <si>
     <t>Thách đấu theo chủ đề từ vựng / ngữ pháp</t>
@@ -2248,19 +2311,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A7)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$71,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A7)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;""))</f>
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A7)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$71)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A7)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")),"")</f>
         <v>1.6666666666666667</v>
       </c>
       <c r="E7" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A7)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A7)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$71)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A7)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")),"")</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="F7" s="6">
@@ -2277,19 +2340,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A8)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$71,$A8)</f>
         <v>7</v>
       </c>
       <c r="C8" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A8)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;""))</f>
         <v>1</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A8)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$71)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A8)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E8" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A8)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A8)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$71)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A8)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="F8" s="6">
@@ -2306,24 +2369,24 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A9)</f>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$71,$A9)</f>
+        <v>11</v>
+      </c>
+      <c r="C9" s="5">
+        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A9)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;""))</f>
         <v>8</v>
       </c>
-      <c r="C9" s="5">
-        <f>SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;""))</f>
-        <v>5</v>
-      </c>
       <c r="D9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A9)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")*'So sánh chi tiết'!$D$2:$D$71)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A9)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")),"")</f>
         <v>2</v>
       </c>
       <c r="E9" s="6">
-        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$66)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$66=$A9)*('So sánh chi tiết'!$D$2:$D$66&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$66&lt;&gt;"")),"")</f>
-        <v>0.8</v>
+        <f>IFERROR(SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A9)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")*'So sánh chi tiết'!$F$2:$F$71)/SUMPRODUCT(('So sánh chi tiết'!$A$2:$A$71=$A9)*('So sánh chi tiết'!$D$2:$D$71&lt;&gt;"")*('So sánh chi tiết'!$F$2:$F$71&lt;&gt;"")),"")</f>
+        <v>0.625</v>
       </c>
       <c r="F9" s="6">
         <f>IFERROR(E9-D9,"")</f>
-        <v>-1.2</v>
+        <v>-1.375</v>
       </c>
       <c r="G9" s="7" t="str">
         <f>IF(OR(C9&lt;3,F9=""),"quá ít mục",IF(F9&gt;0.25,"FRACILE",IF(F9&lt;-0.25,"Vivoire","ngang nhau")))</f>
@@ -2335,24 +2398,24 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$66,$A10)</f>
-        <v>15</v>
+        <f>COUNTIF('So sánh chi tiết'!$A$2:$A$71,$A10)</f>
+        <v>16</v>
       </c>
       <c r="C10" s="5">
-        <f>SUMPRODUCT(('So sán